<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 12/09/2026 08:11
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -43,7 +43,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -62,17 +62,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E6D9F2"/>
+        <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
+        <fgColor rgb="00E6D9F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -88,7 +93,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -101,6 +106,7 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -466,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O33"/>
+  <dimension ref="A1:O31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -643,47 +649,47 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Áridos</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>06/2026</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Transporte de dos mil metros cúbicos (2.000 m³) de ripio arcilloso destinados al mantenimiento y mejoramiento de caminos de la jurisdicción comunal de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
           <t>14/09/2026</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>016/2026</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de mano de obra, materiales y equipamiento para ejecuc ión de restitución de galibo y repavimentación en Avenida Belgrano y Avenida 1° de Mayo de esta ciudad de chajari</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>02/10/2026</t>
-        </is>
-      </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>02 DE OCTUBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>14 de septiembre de 2026 - Hora: 10:00</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -691,11 +697,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>$ 100.000, 00.- (PESOS CIEN MIL CON 00/100)</t>
-        </is>
-      </c>
+      <c r="K3" s="4" t="inlineStr"/>
       <c r="L3" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -713,14 +715,14 @@
       </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
-          <t>id-53f1430f94acb0b0</t>
+          <t>id-85e6cfd11c8a8889</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>16/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -728,44 +730,44 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>MINISTERIO DE SALUD</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Licitación Publica</t>
+          <t>LICITACIÓN PÚBLICA</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>17/26</t>
+          <t>76/2026</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Adquirir Una (01) Mesa de Anestesia. Destino: Hospital “San José” de Diamante, dependiente del Ministerio de Salud de la Provincia de Entre Ríos</t>
+          <t>ADQUICION DE CAMIONES COMPACTADORES DE CARGA TRASERA RSU</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>Sala de reuniones de la Dirección de Contrataciones del Minister io de Salud, sito en calle 25 de Mayo N° 181, segundo p</t>
+          <t>14-09-2026 08:00</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr"/>
@@ -781,19 +783,19 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
-          <t>id-3312d89e1a3e2e53</t>
+          <t>id-ccdfae2a7ede4696</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>16/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -801,14 +803,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE CONCEPCIÓN DEL URUGUAY</t>
+          <t>MUNICIPALIDAD DE HERRERA — DPTO. URUGUAY, ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -818,22 +820,22 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>31/2026</t>
+          <t>01-2026</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>“Pavimento Rígido – 03 (tres) Cuadras Barrio San Felipe”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>Adquisición de vehículo 0 km destinado al traslado de personas tipo van, con capacidad para 11 plazas (1 conductor + 10 pasajeros), motorización a nafta/diesel, según pliego de especificaciones técnicas</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>07 de octubre de 2026 Hora: 10:00</t>
+          <t>DE LAS OFERTAS: el día 15/09/2026, a las 11:00 hs. en el Edificio Municipal de Herrera, sito en Av. H. Bozzolo, Nº 165,</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -841,7 +843,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr"/>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L5" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -859,7 +865,7 @@
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>id-76d9566cb30a6df5</t>
+          <t>id-28313c7a9524d0ee</t>
         </is>
       </c>
     </row>
@@ -874,39 +880,39 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>76/2026</t>
+          <t>014/2026</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>ADQUICION DE CAMIONES COMPACTADORES DE CARGA TRASERA RSU</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de materiales – 500 (quinientos) m3 de Hormigón elaborado Tipo H30, Reglamento CIRSOC 201, para ser utilizados en la obra de construcción de pavimento en c alle Moreno entre Av. 1° de Mayo y Guarumba de nuestra ciudad</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>14-09-2026 08:00</t>
+          <t>15 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -914,7 +920,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr"/>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>$ 82.500,00. - (PESOS OCHENTA Y DOS MIL QUINIENTOS CON 00/100)</t>
+        </is>
+      </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -927,12 +937,12 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>id-ccdfae2a7ede4696</t>
+          <t>id-9e58cc9ec0b69356</t>
         </is>
       </c>
     </row>
@@ -947,14 +957,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCIÓN DEL URUGUAY</t>
+          <t>MINISTERIO DE PLANEAMIENTO E INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -964,22 +974,22 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>27/2026</t>
+          <t>08/26</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>“Adquisición de seiscientas (600) Luminarias Leds para Alumbrado Público”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás docum entación</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “NUEVA INSTALACION ELECTRICA, CUBIERTA DE TECHO Y REFACCION DE BAÑOS ESCUELA Nº 1 “JOSE MARIA TEXIER” -SAN SALVADOR-DEPARTAMENTO SAN SALVADOR.”</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>16/09/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>16 de septiembre de 2026 - Hora: 10:00</t>
+          <t>DE LAS OFERTAS: el día 15 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -987,7 +997,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr"/>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>$ 100 (Cien)</t>
+        </is>
+      </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1005,7 +1019,7 @@
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>id-608017f47f903d65</t>
+          <t>id-fb80c8ade7a8651d</t>
         </is>
       </c>
     </row>
@@ -1020,14 +1034,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>GOBIERNO DE ENTRE RÍOS — UNIDAD CENTRAL DE CONTRATACIONES</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1037,22 +1051,22 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>06/26</t>
+          <t>08/2026</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Adquirir materiales de construcción (chapas, rollos de film de polietileno, tirantes, clavos y clavadoras)</t>
+          <t>Nueva instalación eléctrica, cubierta de techo y refacción de baños Escuela N° 1 "José María Texier", San Salvador</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Unidad Central de Contrataciones, el día 17/09/26 a las 09:00 horas</t>
+          <t>martes, 15 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -1060,11 +1074,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr">
-        <is>
-          <t>PESOS CINCUENTA MIL ($ 50.000)</t>
-        </is>
-      </c>
+      <c r="K8" s="4" t="inlineStr"/>
       <c r="L8" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1077,12 +1087,12 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>id-9dbdaa6090d92bd4</t>
+          <t>id-952aef4c115d8f12</t>
         </is>
       </c>
     </row>
@@ -1099,12 +1109,12 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Materiales</t>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE SEGUÍ</t>
+          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCIÓN DEL URUGUAY</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1114,22 +1124,22 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>27/2026</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Us os Múltiples – Gimnasio Municipal”</t>
+          <t>“Adquisición de seiscientas (600) Luminarias Leds para Alumbrado Público”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás docum entación</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>16/09/2026</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026 a las 10:00 hs, en el Edificio Municipal</t>
+          <t>16 de septiembre de 2026 - Hora: 10:00</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1137,11 +1147,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>Gratuito</t>
-        </is>
-      </c>
+      <c r="K9" s="4" t="inlineStr"/>
       <c r="L9" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1159,7 +1165,7 @@
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>id-90c3d1f38f49418a</t>
+          <t>id-608017f47f903d65</t>
         </is>
       </c>
     </row>
@@ -1174,14 +1180,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
+          <t>GOBIERNO DE ENTRE RÍOS — UNIDAD CENTRAL DE CONTRATACIONES</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1191,22 +1197,22 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>015/2026</t>
+          <t>06/26</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
+          <t>Adquirir materiales de construcción (chapas, rollos de film de polietileno, tirantes, clavos y clavadoras)</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>Unidad Central de Contrataciones, el día 17/09/26 a las 09:00 horas</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1216,7 +1222,7 @@
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>$ 90.000,00. - (PESOS NOVENTA MIL CON 00/100)</t>
+          <t>PESOS CINCUENTA MIL ($ 50.000)</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr">
@@ -1236,7 +1242,7 @@
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>id-74dfdad7e5f9d048</t>
+          <t>id-9dbdaa6090d92bd4</t>
         </is>
       </c>
     </row>
@@ -1251,14 +1257,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>MUNICIPALIDAD DE SEGUÍ</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1268,22 +1274,22 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>09/26</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “AMPLIACION - RECONSTRUCCION DE PISOS Y CONTRAPISOS -IMPERMEABILIZACION LOSAS- INSTALACION ELECTRICA-ESCUELA SECUNDARIA ADULTOS Nº 1 “DR. LUIS AGOTE” -NOGOYA-DEPARTAMENTO NOGOYA.”</t>
+          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Us os Múltiples – Gimnasio Municipal”</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 18 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>17/09/2026 a las 10:00 hs, en el Edificio Municipal</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1293,7 +1299,7 @@
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>$ 100 (Cien)</t>
+          <t>Gratuito</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
@@ -1313,7 +1319,7 @@
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>id-6a4a84712fd41a03</t>
+          <t>id-90c3d1f38f49418a</t>
         </is>
       </c>
     </row>
@@ -1328,14 +1334,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1345,12 +1351,12 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>015/2026</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -1360,7 +1366,7 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
+          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
@@ -1368,7 +1374,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr"/>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>$ 90.000,00. - (PESOS NOVENTA MIL CON 00/100)</t>
+        </is>
+      </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1381,12 +1391,12 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>id-885d4847519dfd48</t>
+          <t>id-74dfdad7e5f9d048</t>
         </is>
       </c>
     </row>
@@ -1408,7 +1418,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1418,22 +1428,22 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>07/2026</t>
+          <t>09/26</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “AMPLIACION - RECONSTRUCCION DE PISOS Y CONTRAPISOS -IMPERMEABILIZACION LOSAS- INSTALACION ELECTRICA-ESCUELA SECUNDARIA ADULTOS Nº 1 “DR. LUIS AGOTE” -NOGOYA-DEPARTAMENTO NOGOYA.”</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>21/09/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>21/09/2026 HORA: 10:00 HS</t>
+          <t>DE LAS OFERTAS: el día 18 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -1443,7 +1453,7 @@
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>SIN COSTO</t>
+          <t>$ 100 (Cien)</t>
         </is>
       </c>
       <c r="L13" s="6" t="inlineStr">
@@ -1463,7 +1473,7 @@
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>id-6ddfa0f2f1aa296d</t>
+          <t>id-6a4a84712fd41a03</t>
         </is>
       </c>
     </row>
@@ -1478,14 +1488,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>COLON — MUNICIPALIDAD DE COLON</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1493,20 +1503,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr"/>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>09/2026</t>
+        </is>
+      </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
+          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>24 de SEPTIEMBRE de 2026</t>
+          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1514,11 +1528,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K14" s="4" t="inlineStr">
-        <is>
-          <t>Sin Cargo</t>
-        </is>
-      </c>
+      <c r="K14" s="4" t="inlineStr"/>
       <c r="L14" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1531,12 +1541,12 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>id-bc610b64999d147d</t>
+          <t>id-885d4847519dfd48</t>
         </is>
       </c>
     </row>
@@ -1558,7 +1568,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1568,30 +1578,34 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>07/2026</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>21/09/2026</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIU</t>
+          <t>21/09/2026 HORA: 10:00 HS</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="K15" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L15" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1609,7 +1623,7 @@
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>id-d97b43a99f1e1824</t>
+          <t>id-6ddfa0f2f1aa296d</t>
         </is>
       </c>
     </row>
@@ -1624,14 +1638,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>COLON — MUNICIPALIDAD DE COLON</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1639,14 +1653,10 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>09/2026</t>
-        </is>
-      </c>
+      <c r="F16" s="4" t="inlineStr"/>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
@@ -1656,15 +1666,19 @@
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CI</t>
+          <t>24 de SEPTIEMBRE de 2026</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="K16" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>Sin Cargo</t>
+        </is>
+      </c>
       <c r="L16" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1677,19 +1691,19 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos + CAFESG (Salto Grande)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>id-f8fab7a7b3a06a2d</t>
+          <t>id-bc610b64999d147d</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1697,14 +1711,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE CRESPO -- ENTRE RÍOS</t>
+          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1714,27 +1728,27 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>05/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 145 metros lineales de modulo canal premoldeado cajón tipo pórtico de 2,00 X 1,00 (interior) X 1,00 mts. de longitud de hormigón para canalizar calle Los Quechuas al final</t>
+          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>28 de septiembre de 2026 10:00 Hs. Lugar: Sección Suministros, Palacio Municipal sito en 25 de mayo Nº 943, C</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIU</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="K17" s="4" t="inlineStr"/>
@@ -1755,7 +1769,7 @@
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>id-61e8747a99305fe9</t>
+          <t>id-d97b43a99f1e1824</t>
         </is>
       </c>
     </row>
@@ -1770,51 +1784,47 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Municipalidad de Crespo</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>5/2026</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 145 metros lineales de módulo canal premoldeado.</t>
+          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>28/9/2026 – 10:00 horas</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CI</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
-        </is>
-      </c>
-      <c r="K18" s="4" t="inlineStr">
-        <is>
-          <t>$25.000,00</t>
-        </is>
-      </c>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1827,12 +1837,12 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Municipalidad de Crespo</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>id-1609ce58e128c413</t>
+          <t>id-f8fab7a7b3a06a2d</t>
         </is>
       </c>
     </row>
@@ -1847,49 +1857,49 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>Municipalidad de Crespo</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>08/2026</t>
+          <t>5/2026</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCL UIDO</t>
+          <t>Adquisición de 145 metros lineales de módulo canal premoldeado.</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>29/09/2026</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>29/09/2026</t>
+          <t>28/9/2026 – 10:00 horas</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>SIN COSTO</t>
+          <t>$25.000,00</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr">
@@ -1904,12 +1914,12 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Crespo</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>id-1590925c21c7e363</t>
+          <t>id-1609ce58e128c413</t>
         </is>
       </c>
     </row>
@@ -1924,14 +1934,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1941,22 +1951,22 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>10/26</t>
+          <t>08/2026</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
+          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCL UIDO</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1966,7 +1976,7 @@
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>$ 100 (Cien)</t>
+          <t>SIN COSTO</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
@@ -1986,7 +1996,7 @@
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>id-75a5c9dd5b4aa6f3</t>
+          <t>id-1590925c21c7e363</t>
         </is>
       </c>
     </row>
@@ -2008,7 +2018,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2018,12 +2028,12 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>10/26</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -2033,7 +2043,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
+          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -2041,7 +2051,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K21" s="4" t="inlineStr"/>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>$ 100 (Cien)</t>
+        </is>
+      </c>
       <c r="L21" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2054,12 +2068,12 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-46c6d9f1f9210d1e</t>
+          <t>id-75a5c9dd5b4aa6f3</t>
         </is>
       </c>
     </row>
@@ -2069,9 +2083,9 @@
           <t>11/09/2026</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
@@ -2081,7 +2095,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2091,18 +2105,22 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>001-2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr"/>
+          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
+          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -2110,11 +2128,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K22" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K22" s="4" t="inlineStr"/>
       <c r="L22" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2127,12 +2141,12 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-b7b0120caf49d551</t>
+          <t>id-46c6d9f1f9210d1e</t>
         </is>
       </c>
     </row>
@@ -2147,14 +2161,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE URDINARRAIN</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2164,18 +2178,18 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>001-2026</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
+          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr"/>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2183,7 +2197,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K23" s="4" t="inlineStr"/>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L23" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2201,7 +2219,7 @@
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-7a200161bcc9b02b</t>
+          <t>id-b7b0120caf49d551</t>
         </is>
       </c>
     </row>
@@ -2216,14 +2234,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
+          <t>MUNICIPALIDAD DE URDINARRAIN</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2233,12 +2251,12 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
+          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr"/>
@@ -2270,7 +2288,7 @@
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-511256e6329e386a</t>
+          <t>id-7a200161bcc9b02b</t>
         </is>
       </c>
     </row>
@@ -2285,14 +2303,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2302,18 +2320,18 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr"/>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2321,11 +2339,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K25" s="4" t="inlineStr">
-        <is>
-          <t>$ 120.976,01</t>
-        </is>
-      </c>
+      <c r="K25" s="4" t="inlineStr"/>
       <c r="L25" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2338,12 +2352,12 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-07ddb93a12c5a870</t>
+          <t>id-511256e6329e386a</t>
         </is>
       </c>
     </row>
@@ -2358,7 +2372,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
+      <c r="C26" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2380,13 +2394,13 @@
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Concurso de Precio N° 02/2025</t>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
+          <t>Publicada 06/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2394,7 +2408,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K26" s="4" t="inlineStr"/>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>$ 120.976,01</t>
+        </is>
+      </c>
       <c r="L26" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2412,14 +2430,14 @@
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-7c1bf02160a66f67</t>
+          <t>id-07ddb93a12c5a870</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2429,29 +2447,33 @@
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>Materiales</t>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>02/2025</t>
+        </is>
+      </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
+          <t>Concurso de Precio N° 02/2025</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 19/06/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2472,12 +2494,12 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-654eebef400f89cd</t>
+          <t>id-7c1bf02160a66f67</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2514,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr">
+      <c r="C28" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2561,7 +2583,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C29" s="8" t="inlineStr">
+      <c r="C29" s="10" t="inlineStr">
         <is>
           <t>Materiales</t>
         </is>
@@ -2757,146 +2779,8 @@
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>14/09/2026</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C32" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Poder Judicial de Entre Ríos</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Solicitud de Cotización</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>232/26</t>
-        </is>
-      </c>
-      <c r="G32" s="5" t="inlineStr">
-        <is>
-          <t>SERVICIO DE REACONDICIONAMIENTO Y REPARACIÓN EN SECTOR POSTERIOR DEL INMUEBLE ALQUILADO DEL JUZGADO DE PAZ DE SAN JAIME DE LA FRONTERA</t>
-        </is>
-      </c>
-      <c r="H32" s="4" t="inlineStr"/>
-      <c r="I32" s="4" t="inlineStr">
-        <is>
-          <t>Ver el sitio</t>
-        </is>
-      </c>
-      <c r="J32" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K32" s="4" t="inlineStr"/>
-      <c r="L32" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M32" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>Poder Judicial de Entre Ríos</t>
-        </is>
-      </c>
-      <c r="O32" s="4" t="inlineStr">
-        <is>
-          <t>id-5a01c3fd726f10dc</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>14/09/2026</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C33" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Poder Judicial de Entre Ríos</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Solicitud de Cotización</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>228/26</t>
-        </is>
-      </c>
-      <c r="G33" s="5" t="inlineStr">
-        <is>
-          <t>Solicitud de Cotización Nº 228/26, porContratación del servicio de recarga, revisión, prueba hidráulica y mantenimiento de los matafuegos ubicados en los Edificios de calle San Martín Nº15, Mitre Nº581 y Sarmiento Nº356 de la localidad de Victoria</t>
-        </is>
-      </c>
-      <c r="H33" s="4" t="inlineStr"/>
-      <c r="I33" s="4" t="inlineStr">
-        <is>
-          <t>Ver el sitio</t>
-        </is>
-      </c>
-      <c r="J33" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K33" s="4" t="inlineStr"/>
-      <c r="L33" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M33" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>Poder Judicial de Entre Ríos</t>
-        </is>
-      </c>
-      <c r="O33" s="4" t="inlineStr">
-        <is>
-          <t>id-e125fe54abc33d69</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:O33"/>
+  <autoFilter ref="A1:O31"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -2958,10 +2842,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId64"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 14/09/2026 08:01
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O31"/>
+  <dimension ref="A1:O41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -737,32 +737,32 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>MUNICIPALIDAD DE HERRERA — DPTO. URUGUAY, ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>76/2026</t>
+          <t>01-2026</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>ADQUICION DE CAMIONES COMPACTADORES DE CARGA TRASERA RSU</t>
+          <t>Adquisición de vehículo 0 km destinado al traslado de personas tipo van, con capacidad para 11 plazas (1 conductor + 10 pasajeros), motorización a nafta/diesel, según pliego de especificaciones técnicas</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>14-09-2026 08:00</t>
+          <t>DE LAS OFERTAS: el día 15/09/2026, a las 11:00 hs. en el Edificio Municipal de Herrera, sito en Av. H. Bozzolo, Nº 165,</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -770,7 +770,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr"/>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L4" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -783,12 +787,12 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
-          <t>id-ccdfae2a7ede4696</t>
+          <t>id-28313c7a9524d0ee</t>
         </is>
       </c>
     </row>
@@ -803,14 +807,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE HERRERA — DPTO. URUGUAY, ENTRE RÍOS</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -820,12 +824,12 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>01-2026</t>
+          <t>014/2026</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de vehículo 0 km destinado al traslado de personas tipo van, con capacidad para 11 plazas (1 conductor + 10 pasajeros), motorización a nafta/diesel, según pliego de especificaciones técnicas</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de materiales – 500 (quinientos) m3 de Hormigón elaborado Tipo H30, Reglamento CIRSOC 201, para ser utilizados en la obra de construcción de pavimento en c alle Moreno entre Av. 1° de Mayo y Guarumba de nuestra ciudad</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -835,7 +839,7 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 15/09/2026, a las 11:00 hs. en el Edificio Municipal de Herrera, sito en Av. H. Bozzolo, Nº 165,</t>
+          <t>15 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -845,7 +849,7 @@
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>SIN COSTO</t>
+          <t>$ 82.500,00. - (PESOS OCHENTA Y DOS MIL QUINIENTOS CON 00/100)</t>
         </is>
       </c>
       <c r="L5" s="6" t="inlineStr">
@@ -865,7 +869,7 @@
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>id-28313c7a9524d0ee</t>
+          <t>id-9e58cc9ec0b69356</t>
         </is>
       </c>
     </row>
@@ -880,14 +884,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
+          <t>MINISTERIO DE PLANEAMIENTO E INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -897,12 +901,12 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>014/2026</t>
+          <t>08/26</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de materiales – 500 (quinientos) m3 de Hormigón elaborado Tipo H30, Reglamento CIRSOC 201, para ser utilizados en la obra de construcción de pavimento en c alle Moreno entre Av. 1° de Mayo y Guarumba de nuestra ciudad</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “NUEVA INSTALACION ELECTRICA, CUBIERTA DE TECHO Y REFACCION DE BAÑOS ESCUELA Nº 1 “JOSE MARIA TEXIER” -SAN SALVADOR-DEPARTAMENTO SAN SALVADOR.”</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -912,7 +916,7 @@
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>15 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>DE LAS OFERTAS: el día 15 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -922,7 +926,7 @@
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>$ 82.500,00. - (PESOS OCHENTA Y DOS MIL QUINIENTOS CON 00/100)</t>
+          <t>$ 100 (Cien)</t>
         </is>
       </c>
       <c r="L6" s="6" t="inlineStr">
@@ -942,7 +946,7 @@
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>id-9e58cc9ec0b69356</t>
+          <t>id-fb80c8ade7a8651d</t>
         </is>
       </c>
     </row>
@@ -964,7 +968,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>MINISTERIO DE PLANEAMIENTO E INFRAESTRUCTURA</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -974,12 +978,12 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>08/26</t>
+          <t>08/2026</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “NUEVA INSTALACION ELECTRICA, CUBIERTA DE TECHO Y REFACCION DE BAÑOS ESCUELA Nº 1 “JOSE MARIA TEXIER” -SAN SALVADOR-DEPARTAMENTO SAN SALVADOR.”</t>
+          <t>Nueva instalación eléctrica, cubierta de techo y refacción de baños Escuela N° 1 "José María Texier", San Salvador</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -989,7 +993,7 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 15 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>martes, 15 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -997,11 +1001,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr">
-        <is>
-          <t>$ 100 (Cien)</t>
-        </is>
-      </c>
+      <c r="K7" s="4" t="inlineStr"/>
       <c r="L7" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1014,12 +1014,12 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>id-fb80c8ade7a8651d</t>
+          <t>id-952aef4c115d8f12</t>
         </is>
       </c>
     </row>
@@ -1034,14 +1034,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCIÓN DEL URUGUAY</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1051,22 +1051,22 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>08/2026</t>
+          <t>27/2026</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Nueva instalación eléctrica, cubierta de techo y refacción de baños Escuela N° 1 "José María Texier", San Salvador</t>
+          <t>“Adquisición de seiscientas (600) Luminarias Leds para Alumbrado Público”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás docum entación</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
+          <t>16/09/2026</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>martes, 15 de septiembre de 2026 - 10:00hs</t>
+          <t>16 de septiembre de 2026 - Hora: 10:00</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -1087,12 +1087,12 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>id-952aef4c115d8f12</t>
+          <t>id-608017f47f903d65</t>
         </is>
       </c>
     </row>
@@ -1107,14 +1107,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCIÓN DEL URUGUAY</t>
+          <t>GOBIERNO DE ENTRE RÍOS — UNIDAD CENTRAL DE CONTRATACIONES</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1124,22 +1124,22 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>27/2026</t>
+          <t>06/26</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>“Adquisición de seiscientas (600) Luminarias Leds para Alumbrado Público”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás docum entación</t>
+          <t>Adquirir materiales de construcción (chapas, rollos de film de polietileno, tirantes, clavos y clavadoras)</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>16/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>16 de septiembre de 2026 - Hora: 10:00</t>
+          <t>Unidad Central de Contrataciones, el día 17/09/26 a las 09:00 horas</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1147,7 +1147,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr"/>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>PESOS CINCUENTA MIL ($ 50.000)</t>
+        </is>
+      </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1165,7 +1169,7 @@
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>id-608017f47f903d65</t>
+          <t>id-9dbdaa6090d92bd4</t>
         </is>
       </c>
     </row>
@@ -1187,7 +1191,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>GOBIERNO DE ENTRE RÍOS — UNIDAD CENTRAL DE CONTRATACIONES</t>
+          <t>MUNICIPALIDAD DE SEGUÍ</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1197,12 +1201,12 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>06/26</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Adquirir materiales de construcción (chapas, rollos de film de polietileno, tirantes, clavos y clavadoras)</t>
+          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Us os Múltiples – Gimnasio Municipal”</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -1212,7 +1216,7 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>Unidad Central de Contrataciones, el día 17/09/26 a las 09:00 horas</t>
+          <t>17/09/2026 a las 10:00 hs, en el Edificio Municipal</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1222,7 +1226,7 @@
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>PESOS CINCUENTA MIL ($ 50.000)</t>
+          <t>Gratuito</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr">
@@ -1242,7 +1246,7 @@
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>id-9dbdaa6090d92bd4</t>
+          <t>id-90c3d1f38f49418a</t>
         </is>
       </c>
     </row>
@@ -1257,14 +1261,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE SEGUÍ</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1274,22 +1278,22 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>015/2026</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Us os Múltiples – Gimnasio Municipal”</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026 a las 10:00 hs, en el Edificio Municipal</t>
+          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1299,7 +1303,7 @@
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>Gratuito</t>
+          <t>$ 90.000,00. - (PESOS NOVENTA MIL CON 00/100)</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
@@ -1319,7 +1323,7 @@
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>id-90c3d1f38f49418a</t>
+          <t>id-74dfdad7e5f9d048</t>
         </is>
       </c>
     </row>
@@ -1334,14 +1338,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
+          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1351,12 +1355,12 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>015/2026</t>
+          <t>09/26</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “AMPLIACION - RECONSTRUCCION DE PISOS Y CONTRAPISOS -IMPERMEABILIZACION LOSAS- INSTALACION ELECTRICA-ESCUELA SECUNDARIA ADULTOS Nº 1 “DR. LUIS AGOTE” -NOGOYA-DEPARTAMENTO NOGOYA.”</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -1366,7 +1370,7 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>DE LAS OFERTAS: el día 18 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
@@ -1376,7 +1380,7 @@
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>$ 90.000,00. - (PESOS NOVENTA MIL CON 00/100)</t>
+          <t>$ 100 (Cien)</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
@@ -1396,7 +1400,7 @@
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>id-74dfdad7e5f9d048</t>
+          <t>id-6a4a84712fd41a03</t>
         </is>
       </c>
     </row>
@@ -1418,7 +1422,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1428,12 +1432,12 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>09/26</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “AMPLIACION - RECONSTRUCCION DE PISOS Y CONTRAPISOS -IMPERMEABILIZACION LOSAS- INSTALACION ELECTRICA-ESCUELA SECUNDARIA ADULTOS Nº 1 “DR. LUIS AGOTE” -NOGOYA-DEPARTAMENTO NOGOYA.”</t>
+          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
@@ -1443,7 +1447,7 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 18 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -1451,11 +1455,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K13" s="4" t="inlineStr">
-        <is>
-          <t>$ 100 (Cien)</t>
-        </is>
-      </c>
+      <c r="K13" s="4" t="inlineStr"/>
       <c r="L13" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1468,12 +1468,12 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>id-6a4a84712fd41a03</t>
+          <t>id-885d4847519dfd48</t>
         </is>
       </c>
     </row>
@@ -1495,7 +1495,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1505,22 +1505,22 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>07/2026</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
+          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>21/09/2026</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
+          <t>21/09/2026 HORA: 10:00 HS</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1528,7 +1528,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K14" s="4" t="inlineStr"/>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L14" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1541,12 +1545,12 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>id-885d4847519dfd48</t>
+          <t>id-6ddfa0f2f1aa296d</t>
         </is>
       </c>
     </row>
@@ -1561,14 +1565,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>COLON — MUNICIPALIDAD DE COLON</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1576,24 +1580,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>07/2026</t>
-        </is>
-      </c>
+      <c r="F15" s="4" t="inlineStr"/>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”</t>
+          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>21/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>21/09/2026 HORA: 10:00 HS</t>
+          <t>24 de SEPTIEMBRE de 2026</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>SIN COSTO</t>
+          <t>Sin Cargo</t>
         </is>
       </c>
       <c r="L15" s="6" t="inlineStr">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>id-6ddfa0f2f1aa296d</t>
+          <t>id-bc610b64999d147d</t>
         </is>
       </c>
     </row>
@@ -1638,14 +1638,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>COLON — MUNICIPALIDAD DE COLON</t>
+          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1653,10 +1653,14 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr"/>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>10/2026</t>
+        </is>
+      </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
+          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
@@ -1666,19 +1670,15 @@
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>24 de SEPTIEMBRE de 2026</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIU</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K16" s="4" t="inlineStr">
-        <is>
-          <t>Sin Cargo</t>
-        </is>
-      </c>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>id-bc610b64999d147d</t>
+          <t>id-d97b43a99f1e1824</t>
         </is>
       </c>
     </row>
@@ -1718,7 +1718,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1728,12 +1728,12 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -1743,7 +1743,7 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIU</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CI</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1764,12 +1764,12 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Boletín Oficial de Entre Ríos + CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>id-d97b43a99f1e1824</t>
+          <t>id-f8fab7a7b3a06a2d</t>
         </is>
       </c>
     </row>
@@ -1784,47 +1784,51 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>Municipalidad de Crespo</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>5/2026</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>Adquisición de 145 metros lineales de módulo canal premoldeado.</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CI</t>
+          <t>28/9/2026 – 10:00 horas</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="K18" s="4" t="inlineStr"/>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t>$25.000,00</t>
+        </is>
+      </c>
       <c r="L18" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1837,12 +1841,12 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Crespo</t>
         </is>
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>id-f8fab7a7b3a06a2d</t>
+          <t>id-1609ce58e128c413</t>
         </is>
       </c>
     </row>
@@ -1857,49 +1861,49 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Municipalidad de Crespo</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>5/2026</t>
+          <t>08/2026</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 145 metros lineales de módulo canal premoldeado.</t>
+          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCL UIDO</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>28/9/2026 – 10:00 horas</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>$25.000,00</t>
+          <t>SIN COSTO</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr">
@@ -1914,12 +1918,12 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Municipalidad de Crespo</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>id-1609ce58e128c413</t>
+          <t>id-1590925c21c7e363</t>
         </is>
       </c>
     </row>
@@ -1934,14 +1938,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1951,22 +1955,22 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>08/2026</t>
+          <t>10/26</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCL UIDO</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>29/09/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>29/09/2026</t>
+          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1976,7 +1980,7 @@
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>SIN COSTO</t>
+          <t>$ 100 (Cien)</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
@@ -1996,7 +2000,7 @@
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>id-1590925c21c7e363</t>
+          <t>id-75a5c9dd5b4aa6f3</t>
         </is>
       </c>
     </row>
@@ -2018,7 +2022,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2028,12 +2032,12 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>10/26</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
+          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -2043,7 +2047,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -2051,11 +2055,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K21" s="4" t="inlineStr">
-        <is>
-          <t>$ 100 (Cien)</t>
-        </is>
-      </c>
+      <c r="K21" s="4" t="inlineStr"/>
       <c r="L21" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2068,12 +2068,12 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-75a5c9dd5b4aa6f3</t>
+          <t>id-46c6d9f1f9210d1e</t>
         </is>
       </c>
     </row>
@@ -2083,9 +2083,9 @@
           <t>11/09/2026</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
@@ -2095,7 +2095,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2105,22 +2105,18 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>001-2026</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr">
-        <is>
-          <t>30/09/2026</t>
-        </is>
-      </c>
+          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr"/>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
+          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -2128,7 +2124,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K22" s="4" t="inlineStr"/>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L22" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2141,12 +2141,12 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-46c6d9f1f9210d1e</t>
+          <t>id-b7b0120caf49d551</t>
         </is>
       </c>
     </row>
@@ -2161,14 +2161,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
+          <t>MUNICIPALIDAD DE URDINARRAIN</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2178,18 +2178,18 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>001-2026</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
+          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr"/>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2197,11 +2197,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K23" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K23" s="4" t="inlineStr"/>
       <c r="L23" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2219,7 +2215,7 @@
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-b7b0120caf49d551</t>
+          <t>id-7a200161bcc9b02b</t>
         </is>
       </c>
     </row>
@@ -2234,14 +2230,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C24" s="10" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE URDINARRAIN</t>
+          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2251,12 +2247,12 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
+          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr"/>
@@ -2288,14 +2284,14 @@
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-7a200161bcc9b02b</t>
+          <t>id-511256e6329e386a</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2303,14 +2299,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2320,18 +2316,18 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>03/26</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr"/>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2352,19 +2348,19 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-511256e6329e386a</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2389,18 +2385,18 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2408,11 +2404,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K26" s="4" t="inlineStr">
-        <is>
-          <t>$ 120.976,01</t>
-        </is>
-      </c>
+      <c r="K26" s="4" t="inlineStr"/>
       <c r="L26" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2430,14 +2422,14 @@
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-07ddb93a12c5a870</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2462,18 +2454,18 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>Concurso de Precio N° 02/2025</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2499,14 +2491,14 @@
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-7c1bf02160a66f67</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2521,28 +2513,28 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Concurso</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>01/26</t>
+          <t>05/2025</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2563,19 +2555,19 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-9a16884dd5a64a49</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2583,35 +2575,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C29" s="10" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>2026-1227</t>
+          <t>06/2025</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2632,19 +2624,19 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-0691eb485d7548eb</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2652,14 +2644,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C30" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2667,20 +2659,16 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>10-2026</t>
-        </is>
-      </c>
+      <c r="F30" s="4" t="inlineStr"/>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego — figura como Pendiente</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2701,19 +2689,19 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-bdd0abb0374c3f42</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2721,35 +2709,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C31" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Licitación Privada</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>04/2025</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego — figura como Pendiente</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2770,17 +2758,703 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
+          <t>IAPV — Viviendas</t>
+        </is>
+      </c>
+      <c r="O31" s="4" t="inlineStr">
+        <is>
+          <t>id-34c85bcdb9b1123f</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>IAPV (Vivienda)</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>03/2025</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr"/>
+      <c r="I32" s="4" t="inlineStr">
+        <is>
+          <t>Publicada 08/10/2025 — ver pliego</t>
+        </is>
+      </c>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K32" s="4" t="inlineStr"/>
+      <c r="L32" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M32" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>IAPV — Viviendas</t>
+        </is>
+      </c>
+      <c r="O32" s="4" t="inlineStr">
+        <is>
+          <t>id-75bfffae63b7eedc</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>IAPV (Vivienda)</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>02/2025</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr"/>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>Publicada 06/10/2025 — ver pliego</t>
+        </is>
+      </c>
+      <c r="J33" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K33" s="4" t="inlineStr"/>
+      <c r="L33" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M33" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>IAPV — Viviendas</t>
+        </is>
+      </c>
+      <c r="O33" s="4" t="inlineStr">
+        <is>
+          <t>id-07ddb93a12c5a870</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>IAPV (Vivienda)</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>02/2025</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>Concurso de Precio N° 02/2025</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr"/>
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t>Publicada 19/06/2025 — ver pliego</t>
+        </is>
+      </c>
+      <c r="J34" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K34" s="4" t="inlineStr"/>
+      <c r="L34" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M34" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>IAPV — Viviendas</t>
+        </is>
+      </c>
+      <c r="O34" s="4" t="inlineStr">
+        <is>
+          <t>id-7c1bf02160a66f67</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C35" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr"/>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr"/>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K35" s="4" t="inlineStr"/>
+      <c r="L35" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M35" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="O35" s="4" t="inlineStr">
+        <is>
+          <t>id-654eebef400f89cd</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Concurso</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>01/26</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr"/>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K36" s="4" t="inlineStr"/>
+      <c r="L36" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M36" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="O36" s="4" t="inlineStr">
+        <is>
+          <t>id-9a16884dd5a64a49</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C37" s="10" t="inlineStr">
+        <is>
+          <t>Materiales</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>ENERSA</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Licitación</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>2026-1227</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr"/>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J37" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K37" s="4" t="inlineStr"/>
+      <c r="L37" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M37" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>ENERSA</t>
+        </is>
+      </c>
+      <c r="O37" s="4" t="inlineStr">
+        <is>
+          <t>id-0691eb485d7548eb</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C38" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
           <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
-      <c r="O31" s="4" t="inlineStr">
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>10-2026</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="inlineStr"/>
+      <c r="I38" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego — figura como Pendiente</t>
+        </is>
+      </c>
+      <c r="J38" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K38" s="4" t="inlineStr"/>
+      <c r="L38" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M38" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="O38" s="4" t="inlineStr">
+        <is>
+          <t>id-bdd0abb0374c3f42</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Licitación Privada</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>04-2026</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr"/>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego — figura como Pendiente</t>
+        </is>
+      </c>
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K39" s="4" t="inlineStr"/>
+      <c r="L39" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M39" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="O39" s="4" t="inlineStr">
         <is>
           <t>id-023b6b75e7014a9c</t>
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Poder Judicial de Entre Ríos</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Solicitud de Cotización</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>228/26</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>Solicitud de Cotización Nº 228/26, porContratación del servicio de recarga, revisión, prueba hidráulica y mantenimiento de los matafuegos ubicados en los Edificios de calle San Martín Nº15, Mitre Nº581 y Sarmiento Nº356 de la localidad de Victoria</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="inlineStr"/>
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>Ver el sitio</t>
+        </is>
+      </c>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K40" s="4" t="inlineStr"/>
+      <c r="L40" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M40" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Poder Judicial de Entre Ríos</t>
+        </is>
+      </c>
+      <c r="O40" s="4" t="inlineStr">
+        <is>
+          <t>id-e125fe54abc33d69</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C41" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Poder Judicial de Entre Ríos</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Solicitud de Cotización</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>230/26</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>“Provisión de manteriales y contratación del servicio de reparación de dos ascensores centrales ubicados en Edificio Tribunales de Concepción del Uruguay de calle San Martín Nº 665”</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr"/>
+      <c r="I41" s="4" t="inlineStr">
+        <is>
+          <t>Ver el sitio</t>
+        </is>
+      </c>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K41" s="4" t="inlineStr"/>
+      <c r="L41" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M41" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Poder Judicial de Entre Ríos</t>
+        </is>
+      </c>
+      <c r="O41" s="4" t="inlineStr">
+        <is>
+          <t>id-8ba9b58bf86dac2c</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O31"/>
+  <autoFilter ref="A1:O41"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -2842,6 +3516,26 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M30" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M31" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L38" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId80"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 15/09/2026 08:32
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -43,7 +43,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -58,11 +58,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
@@ -93,7 +88,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -106,7 +101,6 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -472,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O41"/>
+  <dimension ref="A1:O42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -649,7 +643,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -659,12 +653,12 @@
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>Áridos</t>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -674,22 +668,22 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>06/2026</t>
+          <t>016/2026</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>Transporte de dos mil metros cúbicos (2.000 m³) de ripio arcilloso destinados al mantenimiento y mejoramiento de caminos de la jurisdicción comunal de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de mano de obra, materiales y equipamiento para ejecución de restitución de galibo y repavimentación en Av enida Belgrano y Avenida 1° de Mayo de esta ciudad de chajari</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>02/10/2026</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>14 de septiembre de 2026 - Hora: 10:00</t>
+          <t>02 DE OCTUBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -697,7 +691,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr"/>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>$ 100.000, 00. - (PESOS CIEN MIL CON 00/100)</t>
+        </is>
+      </c>
       <c r="L3" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -715,7 +713,7 @@
       </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
-          <t>id-85e6cfd11c8a8889</t>
+          <t>id-53f1430f94acb0b0</t>
         </is>
       </c>
     </row>
@@ -807,7 +805,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -884,7 +882,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
@@ -961,7 +959,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
@@ -1034,7 +1032,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -1107,7 +1105,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>Materiales</t>
         </is>
@@ -1184,7 +1182,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C10" s="10" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>Materiales</t>
         </is>
@@ -1261,7 +1259,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -1338,7 +1336,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
@@ -1415,7 +1413,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
@@ -1488,7 +1486,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
@@ -1565,7 +1563,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t>Materiales</t>
         </is>
@@ -1638,7 +1636,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
@@ -1711,7 +1709,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
@@ -1776,7 +1774,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1784,29 +1782,29 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C18" s="10" t="inlineStr">
+      <c r="C18" s="9" t="inlineStr">
         <is>
           <t>Materiales</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Municipalidad de Crespo</t>
+          <t>MUNICIPALIDAD DE CRESPO -- ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>5/2026</t>
+          <t>05/2026</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 145 metros lineales de módulo canal premoldeado.</t>
+          <t>Adquisición de 145 metros lineales de modulo canal premoldeado cajón tipo pórtico de 2,00 X 1,00 (interior) X 1,00 mts. de longitud de hormigón para canalizar calle Los Quechuas al final</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1816,19 +1814,15 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>28/9/2026 – 10:00 horas</t>
+          <t>28 de septiembre de 2026 10:00 Hs. Lugar: Sección Suministros, Palacio Municipal sito en 25 de mayo Nº 943, C</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
-        </is>
-      </c>
-      <c r="K18" s="4" t="inlineStr">
-        <is>
-          <t>$25.000,00</t>
-        </is>
-      </c>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1841,12 +1835,12 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Municipalidad de Crespo</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>id-1609ce58e128c413</t>
+          <t>id-61e8747a99305fe9</t>
         </is>
       </c>
     </row>
@@ -1861,49 +1855,49 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>Municipalidad de Crespo</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>08/2026</t>
+          <t>5/2026</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCL UIDO</t>
+          <t>Adquisición de 145 metros lineales de módulo canal premoldeado.</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>29/09/2026</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>29/09/2026</t>
+          <t>28/9/2026 – 10:00 horas</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>SIN COSTO</t>
+          <t>$25.000,00</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr">
@@ -1918,12 +1912,12 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Crespo</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>id-1590925c21c7e363</t>
+          <t>id-1609ce58e128c413</t>
         </is>
       </c>
     </row>
@@ -1938,14 +1932,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1955,22 +1949,22 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>10/26</t>
+          <t>08/2026</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
+          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCL UIDO</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1980,7 +1974,7 @@
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>$ 100 (Cien)</t>
+          <t>SIN COSTO</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
@@ -2000,7 +1994,7 @@
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>id-75a5c9dd5b4aa6f3</t>
+          <t>id-1590925c21c7e363</t>
         </is>
       </c>
     </row>
@@ -2015,14 +2009,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2032,12 +2026,12 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>10/26</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -2047,7 +2041,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
+          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -2055,7 +2049,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K21" s="4" t="inlineStr"/>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>$ 100 (Cien)</t>
+        </is>
+      </c>
       <c r="L21" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2068,12 +2066,12 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-46c6d9f1f9210d1e</t>
+          <t>id-75a5c9dd5b4aa6f3</t>
         </is>
       </c>
     </row>
@@ -2083,19 +2081,19 @@
           <t>11/09/2026</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C22" s="9" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2105,18 +2103,22 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>001-2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr"/>
+          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
+          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -2124,11 +2126,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K22" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K22" s="4" t="inlineStr"/>
       <c r="L22" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2141,12 +2139,12 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-b7b0120caf49d551</t>
+          <t>id-46c6d9f1f9210d1e</t>
         </is>
       </c>
     </row>
@@ -2161,14 +2159,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C23" s="10" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE URDINARRAIN</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2178,18 +2176,18 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>001-2026</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
+          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr"/>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2197,7 +2195,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K23" s="4" t="inlineStr"/>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L23" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2215,7 +2217,7 @@
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-7a200161bcc9b02b</t>
+          <t>id-b7b0120caf49d551</t>
         </is>
       </c>
     </row>
@@ -2230,14 +2232,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
+          <t>MUNICIPALIDAD DE URDINARRAIN</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2247,12 +2249,12 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
+          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr"/>
@@ -2284,14 +2286,14 @@
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-511256e6329e386a</t>
+          <t>id-7a200161bcc9b02b</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2299,14 +2301,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C25" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2316,18 +2318,18 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>03/26</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr"/>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2348,12 +2350,12 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-511256e6329e386a</t>
         </is>
       </c>
     </row>
@@ -2368,7 +2370,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C26" s="8" t="inlineStr">
+      <c r="C26" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2385,18 +2387,18 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>02/2026</t>
+          <t>03/26</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2422,7 +2424,7 @@
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
@@ -2437,7 +2439,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C27" s="8" t="inlineStr">
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2454,18 +2456,18 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2491,7 +2493,7 @@
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
@@ -2506,7 +2508,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C28" s="8" t="inlineStr">
+      <c r="C28" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2523,18 +2525,18 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>05/2025</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2560,7 +2562,7 @@
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
@@ -2575,7 +2577,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C29" s="8" t="inlineStr">
+      <c r="C29" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2592,18 +2594,18 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>06/2025</t>
+          <t>05/2025</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2629,7 +2631,7 @@
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
@@ -2644,7 +2646,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C30" s="8" t="inlineStr">
+      <c r="C30" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2659,16 +2661,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F30" s="4" t="inlineStr"/>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>06/2025</t>
+        </is>
+      </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2694,7 +2700,7 @@
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-ebeeb6a87e688d85</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
@@ -2709,7 +2715,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C31" s="8" t="inlineStr">
+      <c r="C31" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2724,20 +2730,16 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>04/2025</t>
-        </is>
-      </c>
+      <c r="F31" s="4" t="inlineStr"/>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2763,7 +2765,7 @@
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-34c85bcdb9b1123f</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
@@ -2778,7 +2780,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C32" s="8" t="inlineStr">
+      <c r="C32" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2795,18 +2797,18 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>03/2025</t>
+          <t>04/2025</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2832,14 +2834,14 @@
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-75bfffae63b7eedc</t>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2847,7 +2849,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C33" s="8" t="inlineStr">
+      <c r="C33" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2864,18 +2866,18 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>03/2025</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2901,7 +2903,7 @@
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-07ddb93a12c5a870</t>
+          <t>id-75bfffae63b7eedc</t>
         </is>
       </c>
     </row>
@@ -2916,7 +2918,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C34" s="8" t="inlineStr">
+      <c r="C34" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2938,13 +2940,13 @@
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>Concurso de Precio N° 02/2025</t>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
+          <t>Publicada 06/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -2970,14 +2972,14 @@
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-7c1bf02160a66f67</t>
+          <t>id-07ddb93a12c5a870</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2985,31 +2987,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C35" s="10" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F35" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>02/2025</t>
+        </is>
+      </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
+          <t>Concurso de Precio N° 02/2025</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 19/06/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3030,19 +3036,19 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-654eebef400f89cd</t>
+          <t>id-7c1bf02160a66f67</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3050,9 +3056,9 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C36" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C36" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -3062,17 +3068,13 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Concurso</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>01/26</t>
-        </is>
-      </c>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr"/>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
@@ -3104,7 +3106,7 @@
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>id-9a16884dd5a64a49</t>
+          <t>id-654eebef400f89cd</t>
         </is>
       </c>
     </row>
@@ -3119,29 +3121,29 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C37" s="10" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Concurso</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>2026-1227</t>
+          <t>01/26</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
@@ -3168,12 +3170,12 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>id-0691eb485d7548eb</t>
+          <t>id-9a16884dd5a64a49</t>
         </is>
       </c>
     </row>
@@ -3190,33 +3192,33 @@
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>10-2026</t>
+          <t>2026-1227</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego — figura como Pendiente</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -3237,12 +3239,12 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>id-bdd0abb0374c3f42</t>
+          <t>id-0691eb485d7548eb</t>
         </is>
       </c>
     </row>
@@ -3257,7 +3259,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C39" s="9" t="inlineStr">
+      <c r="C39" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
@@ -3269,17 +3271,17 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Licitación Privada</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>10-2026</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
+          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
@@ -3311,14 +3313,14 @@
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
-          <t>id-023b6b75e7014a9c</t>
+          <t>id-bdd0abb0374c3f42</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3328,33 +3330,33 @@
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>Infraestructura</t>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Solicitud de Cotización</t>
+          <t>Licitación Privada</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>228/26</t>
+          <t>04-2026</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>Solicitud de Cotización Nº 228/26, porContratación del servicio de recarga, revisión, prueba hidráulica y mantenimiento de los matafuegos ubicados en los Edificios de calle San Martín Nº15, Mitre Nº581 y Sarmiento Nº356 de la localidad de Victoria</t>
+          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr"/>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Ver el sitio</t>
+          <t>Ver pliego — figura como Pendiente</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
@@ -3375,19 +3377,19 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
-          <t>id-e125fe54abc33d69</t>
+          <t>id-023b6b75e7014a9c</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3395,7 +3397,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C41" s="9" t="inlineStr">
+      <c r="C41" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
@@ -3412,12 +3414,12 @@
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>230/26</t>
+          <t>232/26</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>“Provisión de manteriales y contratación del servicio de reparación de dos ascensores centrales ubicados en Edificio Tribunales de Concepción del Uruguay de calle San Martín Nº 665”</t>
+          <t>SERVICIO DE REACONDICIONAMIENTO Y REPARACIÓN EN SECTOR POSTERIOR DEL INMUEBLE ALQUILADO DEL JUZGADO DE PAZ DE SAN JAIME DE LA FRONTERA</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
@@ -3449,12 +3451,81 @@
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
-          <t>id-8ba9b58bf86dac2c</t>
+          <t>id-5a01c3fd726f10dc</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Poder Judicial de Entre Ríos</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Solicitud de Cotización</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>228/26</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>Solicitud de Cotización Nº 228/26, porContratación del servicio de recarga, revisión, prueba hidráulica y mantenimiento de los matafuegos ubicados en los Edificios de calle San Martín Nº15, Mitre Nº581 y Sarmiento Nº356 de la localidad de Victoria</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="inlineStr"/>
+      <c r="I42" s="4" t="inlineStr">
+        <is>
+          <t>Ver el sitio</t>
+        </is>
+      </c>
+      <c r="J42" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K42" s="4" t="inlineStr"/>
+      <c r="L42" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M42" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Poder Judicial de Entre Ríos</t>
+        </is>
+      </c>
+      <c r="O42" s="4" t="inlineStr">
+        <is>
+          <t>id-e125fe54abc33d69</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O41"/>
+  <autoFilter ref="A1:O42"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -3536,6 +3607,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId78"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId79"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId82"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 16/09/2026 09:00
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$38</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -67,12 +67,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
+        <fgColor rgb="00E6D9F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E6D9F2"/>
+        <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O42"/>
+  <dimension ref="A1:O38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -673,7 +673,7 @@
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de mano de obra, materiales y equipamiento para ejecución de restitución de galibo y repavimentación en Av enida Belgrano y Avenida 1° de Mayo de esta ciudad de chajari</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de mano de obra, materiales y equipamiento para ejecución de restitución de galibo y repavimentación en Avenida Belgrano y Avenida 1° de Mayo de esta ciudad de chajari</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>$ 100.000, 00. - (PESOS CIEN MIL CON 00/100)</t>
+          <t>$ 100.000, 00.- (PESOS CIEN MIL CON 00/100)</t>
         </is>
       </c>
       <c r="L3" s="6" t="inlineStr">
@@ -728,14 +728,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE HERRERA — DPTO. URUGUAY, ENTRE RÍOS</t>
+          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCIÓN DEL URUGUAY</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -745,22 +745,22 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>01-2026</t>
+          <t>27/2026</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de vehículo 0 km destinado al traslado de personas tipo van, con capacidad para 11 plazas (1 conductor + 10 pasajeros), motorización a nafta/diesel, según pliego de especificaciones técnicas</t>
+          <t>“Adquisición de seiscientas (600) Luminarias Leds para Alumbrado Público”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás docum entación</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
+          <t>16/09/2026</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 15/09/2026, a las 11:00 hs. en el Edificio Municipal de Herrera, sito en Av. H. Bozzolo, Nº 165,</t>
+          <t>16 de septiembre de 2026 - Hora: 10:00</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -768,11 +768,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K4" s="4" t="inlineStr"/>
       <c r="L4" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -790,7 +786,7 @@
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
-          <t>id-28313c7a9524d0ee</t>
+          <t>id-608017f47f903d65</t>
         </is>
       </c>
     </row>
@@ -805,14 +801,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
+          <t>GOBIERNO DE ENTRE RÍOS — UNIDAD CENTRAL DE CONTRATACIONES</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -822,22 +818,22 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>014/2026</t>
+          <t>06/26</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de materiales – 500 (quinientos) m3 de Hormigón elaborado Tipo H30, Reglamento CIRSOC 201, para ser utilizados en la obra de construcción de pavimento en c alle Moreno entre Av. 1° de Mayo y Guarumba de nuestra ciudad</t>
+          <t>Adquirir materiales de construcción (chapas, rollos de film de polietileno, tirantes, clavos y clavadoras)</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>15 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>Unidad Central de Contrataciones, el día 17/09/26 a las 09:00 horas</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -847,7 +843,7 @@
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>$ 82.500,00. - (PESOS OCHENTA Y DOS MIL QUINIENTOS CON 00/100)</t>
+          <t>PESOS CINCUENTA MIL ($ 50.000)</t>
         </is>
       </c>
       <c r="L5" s="6" t="inlineStr">
@@ -867,7 +863,7 @@
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>id-9e58cc9ec0b69356</t>
+          <t>id-9dbdaa6090d92bd4</t>
         </is>
       </c>
     </row>
@@ -884,12 +880,12 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>MINISTERIO DE PLANEAMIENTO E INFRAESTRUCTURA</t>
+          <t>MUNICIPALIDAD DE SEGUÍ</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -899,22 +895,22 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>08/26</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “NUEVA INSTALACION ELECTRICA, CUBIERTA DE TECHO Y REFACCION DE BAÑOS ESCUELA Nº 1 “JOSE MARIA TEXIER” -SAN SALVADOR-DEPARTAMENTO SAN SALVADOR.”</t>
+          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Us os Múltiples – Gimnasio Municipal”</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 15 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>17/09/2026 a las 10:00 hs, en el Edificio Municipal</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -924,7 +920,7 @@
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>$ 100 (Cien)</t>
+          <t>Gratuito</t>
         </is>
       </c>
       <c r="L6" s="6" t="inlineStr">
@@ -944,7 +940,7 @@
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>id-fb80c8ade7a8651d</t>
+          <t>id-90c3d1f38f49418a</t>
         </is>
       </c>
     </row>
@@ -959,14 +955,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -976,22 +972,22 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>08/2026</t>
+          <t>015/2026</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Nueva instalación eléctrica, cubierta de techo y refacción de baños Escuela N° 1 "José María Texier", San Salvador</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>martes, 15 de septiembre de 2026 - 10:00hs</t>
+          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -999,7 +995,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr"/>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>$ 90.000,00. - (PESOS NOVENTA MIL CON 00/100)</t>
+        </is>
+      </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1012,12 +1012,12 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>id-952aef4c115d8f12</t>
+          <t>id-74dfdad7e5f9d048</t>
         </is>
       </c>
     </row>
@@ -1032,14 +1032,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCIÓN DEL URUGUAY</t>
+          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1049,22 +1049,22 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>27/2026</t>
+          <t>09/26</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>“Adquisición de seiscientas (600) Luminarias Leds para Alumbrado Público”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás docum entación</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “AMPLIACION - RECONSTRUCCION DE PISOS Y CONTRAPISOS -IMPERMEABILIZACION LOSAS- INSTALACION ELECTRICA-ESCUELA SECUNDARIA ADULTOS Nº 1 “DR. LUIS AGOTE” -NOGOYA-DEPARTAMENTO NOGOYA.”</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>16/09/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>16 de septiembre de 2026 - Hora: 10:00</t>
+          <t>DE LAS OFERTAS: el día 18 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -1072,7 +1072,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr"/>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>$ 100 (Cien)</t>
+        </is>
+      </c>
       <c r="L8" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1090,7 +1094,7 @@
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>id-608017f47f903d65</t>
+          <t>id-6a4a84712fd41a03</t>
         </is>
       </c>
     </row>
@@ -1107,12 +1111,12 @@
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Materiales</t>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>GOBIERNO DE ENTRE RÍOS — UNIDAD CENTRAL DE CONTRATACIONES</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1122,22 +1126,22 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>06/26</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Adquirir materiales de construcción (chapas, rollos de film de polietileno, tirantes, clavos y clavadoras)</t>
+          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Unidad Central de Contrataciones, el día 17/09/26 a las 09:00 horas</t>
+          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1145,11 +1149,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>PESOS CINCUENTA MIL ($ 50.000)</t>
-        </is>
-      </c>
+      <c r="K9" s="4" t="inlineStr"/>
       <c r="L9" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1162,12 +1162,12 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>id-9dbdaa6090d92bd4</t>
+          <t>id-885d4847519dfd48</t>
         </is>
       </c>
     </row>
@@ -1184,12 +1184,12 @@
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Materiales</t>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE SEGUÍ</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1199,22 +1199,22 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>07/2026</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Us os Múltiples – Gimnasio Municipal”</t>
+          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>21/09/2026</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026 a las 10:00 hs, en el Edificio Municipal</t>
+          <t>21/09/2026 HORA: 10:00 HS</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>Gratuito</t>
+          <t>SIN COSTO</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr">
@@ -1244,7 +1244,7 @@
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>id-90c3d1f38f49418a</t>
+          <t>id-6ddfa0f2f1aa296d</t>
         </is>
       </c>
     </row>
@@ -1259,14 +1259,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
+          <t>COLON — MUNICIPALIDAD DE COLON</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1274,24 +1274,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>015/2026</t>
-        </is>
-      </c>
+      <c r="F11" s="4" t="inlineStr"/>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
+          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>24 de SEPTIEMBRE de 2026</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1301,7 +1297,7 @@
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>$ 90.000,00. - (PESOS NOVENTA MIL CON 00/100)</t>
+          <t>Sin Cargo</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
@@ -1321,7 +1317,7 @@
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>id-74dfdad7e5f9d048</t>
+          <t>id-bc610b64999d147d</t>
         </is>
       </c>
     </row>
@@ -1336,14 +1332,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1353,34 +1349,30 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>09/26</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “AMPLIACION - RECONSTRUCCION DE PISOS Y CONTRAPISOS -IMPERMEABILIZACION LOSAS- INSTALACION ELECTRICA-ESCUELA SECUNDARIA ADULTOS Nº 1 “DR. LUIS AGOTE” -NOGOYA-DEPARTAMENTO NOGOYA.”</t>
+          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 18 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIU</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K12" s="4" t="inlineStr">
-        <is>
-          <t>$ 100 (Cien)</t>
-        </is>
-      </c>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr"/>
       <c r="L12" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1398,7 +1390,7 @@
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>id-6a4a84712fd41a03</t>
+          <t>id-d97b43a99f1e1824</t>
         </is>
       </c>
     </row>
@@ -1413,14 +1405,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1435,22 +1427,22 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
+          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CI</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr"/>
@@ -1466,19 +1458,19 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>id-885d4847519dfd48</t>
+          <t>id-f8fab7a7b3a06a2d</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1488,12 +1480,12 @@
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>MUNICIPALIDAD DE CRESPO -- ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1503,34 +1495,30 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>07/2026</t>
+          <t>05/2026</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”</t>
+          <t>Adquisición de 145 metros lineales de modulo canal premoldeado caj ón tipo pórtico de 2,00 X 1,00 (interior) X 1,00 mts. de longitud de hormigón para canalizar calle Los Quechuas al final</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>21/09/2026</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>21/09/2026 HORA: 10:00 HS</t>
+          <t>28 de septiembre de 2026 10:00 Hs. Lugar: Sección Suministros, Palacio Municipal sito en 25 de mayo Nº 943, C</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K14" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr"/>
       <c r="L14" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1548,7 +1536,7 @@
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>id-6ddfa0f2f1aa296d</t>
+          <t>id-61e8747a99305fe9</t>
         </is>
       </c>
     </row>
@@ -1563,45 +1551,49 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>Materiales</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>COLON — MUNICIPALIDAD DE COLON</t>
+          <t>Municipalidad de Crespo</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr"/>
+          <t>Licitación</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>5/2026</t>
+        </is>
+      </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
+          <t>Adquisición de 145 metros lineales de módulo canal premoldeado.</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>24 de SEPTIEMBRE de 2026</t>
+          <t>28/9/2026 – 10:00 horas</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>Sin Cargo</t>
+          <t>$25.000,00</t>
         </is>
       </c>
       <c r="L15" s="6" t="inlineStr">
@@ -1616,12 +1608,12 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Crespo</t>
         </is>
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>id-bc610b64999d147d</t>
+          <t>id-1609ce58e128c413</t>
         </is>
       </c>
     </row>
@@ -1636,14 +1628,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1653,30 +1645,34 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>08/2026</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCL UIDO</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIU</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="K16" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L16" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1694,7 +1690,7 @@
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>id-d97b43a99f1e1824</t>
+          <t>id-1590925c21c7e363</t>
         </is>
       </c>
     </row>
@@ -1709,14 +1705,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C17" s="9" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1726,30 +1722,34 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>10/26</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CI</t>
+          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="K17" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>$ 100 (Cien)</t>
+        </is>
+      </c>
       <c r="L17" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1762,19 +1762,19 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos + CAFESG (Salto Grande)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>id-f8fab7a7b3a06a2d</t>
+          <t>id-75a5c9dd5b4aa6f3</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1784,12 +1784,12 @@
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>Materiales</t>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE CRESPO -- ENTRE RÍOS</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1799,27 +1799,27 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>05/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 145 metros lineales de modulo canal premoldeado cajón tipo pórtico de 2,00 X 1,00 (interior) X 1,00 mts. de longitud de hormigón para canalizar calle Los Quechuas al final</t>
+          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>28 de septiembre de 2026 10:00 Hs. Lugar: Sección Suministros, Palacio Municipal sito en 25 de mayo Nº 943, C</t>
+          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr"/>
@@ -1835,12 +1835,12 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>id-61e8747a99305fe9</t>
+          <t>id-46c6d9f1f9210d1e</t>
         </is>
       </c>
     </row>
@@ -1850,54 +1850,50 @@
           <t>11/09/2026</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>Materiales</t>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Municipalidad de Crespo</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>5/2026</t>
+          <t>001-2026</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 145 metros lineales de módulo canal premoldeado.</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t>28/09/2026</t>
-        </is>
-      </c>
+          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr"/>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>28/9/2026 – 10:00 horas</t>
+          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>$25.000,00</t>
+          <t>SIN COSTO</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr">
@@ -1912,12 +1908,12 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Municipalidad de Crespo</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>id-1609ce58e128c413</t>
+          <t>id-b7b0120caf49d551</t>
         </is>
       </c>
     </row>
@@ -1927,19 +1923,19 @@
           <t>11/09/2026</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>MUNICIPALIDAD DE URDINARRAIN</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1949,22 +1945,18 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>08/2026</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCL UIDO</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>29/09/2026</t>
-        </is>
-      </c>
+          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr"/>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>29/09/2026</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1972,11 +1964,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K20" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K20" s="4" t="inlineStr"/>
       <c r="L20" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1994,7 +1982,7 @@
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>id-1590925c21c7e363</t>
+          <t>id-7a200161bcc9b02b</t>
         </is>
       </c>
     </row>
@@ -2004,19 +1992,19 @@
           <t>11/09/2026</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2026,22 +2014,18 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>10/26</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>30/09/2026</t>
-        </is>
-      </c>
+          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr"/>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -2049,11 +2033,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K21" s="4" t="inlineStr">
-        <is>
-          <t>$ 100 (Cien)</t>
-        </is>
-      </c>
+      <c r="K21" s="4" t="inlineStr"/>
       <c r="L21" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2071,29 +2051,29 @@
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-75a5c9dd5b4aa6f3</t>
+          <t>id-511256e6329e386a</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2103,22 +2083,18 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>03/26</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr">
-        <is>
-          <t>30/09/2026</t>
-        </is>
-      </c>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr"/>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -2139,19 +2115,19 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-46c6d9f1f9210d1e</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2159,14 +2135,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2176,18 +2152,18 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>001-2026</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr"/>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2195,11 +2171,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K23" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K23" s="4" t="inlineStr"/>
       <c r="L23" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2212,19 +2184,19 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-b7b0120caf49d551</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2232,14 +2204,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE URDINARRAIN</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2249,18 +2221,18 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr"/>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -2281,19 +2253,19 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-7a200161bcc9b02b</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2301,14 +2273,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2318,18 +2290,18 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>05/2025</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr"/>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2350,12 +2322,12 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-511256e6329e386a</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
@@ -2387,18 +2359,18 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>03/26</t>
+          <t>06/2025</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2424,7 +2396,7 @@
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
@@ -2454,20 +2426,16 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>02/2026</t>
-        </is>
-      </c>
+      <c r="F27" s="4" t="inlineStr"/>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2493,7 +2461,7 @@
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
@@ -2525,18 +2493,18 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>04/2025</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2562,7 +2530,7 @@
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
@@ -2594,18 +2562,18 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>05/2025</t>
+          <t>03/2025</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2631,14 +2599,14 @@
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-75bfffae63b7eedc</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2663,18 +2631,18 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>06/2025</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Publicada 06/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2700,14 +2668,14 @@
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
+          <t>id-07ddb93a12c5a870</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2730,16 +2698,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F31" s="4" t="inlineStr"/>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>02/2025</t>
+        </is>
+      </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+          <t>Concurso de Precio N° 02/2025</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
+          <t>Publicada 19/06/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2765,7 +2737,7 @@
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-ebeeb6a87e688d85</t>
+          <t>id-7c1bf02160a66f67</t>
         </is>
       </c>
     </row>
@@ -2780,35 +2752,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C32" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>04/2025</t>
-        </is>
-      </c>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr"/>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2829,19 +2797,19 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-34c85bcdb9b1123f</t>
+          <t>id-654eebef400f89cd</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2856,28 +2824,28 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Concurso</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>03/2025</t>
+          <t>01/26</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2898,19 +2866,19 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-75bfffae63b7eedc</t>
+          <t>id-9a16884dd5a64a49</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2918,35 +2886,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Solicitud de Cotización</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>232/26</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>SERVICIO DE REACONDICIONAMIENTO Y REPARACIÓN EN SECTOR POSTERIOR DEL INMUEBLE ALQUILADO DEL JUZGADO DE PAZ DE SAN JAIME DE LA FRONTERA</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>Ver el sitio</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -2967,19 +2935,19 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-07ddb93a12c5a870</t>
+          <t>id-5a01c3fd726f10dc</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2994,28 +2962,28 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Solicitud de Cotización</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>228/26</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>Concurso de Precio N° 02/2025</t>
+          <t>Solicitud de Cotización Nº 228/26, porContratación del servicio de recarga, revisión, prueba hidráulica y mantenimiento de los matafuegos ubicados en los Edificios de calle San Martín Nº15, Mitre Nº581 y Sarmiento Nº356 de la localidad de Victoria</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
+          <t>Ver el sitio</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3036,19 +3004,19 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-7c1bf02160a66f67</t>
+          <t>id-e125fe54abc33d69</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3056,25 +3024,29 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C36" s="9" t="inlineStr">
+      <c r="C36" s="8" t="inlineStr">
         <is>
           <t>Materiales</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr"/>
+          <t>Licitación</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>2026-1227</t>
+        </is>
+      </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
@@ -3101,12 +3073,12 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>id-654eebef400f89cd</t>
+          <t>id-0691eb485d7548eb</t>
         </is>
       </c>
     </row>
@@ -3121,35 +3093,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C37" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C37" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Concurso</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>01/26</t>
+          <t>10-2026</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Ver pliego — figura como Pendiente</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3170,12 +3142,12 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>id-9a16884dd5a64a49</t>
+          <t>id-bdd0abb0374c3f42</t>
         </is>
       </c>
     </row>
@@ -3192,33 +3164,33 @@
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>Materiales</t>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Privada</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>2026-1227</t>
+          <t>04-2026</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Ver pliego — figura como Pendiente</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -3239,293 +3211,17 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>id-0691eb485d7548eb</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>11/09/2026</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>CAFESG (Salto Grande)</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F39" s="4" t="inlineStr">
-        <is>
-          <t>10-2026</t>
-        </is>
-      </c>
-      <c r="G39" s="5" t="inlineStr">
-        <is>
-          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
-        </is>
-      </c>
-      <c r="H39" s="4" t="inlineStr"/>
-      <c r="I39" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego — figura como Pendiente</t>
-        </is>
-      </c>
-      <c r="J39" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K39" s="4" t="inlineStr"/>
-      <c r="L39" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M39" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>CAFESG (Salto Grande)</t>
-        </is>
-      </c>
-      <c r="O39" s="4" t="inlineStr">
-        <is>
-          <t>id-bdd0abb0374c3f42</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>11/09/2026</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C40" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>CAFESG (Salto Grande)</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Licitación Privada</t>
-        </is>
-      </c>
-      <c r="F40" s="4" t="inlineStr">
-        <is>
-          <t>04-2026</t>
-        </is>
-      </c>
-      <c r="G40" s="5" t="inlineStr">
-        <is>
-          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
-        </is>
-      </c>
-      <c r="H40" s="4" t="inlineStr"/>
-      <c r="I40" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego — figura como Pendiente</t>
-        </is>
-      </c>
-      <c r="J40" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K40" s="4" t="inlineStr"/>
-      <c r="L40" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M40" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N40" t="inlineStr">
-        <is>
-          <t>CAFESG (Salto Grande)</t>
-        </is>
-      </c>
-      <c r="O40" s="4" t="inlineStr">
-        <is>
           <t>id-023b6b75e7014a9c</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>15/09/2026</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Poder Judicial de Entre Ríos</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Solicitud de Cotización</t>
-        </is>
-      </c>
-      <c r="F41" s="4" t="inlineStr">
-        <is>
-          <t>232/26</t>
-        </is>
-      </c>
-      <c r="G41" s="5" t="inlineStr">
-        <is>
-          <t>SERVICIO DE REACONDICIONAMIENTO Y REPARACIÓN EN SECTOR POSTERIOR DEL INMUEBLE ALQUILADO DEL JUZGADO DE PAZ DE SAN JAIME DE LA FRONTERA</t>
-        </is>
-      </c>
-      <c r="H41" s="4" t="inlineStr"/>
-      <c r="I41" s="4" t="inlineStr">
-        <is>
-          <t>Ver el sitio</t>
-        </is>
-      </c>
-      <c r="J41" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K41" s="4" t="inlineStr"/>
-      <c r="L41" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M41" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>Poder Judicial de Entre Ríos</t>
-        </is>
-      </c>
-      <c r="O41" s="4" t="inlineStr">
-        <is>
-          <t>id-5a01c3fd726f10dc</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>14/09/2026</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C42" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Poder Judicial de Entre Ríos</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Solicitud de Cotización</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="inlineStr">
-        <is>
-          <t>228/26</t>
-        </is>
-      </c>
-      <c r="G42" s="5" t="inlineStr">
-        <is>
-          <t>Solicitud de Cotización Nº 228/26, porContratación del servicio de recarga, revisión, prueba hidráulica y mantenimiento de los matafuegos ubicados en los Edificios de calle San Martín Nº15, Mitre Nº581 y Sarmiento Nº356 de la localidad de Victoria</t>
-        </is>
-      </c>
-      <c r="H42" s="4" t="inlineStr"/>
-      <c r="I42" s="4" t="inlineStr">
-        <is>
-          <t>Ver el sitio</t>
-        </is>
-      </c>
-      <c r="J42" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K42" s="4" t="inlineStr"/>
-      <c r="L42" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M42" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>Poder Judicial de Entre Ríos</t>
-        </is>
-      </c>
-      <c r="O42" s="4" t="inlineStr">
-        <is>
-          <t>id-e125fe54abc33d69</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:O42"/>
+  <autoFilter ref="A1:O38"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -3601,14 +3297,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L38" r:id="rId73"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId82"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 17/09/2026 08:13
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$37</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -67,12 +67,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
+        <fgColor rgb="00E6D9F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E6D9F2"/>
+        <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O35"/>
+  <dimension ref="A1:O37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -693,7 +693,7 @@
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>$ 100.000, 00. - (PESOS CIEN MIL CON 00/100)</t>
+          <t>$ 100.000, 00.- (PESOS CIEN MIL CON 00/100)</t>
         </is>
       </c>
       <c r="L3" s="6" t="inlineStr">
@@ -720,55 +720,59 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Materiales</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>GOBIERNO DE ENTRE RÍOS — UNIDAD CENTRAL DE CONTRATACIONES</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>06/26</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Adquirir materiales de construcción (chapas, rollos de film de polietileno, tirantes, clavos y clavadoras)</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
           <t>17/09/2026</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>P ARANA — MINISTERIO DE SALUD</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Licitación Publica</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>17/26</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>Adquirir Una (01) Mesa de Anestesia. Destino: Hospital “San José” de Diamante, dependiente del Ministerio de Salud de la Provincia de Entre Ríos</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>06/10/2026</t>
-        </is>
-      </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
+          <t>Unidad Central de Contrataciones, el día 17/09/26 a las 09:00 horas</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>PESOS CINCUENTA MIL ($ 50.000)</t>
+        </is>
+      </c>
       <c r="L4" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -786,54 +790,54 @@
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
-          <t>id-3312d89e1a3e2e53</t>
+          <t>id-9dbdaa6090d92bd4</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Materiales</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>MUNICIPALIDAD DE SEGUÍ</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>08-2026</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Us os Múltiples – Gimnasio Municipal”</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
           <t>17/09/2026</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>MUNICIPALIDAD DE CONCEPCIÓN DEL URUGUAY</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>31/2026</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>“Pavimento Rígido – 03 (tres) Cuadras Barrio San Felipe”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>07/10/2026</t>
-        </is>
-      </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>07 de octubre de 2026 Hora: 10:00</t>
+          <t>17/09/2026 a las 10:00 hs, en el Edificio Municipal</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -841,7 +845,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr"/>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>Gratuito</t>
+        </is>
+      </c>
       <c r="L5" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -859,14 +867,14 @@
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>id-76d9566cb30a6df5</t>
+          <t>id-90c3d1f38f49418a</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -874,14 +882,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -891,30 +899,34 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>11/2026</t>
+          <t>015/2026</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>REFACCION EN ESCUELA N° 65 “ALMIRANTE BROWN” – CIUDAD DE CONCORDIA - DEPARTAMENTO CONCORDIA - PROVINCIA DE ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026. - Hora: 09:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDA</t>
+          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>$ 90.000,00. - (PESOS NOVENTA MIL CON 00/100)</t>
+        </is>
+      </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -932,14 +944,14 @@
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>id-fc30d5c0b0589a79</t>
+          <t>id-74dfdad7e5f9d048</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -947,14 +959,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
+          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -964,30 +976,34 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>13/2026</t>
+          <t>09/26</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>REPARACIONES VARIAS EN C . P. E. F. Nº 3 “PROFESOR HUGO LA NASA” – CIUDAD DE CONCEPCION DEL URUGUAY - DEPARTAMENTO URUGUAY - PROVINCIA DE ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “AMPLIACION - RECONSTRUCCION DE PISOS Y CONTRAPISOS -IMPERMEABILIZACION LOSAS- INSTALACION ELECTRICA-ESCUELA SECUNDARIA ADULTOS Nº 1 “DR. LUIS AGOTE” -NOGOYA-DEPARTAMENTO NOGOYA.”</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026. - Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDA</t>
+          <t>DE LAS OFERTAS: el día 18 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
-        </is>
-      </c>
-      <c r="K7" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>$ 100 (Cien)</t>
+        </is>
+      </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1005,14 +1021,14 @@
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>id-9d3847fb0e2b0929</t>
+          <t>id-6a4a84712fd41a03</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1020,14 +1036,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1037,27 +1053,27 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>12/2026</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>RECAMBIO DE CUBIERTA Y REPARACIONES VARIAS EN ESCUELA Nº 92 “CONGRESO DE TUCUMAN” – CONCEPCION DEL URUGUAY - DPTO. URUGUAY – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026. - Hora: 10:30 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDA</t>
+          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr"/>
@@ -1073,12 +1089,12 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>id-059239b424b9c936</t>
+          <t>id-885d4847519dfd48</t>
         </is>
       </c>
     </row>
@@ -1095,12 +1111,12 @@
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Materiales</t>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>GOBIERNO DE ENTRE RÍOS — UNIDAD CENTRAL DE CONTRATACIONES</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1110,22 +1126,22 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>06/26</t>
+          <t>07/2026</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Adquirir materiales de construcción (chapas, rollos de film de polietileno, tirantes, clavos y clavadoras)</t>
+          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>21/09/2026</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Unidad Central de Contrataciones, el día 17/09/26 a las 09:00 horas</t>
+          <t>21/09/2026 HORA: 10:00 HS</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1135,7 +1151,7 @@
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>PESOS CINCUENTA MIL ($ 50.000)</t>
+          <t>SIN COSTO</t>
         </is>
       </c>
       <c r="L9" s="6" t="inlineStr">
@@ -1155,7 +1171,7 @@
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>id-9dbdaa6090d92bd4</t>
+          <t>id-6ddfa0f2f1aa296d</t>
         </is>
       </c>
     </row>
@@ -1170,14 +1186,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>Materiales</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE SEGUÍ</t>
+          <t>COLON — MUNICIPALIDAD DE COLON</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1185,24 +1201,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>08-2026</t>
-        </is>
-      </c>
+      <c r="F10" s="4" t="inlineStr"/>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Us os Múltiples – Gimnasio Municipal”</t>
+          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026 a las 10:00 hs, en el Edificio Municipal</t>
+          <t>24 de SEPTIEMBRE de 2026</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1212,7 +1224,7 @@
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>Gratuito</t>
+          <t>Sin Cargo</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr">
@@ -1232,7 +1244,7 @@
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>id-90c3d1f38f49418a</t>
+          <t>id-bc610b64999d147d</t>
         </is>
       </c>
     </row>
@@ -1247,14 +1259,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
+          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1264,34 +1276,30 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>015/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
+          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIU</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K11" s="4" t="inlineStr">
-        <is>
-          <t>$ 90.000,00. - (PESOS NOVENTA MIL CON 00/100)</t>
-        </is>
-      </c>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr"/>
       <c r="L11" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1309,7 +1317,7 @@
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>id-74dfdad7e5f9d048</t>
+          <t>id-d97b43a99f1e1824</t>
         </is>
       </c>
     </row>
@@ -1324,14 +1332,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1341,34 +1349,30 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>09/26</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “AMPLIACION - RECONSTRUCCION DE PISOS Y CONTRAPISOS -IMPERMEABILIZACION LOSAS- INSTALACION ELECTRICA-ESCUELA SECUNDARIA ADULTOS Nº 1 “DR. LUIS AGOTE” -NOGOYA-DEPARTAMENTO NOGOYA.”</t>
+          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 18 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CI</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K12" s="4" t="inlineStr">
-        <is>
-          <t>$ 100 (Cien)</t>
-        </is>
-      </c>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr"/>
       <c r="L12" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1386,14 +1390,14 @@
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>id-6a4a84712fd41a03</t>
+          <t>id-f8fab7a7b3a06a2d</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1403,12 +1407,12 @@
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>MUNICIPALIDAD DE CRESPO -- ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1418,27 +1422,27 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>05/2026</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
+          <t>Adquisición de 145 metros lineales de modulo canal premoldeado caj ón tipo pórtico de 2,00 X 1,00 (interior) X 1,00 mts. de longitud de hormigón para canalizar calle Los Quechuas al final</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
+          <t>28 de septiembre de 2026 10:00 Hs. Lugar: Sección Suministros, Palacio Municipal sito en 25 de mayo Nº 943, C</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr"/>
@@ -1454,12 +1458,12 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>id-885d4847519dfd48</t>
+          <t>id-61e8747a99305fe9</t>
         </is>
       </c>
     </row>
@@ -1476,47 +1480,47 @@
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>Municipalidad de Crespo</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>07/2026</t>
+          <t>5/2026</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”</t>
+          <t>Adquisición de 145 metros lineales de módulo canal premoldeado.</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>21/09/2026</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>21/09/2026 HORA: 10:00 HS</t>
+          <t>28/9/2026 – 10:00 horas</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
-          <t>SIN COSTO</t>
+          <t>$25.000,00</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr">
@@ -1531,12 +1535,12 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Crespo</t>
         </is>
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>id-6ddfa0f2f1aa296d</t>
+          <t>id-1609ce58e128c413</t>
         </is>
       </c>
     </row>
@@ -1551,14 +1555,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>COLON — MUNICIPALIDAD DE COLON</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1566,20 +1570,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr"/>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>08/2026</t>
+        </is>
+      </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
+          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCL UIDO</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>24 de SEPTIEMBRE de 2026</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1589,7 +1597,7 @@
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>Sin Cargo</t>
+          <t>SIN COSTO</t>
         </is>
       </c>
       <c r="L15" s="6" t="inlineStr">
@@ -1609,7 +1617,7 @@
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>id-bc610b64999d147d</t>
+          <t>id-1590925c21c7e363</t>
         </is>
       </c>
     </row>
@@ -1624,14 +1632,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1641,30 +1649,34 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>10/26</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIU</t>
+          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="K16" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>$ 100 (Cien)</t>
+        </is>
+      </c>
       <c r="L16" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1682,7 +1694,7 @@
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>id-d97b43a99f1e1824</t>
+          <t>id-75a5c9dd5b4aa6f3</t>
         </is>
       </c>
     </row>
@@ -1697,14 +1709,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C17" s="9" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1714,27 +1726,27 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CI</t>
+          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K17" s="4" t="inlineStr"/>
@@ -1750,34 +1762,34 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos + CAFESG (Salto Grande)</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>id-f8fab7a7b3a06a2d</t>
+          <t>id-46c6d9f1f9210d1e</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>Materiales</t>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE CRESPO -- ENTRE RÍOS</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1787,30 +1799,30 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>05/2026</t>
+          <t>001-2026</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 145 metros lineales de modulo canal premoldeado cajón tipo pórtico de 2,00 X 1,00 (interior) X 1,00 mts. de longitud de hormigón para canalizar calle Los Quechuas al final</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>28/09/2026</t>
-        </is>
-      </c>
+          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr"/>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>28 de septiembre de 2026 10:00 Hs. Lugar: Sección Suministros, Palacio Municipal sito en 25 de mayo Nº 943, C</t>
+          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
-        </is>
-      </c>
-      <c r="K18" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L18" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1828,7 +1840,7 @@
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>id-61e8747a99305fe9</t>
+          <t>id-b7b0120caf49d551</t>
         </is>
       </c>
     </row>
@@ -1838,56 +1850,48 @@
           <t>11/09/2026</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C19" s="9" t="inlineStr">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>Materiales</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Municipalidad de Crespo</t>
+          <t>MUNICIPALIDAD DE URDINARRAIN</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>5/2026</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 145 metros lineales de módulo canal premoldeado.</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t>28/09/2026</t>
-        </is>
-      </c>
+          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr"/>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>28/9/2026 – 10:00 horas</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
-        </is>
-      </c>
-      <c r="K19" s="4" t="inlineStr">
-        <is>
-          <t>$25.000,00</t>
-        </is>
-      </c>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K19" s="4" t="inlineStr"/>
       <c r="L19" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1900,12 +1904,12 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Municipalidad de Crespo</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>id-1609ce58e128c413</t>
+          <t>id-7a200161bcc9b02b</t>
         </is>
       </c>
     </row>
@@ -1915,9 +1919,9 @@
           <t>11/09/2026</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -1927,7 +1931,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1937,22 +1941,18 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>08/2026</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCL UIDO</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>29/09/2026</t>
-        </is>
-      </c>
+          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr"/>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>29/09/2026</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1960,11 +1960,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K20" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K20" s="4" t="inlineStr"/>
       <c r="L20" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1982,29 +1978,29 @@
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>id-1590925c21c7e363</t>
+          <t>id-511256e6329e386a</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2014,22 +2010,18 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>10/26</t>
+          <t>03/26</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>30/09/2026</t>
-        </is>
-      </c>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr"/>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -2037,11 +2029,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K21" s="4" t="inlineStr">
-        <is>
-          <t>$ 100 (Cien)</t>
-        </is>
-      </c>
+      <c r="K21" s="4" t="inlineStr"/>
       <c r="L21" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2054,34 +2042,34 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-75a5c9dd5b4aa6f3</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+          <t>14/09/2026</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2091,22 +2079,18 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr">
-        <is>
-          <t>30/09/2026</t>
-        </is>
-      </c>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr"/>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -2127,19 +2111,19 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-46c6d9f1f9210d1e</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2147,14 +2131,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2164,18 +2148,18 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>001-2026</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr"/>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2183,11 +2167,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K23" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K23" s="4" t="inlineStr"/>
       <c r="L23" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2200,19 +2180,19 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-b7b0120caf49d551</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2220,14 +2200,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE URDINARRAIN</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2237,18 +2217,18 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>05/2025</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr"/>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -2269,19 +2249,19 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-7a200161bcc9b02b</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2289,14 +2269,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2306,18 +2286,18 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>06/2025</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr"/>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2338,19 +2318,19 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-511256e6329e386a</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2373,20 +2353,16 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>02/2025</t>
-        </is>
-      </c>
+      <c r="F26" s="4" t="inlineStr"/>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2394,11 +2370,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K26" s="4" t="inlineStr">
-        <is>
-          <t>$ 120.976,01</t>
-        </is>
-      </c>
+      <c r="K26" s="4" t="inlineStr"/>
       <c r="L26" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2416,14 +2388,14 @@
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-07ddb93a12c5a870</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2448,18 +2420,18 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>04/2025</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>Concurso de Precio N° 02/2025</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2485,7 +2457,7 @@
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-7c1bf02160a66f67</t>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
@@ -2500,31 +2472,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C28" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>03/2025</t>
+        </is>
+      </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2545,12 +2521,12 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-654eebef400f89cd</t>
+          <t>id-75bfffae63b7eedc</t>
         </is>
       </c>
     </row>
@@ -2572,28 +2548,28 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Concurso</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>01/26</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 06/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2614,12 +2590,12 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-9a16884dd5a64a49</t>
+          <t>id-07ddb93a12c5a870</t>
         </is>
       </c>
     </row>
@@ -2634,35 +2610,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C30" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>2026-1227</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+          <t>Concurso de Precio N° 02/2025</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 19/06/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2683,19 +2659,19 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-0691eb485d7548eb</t>
+          <t>id-7c1bf02160a66f67</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2705,33 +2681,29 @@
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>10-2026</t>
-        </is>
-      </c>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr"/>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
+          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego — figura como Pendiente</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2752,12 +2724,12 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-bdd0abb0374c3f42</t>
+          <t>id-654eebef400f89cd</t>
         </is>
       </c>
     </row>
@@ -2772,35 +2744,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Licitación Privada</t>
+          <t>Concurso</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>01/26</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego — figura como Pendiente</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2821,19 +2793,19 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-023b6b75e7014a9c</t>
+          <t>id-9a16884dd5a64a49</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>15/09/2026</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2841,7 +2813,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C33" s="8" t="inlineStr">
+      <c r="C33" s="9" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
@@ -2858,12 +2830,12 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>233/26</t>
+          <t>232/26</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>Reemplazo, provisión e instalación de las barreras vehiculares automáticas en el Edificio Central de Tribunales, de Paraná (sito Laprida N°250).</t>
+          <t>SERVICIO DE REACONDICIONAMIENTO Y REPARACIÓN EN SECTOR POSTERIOR DEL INMUEBLE ALQUILADO DEL JUZGADO DE PAZ DE SAN JAIME DE LA FRONTERA</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
@@ -2895,14 +2867,14 @@
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-f48b8e7889aac66c</t>
+          <t>id-5a01c3fd726f10dc</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>14/09/2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2910,9 +2882,9 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C34" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2922,17 +2894,17 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Concurso</t>
+          <t>Solicitud de Cotización</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>04/26</t>
+          <t>228/26</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>Edif. Tribunales – Chajarí, departamento de Federación. Obra “Reparaciones generales de baños e instalación eléctrica – 2° piso”</t>
+          <t>Solicitud de Cotización Nº 228/26, porContratación del servicio de recarga, revisión, prueba hidráulica y mantenimiento de los matafuegos ubicados en los Edificios de calle San Martín Nº15, Mitre Nº581 y Sarmiento Nº356 de la localidad de Victoria</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
@@ -2964,14 +2936,14 @@
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-2466cef612391e08</t>
+          <t>id-e125fe54abc33d69</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2981,33 +2953,33 @@
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Solicitud de Cotización</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>232/26</t>
+          <t>2026-1227</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE REACONDICIONAMIENTO Y REPARACIÓN EN SECTOR POSTERIOR DEL INMUEBLE ALQUILADO DEL JUZGADO DE PAZ DE SAN JAIME DE LA FRONTERA</t>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Ver el sitio</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3028,17 +3000,155 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-5a01c3fd726f10dc</t>
+          <t>id-0691eb485d7548eb</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>10-2026</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr"/>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego — figura como Pendiente</t>
+        </is>
+      </c>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K36" s="4" t="inlineStr"/>
+      <c r="L36" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M36" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="O36" s="4" t="inlineStr">
+        <is>
+          <t>id-bdd0abb0374c3f42</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C37" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Licitación Privada</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>04-2026</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr"/>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego — figura como Pendiente</t>
+        </is>
+      </c>
+      <c r="J37" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K37" s="4" t="inlineStr"/>
+      <c r="L37" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M37" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="O37" s="4" t="inlineStr">
+        <is>
+          <t>id-023b6b75e7014a9c</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O35"/>
+  <autoFilter ref="A1:O37"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -3108,6 +3218,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId67"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId72"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Arreglar los timeouts: era saturación propia, no sitios caídos
ENERSA, Oro Verde y CAFESG figuraban en ERROR por timeout, pero pedidas sueltas
responden en 2 a 5 segundos. El problema era el paralelismo: 6 fuentes a la vez
y el Boletín abriendo por dentro otras 6 descargas de PDFs de 2 MB, hasta 36
simultáneas ahogando la conexión.

Ahora 4 fuentes a la vez, 3 descargas dentro del Boletín, más margen de lectura
y un reintento ante timeout. Las 20 fuentes responden 200, cero errores.

Se reactiva Paraná: el bloqueo de Cloudflare resultó intermitente, no
permanente. Hoy trajo la 82/2026 (acondicionamiento de techo) y la 304/2026.
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -67,12 +67,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E6D9F2"/>
+        <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
+        <fgColor rgb="00E6D9F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -566,7 +566,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -643,7 +643,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>$ 100.000, 00.- (PESOS CIEN MIL CON 00/100)</t>
+          <t>$ 100.000, 00. - (PESOS CIEN MIL CON 00/100)</t>
         </is>
       </c>
       <c r="L3" s="6" t="inlineStr">
@@ -720,7 +720,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -728,51 +728,47 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>GOBIERNO DE ENTRE RÍOS — UNIDAD CENTRAL DE CONTRATACIONES</t>
+          <t>P ARANA — MINISTERIO DE SALUD</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación Publica</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>06/26</t>
+          <t>17/26</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Adquirir materiales de construcción (chapas, rollos de film de polietileno, tirantes, clavos y clavadoras)</t>
+          <t>Adquirir Una (01) Mesa de Anestesia. Destino: Hospital “San José” de Diamante, dependiente del Ministerio de Salud de la Provincia de Entre Ríos</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>06/10/2026</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>Unidad Central de Contrataciones, el día 17/09/26 a las 09:00 horas</t>
+          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>PESOS CINCUENTA MIL ($ 50.000)</t>
-        </is>
-      </c>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr"/>
       <c r="L4" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -790,14 +786,14 @@
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
-          <t>id-9dbdaa6090d92bd4</t>
+          <t>id-3312d89e1a3e2e53</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -805,14 +801,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE SEGUÍ</t>
+          <t>MUNICIPALIDAD DE CONCEPCIÓN DEL URUGUAY</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -822,22 +818,22 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>31/2026</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Us os Múltiples – Gimnasio Municipal”</t>
+          <t>“Pavimento Rígido – 03 (tres) Cuadras Barrio San Felipe”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026 a las 10:00 hs, en el Edificio Municipal</t>
+          <t>07 de octubre de 2026 Hora: 10:00</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -845,11 +841,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t>Gratuito</t>
-        </is>
-      </c>
+      <c r="K5" s="4" t="inlineStr"/>
       <c r="L5" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -867,14 +859,14 @@
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>id-90c3d1f38f49418a</t>
+          <t>id-76d9566cb30a6df5</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -882,14 +874,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -899,34 +891,30 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>015/2026</t>
+          <t>11/2026</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
+          <t>REFACCION EN ESCUELA N° 65 “ALMIRANTE BROWN” – CIUDAD DE CONCORDIA - DEPARTAMENTO CONCORDIA - PROVINCIA DE ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026. - Hora: 09:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDA</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t>$ 90.000,00. - (PESOS NOVENTA MIL CON 00/100)</t>
-        </is>
-      </c>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr"/>
       <c r="L6" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -944,14 +932,14 @@
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>id-74dfdad7e5f9d048</t>
+          <t>id-fc30d5c0b0589a79</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -959,14 +947,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -976,34 +964,30 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>09/26</t>
+          <t>13/2026</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “AMPLIACION - RECONSTRUCCION DE PISOS Y CONTRAPISOS -IMPERMEABILIZACION LOSAS- INSTALACION ELECTRICA-ESCUELA SECUNDARIA ADULTOS Nº 1 “DR. LUIS AGOTE” -NOGOYA-DEPARTAMENTO NOGOYA.”</t>
+          <t>REPARACIONES VARIAS EN C . P. E. F. Nº 3 “PROFESOR HUGO LA NASA” – CIUDAD DE CONCEPCION DEL URUGUAY - DEPARTAMENTO URUGUAY - PROVINCIA DE ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 18 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026. - Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDA</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K7" s="4" t="inlineStr">
-        <is>
-          <t>$ 100 (Cien)</t>
-        </is>
-      </c>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr"/>
       <c r="L7" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1021,14 +1005,14 @@
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>id-6a4a84712fd41a03</t>
+          <t>id-9d3847fb0e2b0929</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1036,14 +1020,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1053,27 +1037,27 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>12/2026</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
+          <t>RECAMBIO DE CUBIERTA Y REPARACIONES VARIAS EN ESCUELA Nº 92 “CONGRESO DE TUCUMAN” – CONCEPCION DEL URUGUAY - DPTO. URUGUAY – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026. - Hora: 10:30 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDA</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>06/10/2026</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr"/>
@@ -1089,19 +1073,19 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>id-885d4847519dfd48</t>
+          <t>id-059239b424b9c936</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1111,12 +1095,12 @@
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>GOBIERNO DE ENTRE RÍOS — UNIDAD CENTRAL DE CONTRATACIONES</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1126,22 +1110,22 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>07/2026</t>
+          <t>06/26</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”</t>
+          <t>Adquirir materiales de construcción (chapas, rollos de film de polietileno, tirantes, clavos y clavadoras)</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>21/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>21/09/2026 HORA: 10:00 HS</t>
+          <t>Unidad Central de Contrataciones, el día 17/09/26 a las 09:00 horas</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1151,7 +1135,7 @@
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>SIN COSTO</t>
+          <t>PESOS CINCUENTA MIL ($ 50.000)</t>
         </is>
       </c>
       <c r="L9" s="6" t="inlineStr">
@@ -1171,14 +1155,14 @@
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>id-6ddfa0f2f1aa296d</t>
+          <t>id-9dbdaa6090d92bd4</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1186,14 +1170,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>Materiales</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>COLON — MUNICIPALIDAD DE COLON</t>
+          <t>MUNICIPALIDAD DE SEGUÍ</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1201,20 +1185,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr"/>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>08-2026</t>
+        </is>
+      </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
+          <t>Adquisición de Materiales para la Obra Pública, según Planificación del “Proyecto: Vestuarios, Sanitarios y Salón de Us os Múltiples – Gimnasio Municipal”</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>24 de SEPTIEMBRE de 2026</t>
+          <t>17/09/2026 a las 10:00 hs, en el Edificio Municipal</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1224,7 +1212,7 @@
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>Sin Cargo</t>
+          <t>Gratuito</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr">
@@ -1244,14 +1232,14 @@
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>id-bc610b64999d147d</t>
+          <t>id-90c3d1f38f49418a</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1259,14 +1247,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1276,30 +1264,34 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>015/2026</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIU</t>
+          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="K11" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>$ 90.000,00. - (PESOS NOVENTA MIL CON 00/100)</t>
+        </is>
+      </c>
       <c r="L11" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1317,14 +1309,14 @@
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>id-d97b43a99f1e1824</t>
+          <t>id-74dfdad7e5f9d048</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1332,14 +1324,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1349,30 +1341,34 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>09/26</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “AMPLIACION - RECONSTRUCCION DE PISOS Y CONTRAPISOS -IMPERMEABILIZACION LOSAS- INSTALACION ELECTRICA-ESCUELA SECUNDARIA ADULTOS Nº 1 “DR. LUIS AGOTE” -NOGOYA-DEPARTAMENTO NOGOYA.”</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CI</t>
+          <t>DE LAS OFERTAS: el día 18 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="K12" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>$ 100 (Cien)</t>
+        </is>
+      </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1390,14 +1386,14 @@
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>id-f8fab7a7b3a06a2d</t>
+          <t>id-6a4a84712fd41a03</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1407,12 +1403,12 @@
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Materiales</t>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE CRESPO -- ENTRE RÍOS</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1422,27 +1418,27 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>05/2026</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 145 metros lineales de modulo canal premoldeado caj ón tipo pórtico de 2,00 X 1,00 (interior) X 1,00 mts. de longitud de hormigón para canalizar calle Los Quechuas al final</t>
+          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>28 de septiembre de 2026 10:00 Hs. Lugar: Sección Suministros, Palacio Municipal sito en 25 de mayo Nº 943, C</t>
+          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr"/>
@@ -1458,19 +1454,19 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>id-61e8747a99305fe9</t>
+          <t>id-885d4847519dfd48</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1480,47 +1476,47 @@
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Materiales</t>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Municipalidad de Crespo</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>5/2026</t>
+          <t>07/2026</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 145 metros lineales de módulo canal premoldeado.</t>
+          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>21/09/2026</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>28/9/2026 – 10:00 horas</t>
+          <t>21/09/2026 HORA: 10:00 HS</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
-          <t>$25.000,00</t>
+          <t>SIN COSTO</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr">
@@ -1535,19 +1531,19 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Municipalidad de Crespo</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>id-1609ce58e128c413</t>
+          <t>id-6ddfa0f2f1aa296d</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1555,39 +1551,39 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>CONCURSO DE PRECIOS</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>08/2026</t>
+          <t>304/2026</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCL UIDO</t>
+          <t>PROVISION E INSTALACION DE SISTEMA DE ILUMINACION</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>29/09/2026</t>
+          <t>21/09/2026</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>29/09/2026</t>
+          <t>21-09-2026 08:15</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1595,11 +1591,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K15" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K15" s="4" t="inlineStr"/>
       <c r="L15" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1612,19 +1604,19 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>id-1590925c21c7e363</t>
+          <t>id-cb965eafa60519ea</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1632,39 +1624,39 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>LICITACIÓN PÚBLICA</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>10/26</t>
+          <t>82/2026</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
+          <t>CONTRATACION DE SERVICIO DE MANO DE OBRA PARA ACONDICIONAMIENTO DE TECHO</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>22/09/2026</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>22-09-2026 08:00</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -1672,11 +1664,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K16" s="4" t="inlineStr">
-        <is>
-          <t>$ 100 (Cien)</t>
-        </is>
-      </c>
+      <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1689,19 +1677,19 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>id-75a5c9dd5b4aa6f3</t>
+          <t>id-e31ab37f1904ce3b</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1711,12 +1699,12 @@
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>COLON — MUNICIPALIDAD DE COLON</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1724,24 +1712,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>10/2026</t>
-        </is>
-      </c>
+      <c r="F17" s="4" t="inlineStr"/>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
+          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
+          <t>24 de SEPTIEMBRE de 2026</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1749,7 +1733,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K17" s="4" t="inlineStr"/>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>Sin Cargo</t>
+        </is>
+      </c>
       <c r="L17" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1762,34 +1750,34 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>id-46c6d9f1f9210d1e</t>
+          <t>id-bc610b64999d147d</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C18" s="9" t="inlineStr">
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
+          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1799,30 +1787,30 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>001-2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr"/>
+          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIU</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K18" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1840,29 +1828,29 @@
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>id-b7b0120caf49d551</t>
+          <t>id-d97b43a99f1e1824</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>Materiales</t>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE URDINARRAIN</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1872,23 +1860,27 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr"/>
+          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CI</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr"/>
@@ -1904,34 +1896,34 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Boletín Oficial de Entre Ríos + CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>id-7a200161bcc9b02b</t>
+          <t>id-f8fab7a7b3a06a2d</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
+          <t>MUNICIPALIDAD DE CRESPO -- ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1941,23 +1933,27 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>05/2026</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="inlineStr"/>
+          <t>Adquisición de 145 metros lineales de modulo canal premoldeado cajón tipo pórtico de 2,00 X 1,00 (interior) X 1,00 mts. de longitud de hormigón para canalizar calle Los Quechuas al final</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>28 de septiembre de 2026 10:00 Hs. Lugar: Sección Suministros, Palacio Municipal sito en 25 de mayo Nº 943, C</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="K20" s="4" t="inlineStr"/>
@@ -1978,58 +1974,66 @@
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>id-511256e6329e386a</t>
+          <t>id-61e8747a99305fe9</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Municipalidad de Crespo</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>03/26</t>
+          <t>5/2026</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr"/>
+          <t>Adquisición de 145 metros lineales de módulo canal premoldeado.</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>28/9/2026 – 10:00 horas</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K21" s="4" t="inlineStr"/>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>$25.000,00</t>
+        </is>
+      </c>
       <c r="L21" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2042,34 +2046,34 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Municipalidad de Crespo</t>
         </is>
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-1609ce58e128c413</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2079,18 +2083,22 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>02/2026</t>
+          <t>08/2026</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr"/>
+          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCL UIDO</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -2098,7 +2106,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K22" s="4" t="inlineStr"/>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L22" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2111,34 +2123,34 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-1590925c21c7e363</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2148,18 +2160,22 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>10/26</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr"/>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2167,7 +2183,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K23" s="4" t="inlineStr"/>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>$ 100 (Cien)</t>
+        </is>
+      </c>
       <c r="L23" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2180,34 +2200,34 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-75a5c9dd5b4aa6f3</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C24" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2217,18 +2237,22 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>05/2025</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr"/>
+          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -2249,19 +2273,19 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-46c6d9f1f9210d1e</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2269,14 +2293,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2286,18 +2310,18 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>06/2025</t>
+          <t>001-2026</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr"/>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2305,7 +2329,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K25" s="4" t="inlineStr"/>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L25" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2318,19 +2346,19 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
+          <t>id-b7b0120caf49d551</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2338,14 +2366,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>MUNICIPALIDAD DE URDINARRAIN</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2353,16 +2381,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr"/>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2383,19 +2415,19 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-ebeeb6a87e688d85</t>
+          <t>id-7a200161bcc9b02b</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2403,14 +2435,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2420,18 +2452,18 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>04/2025</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2452,19 +2484,19 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-34c85bcdb9b1123f</t>
+          <t>id-511256e6329e386a</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2489,18 +2521,18 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>03/2025</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
+          <t>Publicada 06/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2508,7 +2540,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K28" s="4" t="inlineStr"/>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>$ 120.976,01</t>
+        </is>
+      </c>
       <c r="L28" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2526,14 +2562,14 @@
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-75bfffae63b7eedc</t>
+          <t>id-07ddb93a12c5a870</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2563,13 +2599,13 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>Concurso de Precio N° 02/2025</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>Publicada 19/06/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2595,14 +2631,14 @@
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-07ddb93a12c5a870</t>
+          <t>id-7c1bf02160a66f67</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2610,35 +2646,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C30" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>02/2025</t>
-        </is>
-      </c>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr"/>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>Concurso de Precio N° 02/2025</t>
+          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2659,19 +2691,19 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-7c1bf02160a66f67</t>
+          <t>id-654eebef400f89cd</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2679,9 +2711,9 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2691,13 +2723,17 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr"/>
+          <t>Concurso</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>01/26</t>
+        </is>
+      </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
@@ -2729,14 +2765,14 @@
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-654eebef400f89cd</t>
+          <t>id-9a16884dd5a64a49</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2744,29 +2780,29 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C32" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Concurso</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>01/26</t>
+          <t>2026-1227</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
@@ -2793,19 +2829,19 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-9a16884dd5a64a49</t>
+          <t>id-0691eb485d7548eb</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2813,35 +2849,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C33" s="9" t="inlineStr">
+      <c r="C33" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Solicitud de Cotización</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>232/26</t>
+          <t>10-2026</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE REACONDICIONAMIENTO Y REPARACIÓN EN SECTOR POSTERIOR DEL INMUEBLE ALQUILADO DEL JUZGADO DE PAZ DE SAN JAIME DE LA FRONTERA</t>
+          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Ver el sitio</t>
+          <t>Ver pliego — figura como Pendiente</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2862,19 +2898,19 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-5a01c3fd726f10dc</t>
+          <t>id-bdd0abb0374c3f42</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>14/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2882,35 +2918,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Solicitud de Cotización</t>
+          <t>Licitación Privada</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>228/26</t>
+          <t>04-2026</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>Solicitud de Cotización Nº 228/26, porContratación del servicio de recarga, revisión, prueba hidráulica y mantenimiento de los matafuegos ubicados en los Edificios de calle San Martín Nº15, Mitre Nº581 y Sarmiento Nº356 de la localidad de Victoria</t>
+          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Ver el sitio</t>
+          <t>Ver pliego — figura como Pendiente</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -2931,19 +2967,19 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-e125fe54abc33d69</t>
+          <t>id-023b6b75e7014a9c</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2953,33 +2989,33 @@
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>Materiales</t>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Solicitud de Cotización</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>2026-1227</t>
+          <t>233/26</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+          <t>Reemplazo, provisión e instalación de las barreras vehiculares automáticas en el Edificio Central de Tribunales, de Paraná (sito Laprida N°250).</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Ver el sitio</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3000,19 +3036,19 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-0691eb485d7548eb</t>
+          <t>id-f48b8e7889aac66c</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3020,35 +3056,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C36" s="9" t="inlineStr">
+      <c r="C36" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Concurso</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>10-2026</t>
+          <t>04/26</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
+          <t>Edif. Tribunales – Chajarí, departamento de Federación. Obra “Reparaciones generales de baños e instalación eléctrica – 2° piso”</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego — figura como Pendiente</t>
+          <t>Ver el sitio</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3069,19 +3105,19 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>id-bdd0abb0374c3f42</t>
+          <t>id-2466cef612391e08</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3089,35 +3125,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C37" s="9" t="inlineStr">
+      <c r="C37" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Licitación Privada</t>
+          <t>Solicitud de Cotización</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>232/26</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
+          <t>SERVICIO DE REACONDICIONAMIENTO Y REPARACIÓN EN SECTOR POSTERIOR DEL INMUEBLE ALQUILADO DEL JUZGADO DE PAZ DE SAN JAIME DE LA FRONTERA</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego — figura como Pendiente</t>
+          <t>Ver el sitio</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3138,12 +3174,12 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>id-023b6b75e7014a9c</t>
+          <t>id-5a01c3fd726f10dc</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 18/09/2026 08:09
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -43,7 +43,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -53,6 +53,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F3A5F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -70,16 +75,6 @@
         <fgColor rgb="00E6D9F2"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -93,7 +88,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -106,7 +101,6 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -472,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O39"/>
+  <dimension ref="A1:O35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -582,12 +576,12 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Infraestructura</t>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
+          <t>COLON — MUNICIPALIDAD DE VILLA ELISA (E.R.)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -597,22 +591,22 @@
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>016/2026</t>
+          <t>004/26</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de mano de obra, materiales y equipamiento para ejecución de restitución de galibo y repavimentación en Avenida Belgrano y Avenida 1° de Mayo de esta ciudad de chajari</t>
+          <t>ADQUISICIÓN DE UN (1) VEHÍCULO PARA TRANSPORTE DE PASAJEROS DE (5) CINCO PLAZAS 0 KM - MODELO/AÑO 2026, PARA LA MUNICIPALIDAD DE LA CIUDAD DE VILLA ELISA, ENTRE RÍOS</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>02/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>02 DE OCTUBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>01 de OCTUBRE de 2026 a la hora 10:00 en la Oficina de Compras de la Municipalidad de Villa Elisa, Entre Ríos</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
@@ -622,7 +616,7 @@
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>$ 100.000, 00. - (PESOS CIEN MIL CON 00/100)</t>
+          <t xml:space="preserve">$ 20.000,00 (Pesos Veinte mil con 00/100) el que se puede adquirir en </t>
         </is>
       </c>
       <c r="L2" s="6" t="inlineStr">
@@ -642,14 +636,14 @@
       </c>
       <c r="O2" s="4" t="inlineStr">
         <is>
-          <t>id-53f1430f94acb0b0</t>
+          <t>id-0132097e777a3442</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>25/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -659,12 +653,12 @@
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -674,22 +668,22 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>07/2026</t>
+          <t>016/2026</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”, destinada a la obra denominada “Nueva Pileta en el Polideportivo El Aguará”,</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de mano de obra, materiales y equipamiento para ejecución de restitución de galibo y repavimentación en Avenida Belgrano y Avenida 1° de Mayo de esta ciudad de chajari</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
+          <t>02/10/2026</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026 HORA: 11:00 HS</t>
+          <t>02 DE OCTUBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -699,7 +693,7 @@
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>SIN COSTO</t>
+          <t>$ 100.000, 00. - (PESOS CIEN MIL CON 00/100)</t>
         </is>
       </c>
       <c r="L3" s="6" t="inlineStr">
@@ -719,7 +713,7 @@
       </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
-          <t>id-65d18d99bf0b2c6c</t>
+          <t>id-53f1430f94acb0b0</t>
         </is>
       </c>
     </row>
@@ -734,14 +728,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE SALUD</t>
+          <t>P ARANA — MINISTERIO DE SALUD</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -807,14 +801,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
+          <t>MUNICIPALIDAD DE CONCEPCIÓN DEL URUGUAY</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -872,7 +866,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>21/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -882,12 +876,12 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Materiales</t>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -897,27 +891,27 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>32/2026</t>
+          <t>11/2026</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>"Adquisición de 835 m3 de Hormigón Calidad H25 para 08 cuadras de Pavimento", en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>REFACCION EN ESCUELA N° 65 “ALMIRANTE BROWN” – CIUDAD DE CONCORDIA - DEPARTAMENTO CONCORDIA - PROVINCIA DE ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>08 de octubre de 2026 Hora: 10:00</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026. - Hora: 09:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDA</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>06/10/2026</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr"/>
@@ -938,14 +932,14 @@
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>id-0ace7de8f16d3baf</t>
+          <t>id-fc30d5c0b0589a79</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>21/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -953,14 +947,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -970,27 +964,27 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>33/2026</t>
+          <t>13/2026</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>“Pavimento Rígido – 04 (cuatro) Cuadras Barrio San Roque y 01 (una) Cuadra Barrio Vicente Obrego”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>REPARACIONES VARIAS EN C . P. E. F. Nº 3 “PROFESOR HUGO LA NASA” – CIUDAD DE CONCEPCION DEL URUGUAY - DEPARTAMENTO URUGUAY - PROVINCIA DE ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>08 de octubre de 2026 Hora: 11:00</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026. - Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDA</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>06/10/2026</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr"/>
@@ -1011,14 +1005,14 @@
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>id-fe71ac2aaf71b8d8</t>
+          <t>id-9d3847fb0e2b0929</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>21/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1026,14 +1020,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1043,27 +1037,27 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>34/2026</t>
+          <t>12/2026</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>“Concesión de la Explotación Comercial de un (01) Camión de Comidas Rápidas (para cubrir el total de cuatro puestos) en la Zona Joven – Parque La Salamanca de la Municipalidad de Concepción del Uruguay – Entre Ríos”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>RECAMBIO DE CUBIERTA Y REPARACIONES VARIAS EN ESCUELA Nº 92 “CONGRESO DE TUCUMAN” – CONCEPCION DEL URUGUAY - DPTO. URUGUAY – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>09 de octubre de 2026 Hora: 10:00</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026. - Hora: 10:30 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDA</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>06/10/2026</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr"/>
@@ -1084,54 +1078,54 @@
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>id-b147fbd9d3081bfc</t>
+          <t>id-059239b424b9c936</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>015/2026</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
           <t>18/09/2026</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>10/2026</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>“PROVISIÓN DE UNA (1) MINICARGADORA 0 KM, CON CUCHARÓN FRONTAL DE USO GENERAL, UN (1) MARTILLO HIDRÁULICO Y UN (1) COMPACTADOR/RODILLO VIBRATORIO LISO”</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>09/10/2026</t>
-        </is>
-      </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>09/10/2026 HORA: 10:00 HS</t>
+          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1141,7 +1135,7 @@
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>($ 270.000,00) PESOS DOSCIENTOS SETENTA MIL</t>
+          <t>$ 90.000,00. - (PESOS NOVENTA MIL CON 00/100)</t>
         </is>
       </c>
       <c r="L9" s="6" t="inlineStr">
@@ -1161,54 +1155,54 @@
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>id-779e4cd290f2e64e</t>
+          <t>id-74dfdad7e5f9d048</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>09/26</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “AMPLIACION - RECONSTRUCCION DE PISOS Y CONTRAPISOS -IMPERMEABILIZACION LOSAS- INSTALACION ELECTRICA-ESCUELA SECUNDARIA ADULTOS Nº 1 “DR. LUIS AGOTE” -NOGOYA-DEPARTAMENTO NOGOYA.”</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
           <t>18/09/2026</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>MUNICIPALIDAD DE SANTA ELENA</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>11/2026</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>OBRA "PAVIMENTACION URBANA CALLE TRATADO DEL PILAR B° 3 DE FEBRERO - MUNICIPALIDAD DE SANTA ELENA" (Según Pliegos de Bases y condi ciones)</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>13/10/2026</t>
-        </is>
-      </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026 HORA: 10: 00 HS</t>
+          <t>DE LAS OFERTAS: el día 18 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1218,7 +1212,7 @@
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>$ 728.000,00 PESOS SETECIENTOS VEINTIOCHO MIL</t>
+          <t>$ 100 (Cien)</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr">
@@ -1238,7 +1232,7 @@
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>id-1a2561509308b1b6</t>
+          <t>id-6a4a84712fd41a03</t>
         </is>
       </c>
     </row>
@@ -1253,14 +1247,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1270,27 +1264,27 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>11/2026</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>REFACCION EN ESCUELA N° 65 “ALMIRANTE BROWN” – CIUDAD DE CONCORDIA - DEPARTAMENTO CONCORDIA - PROVINCIA DE ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 09:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
+          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr"/>
@@ -1306,12 +1300,12 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>id-fc30d5c0b0589a79</t>
+          <t>id-885d4847519dfd48</t>
         </is>
       </c>
     </row>
@@ -1326,14 +1320,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1343,30 +1337,34 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>13/2026</t>
+          <t>07/2026</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>REPARACIONES VARIAS EN C. P. E. F. Nº 3 “PROFESOR HUGO LA NASA” – CIUDAD DE CONCEPCION DEL URUGUAY - DEPARTAMENTO URUGUAY - PROVINCIA D E ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026</t>
+          <t>21/09/2026</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
+          <t>21/09/2026 HORA: 10:00 HS</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
-        </is>
-      </c>
-      <c r="K12" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1384,7 +1382,7 @@
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>id-9d3847fb0e2b0929</t>
+          <t>id-6ddfa0f2f1aa296d</t>
         </is>
       </c>
     </row>
@@ -1401,42 +1399,42 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>CONCURSO DE PRECIOS</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>12/2026</t>
+          <t>304/2026</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>RECAMBIO DE CUBIERTA Y REPARACIONES VARIAS EN ESCUELA Nº 92 “CONGRESO DE TUCUMAN” – CONCEPCION DEL URUGUAY - DPTO. URUGUAY – PROVINCIA DE ENTRE RIOS de acuerdo a las c ondiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>PROVISION E INSTALACION DE SISTEMA DE ILUMINACION</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026</t>
+          <t>21/09/2026</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 10:30 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
+          <t>21-09-2026 08:15</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr"/>
@@ -1452,19 +1450,19 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>id-059239b424b9c936</t>
+          <t>id-cb965eafa60519ea</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1472,35 +1470,39 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE COLON</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr"/>
+          <t>LICITACIÓN PÚBLICA</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>82/2026</t>
+        </is>
+      </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN DE MATERIALES ELÉCTRICOS PARA EJECUCIÓN DEL PROYECTO DE RECONVERSIÓN Y OPTIMIZACIÓN DEL ALUMBRADO PÚBLICO DE LA CIUDAD DE COLÓN”</t>
+          <t>CONTRATACION DE SERVICIO DE MANO DE OBRA PARA ACONDICIONAMIENTO DE TECHO</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>14/10/2026</t>
+          <t>22/09/2026</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>14 de OCTUBRE de 2026</t>
+          <t>22-09-2026 08:00</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1508,11 +1510,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K14" s="4" t="inlineStr">
-        <is>
-          <t>Sin Cargo</t>
-        </is>
-      </c>
+      <c r="K14" s="4" t="inlineStr"/>
       <c r="L14" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1525,19 +1523,19 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>id-9e122d52de12ffef</t>
+          <t>id-e31ab37f1904ce3b</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1545,14 +1543,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t>Materiales</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>DIAMANTE — COMUNA ALDEA PROTESTANTE -- DIAMANTE -- ENTRE RÍOS</t>
+          <t>COLON — MUNICIPALIDAD DE COLON</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1560,24 +1558,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>03/2026</t>
-        </is>
-      </c>
+      <c r="F15" s="4" t="inlineStr"/>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Conforme a lo autorizado por decreto Nº 290/26 llámese a licitación pública Nº 03/26 con el objeto de comprar 10 toneladas de emulsión catiónica súper estable (asfalto de imprimación), puesto en Aldea Protestante</t>
+          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>14/10/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>miércoles 14 de octubre de 2026 – Hora nueve (09:00) Lugar de presentación de la oferta: Sede Comuna Aldea Protestan</t>
+          <t>24 de SEPTIEMBRE de 2026</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1585,7 +1579,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K15" s="4" t="inlineStr"/>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>Sin Cargo</t>
+        </is>
+      </c>
       <c r="L15" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1603,14 +1601,14 @@
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>id-c2f3a25cfb37fd38</t>
+          <t>id-bc610b64999d147d</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1618,14 +1616,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
+          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1635,34 +1633,30 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>017/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de UNA (1) MOTONIVELADORA, nueva, sin uso, cero km, con una potencia entre 220/240 HP, con opción a implementos, que será utilizada para el área del corralón municipal</t>
+          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>14/10/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>14 DE OCTUBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIU</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K16" s="4" t="inlineStr">
-        <is>
-          <t>$100.000,00. - (PESOS CIEN MIL CON 00/100) PRESUPUESTO OFICIAL ESTIMAD</t>
-        </is>
-      </c>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1680,14 +1674,14 @@
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>id-4c3b33859e596759</t>
+          <t>id-d97b43a99f1e1824</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>23/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1695,14 +1689,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>VICTORIA — MUNICIPALIDAD DE VICTORIA</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1712,27 +1706,27 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>008/2026</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Proveer a la Municipalidad de Victoria, Entre Ríos, de Veinticinco Mil (25.000) litros de Diésel 500, para movilidad de vehículos y maquinarias viales , Ocho Mil (8.000) litros de Gasoil Tipo euro o similar y Ocho (8.000) litros de nafta súper para vehículos y áreas afectadas a la Secretaria de Planeamiento y Dirección de Ambiente y Desarrollo sostenible;</t>
+          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>14/10/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>14 de octubre de 2026 a las 09:00 hs., en la Oficina de Compras de la Municipalidad de Victoria, Entr</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CI</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="K17" s="4" t="inlineStr"/>
@@ -1753,66 +1747,62 @@
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>id-a9af9f59c8c487c8</t>
+          <t>id-f8fab7a7b3a06a2d</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>MUNICIPALIDAD DE CRESPO -- ENTRE RÍOS</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>Adquisición de 145 metros lineales de modulo canal premoldeado cajón tipo pórtico de 2,00 X 1,00 (interior) X 1,00 mts. de longitud de hormigón para canalizar calle Los Quechuas al final</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
           <t>28/09/2026</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>MINISTERIO DE SALUD — GOBIERNO DE ENTRE RIOS</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>18/26</t>
-        </is>
-      </c>
-      <c r="G18" s="5" t="inlineStr">
-        <is>
-          <t>Adquirir Sesenta Mil (60.000) Kilogramos de Leche Entera en Polvo Instantánea, Fortificada con Hierro, Zinc y Ácido Ascórbico</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>16/10/2026</t>
-        </is>
-      </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
+          <t>28 de septiembre de 2026 10:00 Hs. Lugar: Sección Suministros, Palacio Municipal sito en 25 de mayo Nº 943, C</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K18" s="4" t="inlineStr">
-        <is>
-          <t>PESOS TRES MIL QUINIENTOS ($ 3.500,00)</t>
-        </is>
-      </c>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1830,60 +1820,64 @@
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>id-04a917d50ccab2e3</t>
+          <t>id-61e8747a99305fe9</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Municipalidad de Crespo</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Licitación</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>5/2026</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>Adquisición de 145 metros lineales de módulo canal premoldeado.</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
           <t>28/09/2026</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>VILLAGUAY — MUNICIPALIDAD DE VILLAGUAY</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr"/>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>Contratación, ejecución, liquidación, pago y recepción de la obra destinada a la elaboración del Proyecto Ejecutivo, provisión de materiales, mano de obra, equipos, ejecución, ensayos, habilitación y puesta en servicio de la instalación de gas natural para la Planta Municipal de Elaboración de Mezcla Asfáltica en Caliente, ubicada en el Lote N.º 4 de la Chacra N.º 263 del Parque Industrial de Villaguay, Provincia de Entre Ríos. La contratación comprenderá una solución i ntegral bajo modalidad “llave en mano”, incluyendo todos los trabajos, provisiones, trámites, representaciones técnicas, insp</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t>16/10/2026</t>
-        </is>
-      </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>16 de octubre del año 2026 a las 10:00 Horas, la que se realizara en la Ofici na de suministros de la Municipalidad de V</t>
+          <t>28/9/2026 – 10:00 horas</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>$ 50.000,00</t>
+          <t>$25.000,00</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr">
@@ -1898,19 +1892,19 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Crespo</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>id-55f1e5ca423a9262</t>
+          <t>id-1609ce58e128c413</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1920,12 +1914,12 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Infraestructura</t>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>SALUD ENTRE RÍOS S.A.U</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1933,20 +1927,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr"/>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>08/2026</t>
+        </is>
+      </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Contratación de Servicio de Viandas para el Hospital de la Baxada</t>
+          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCL UIDO</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>Hospital de la Baxada, calle Gral. Al varado Nº 2.250 Paraná, Entre Ríos, el día 19/10/2026 a las 10:00 hs</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1956,7 +1954,7 @@
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>SIN COSTO</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
@@ -1976,7 +1974,7 @@
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>id-d35d5e849089d7ac</t>
+          <t>id-1590925c21c7e363</t>
         </is>
       </c>
     </row>
@@ -1991,39 +1989,39 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>CONCURSO DE PRECIOS</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>304/2026</t>
+          <t>10/26</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>PROVISION E INSTALACION DE SISTEMA DE ILUMINACION</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>21/09/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>21-09-2026 08:15</t>
+          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -2031,7 +2029,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K21" s="4" t="inlineStr"/>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>$ 100 (Cien)</t>
+        </is>
+      </c>
       <c r="L21" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2044,19 +2046,19 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-cb965eafa60519ea</t>
+          <t>id-75a5c9dd5b4aa6f3</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -2064,14 +2066,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>PARANA — SALUD ENTRE RÍOS S.A.U</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2079,20 +2081,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr"/>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>10/2026</t>
+        </is>
+      </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Servicio de Recolección, Lavado, Desinfección, Secado, Planchado y Transporte de Ropa Hospitalaria</t>
+          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>21/10/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Hospital de la Baxada, calle Gral. Alvarado Nº 2.250 Paraná, Entre Ríos, el día 21/10/2026 a las 10:00 hs</t>
+          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -2100,11 +2106,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K22" s="4" t="inlineStr">
-        <is>
-          <t>Ninguno</t>
-        </is>
-      </c>
+      <c r="K22" s="4" t="inlineStr"/>
       <c r="L22" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2117,12 +2119,12 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-6b955df9d3f6241a</t>
+          <t>id-46c6d9f1f9210d1e</t>
         </is>
       </c>
     </row>
@@ -2132,44 +2134,40 @@
           <t>17/09/2026</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>82/2026</t>
+          <t>001-2026</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>CONTRATACION DE SERVICIO DE MANO DE OBRA PARA ACONDICIONAMIENTO DE TECHO</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t>22/09/2026</t>
-        </is>
-      </c>
+          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr"/>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>22-09-2026 08:00</t>
+          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2177,7 +2175,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K23" s="4" t="inlineStr"/>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L23" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2190,34 +2192,34 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-e31ab37f1904ce3b</t>
+          <t>id-b7b0120caf49d551</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C24" s="7" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>MUNICIPALIDAD DE URDINARRAIN</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2227,22 +2229,18 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>11/26</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “TERMINACION ESCUELA Nº 40 “JOSÉ ENRIQUE RODÓ”-SEPTIMO DISTRITO-DEPARTAMENTO GUALEGUAY.”</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>23/10/2026</t>
-        </is>
-      </c>
+          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr"/>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 23 de Octubre de 2026 a las 10:00 hs</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -2250,11 +2248,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K24" s="4" t="inlineStr">
-        <is>
-          <t>$ 100 (Cien)</t>
-        </is>
-      </c>
+      <c r="K24" s="4" t="inlineStr"/>
       <c r="L24" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2272,29 +2266,29 @@
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-86cc9c230734c462</t>
+          <t>id-7a200161bcc9b02b</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2304,22 +2298,18 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>11/2026</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>Terminación Escuela N° 40 "José Enrique Rodó", Séptimo Distrito</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>23/10/2026</t>
-        </is>
-      </c>
+          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr"/>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>viernes, 23 de octubre de 2026 - 10:00hs</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2340,12 +2330,12 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-322a40f5e43af35d</t>
+          <t>id-511256e6329e386a</t>
         </is>
       </c>
     </row>
@@ -2355,19 +2345,19 @@
           <t>17/09/2026</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2377,22 +2367,18 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>10/26</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
-        </is>
-      </c>
-      <c r="H26" s="4" t="inlineStr">
-        <is>
-          <t>30/09/2026</t>
-        </is>
-      </c>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>Publicada 06/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2402,7 +2388,7 @@
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>$ 100 (Cien)</t>
+          <t>$ 120.976,01</t>
         </is>
       </c>
       <c r="L26" s="6" t="inlineStr">
@@ -2417,12 +2403,12 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-75a5c9dd5b4aa6f3</t>
+          <t>id-07ddb93a12c5a870</t>
         </is>
       </c>
     </row>
@@ -2432,19 +2418,19 @@
           <t>17/09/2026</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2454,22 +2440,18 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="inlineStr">
-        <is>
-          <t>30/09/2026</t>
-        </is>
-      </c>
+          <t>Concurso de Precio N° 02/2025</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
+          <t>Publicada 19/06/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2490,19 +2472,19 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-46c6d9f1f9210d1e</t>
+          <t>id-7c1bf02160a66f67</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>25/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2512,33 +2494,29 @@
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>Vehículos</t>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>001/26</t>
-        </is>
-      </c>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr"/>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN de UN (1) FURGON UTILITARIO CHICO con 5 asientos 0 KM. con destino a Subsecretaria de Asistencia Directa y Emergencia</t>
+          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>DE LAS PROPUESTAS: 20 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2559,19 +2537,19 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-ca205f0874380f69</t>
+          <t>id-654eebef400f89cd</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2579,35 +2557,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C29" s="10" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Concurso</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>07/2026</t>
+          <t>01/26</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Transporte de mil doscientos cincuenta metros cúbicos (1.250 m³) de broza grillada desde Cantera “Tayreta” (Ruta Nacional N° 14 km 135) hasta jurisdicción de la comuna, de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Viernes 09 de octubre del corriente año a las 10:00 hs en la Oficina de la Sede de la Comuna</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2628,19 +2606,19 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-24e9015ecceeff7f</t>
+          <t>id-9a16884dd5a64a49</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2648,14 +2626,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>INSTITUTO CARBÓ S.R.L</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2663,16 +2641,20 @@
           <t>Licitación</t>
         </is>
       </c>
-      <c r="F30" s="4" t="inlineStr"/>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>2026-1227</t>
+        </is>
+      </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>sin internación en materia de salud, pre- hospitalarias, atención médica, domiciliaria y traslados sanitarios de alta</t>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2693,19 +2675,19 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-6aa57c7437a30ca3</t>
+          <t>id-0691eb485d7548eb</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>21/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2713,14 +2695,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE VIALE</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2730,18 +2712,18 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>08/26</t>
+          <t>10-2026</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>de asf alto 70-16 destinado a la producción de pavimento de la Planta Asfáltica, y que a continuación se detalla y</t>
+          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Ver pliego — figura como Pendiente</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2762,12 +2744,12 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-ef1ddb923c7e7fdb</t>
+          <t>id-bdd0abb0374c3f42</t>
         </is>
       </c>
     </row>
@@ -2782,35 +2764,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C32" s="7" t="inlineStr">
+      <c r="C32" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación Privada</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>001-2026</t>
+          <t>04-2026</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
+          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
+          <t>Ver pliego — figura como Pendiente</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2818,11 +2800,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K32" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K32" s="4" t="inlineStr"/>
       <c r="L32" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2835,12 +2813,12 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-b7b0120caf49d551</t>
+          <t>id-023b6b75e7014a9c</t>
         </is>
       </c>
     </row>
@@ -2857,33 +2835,33 @@
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>Materiales</t>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE URDINARRAIN</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Solicitud de Cotización</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>233/26</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
+          <t>Reemplazo, provisión e instalación de las barreras vehiculares automáticas en el Edificio Central de Tribunales, de Paraná (sito Laprida N°250).</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Ver el sitio</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2904,12 +2882,12 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-7a200161bcc9b02b</t>
+          <t>id-f48b8e7889aac66c</t>
         </is>
       </c>
     </row>
@@ -2924,35 +2902,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Concurso</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>04/26</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>Edif. Tribunales – Chajarí, departamento de Federación. Obra “Reparaciones generales de baños e instalación eléctrica – 2° piso”</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>Ver el sitio</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -2960,11 +2938,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K34" s="4" t="inlineStr">
-        <is>
-          <t>$ 120.976,01</t>
-        </is>
-      </c>
+      <c r="K34" s="4" t="inlineStr"/>
       <c r="L34" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2977,12 +2951,12 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-07ddb93a12c5a870</t>
+          <t>id-2466cef612391e08</t>
         </is>
       </c>
     </row>
@@ -2997,35 +2971,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Solicitud de Cotización</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>232/26</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>Concurso de Precio N° 02/2025</t>
+          <t>SERVICIO DE REACONDICIONAMIENTO Y REPARACIÓN EN SECTOR POSTERIOR DEL INMUEBLE ALQUILADO DEL JUZGADO DE PAZ DE SAN JAIME DE LA FRONTERA</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
+          <t>Ver el sitio</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3046,289 +3020,17 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-7c1bf02160a66f67</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr"/>
-      <c r="G36" s="5" t="inlineStr">
-        <is>
-          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
-        </is>
-      </c>
-      <c r="H36" s="4" t="inlineStr"/>
-      <c r="I36" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J36" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K36" s="4" t="inlineStr"/>
-      <c r="L36" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M36" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N36" t="inlineStr">
-        <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
-        </is>
-      </c>
-      <c r="O36" s="4" t="inlineStr">
-        <is>
-          <t>id-654eebef400f89cd</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Concurso</t>
-        </is>
-      </c>
-      <c r="F37" s="4" t="inlineStr">
-        <is>
-          <t>01/26</t>
-        </is>
-      </c>
-      <c r="G37" s="5" t="inlineStr">
-        <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
-        </is>
-      </c>
-      <c r="H37" s="4" t="inlineStr"/>
-      <c r="I37" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J37" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K37" s="4" t="inlineStr"/>
-      <c r="L37" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M37" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N37" t="inlineStr">
-        <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
-        </is>
-      </c>
-      <c r="O37" s="4" t="inlineStr">
-        <is>
-          <t>id-9a16884dd5a64a49</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>25/09/2026</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C38" s="7" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Poder Judicial de Entre Ríos</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F38" s="4" t="inlineStr">
-        <is>
-          <t>08/26</t>
-        </is>
-      </c>
-      <c r="G38" s="5" t="inlineStr">
-        <is>
-          <t>Obra “Readecuación del sistema de climatización –ala sur- Edificio Tribunales Gualeguay”.</t>
-        </is>
-      </c>
-      <c r="H38" s="4" t="inlineStr"/>
-      <c r="I38" s="4" t="inlineStr">
-        <is>
-          <t>Ver el sitio</t>
-        </is>
-      </c>
-      <c r="J38" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K38" s="4" t="inlineStr"/>
-      <c r="L38" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M38" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N38" t="inlineStr">
-        <is>
-          <t>Poder Judicial de Entre Ríos</t>
-        </is>
-      </c>
-      <c r="O38" s="4" t="inlineStr">
-        <is>
-          <t>id-9ca2387eef6d6fc1</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>ENERSA</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Licitación</t>
-        </is>
-      </c>
-      <c r="F39" s="4" t="inlineStr">
-        <is>
-          <t>2026-1227</t>
-        </is>
-      </c>
-      <c r="G39" s="5" t="inlineStr">
-        <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
-        </is>
-      </c>
-      <c r="H39" s="4" t="inlineStr"/>
-      <c r="I39" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J39" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K39" s="4" t="inlineStr"/>
-      <c r="L39" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M39" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>ENERSA</t>
-        </is>
-      </c>
-      <c r="O39" s="4" t="inlineStr">
-        <is>
-          <t>id-0691eb485d7548eb</t>
+          <t>id-5a01c3fd726f10dc</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O39"/>
+  <autoFilter ref="A1:O35"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -3398,14 +3100,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId67"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L38" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId76"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 19/09/2026 17:07
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$33</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O35"/>
+  <dimension ref="A1:O33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1093,14 +1093,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1110,12 +1110,12 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>015/2026</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la Provisión de 400 (CUATROCIENTOS) Equipos de luminarias para iluminación pública con tecnología LED 150, para ser colocadas en distintos sectores, con el fin de mejorar el aspecto de nuestra ciudad</t>
+          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>18 DE SEPTIEMBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1133,11 +1133,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>$ 90.000,00. - (PESOS NOVENTA MIL CON 00/100)</t>
-        </is>
-      </c>
+      <c r="K9" s="4" t="inlineStr"/>
       <c r="L9" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1150,12 +1146,12 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>id-74dfdad7e5f9d048</t>
+          <t>id-885d4847519dfd48</t>
         </is>
       </c>
     </row>
@@ -1177,7 +1173,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1187,22 +1183,22 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>09/26</t>
+          <t>07/2026</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “AMPLIACION - RECONSTRUCCION DE PISOS Y CONTRAPISOS -IMPERMEABILIZACION LOSAS- INSTALACION ELECTRICA-ESCUELA SECUNDARIA ADULTOS Nº 1 “DR. LUIS AGOTE” -NOGOYA-DEPARTAMENTO NOGOYA.”</t>
+          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>21/09/2026</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 18 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>21/09/2026 HORA: 10:00 HS</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1212,7 +1208,7 @@
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>$ 100 (Cien)</t>
+          <t>SIN COSTO</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr">
@@ -1232,7 +1228,7 @@
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>id-6a4a84712fd41a03</t>
+          <t>id-6ddfa0f2f1aa296d</t>
         </is>
       </c>
     </row>
@@ -1247,39 +1243,39 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>CONCURSO DE PRECIOS</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>304/2026</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
+          <t>PROVISION E INSTALACION DE SISTEMA DE ILUMINACION</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>21/09/2026</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
+          <t>21-09-2026 08:15</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1300,12 +1296,12 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>id-885d4847519dfd48</t>
+          <t>id-cb965eafa60519ea</t>
         </is>
       </c>
     </row>
@@ -1327,32 +1323,32 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>LICITACIÓN PÚBLICA</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>07/2026</t>
+          <t>82/2026</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”</t>
+          <t>CONTRATACION DE SERVICIO DE MANO DE OBRA PARA ACONDICIONAMIENTO DE TECHO</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>21/09/2026</t>
+          <t>22/09/2026</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>21/09/2026 HORA: 10:00 HS</t>
+          <t>22-09-2026 08:00</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
@@ -1360,11 +1356,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K12" s="4" t="inlineStr"/>
       <c r="L12" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1377,12 +1369,12 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>id-6ddfa0f2f1aa296d</t>
+          <t>id-e31ab37f1904ce3b</t>
         </is>
       </c>
     </row>
@@ -1397,39 +1389,35 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>COLON — MUNICIPALIDAD DE COLON</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>CONCURSO DE PRECIOS</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>304/2026</t>
-        </is>
-      </c>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr"/>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>PROVISION E INSTALACION DE SISTEMA DE ILUMINACION</t>
+          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>21/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>21-09-2026 08:15</t>
+          <t>24 de SEPTIEMBRE de 2026</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -1437,7 +1425,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K13" s="4" t="inlineStr"/>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>Sin Cargo</t>
+        </is>
+      </c>
       <c r="L13" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1450,12 +1442,12 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>id-cb965eafa60519ea</t>
+          <t>id-bc610b64999d147d</t>
         </is>
       </c>
     </row>
@@ -1477,37 +1469,37 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>82/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>CONTRATACION DE SERVICIO DE MANO DE OBRA PARA ACONDICIONAMIENTO DE TECHO</t>
+          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>22/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>22-09-2026 08:00</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIU</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr"/>
@@ -1523,12 +1515,12 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>id-e31ab37f1904ce3b</t>
+          <t>id-d97b43a99f1e1824</t>
         </is>
       </c>
     </row>
@@ -1543,14 +1535,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>COLON — MUNICIPALIDAD DE COLON</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1558,10 +1550,14 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr"/>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>09/2026</t>
+        </is>
+      </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
+          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
@@ -1571,19 +1567,15 @@
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>24 de SEPTIEMBRE de 2026</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CI</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K15" s="4" t="inlineStr">
-        <is>
-          <t>Sin Cargo</t>
-        </is>
-      </c>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr"/>
       <c r="L15" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1596,12 +1588,12 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Boletín Oficial de Entre Ríos + CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>id-bc610b64999d147d</t>
+          <t>id-f8fab7a7b3a06a2d</t>
         </is>
       </c>
     </row>
@@ -1616,14 +1608,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>MUNICIPALIDAD DE CRESPO -- ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1633,27 +1625,27 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>05/2026</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>Adquisición de 145 metros lineales de modulo canal premoldeado cajón tipo pórtico de 2,00 X 1,00 (interior) X 1,00 mts. de longitud de hormigón para canalizar calle Los Quechuas al final</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIU</t>
+          <t>28 de septiembre de 2026 10:00 Hs. Lugar: Sección Suministros, Palacio Municipal sito en 25 de mayo Nº 943, C</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr"/>
@@ -1674,7 +1666,7 @@
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>id-d97b43a99f1e1824</t>
+          <t>id-61e8747a99305fe9</t>
         </is>
       </c>
     </row>
@@ -1689,47 +1681,51 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>Municipalidad de Crespo</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>5/2026</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>Adquisición de 145 metros lineales de módulo canal premoldeado.</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CI</t>
+          <t>28/9/2026 – 10:00 horas</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="K17" s="4" t="inlineStr"/>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>$25.000,00</t>
+        </is>
+      </c>
       <c r="L17" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1742,12 +1738,12 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Crespo</t>
         </is>
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>id-f8fab7a7b3a06a2d</t>
+          <t>id-1609ce58e128c413</t>
         </is>
       </c>
     </row>
@@ -1762,14 +1758,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE CRESPO -- ENTRE RÍOS</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1779,30 +1775,34 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>05/2026</t>
+          <t>08/2026</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 145 metros lineales de modulo canal premoldeado cajón tipo pórtico de 2,00 X 1,00 (interior) X 1,00 mts. de longitud de hormigón para canalizar calle Los Quechuas al final</t>
+          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCL UIDO</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>28 de septiembre de 2026 10:00 Hs. Lugar: Sección Suministros, Palacio Municipal sito en 25 de mayo Nº 943, C</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
-        </is>
-      </c>
-      <c r="K18" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L18" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1820,7 +1820,7 @@
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>id-61e8747a99305fe9</t>
+          <t>id-1590925c21c7e363</t>
         </is>
       </c>
     </row>
@@ -1835,49 +1835,49 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Municipalidad de Crespo</t>
+          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>5/2026</t>
+          <t>10/26</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 145 metros lineales de módulo canal premoldeado.</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>28/9/2026 – 10:00 horas</t>
+          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>$25.000,00</t>
+          <t>$ 100 (Cien)</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr">
@@ -1892,12 +1892,12 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Municipalidad de Crespo</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>id-1609ce58e128c413</t>
+          <t>id-75a5c9dd5b4aa6f3</t>
         </is>
       </c>
     </row>
@@ -1912,14 +1912,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1929,22 +1929,22 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>08/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCL UIDO</t>
+          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>29/09/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>29/09/2026</t>
+          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1952,11 +1952,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K20" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K20" s="4" t="inlineStr"/>
       <c r="L20" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1969,12 +1965,12 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>id-1590925c21c7e363</t>
+          <t>id-46c6d9f1f9210d1e</t>
         </is>
       </c>
     </row>
@@ -1984,9 +1980,9 @@
           <t>17/09/2026</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
@@ -1996,7 +1992,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2006,22 +2002,18 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>10/26</t>
+          <t>001-2026</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>30/09/2026</t>
-        </is>
-      </c>
+          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr"/>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -2031,7 +2023,7 @@
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>$ 100 (Cien)</t>
+          <t>SIN COSTO</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr">
@@ -2051,7 +2043,7 @@
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-75a5c9dd5b4aa6f3</t>
+          <t>id-b7b0120caf49d551</t>
         </is>
       </c>
     </row>
@@ -2061,19 +2053,19 @@
           <t>17/09/2026</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>MUNICIPALIDAD DE URDINARRAIN</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2083,22 +2075,18 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr">
-        <is>
-          <t>30/09/2026</t>
-        </is>
-      </c>
+          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr"/>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -2119,12 +2107,12 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-46c6d9f1f9210d1e</t>
+          <t>id-7a200161bcc9b02b</t>
         </is>
       </c>
     </row>
@@ -2139,14 +2127,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
+          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2156,18 +2144,18 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>001-2026</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
+          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr"/>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2175,11 +2163,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K23" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K23" s="4" t="inlineStr"/>
       <c r="L23" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2197,7 +2181,7 @@
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-b7b0120caf49d551</t>
+          <t>id-511256e6329e386a</t>
         </is>
       </c>
     </row>
@@ -2219,28 +2203,28 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE URDINARRAIN</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>2026-1227</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr"/>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -2261,12 +2245,12 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-7a200161bcc9b02b</t>
+          <t>id-0691eb485d7548eb</t>
         </is>
       </c>
     </row>
@@ -2281,14 +2265,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2298,18 +2282,18 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>10-2026</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
+          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr"/>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Ver pliego — figura como Pendiente</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2330,12 +2314,12 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-511256e6329e386a</t>
+          <t>id-bdd0abb0374c3f42</t>
         </is>
       </c>
     </row>
@@ -2350,35 +2334,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación Privada</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>04-2026</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>Ver pliego — figura como Pendiente</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2386,11 +2370,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K26" s="4" t="inlineStr">
-        <is>
-          <t>$ 120.976,01</t>
-        </is>
-      </c>
+      <c r="K26" s="4" t="inlineStr"/>
       <c r="L26" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2403,19 +2383,19 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-07ddb93a12c5a870</t>
+          <t>id-023b6b75e7014a9c</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>19/09/2026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2423,35 +2403,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Solicitud de Cotización</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>235/26</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>Concurso de Precio N° 02/2025</t>
+          <t>Contratación de servicio para puesta en marcha de Grupo Electrógeno 30KVA, ubicado en el Edificio Tribunales de C. del Uruguay, calle San Martín Nº665.</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
+          <t>Ver el sitio</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2472,12 +2452,12 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-7c1bf02160a66f67</t>
+          <t>id-d3938e7b907594a8</t>
         </is>
       </c>
     </row>
@@ -2492,31 +2472,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C28" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr"/>
+          <t>Solicitud de Cotización</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>233/26</t>
+        </is>
+      </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
+          <t>Reemplazo, provisión e instalación de las barreras vehiculares automáticas en el Edificio Central de Tribunales, de Paraná (sito Laprida N°250).</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Ver el sitio</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2537,12 +2521,12 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-654eebef400f89cd</t>
+          <t>id-f48b8e7889aac66c</t>
         </is>
       </c>
     </row>
@@ -2557,14 +2541,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2574,18 +2558,18 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>01/26</t>
+          <t>04/26</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>Edif. Tribunales – Chajarí, departamento de Federación. Obra “Reparaciones generales de baños e instalación eléctrica – 2° piso”</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Ver el sitio</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2606,12 +2590,12 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-9a16884dd5a64a49</t>
+          <t>id-2466cef612391e08</t>
         </is>
       </c>
     </row>
@@ -2626,43 +2610,47 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C30" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>2026-1227</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
+          <t>Publicada 06/10/2025 — ver pliego</t>
+        </is>
+      </c>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="J30" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K30" s="4" t="inlineStr"/>
+      <c r="K30" s="4" t="inlineStr">
+        <is>
+          <t>$ 120.976,01</t>
+        </is>
+      </c>
       <c r="L30" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2675,12 +2663,12 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-0691eb485d7548eb</t>
+          <t>id-07ddb93a12c5a870</t>
         </is>
       </c>
     </row>
@@ -2695,14 +2683,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2712,18 +2700,18 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>10-2026</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
+          <t>Concurso de Precio N° 02/2025</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego — figura como Pendiente</t>
+          <t>Publicada 19/06/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2744,12 +2732,12 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-bdd0abb0374c3f42</t>
+          <t>id-7c1bf02160a66f67</t>
         </is>
       </c>
     </row>
@@ -2764,35 +2752,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Licitación Privada</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>04-2026</t>
-        </is>
-      </c>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr"/>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
+          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego — figura como Pendiente</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2813,12 +2797,12 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-023b6b75e7014a9c</t>
+          <t>id-654eebef400f89cd</t>
         </is>
       </c>
     </row>
@@ -2833,35 +2817,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C33" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Solicitud de Cotización</t>
+          <t>Concurso</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>233/26</t>
+          <t>01/26</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>Reemplazo, provisión e instalación de las barreras vehiculares automáticas en el Edificio Central de Tribunales, de Paraná (sito Laprida N°250).</t>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Ver el sitio</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2882,155 +2866,17 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-f48b8e7889aac66c</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C34" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Poder Judicial de Entre Ríos</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Concurso</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t>04/26</t>
-        </is>
-      </c>
-      <c r="G34" s="5" t="inlineStr">
-        <is>
-          <t>Edif. Tribunales – Chajarí, departamento de Federación. Obra “Reparaciones generales de baños e instalación eléctrica – 2° piso”</t>
-        </is>
-      </c>
-      <c r="H34" s="4" t="inlineStr"/>
-      <c r="I34" s="4" t="inlineStr">
-        <is>
-          <t>Ver el sitio</t>
-        </is>
-      </c>
-      <c r="J34" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K34" s="4" t="inlineStr"/>
-      <c r="L34" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M34" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>Poder Judicial de Entre Ríos</t>
-        </is>
-      </c>
-      <c r="O34" s="4" t="inlineStr">
-        <is>
-          <t>id-2466cef612391e08</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C35" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Poder Judicial de Entre Ríos</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Solicitud de Cotización</t>
-        </is>
-      </c>
-      <c r="F35" s="4" t="inlineStr">
-        <is>
-          <t>232/26</t>
-        </is>
-      </c>
-      <c r="G35" s="5" t="inlineStr">
-        <is>
-          <t>SERVICIO DE REACONDICIONAMIENTO Y REPARACIÓN EN SECTOR POSTERIOR DEL INMUEBLE ALQUILADO DEL JUZGADO DE PAZ DE SAN JAIME DE LA FRONTERA</t>
-        </is>
-      </c>
-      <c r="H35" s="4" t="inlineStr"/>
-      <c r="I35" s="4" t="inlineStr">
-        <is>
-          <t>Ver el sitio</t>
-        </is>
-      </c>
-      <c r="J35" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K35" s="4" t="inlineStr"/>
-      <c r="L35" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M35" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>Poder Judicial de Entre Ríos</t>
-        </is>
-      </c>
-      <c r="O35" s="4" t="inlineStr">
-        <is>
-          <t>id-5a01c3fd726f10dc</t>
+          <t>id-9a16884dd5a64a49</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O35"/>
+  <autoFilter ref="A1:O33"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -3096,10 +2942,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId62"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId63"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId68"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 20/09/2026 08:09
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O33"/>
+  <dimension ref="A1:O44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -735,7 +735,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>P ARANA — MINISTERIO DE SALUD</t>
+          <t>PARANA — MINISTERIO DE SALUD</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -808,7 +808,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE CONCEPCIÓN DEL URUGUAY</t>
+          <t>MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -866,7 +866,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -874,14 +874,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -891,30 +891,34 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>11/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>REFACCION EN ESCUELA N° 65 “ALMIRANTE BROWN” – CIUDAD DE CONCORDIA - DEPARTAMENTO CONCORDIA - PROVINCIA DE ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>“PROVISIÓN DE UNA (1) MINICARGADORA 0 KM, CON CUCHARÓN FRONTAL DE USO GENERAL, UN (1) MARTILLO HIDRÁULICO Y UN (1) COMPACTADOR/RODILLO VIBRATORIO LISO ”</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026. - Hora: 09:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDA</t>
+          <t>09/10/2026 HORA: 10:00 HS</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>($ 270.000,00) PESOS DOSCIENTOS SETENTA MIL</t>
+        </is>
+      </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -932,7 +936,7 @@
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>id-fc30d5c0b0589a79</t>
+          <t>id-779e4cd290f2e64e</t>
         </is>
       </c>
     </row>
@@ -964,12 +968,12 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>13/2026</t>
+          <t>11/2026</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>REPARACIONES VARIAS EN C . P. E. F. Nº 3 “PROFESOR HUGO LA NASA” – CIUDAD DE CONCEPCION DEL URUGUAY - DEPARTAMENTO URUGUAY - PROVINCIA DE ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>REFACCION EN ESCUELA N° 65 “ALMIRANTE BROWN” – CIUDAD DE CONCORDIA - DEPARTAMENTO CONCORDIA - PROVINCIA DE ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -979,7 +983,7 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026. - Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDA</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 09:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -1005,14 +1009,14 @@
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>id-9d3847fb0e2b0929</t>
+          <t>id-fc30d5c0b0589a79</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1020,14 +1024,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
+          <t>MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1037,12 +1041,12 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>12/2026</t>
+          <t>11/2026</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>RECAMBIO DE CUBIERTA Y REPARACIONES VARIAS EN ESCUELA Nº 92 “CONGRESO DE TUCUMAN” – CONCEPCION DEL URUGUAY - DPTO. URUGUAY – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>OBRA "PAVIMENTACION URBANA CALLE TRATADO DEL PILAR B° 3 DE FEBRERO - MUNICIPALIDAD DE SANTA ELENA" (Según Pliegos de Bases y condiciones)</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -1052,15 +1056,19 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026. - Hora: 10:30 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDA</t>
+          <t>13/10/2026 HORA: 10:00 HS</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
-        </is>
-      </c>
-      <c r="K8" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>$ 728.000,00 PESOS SETECIENTOS VEINTIOCHO MIL</t>
+        </is>
+      </c>
       <c r="L8" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1078,7 +1086,7 @@
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>id-059239b424b9c936</t>
+          <t>id-1a2561509308b1b6</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1108,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1110,27 +1118,27 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>13/2026</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Ampliación - Reconstrucción de pisos y contrapisos - Impermeabilización losas - Instalación eléctrica - Escuela Secundaria Adultos N° 1 "Dr. Luis Agote", Nogoyá</t>
+          <t>REPARACIONES VARIAS EN C. P. E. F. Nº 3 “PROFESOR HUGO LA NASA” – CIUDAD DE CONCEPCION DEL URUGUAY - DEPARTAMENTO URUGUAY - PROVINCIA D E ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>18/09/2026</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>viernes, 18 de septiembre de 2026 - 10:00hs</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>06/10/2026</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr"/>
@@ -1146,12 +1154,12 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>id-885d4847519dfd48</t>
+          <t>id-9d3847fb0e2b0929</t>
         </is>
       </c>
     </row>
@@ -1173,7 +1181,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1183,34 +1191,30 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>07/2026</t>
+          <t>12/2026</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”</t>
+          <t>RECAMBIO DE CUBIERTA Y REPARACIONES VARIAS EN ESCUELA Nº 92 “CONGRESO DE TUCUMAN” – CONCEPCION DEL URUGUAY - DPTO. URUGUAY – PROVINCIA DE ENTRE RIOS de acuerdo a las c ondiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>21/09/2026</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>21/09/2026 HORA: 10:00 HS</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 10:30 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K10" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr"/>
       <c r="L10" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1228,14 +1232,14 @@
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>id-6ddfa0f2f1aa296d</t>
+          <t>id-059239b424b9c936</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1250,32 +1254,28 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>SALUD ENTRE RÍOS S.A.U</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>CONCURSO DE PRECIOS</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>304/2026</t>
-        </is>
-      </c>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr"/>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>PROVISION E INSTALACION DE SISTEMA DE ILUMINACION</t>
+          <t>Contratación de Servicio de Viandas para el Hospital de la Baxada</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>21/09/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>21-09-2026 08:15</t>
+          <t>Hospital d e la Baxada, calle Gral. Alvarado Nº 2.250 Paraná, Entre Ríos, el día 19/10/2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1283,7 +1283,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K11" s="4" t="inlineStr"/>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
       <c r="L11" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1296,12 +1300,12 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>id-cb965eafa60519ea</t>
+          <t>id-d35d5e849089d7ac</t>
         </is>
       </c>
     </row>
@@ -1323,32 +1327,32 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>82/2026</t>
+          <t>07/2026</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>CONTRATACION DE SERVICIO DE MANO DE OBRA PARA ACONDICIONAMIENTO DE TECHO</t>
+          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>22/09/2026</t>
+          <t>21/09/2026</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>22-09-2026 08:00</t>
+          <t>21/09/2026 HORA: 10:00 HS</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
@@ -1356,7 +1360,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr"/>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1369,12 +1377,12 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>id-e31ab37f1904ce3b</t>
+          <t>id-6ddfa0f2f1aa296d</t>
         </is>
       </c>
     </row>
@@ -1389,35 +1397,39 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>COLON — MUNICIPALIDAD DE COLON</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr"/>
+          <t>CONCURSO DE PRECIOS</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>304/2026</t>
+        </is>
+      </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
+          <t>PROVISION E INSTALACION DE SISTEMA DE ILUMINACION</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>21/09/2026</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>24 de SEPTIEMBRE de 2026</t>
+          <t>21-09-2026 08:15</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -1425,11 +1437,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K13" s="4" t="inlineStr">
-        <is>
-          <t>Sin Cargo</t>
-        </is>
-      </c>
+      <c r="K13" s="4" t="inlineStr"/>
       <c r="L13" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1442,19 +1450,19 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>id-bc610b64999d147d</t>
+          <t>id-cb965eafa60519ea</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1462,14 +1470,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>SALUD ENTRE RÍOS S.A.U</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1477,32 +1485,32 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>10/2026</t>
-        </is>
-      </c>
+      <c r="F14" s="4" t="inlineStr"/>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>Servicio de Recolección, Lavado, Desinfección, Secado, Planchado y Transporte de Ropa Hospitalaria</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIU</t>
+          <t>Hospital de la Baxada, calle Gral. Alvarado Nº 2.250 Paraná, Entre Ríos, el día 21/10/2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="K14" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
       <c r="L14" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1520,7 +1528,7 @@
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>id-d97b43a99f1e1824</t>
+          <t>id-6b955df9d3f6241a</t>
         </is>
       </c>
     </row>
@@ -1542,37 +1550,37 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>LICITACIÓN PÚBLICA</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>82/2026</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>CONTRATACION DE SERVICIO DE MANO DE OBRA PARA ACONDICIONAMIENTO DE TECHO</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>22/09/2026</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CI</t>
+          <t>22-09-2026 08:00</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr"/>
@@ -1588,12 +1596,12 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos + CAFESG (Salto Grande)</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>id-f8fab7a7b3a06a2d</t>
+          <t>id-e31ab37f1904ce3b</t>
         </is>
       </c>
     </row>
@@ -1615,7 +1623,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE CRESPO -- ENTRE RÍOS</t>
+          <t>COLON — MUNICIPALIDAD DE COLON</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1623,32 +1631,32 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>05/2026</t>
-        </is>
-      </c>
+      <c r="F16" s="4" t="inlineStr"/>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 145 metros lineales de modulo canal premoldeado cajón tipo pórtico de 2,00 X 1,00 (interior) X 1,00 mts. de longitud de hormigón para canalizar calle Los Quechuas al final</t>
+          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>28 de septiembre de 2026 10:00 Hs. Lugar: Sección Suministros, Palacio Municipal sito en 25 de mayo Nº 943, C</t>
+          <t>24 de SEPTIEMBRE de 2026</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
-        </is>
-      </c>
-      <c r="K16" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>Sin Cargo</t>
+        </is>
+      </c>
       <c r="L16" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1666,7 +1674,7 @@
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>id-61e8747a99305fe9</t>
+          <t>id-bc610b64999d147d</t>
         </is>
       </c>
     </row>
@@ -1681,51 +1689,47 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Municipalidad de Crespo</t>
+          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>5/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 145 metros lineales de módulo canal premoldeado.</t>
+          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>28/9/2026 – 10:00 horas</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIU</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
-        </is>
-      </c>
-      <c r="K17" s="4" t="inlineStr">
-        <is>
-          <t>$25.000,00</t>
-        </is>
-      </c>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr"/>
       <c r="L17" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1738,12 +1742,12 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Municipalidad de Crespo</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>id-1609ce58e128c413</t>
+          <t>id-d97b43a99f1e1824</t>
         </is>
       </c>
     </row>
@@ -1758,14 +1762,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1775,34 +1779,30 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>08/2026</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCL UIDO</t>
+          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>29/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>29/09/2026</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CI</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K18" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="K18" s="4" t="inlineStr"/>
       <c r="L18" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1815,12 +1815,12 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Boletín Oficial de Entre Ríos + CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>id-1590925c21c7e363</t>
+          <t>id-f8fab7a7b3a06a2d</t>
         </is>
       </c>
     </row>
@@ -1835,14 +1835,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>MUNICIPALIDAD DE CRESPO -- ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1852,34 +1852,30 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>10/26</t>
+          <t>05/2026</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
+          <t>Adquisición de 145 metros lineales de modulo canal premoldeado cajón tipo pórtico de 2,00 X 1,00 (interior) X 1,00 mts. de longitud de hormigón para canalizar calle Los Quechuas al final</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>28 de septiembre de 2026 10:00 Hs. Lugar: Sección Suministros, Palacio Municipal sito en 25 de mayo Nº 943, C</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K19" s="4" t="inlineStr">
-        <is>
-          <t>$ 100 (Cien)</t>
-        </is>
-      </c>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="K19" s="4" t="inlineStr"/>
       <c r="L19" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1897,7 +1893,7 @@
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>id-75a5c9dd5b4aa6f3</t>
+          <t>id-61e8747a99305fe9</t>
         </is>
       </c>
     </row>
@@ -1912,47 +1908,51 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>Municipalidad de Crespo</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>5/2026</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
+          <t>Adquisición de 145 metros lineales de módulo canal premoldeado.</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
+          <t>28/9/2026 – 10:00 horas</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K20" s="4" t="inlineStr"/>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t>$25.000,00</t>
+        </is>
+      </c>
       <c r="L20" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1965,12 +1965,12 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Municipalidad de Crespo</t>
         </is>
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>id-46c6d9f1f9210d1e</t>
+          <t>id-1609ce58e128c413</t>
         </is>
       </c>
     </row>
@@ -1980,19 +1980,19 @@
           <t>17/09/2026</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2002,18 +2002,22 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>001-2026</t>
+          <t>08/2026</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr"/>
+          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCL UIDO</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -2043,7 +2047,7 @@
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-b7b0120caf49d551</t>
+          <t>id-1590925c21c7e363</t>
         </is>
       </c>
     </row>
@@ -2053,19 +2057,19 @@
           <t>17/09/2026</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE URDINARRAIN</t>
+          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2075,18 +2079,22 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>10/26</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr"/>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -2094,7 +2102,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K22" s="4" t="inlineStr"/>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>$ 100 (Cien)</t>
+        </is>
+      </c>
       <c r="L22" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2112,7 +2124,7 @@
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-7a200161bcc9b02b</t>
+          <t>id-75a5c9dd5b4aa6f3</t>
         </is>
       </c>
     </row>
@@ -2122,19 +2134,19 @@
           <t>17/09/2026</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2144,18 +2156,22 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr"/>
+          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2176,12 +2192,12 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-511256e6329e386a</t>
+          <t>id-46c6d9f1f9210d1e</t>
         </is>
       </c>
     </row>
@@ -2196,43 +2212,47 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>2026-1227</t>
+          <t>001-2026</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr"/>
       <c r="I24" s="4" t="inlineStr">
         <is>
+          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="J24" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K24" s="4" t="inlineStr"/>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L24" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2245,12 +2265,12 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-0691eb485d7548eb</t>
+          <t>id-b7b0120caf49d551</t>
         </is>
       </c>
     </row>
@@ -2265,14 +2285,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C25" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>MUNICIPALIDAD DE URDINARRAIN</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2282,18 +2302,18 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>10-2026</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
+          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr"/>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego — figura como Pendiente</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2314,12 +2334,12 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-bdd0abb0374c3f42</t>
+          <t>id-7a200161bcc9b02b</t>
         </is>
       </c>
     </row>
@@ -2334,35 +2354,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C26" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Licitación Privada</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
+          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego — figura como Pendiente</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2383,19 +2403,19 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-023b6b75e7014a9c</t>
+          <t>id-511256e6329e386a</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>19/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2403,35 +2423,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C27" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Solicitud de Cotización</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>235/26</t>
+          <t>03/26</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>Contratación de servicio para puesta en marcha de Grupo Electrógeno 30KVA, ubicado en el Edificio Tribunales de C. del Uruguay, calle San Martín Nº665.</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Ver el sitio</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2452,19 +2472,19 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-d3938e7b907594a8</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2472,35 +2492,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Solicitud de Cotización</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>233/26</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Reemplazo, provisión e instalación de las barreras vehiculares automáticas en el Edificio Central de Tribunales, de Paraná (sito Laprida N°250).</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Ver el sitio</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2521,19 +2541,19 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-f48b8e7889aac66c</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2541,35 +2561,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C29" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Concurso</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>04/26</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Edif. Tribunales – Chajarí, departamento de Federación. Obra “Reparaciones generales de baños e instalación eléctrica – 2° piso”</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Ver el sitio</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2590,19 +2610,19 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-2466cef612391e08</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2627,18 +2647,18 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>05/2025</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2646,11 +2666,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K30" s="4" t="inlineStr">
-        <is>
-          <t>$ 120.976,01</t>
-        </is>
-      </c>
+      <c r="K30" s="4" t="inlineStr"/>
       <c r="L30" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2668,14 +2684,14 @@
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-07ddb93a12c5a870</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2700,18 +2716,18 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>06/2025</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>Concurso de Precio N° 02/2025</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2737,14 +2753,14 @@
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-7c1bf02160a66f67</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2752,31 +2768,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C32" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr"/>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2797,19 +2813,19 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-654eebef400f89cd</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2824,28 +2840,28 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Concurso</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>01/26</t>
+          <t>04/2025</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2866,17 +2882,772 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
+          <t>IAPV — Viviendas</t>
+        </is>
+      </c>
+      <c r="O33" s="4" t="inlineStr">
+        <is>
+          <t>id-34c85bcdb9b1123f</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>20/09/2026</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>IAPV (Vivienda)</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>03/2025</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr"/>
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t>Publicada 08/10/2025 — ver pliego</t>
+        </is>
+      </c>
+      <c r="J34" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K34" s="4" t="inlineStr"/>
+      <c r="L34" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M34" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>IAPV — Viviendas</t>
+        </is>
+      </c>
+      <c r="O34" s="4" t="inlineStr">
+        <is>
+          <t>id-75bfffae63b7eedc</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>IAPV (Vivienda)</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>02/2025</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr"/>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>Publicada 06/10/2025 — ver pliego</t>
+        </is>
+      </c>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K35" s="4" t="inlineStr"/>
+      <c r="L35" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M35" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>IAPV — Viviendas</t>
+        </is>
+      </c>
+      <c r="O35" s="4" t="inlineStr">
+        <is>
+          <t>id-07ddb93a12c5a870</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>IAPV (Vivienda)</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>02/2025</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>Concurso de Precio N° 02/2025</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr"/>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>Publicada 19/06/2025 — ver pliego</t>
+        </is>
+      </c>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K36" s="4" t="inlineStr"/>
+      <c r="L36" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M36" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>IAPV — Viviendas</t>
+        </is>
+      </c>
+      <c r="O36" s="4" t="inlineStr">
+        <is>
+          <t>id-7c1bf02160a66f67</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C37" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
           <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
-      <c r="O33" s="4" t="inlineStr">
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr"/>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr"/>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J37" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K37" s="4" t="inlineStr"/>
+      <c r="L37" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M37" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="O37" s="4" t="inlineStr">
+        <is>
+          <t>id-654eebef400f89cd</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Concurso</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>01/26</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="inlineStr"/>
+      <c r="I38" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J38" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K38" s="4" t="inlineStr"/>
+      <c r="L38" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M38" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="O38" s="4" t="inlineStr">
         <is>
           <t>id-9a16884dd5a64a49</t>
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>ENERSA</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Licitación</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>2026-1227</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr"/>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K39" s="4" t="inlineStr"/>
+      <c r="L39" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M39" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>ENERSA</t>
+        </is>
+      </c>
+      <c r="O39" s="4" t="inlineStr">
+        <is>
+          <t>id-0691eb485d7548eb</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>10-2026</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="inlineStr"/>
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego — figura como Pendiente</t>
+        </is>
+      </c>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K40" s="4" t="inlineStr"/>
+      <c r="L40" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M40" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="O40" s="4" t="inlineStr">
+        <is>
+          <t>id-bdd0abb0374c3f42</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Licitación Privada</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>04-2026</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr"/>
+      <c r="I41" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego — figura como Pendiente</t>
+        </is>
+      </c>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K41" s="4" t="inlineStr"/>
+      <c r="L41" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M41" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="O41" s="4" t="inlineStr">
+        <is>
+          <t>id-023b6b75e7014a9c</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>19/09/2026</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Poder Judicial de Entre Ríos</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Solicitud de Cotización</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>235/26</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>Contratación de servicio para puesta en marcha de Grupo Electrógeno 30KVA, ubicado en el Edificio Tribunales de C. del Uruguay, calle San Martín Nº665.</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="inlineStr"/>
+      <c r="I42" s="4" t="inlineStr">
+        <is>
+          <t>Ver el sitio</t>
+        </is>
+      </c>
+      <c r="J42" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K42" s="4" t="inlineStr"/>
+      <c r="L42" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M42" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Poder Judicial de Entre Ríos</t>
+        </is>
+      </c>
+      <c r="O42" s="4" t="inlineStr">
+        <is>
+          <t>id-d3938e7b907594a8</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Poder Judicial de Entre Ríos</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Solicitud de Cotización</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>233/26</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>Reemplazo, provisión e instalación de las barreras vehiculares automáticas en el Edificio Central de Tribunales, de Paraná (sito Laprida N°250).</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr"/>
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>Ver el sitio</t>
+        </is>
+      </c>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K43" s="4" t="inlineStr"/>
+      <c r="L43" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M43" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>Poder Judicial de Entre Ríos</t>
+        </is>
+      </c>
+      <c r="O43" s="4" t="inlineStr">
+        <is>
+          <t>id-f48b8e7889aac66c</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Poder Judicial de Entre Ríos</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Concurso</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>04/26</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>Edif. Tribunales – Chajarí, departamento de Federación. Obra “Reparaciones generales de baños e instalación eléctrica – 2° piso”</t>
+        </is>
+      </c>
+      <c r="H44" s="4" t="inlineStr"/>
+      <c r="I44" s="4" t="inlineStr">
+        <is>
+          <t>Ver el sitio</t>
+        </is>
+      </c>
+      <c r="J44" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K44" s="4" t="inlineStr"/>
+      <c r="L44" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M44" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>Poder Judicial de Entre Ríos</t>
+        </is>
+      </c>
+      <c r="O44" s="4" t="inlineStr">
+        <is>
+          <t>id-2466cef612391e08</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O33"/>
+  <autoFilter ref="A1:O44"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -2942,6 +3713,28 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M32" r:id="rId62"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId63"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M33" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L38" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L43" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId86"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 21/09/2026 08:01
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O44"/>
+  <dimension ref="A1:O42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1815,7 +1815,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos + CAFESG (Salto Grande)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O18" s="4" t="inlineStr">
@@ -3304,7 +3304,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>19/09/2026</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3319,28 +3319,28 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Solicitud de Cotización</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>10-2026</t>
+          <t>235/26</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
+          <t>Contratación de servicio para puesta en marcha de Grupo Electrógeno 30KVA, ubicado en el Edificio Tribunales de C. del Uruguay, calle San Martín Nº665.</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr"/>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego — figura como Pendiente</t>
+          <t>Ver el sitio</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
@@ -3361,12 +3361,12 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
-          <t>id-bdd0abb0374c3f42</t>
+          <t>id-d3938e7b907594a8</t>
         </is>
       </c>
     </row>
@@ -3388,28 +3388,28 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Licitación Privada</t>
+          <t>Solicitud de Cotización</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>233/26</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
+          <t>Reemplazo, provisión e instalación de las barreras vehiculares automáticas en el Edificio Central de Tribunales, de Paraná (sito Laprida N°250).</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego — figura como Pendiente</t>
+          <t>Ver el sitio</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
@@ -3430,19 +3430,19 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
-          <t>id-023b6b75e7014a9c</t>
+          <t>id-f48b8e7889aac66c</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>19/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3462,17 +3462,17 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Solicitud de Cotización</t>
+          <t>Concurso</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>235/26</t>
+          <t>04/26</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>Contratación de servicio para puesta en marcha de Grupo Electrógeno 30KVA, ubicado en el Edificio Tribunales de C. del Uruguay, calle San Martín Nº665.</t>
+          <t>Edif. Tribunales – Chajarí, departamento de Federación. Obra “Reparaciones generales de baños e instalación eléctrica – 2° piso”</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr"/>
@@ -3504,150 +3504,12 @@
       </c>
       <c r="O42" s="4" t="inlineStr">
         <is>
-          <t>id-d3938e7b907594a8</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Poder Judicial de Entre Ríos</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Solicitud de Cotización</t>
-        </is>
-      </c>
-      <c r="F43" s="4" t="inlineStr">
-        <is>
-          <t>233/26</t>
-        </is>
-      </c>
-      <c r="G43" s="5" t="inlineStr">
-        <is>
-          <t>Reemplazo, provisión e instalación de las barreras vehiculares automáticas en el Edificio Central de Tribunales, de Paraná (sito Laprida N°250).</t>
-        </is>
-      </c>
-      <c r="H43" s="4" t="inlineStr"/>
-      <c r="I43" s="4" t="inlineStr">
-        <is>
-          <t>Ver el sitio</t>
-        </is>
-      </c>
-      <c r="J43" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K43" s="4" t="inlineStr"/>
-      <c r="L43" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M43" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>Poder Judicial de Entre Ríos</t>
-        </is>
-      </c>
-      <c r="O43" s="4" t="inlineStr">
-        <is>
-          <t>id-f48b8e7889aac66c</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Poder Judicial de Entre Ríos</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>Concurso</t>
-        </is>
-      </c>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t>04/26</t>
-        </is>
-      </c>
-      <c r="G44" s="5" t="inlineStr">
-        <is>
-          <t>Edif. Tribunales – Chajarí, departamento de Federación. Obra “Reparaciones generales de baños e instalación eléctrica – 2° piso”</t>
-        </is>
-      </c>
-      <c r="H44" s="4" t="inlineStr"/>
-      <c r="I44" s="4" t="inlineStr">
-        <is>
-          <t>Ver el sitio</t>
-        </is>
-      </c>
-      <c r="J44" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K44" s="4" t="inlineStr"/>
-      <c r="L44" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M44" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N44" t="inlineStr">
-        <is>
-          <t>Poder Judicial de Entre Ríos</t>
-        </is>
-      </c>
-      <c r="O44" s="4" t="inlineStr">
-        <is>
           <t>id-2466cef612391e08</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O44"/>
+  <autoFilter ref="A1:O42"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -3731,10 +3593,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId80"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId81"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L43" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId86"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 22/09/2026 08:00
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O42"/>
+  <dimension ref="A1:O41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1320,29 +1320,29 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>CONCURSO DE PRECIOS</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>07/2026</t>
+          <t>304/2026</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”</t>
+          <t>PROVISION E INSTALACION DE SISTEMA DE ILUMINACION</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>21/09/2026 HORA: 10:00 HS</t>
+          <t>21-09-2026 08:15</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
@@ -1360,11 +1360,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K12" s="4" t="inlineStr"/>
       <c r="L12" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1377,19 +1373,19 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>id-6ddfa0f2f1aa296d</t>
+          <t>id-cb965eafa60519ea</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1404,32 +1400,28 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>SALUD ENTRE RÍOS S.A.U</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>CONCURSO DE PRECIOS</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>304/2026</t>
-        </is>
-      </c>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr"/>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>PROVISION E INSTALACION DE SISTEMA DE ILUMINACION</t>
+          <t>Servicio de Recolección, Lavado, Desinfección, Secado, Planchado y Transporte de Ropa Hospitalaria</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>21/09/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>21-09-2026 08:15</t>
+          <t>Hospital de la Baxada, calle Gral. Alvarado Nº 2.250 Paraná, Entre Ríos, el día 21/10/2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -1437,7 +1429,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K13" s="4" t="inlineStr"/>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
       <c r="L13" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1450,19 +1446,19 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>id-cb965eafa60519ea</t>
+          <t>id-6b955df9d3f6241a</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1470,35 +1466,39 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>SALUD ENTRE RÍOS S.A.U</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr"/>
+          <t>LICITACIÓN PÚBLICA</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>82/2026</t>
+        </is>
+      </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Servicio de Recolección, Lavado, Desinfección, Secado, Planchado y Transporte de Ropa Hospitalaria</t>
+          <t>CONTRATACION DE SERVICIO DE MANO DE OBRA PARA ACONDICIONAMIENTO DE TECHO</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>21/10/2026</t>
+          <t>22/09/2026</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>Hospital de la Baxada, calle Gral. Alvarado Nº 2.250 Paraná, Entre Ríos, el día 21/10/2026 a las 10:00 hs</t>
+          <t>22-09-2026 08:00</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1506,11 +1506,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K14" s="4" t="inlineStr">
-        <is>
-          <t>Ninguno</t>
-        </is>
-      </c>
+      <c r="K14" s="4" t="inlineStr"/>
       <c r="L14" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1523,12 +1519,12 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>id-6b955df9d3f6241a</t>
+          <t>id-e31ab37f1904ce3b</t>
         </is>
       </c>
     </row>
@@ -1543,39 +1539,35 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>COLON — MUNICIPALIDAD DE COLON</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>82/2026</t>
-        </is>
-      </c>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr"/>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>CONTRATACION DE SERVICIO DE MANO DE OBRA PARA ACONDICIONAMIENTO DE TECHO</t>
+          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>22/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>22-09-2026 08:00</t>
+          <t>24 de SEPTIEMBRE de 2026</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1583,7 +1575,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K15" s="4" t="inlineStr"/>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>Sin Cargo</t>
+        </is>
+      </c>
       <c r="L15" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1596,12 +1592,12 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>id-e31ab37f1904ce3b</t>
+          <t>id-bc610b64999d147d</t>
         </is>
       </c>
     </row>
@@ -1616,14 +1612,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>COLON — MUNICIPALIDAD DE COLON</t>
+          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1631,10 +1627,14 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr"/>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>10/2026</t>
+        </is>
+      </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
+          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
@@ -1644,19 +1644,15 @@
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>24 de SEPTIEMBRE de 2026</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIU</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K16" s="4" t="inlineStr">
-        <is>
-          <t>Sin Cargo</t>
-        </is>
-      </c>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1674,7 +1670,7 @@
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>id-bc610b64999d147d</t>
+          <t>id-d97b43a99f1e1824</t>
         </is>
       </c>
     </row>
@@ -1696,7 +1692,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1706,12 +1702,12 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -1721,7 +1717,7 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIU</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CI</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1747,7 +1743,7 @@
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>id-d97b43a99f1e1824</t>
+          <t>id-f8fab7a7b3a06a2d</t>
         </is>
       </c>
     </row>
@@ -1762,14 +1758,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>MUNICIPALIDAD DE CRESPO -- ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1779,27 +1775,27 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>05/2026</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>Adquisición de 145 metros lineales de modulo canal premoldeado cajón tipo pórtico de 2,00 X 1,00 (interior) X 1,00 mts. de longitud de hormigón para canalizar calle Los Quechuas al final</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CI</t>
+          <t>28 de septiembre de 2026 10:00 Hs. Lugar: Sección Suministros, Palacio Municipal sito en 25 de mayo Nº 943, C</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr"/>
@@ -1820,7 +1816,7 @@
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>id-f8fab7a7b3a06a2d</t>
+          <t>id-61e8747a99305fe9</t>
         </is>
       </c>
     </row>
@@ -1842,22 +1838,22 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE CRESPO -- ENTRE RÍOS</t>
+          <t>Municipalidad de Crespo</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>05/2026</t>
+          <t>5/2026</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 145 metros lineales de modulo canal premoldeado cajón tipo pórtico de 2,00 X 1,00 (interior) X 1,00 mts. de longitud de hormigón para canalizar calle Los Quechuas al final</t>
+          <t>Adquisición de 145 metros lineales de módulo canal premoldeado.</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1867,15 +1863,19 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>28 de septiembre de 2026 10:00 Hs. Lugar: Sección Suministros, Palacio Municipal sito en 25 de mayo Nº 943, C</t>
+          <t>28/9/2026 – 10:00 horas</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
-        </is>
-      </c>
-      <c r="K19" s="4" t="inlineStr"/>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>$25.000,00</t>
+        </is>
+      </c>
       <c r="L19" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1888,12 +1888,12 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Crespo</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>id-61e8747a99305fe9</t>
+          <t>id-1609ce58e128c413</t>
         </is>
       </c>
     </row>
@@ -1908,49 +1908,49 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Municipalidad de Crespo</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>5/2026</t>
+          <t>08/2026</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 145 metros lineales de módulo canal premoldeado.</t>
+          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCL UIDO</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>28/9/2026 – 10:00 horas</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>$25.000,00</t>
+          <t>SIN COSTO</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
@@ -1965,12 +1965,12 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Municipalidad de Crespo</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>id-1609ce58e128c413</t>
+          <t>id-1590925c21c7e363</t>
         </is>
       </c>
     </row>
@@ -1985,14 +1985,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2002,22 +2002,22 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>08/2026</t>
+          <t>10/26</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCL UIDO</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>29/09/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>29/09/2026</t>
+          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -2027,7 +2027,7 @@
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>SIN COSTO</t>
+          <t>$ 100 (Cien)</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr">
@@ -2047,7 +2047,7 @@
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-1590925c21c7e363</t>
+          <t>id-75a5c9dd5b4aa6f3</t>
         </is>
       </c>
     </row>
@@ -2069,7 +2069,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2079,12 +2079,12 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>10/26</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
+          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -2094,7 +2094,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -2102,11 +2102,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K22" s="4" t="inlineStr">
-        <is>
-          <t>$ 100 (Cien)</t>
-        </is>
-      </c>
+      <c r="K22" s="4" t="inlineStr"/>
       <c r="L22" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2119,12 +2115,12 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-75a5c9dd5b4aa6f3</t>
+          <t>id-46c6d9f1f9210d1e</t>
         </is>
       </c>
     </row>
@@ -2134,9 +2130,9 @@
           <t>17/09/2026</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
@@ -2146,7 +2142,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2156,22 +2152,18 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>001-2026</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t>30/09/2026</t>
-        </is>
-      </c>
+          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr"/>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
+          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2179,7 +2171,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K23" s="4" t="inlineStr"/>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L23" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2192,12 +2188,12 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-46c6d9f1f9210d1e</t>
+          <t>id-b7b0120caf49d551</t>
         </is>
       </c>
     </row>
@@ -2212,14 +2208,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C24" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
+          <t>MUNICIPALIDAD DE URDINARRAIN</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2229,18 +2225,18 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>001-2026</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
+          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr"/>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -2248,11 +2244,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K24" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K24" s="4" t="inlineStr"/>
       <c r="L24" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2270,7 +2262,7 @@
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-b7b0120caf49d551</t>
+          <t>id-7a200161bcc9b02b</t>
         </is>
       </c>
     </row>
@@ -2285,14 +2277,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE URDINARRAIN</t>
+          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2302,12 +2294,12 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
+          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr"/>
@@ -2339,14 +2331,14 @@
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-7a200161bcc9b02b</t>
+          <t>id-511256e6329e386a</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2354,14 +2346,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2371,18 +2363,18 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>03/26</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2403,12 +2395,12 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-511256e6329e386a</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
@@ -2440,18 +2432,18 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>03/26</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2477,7 +2469,7 @@
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
@@ -2509,18 +2501,18 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>02/2026</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2546,7 +2538,7 @@
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
@@ -2578,18 +2570,18 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>05/2025</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2615,7 +2607,7 @@
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
@@ -2647,18 +2639,18 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>05/2025</t>
+          <t>06/2025</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2684,7 +2676,7 @@
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
@@ -2714,20 +2706,16 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>06/2025</t>
-        </is>
-      </c>
+      <c r="F31" s="4" t="inlineStr"/>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2753,7 +2741,7 @@
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
@@ -2783,16 +2771,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F32" s="4" t="inlineStr"/>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>04/2025</t>
+        </is>
+      </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2818,7 +2810,7 @@
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-ebeeb6a87e688d85</t>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
@@ -2850,18 +2842,18 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>04/2025</t>
+          <t>03/2025</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2887,14 +2879,14 @@
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-34c85bcdb9b1123f</t>
+          <t>id-75bfffae63b7eedc</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2919,18 +2911,18 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>03/2025</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
+          <t>Publicada 06/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -2956,7 +2948,7 @@
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-75bfffae63b7eedc</t>
+          <t>id-07ddb93a12c5a870</t>
         </is>
       </c>
     </row>
@@ -2993,13 +2985,13 @@
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>Concurso de Precio N° 02/2025</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>Publicada 19/06/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3025,7 +3017,7 @@
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-07ddb93a12c5a870</t>
+          <t>id-7c1bf02160a66f67</t>
         </is>
       </c>
     </row>
@@ -3040,35 +3032,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C36" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C36" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>02/2025</t>
-        </is>
-      </c>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr"/>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>Concurso de Precio N° 02/2025</t>
+          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3089,12 +3077,12 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>id-7c1bf02160a66f67</t>
+          <t>id-654eebef400f89cd</t>
         </is>
       </c>
     </row>
@@ -3109,9 +3097,9 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C37" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -3121,13 +3109,17 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F37" s="4" t="inlineStr"/>
+          <t>Concurso</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>01/26</t>
+        </is>
+      </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
@@ -3159,7 +3151,7 @@
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>id-654eebef400f89cd</t>
+          <t>id-9a16884dd5a64a49</t>
         </is>
       </c>
     </row>
@@ -3174,29 +3166,29 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C38" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C38" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Concurso</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>01/26</t>
+          <t>2026-1227</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
@@ -3223,19 +3215,19 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>id-9a16884dd5a64a49</t>
+          <t>id-0691eb485d7548eb</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>19/09/2026</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3243,35 +3235,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C39" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Solicitud de Cotización</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>2026-1227</t>
+          <t>235/26</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+          <t>Contratación de servicio para puesta en marcha de Grupo Electrógeno 30KVA, ubicado en el Edificio Tribunales de C. del Uruguay, calle San Martín Nº665.</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Ver el sitio</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -3292,19 +3284,19 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
-          <t>id-0691eb485d7548eb</t>
+          <t>id-d3938e7b907594a8</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>19/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3329,12 +3321,12 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>235/26</t>
+          <t>233/26</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>Contratación de servicio para puesta en marcha de Grupo Electrógeno 30KVA, ubicado en el Edificio Tribunales de C. del Uruguay, calle San Martín Nº665.</t>
+          <t>Reemplazo, provisión e instalación de las barreras vehiculares automáticas en el Edificio Central de Tribunales, de Paraná (sito Laprida N°250).</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr"/>
@@ -3366,7 +3358,7 @@
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
-          <t>id-d3938e7b907594a8</t>
+          <t>id-f48b8e7889aac66c</t>
         </is>
       </c>
     </row>
@@ -3393,17 +3385,17 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Solicitud de Cotización</t>
+          <t>Concurso</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>233/26</t>
+          <t>04/26</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>Reemplazo, provisión e instalación de las barreras vehiculares automáticas en el Edificio Central de Tribunales, de Paraná (sito Laprida N°250).</t>
+          <t>Edif. Tribunales – Chajarí, departamento de Federación. Obra “Reparaciones generales de baños e instalación eléctrica – 2° piso”</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
@@ -3435,81 +3427,12 @@
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
-          <t>id-f48b8e7889aac66c</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Poder Judicial de Entre Ríos</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Concurso</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="inlineStr">
-        <is>
-          <t>04/26</t>
-        </is>
-      </c>
-      <c r="G42" s="5" t="inlineStr">
-        <is>
-          <t>Edif. Tribunales – Chajarí, departamento de Federación. Obra “Reparaciones generales de baños e instalación eléctrica – 2° piso”</t>
-        </is>
-      </c>
-      <c r="H42" s="4" t="inlineStr"/>
-      <c r="I42" s="4" t="inlineStr">
-        <is>
-          <t>Ver el sitio</t>
-        </is>
-      </c>
-      <c r="J42" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K42" s="4" t="inlineStr"/>
-      <c r="L42" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M42" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>Poder Judicial de Entre Ríos</t>
-        </is>
-      </c>
-      <c r="O42" s="4" t="inlineStr">
-        <is>
           <t>id-2466cef612391e08</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O42"/>
+  <autoFilter ref="A1:O41"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -3591,8 +3514,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId78"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId79"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId82"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 23/09/2026 08:00
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$48</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -62,17 +62,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00E6D9F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E6D9F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O41"/>
+  <dimension ref="A1:O48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -643,7 +643,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>23/09/2026</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -653,37 +653,37 @@
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>Infraestructura</t>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>LICITACIÓN PÚBLICA</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>016/2026</t>
+          <t>86/2026</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de mano de obra, materiales y equipamiento para ejecución de restitución de galibo y repavimentación en Avenida Belgrano y Avenida 1° de Mayo de esta ciudad de chajari</t>
+          <t>ADQUISICION DE CAL VIVA AEREA</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>02/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>02 DE OCTUBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>01-10-2026 08:00</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -691,11 +691,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>$ 100.000, 00. - (PESOS CIEN MIL CON 00/100)</t>
-        </is>
-      </c>
+      <c r="K3" s="4" t="inlineStr"/>
       <c r="L3" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -708,12 +704,12 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
-          <t>id-53f1430f94acb0b0</t>
+          <t>id-ee4153887a6e1e8d</t>
         </is>
       </c>
     </row>
@@ -728,47 +724,51 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE SALUD</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Licitación Publica</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>17/26</t>
+          <t>016/2026</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Adquirir Una (01) Mesa de Anestesia. Destino: Hospital “San José” de Diamante, dependiente del Ministerio de Salud de la Provincia de Entre Ríos</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de mano de obra, materiales y equipamiento para ejecución de restitución de galibo y repavimentación en Avenida Belgrano y Avenida 1° de Mayo de esta ciudad de chajari</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
+          <t>02/10/2026</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
+          <t>02 DE OCTUBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>$ 100.000, 00. - (PESOS CIEN MIL CON 00/100)</t>
+        </is>
+      </c>
       <c r="L4" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -786,7 +786,7 @@
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
-          <t>id-3312d89e1a3e2e53</t>
+          <t>id-53f1430f94acb0b0</t>
         </is>
       </c>
     </row>
@@ -801,44 +801,44 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
+          <t>PARANA — MINISTERIO DE SALUD</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación Publica</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>31/2026</t>
+          <t>17/26</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>“Pavimento Rígido – 03 (tres) Cuadras Barrio San Felipe”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>Adquirir Una (01) Mesa de Anestesia. Destino: Hospital “San José” de Diamante, dependiente del Ministerio de Salud de la Provincia de Entre Ríos</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>06/10/2026</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>07 de octubre de 2026 Hora: 10:00</t>
+          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>06/10/2026</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr"/>
@@ -859,14 +859,14 @@
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>id-76d9566cb30a6df5</t>
+          <t>id-3312d89e1a3e2e53</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -874,14 +874,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -891,22 +891,22 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>31/2026</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>“PROVISIÓN DE UNA (1) MINICARGADORA 0 KM, CON CUCHARÓN FRONTAL DE USO GENERAL, UN (1) MARTILLO HIDRÁULICO Y UN (1) COMPACTADOR/RODILLO VIBRATORIO LISO ”</t>
+          <t>“Pavimento Rígido – 03 (tres) Cuadras Barrio San Felipe”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>09/10/2026 HORA: 10:00 HS</t>
+          <t>07 de octubre de 2026 Hora: 10:00</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -914,11 +914,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t>($ 270.000,00) PESOS DOSCIENTOS SETENTA MIL</t>
-        </is>
-      </c>
+      <c r="K6" s="4" t="inlineStr"/>
       <c r="L6" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -936,14 +932,14 @@
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>id-779e4cd290f2e64e</t>
+          <t>id-76d9566cb30a6df5</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>23/09/2026</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -951,14 +947,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
+          <t>MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -968,27 +964,27 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>11/2026</t>
+          <t>32/2026</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>REFACCION EN ESCUELA N° 65 “ALMIRANTE BROWN” – CIUDAD DE CONCORDIA - DEPARTAMENTO CONCORDIA - PROVINCIA DE ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>"Adquisición de 835 m3 de Hormigón Calidad H25 para 08 cuadras de Pavimento", en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 09:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
+          <t>08 de octubre de 2026 Hora: 10:00</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr"/>
@@ -1009,14 +1005,14 @@
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>id-fc30d5c0b0589a79</t>
+          <t>id-0ace7de8f16d3baf</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>23/09/2026</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1024,14 +1020,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1041,22 +1037,22 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>11/2026</t>
+          <t>33/2026</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>OBRA "PAVIMENTACION URBANA CALLE TRATADO DEL PILAR B° 3 DE FEBRERO - MUNICIPALIDAD DE SANTA ELENA" (Según Pliegos de Bases y condiciones)</t>
+          <t>“Pavimento Rígido – 04 (cuatro) Cuadras Barrio San Roque y 01 (una) Cuadra Barrio Vicente Obrego”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026 HORA: 10:00 HS</t>
+          <t>08 de octubre de 2026 Hora: 11:00</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -1064,11 +1060,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr">
-        <is>
-          <t>$ 728.000,00 PESOS SETECIENTOS VEINTIOCHO MIL</t>
-        </is>
-      </c>
+      <c r="K8" s="4" t="inlineStr"/>
       <c r="L8" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1086,14 +1078,14 @@
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>id-1a2561509308b1b6</t>
+          <t>id-fe71ac2aaf71b8d8</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1101,14 +1093,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1118,30 +1110,34 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>13/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>REPARACIONES VARIAS EN C. P. E. F. Nº 3 “PROFESOR HUGO LA NASA” – CIUDAD DE CONCEPCION DEL URUGUAY - DEPARTAMENTO URUGUAY - PROVINCIA D E ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>“PROVISIÓN DE UNA (1) MINICARGADORA 0 KM, CON CUCHARÓN FRONTAL DE USO GENERAL, UN (1) MARTILLO HIDRÁULICO Y UN (1) COMPACTADOR/RODILLO VIBRATORIO LISO”</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
+          <t>09/10/2026 HORA: 10:00 HS</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
-        </is>
-      </c>
-      <c r="K9" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>($ 270.000,00) PESOS DOSCIENTOS SETENTA MIL</t>
+        </is>
+      </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1159,14 +1155,14 @@
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>id-9d3847fb0e2b0929</t>
+          <t>id-779e4cd290f2e64e</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>23/09/2026</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1174,14 +1170,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
+          <t>MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1191,27 +1187,27 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>12/2026</t>
+          <t>34/2026</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>RECAMBIO DE CUBIERTA Y REPARACIONES VARIAS EN ESCUELA Nº 92 “CONGRESO DE TUCUMAN” – CONCEPCION DEL URUGUAY - DPTO. URUGUAY – PROVINCIA DE ENTRE RIOS de acuerdo a las c ondiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>“ Concesión de la Explotación Comercial de un (01) Camión de Comidas Rápidas (para cubrir el total de cuatro puestos) en la Zona Joven – Parque La Salamanca de la Municipalidad de Concepción del Uruguay – Entre Ríos”, en un todo de acuerdo a los Pliegos de B ases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 10:30 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
+          <t>09 de octubre de 2026 Hora: 10:00</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr"/>
@@ -1232,7 +1228,7 @@
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>id-059239b424b9c936</t>
+          <t>id-b147fbd9d3081bfc</t>
         </is>
       </c>
     </row>
@@ -1247,14 +1243,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>SALUD ENTRE RÍOS S.A.U</t>
+          <t>MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1262,20 +1258,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr"/>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>11/2026</t>
+        </is>
+      </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Contratación de Servicio de Viandas para el Hospital de la Baxada</t>
+          <t>OBRA "PAVIMENTACION URBANA CALLE TRATADO DEL PILAR B° 3 DE FEBRERO - MUNICIPALIDAD DE SANTA ELENA" (Según Pliegos de Bases y condi ciones)</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>Hospital d e la Baxada, calle Gral. Alvarado Nº 2.250 Paraná, Entre Ríos, el día 19/10/2026 a las 10:00 hs</t>
+          <t>13/10/2026 HORA: 10: 00 HS</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>$ 728.000,00 PESOS SETECIENTOS VEINTIOCHO MIL</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>id-d35d5e849089d7ac</t>
+          <t>id-1a2561509308b1b6</t>
         </is>
       </c>
     </row>
@@ -1320,44 +1320,44 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>CONCURSO DE PRECIOS</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>304/2026</t>
+          <t>11/2026</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>PROVISION E INSTALACION DE SISTEMA DE ILUMINACION</t>
+          <t>REFACCION EN ESCUELA N° 65 “ALMIRANTE BROWN” – CIUDAD DE CONCORDIA - DEPARTAMENTO CONCORDIA - PROVINCIA DE ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>21/09/2026</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>21-09-2026 08:15</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 09:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>06/10/2026</t>
         </is>
       </c>
       <c r="K12" s="4" t="inlineStr"/>
@@ -1373,19 +1373,19 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>id-cb965eafa60519ea</t>
+          <t>id-fc30d5c0b0589a79</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1393,14 +1393,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>SALUD ENTRE RÍOS S.A.U</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1408,32 +1408,32 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr"/>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>13/2026</t>
+        </is>
+      </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Servicio de Recolección, Lavado, Desinfección, Secado, Planchado y Transporte de Ropa Hospitalaria</t>
+          <t>REPARACIONES VARIAS EN C. P. E. F. Nº 3 “PROFESOR HUGO LA NASA” – CIUDAD DE CONCEPCION DEL URUGUAY - DEPARTAMENTO URUGUAY - PROVINCIA D E ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>21/10/2026</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>Hospital de la Baxada, calle Gral. Alvarado Nº 2.250 Paraná, Entre Ríos, el día 21/10/2026 a las 10:00 hs</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K13" s="4" t="inlineStr">
-        <is>
-          <t>Ninguno</t>
-        </is>
-      </c>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="inlineStr"/>
       <c r="L13" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1451,7 +1451,7 @@
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>id-6b955df9d3f6241a</t>
+          <t>id-9d3847fb0e2b0929</t>
         </is>
       </c>
     </row>
@@ -1466,44 +1466,44 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>82/2026</t>
+          <t>12/2026</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>CONTRATACION DE SERVICIO DE MANO DE OBRA PARA ACONDICIONAMIENTO DE TECHO</t>
+          <t>RECAMBIO DE CUBIERTA Y REPARACIONES VARIAS EN ESCUELA Nº 92 “CONGRESO DE TUCUMAN” – CONCEPCION DEL URUGUAY - DPTO. URUGUAY – PROVINCIA DE ENTRE RIOS de acuerdo a las c ondiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>22/09/2026</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>22-09-2026 08:00</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 10:30 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>06/10/2026</t>
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr"/>
@@ -1519,19 +1519,19 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>id-e31ab37f1904ce3b</t>
+          <t>id-059239b424b9c936</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>23/09/2026</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1539,14 +1539,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>COLON — MUNICIPALIDAD DE COLON</t>
+          <t>VICTORIA — MUNICIPALIDAD DE VICTORIA</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1554,20 +1554,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr"/>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>008/2026</t>
+        </is>
+      </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
+          <t>Proveer a la Municipalidad de Victoria, Entre Ríos, de Veinticinco Mil (25.000) litros de Diésel 500, para movilidad de vehículos y maquinarias viales, Ocho Mil (8.000) litros de Gasoil Tipo euro o similar y Ocho (8.000) litros de nafta súper para vehículos y áreas afectadas a la Secretaria de Planeamiento y Dirección de Ambiente y Desarrollo sostenible;</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>14/10/2026</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>24 de SEPTIEMBRE de 2026</t>
+          <t>14 de octubre de 2026 a las 09:00 hs., en la Oficina de Compras de la Municipalidad de Victoria, Entr</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1575,11 +1579,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K15" s="4" t="inlineStr">
-        <is>
-          <t>Sin Cargo</t>
-        </is>
-      </c>
+      <c r="K15" s="4" t="inlineStr"/>
       <c r="L15" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1597,14 +1597,14 @@
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>id-bc610b64999d147d</t>
+          <t>id-a9af9f59c8c487c8</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1614,12 +1614,12 @@
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>SALUD ENTRE RÍOS S.A.U</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1627,32 +1627,32 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>10/2026</t>
-        </is>
-      </c>
+      <c r="F16" s="4" t="inlineStr"/>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>Contratación de Servicio de Viandas para el Hospital de la Baxada</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIU</t>
+          <t>Hospital de la Baxada, calle Gral. Al varado Nº 2.250 Paraná, Entre Ríos, el día 19/10/2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="K16" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
       <c r="L16" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1670,14 +1670,14 @@
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>id-d97b43a99f1e1824</t>
+          <t>id-d35d5e849089d7ac</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1687,12 +1687,12 @@
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>PARANA — SALUD ENTRE RÍOS S.A.U</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1700,32 +1700,32 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>09/2026</t>
-        </is>
-      </c>
+      <c r="F17" s="4" t="inlineStr"/>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>Servicio de Recolección, Lavado, Desinfección, Secado, Planchado y Transporte de Ropa Hospitalaria</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CI</t>
+          <t>Hospital de la Baxada, calle Gral. Alvarado Nº 2.250 Paraná, Entre Ríos, el día 21/10/2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="K17" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
       <c r="L17" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1743,14 +1743,14 @@
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>id-f8fab7a7b3a06a2d</t>
+          <t>id-6b955df9d3f6241a</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>23/09/2026</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1758,44 +1758,44 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE CRESPO -- ENTRE RÍOS</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>CONCURSO DE PRECIOS</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>05/2026</t>
+          <t>308/2026</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 145 metros lineales de modulo canal premoldeado cajón tipo pórtico de 2,00 X 1,00 (interior) X 1,00 mts. de longitud de hormigón para canalizar calle Los Quechuas al final</t>
+          <t>CONTRATACION DE SERVICIO DE ILUMINACION, PANTALLA LED Y SONIDO</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>23/09/2026</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>28 de septiembre de 2026 10:00 Hs. Lugar: Sección Suministros, Palacio Municipal sito en 25 de mayo Nº 943, C</t>
+          <t>23-09-2026 10:30</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr"/>
@@ -1811,12 +1811,12 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>id-61e8747a99305fe9</t>
+          <t>id-e39cbe830cc7226a</t>
         </is>
       </c>
     </row>
@@ -1831,49 +1831,45 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>Materiales</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Municipalidad de Crespo</t>
+          <t>COLON — MUNICIPALIDAD DE COLON</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Licitación</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>5/2026</t>
-        </is>
-      </c>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr"/>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 145 metros lineales de módulo canal premoldeado.</t>
+          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>28/9/2026 – 10:00 horas</t>
+          <t>24 de SEPTIEMBRE de 2026</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>$25.000,00</t>
+          <t>Sin Cargo</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr">
@@ -1888,12 +1884,12 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Municipalidad de Crespo</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>id-1609ce58e128c413</t>
+          <t>id-bc610b64999d147d</t>
         </is>
       </c>
     </row>
@@ -1908,14 +1904,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1925,34 +1921,30 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>08/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCL UIDO</t>
+          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>29/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>29/09/2026</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIU</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K20" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="K20" s="4" t="inlineStr"/>
       <c r="L20" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1970,7 +1962,7 @@
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>id-1590925c21c7e363</t>
+          <t>id-d97b43a99f1e1824</t>
         </is>
       </c>
     </row>
@@ -1985,14 +1977,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
+      <c r="C21" s="9" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2002,34 +1994,30 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>10/26</t>
+          <t>09/2026</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
+          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CI</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K21" s="4" t="inlineStr">
-        <is>
-          <t>$ 100 (Cien)</t>
-        </is>
-      </c>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr"/>
       <c r="L21" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2042,12 +2030,12 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Boletín Oficial de Entre Ríos + CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-75a5c9dd5b4aa6f3</t>
+          <t>id-f8fab7a7b3a06a2d</t>
         </is>
       </c>
     </row>
@@ -2062,14 +2050,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>MUNICIPALIDAD DE CRESPO -- ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2079,27 +2067,27 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>05/2026</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
+          <t>Adquisición de 145 metros lineales de modulo canal premoldeado cajón tipo pórtico de 2,00 X 1,00 (interior) X 1,00 mts. de longitud de hormigón para canalizar calle Los Quechuas al final</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
+          <t>28 de septiembre de 2026 10:00 Hs. Lugar: Sección Suministros, Palacio Municipal sito en 25 de mayo Nº 943, C</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>08/09/2026</t>
         </is>
       </c>
       <c r="K22" s="4" t="inlineStr"/>
@@ -2115,12 +2103,12 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-46c6d9f1f9210d1e</t>
+          <t>id-61e8747a99305fe9</t>
         </is>
       </c>
     </row>
@@ -2130,50 +2118,54 @@
           <t>17/09/2026</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
+          <t>Municipalidad de Crespo</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>001-2026</t>
+          <t>5/2026</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr"/>
+          <t>Adquisición de 145 metros lineales de módulo canal premoldeado.</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
+          <t>28/9/2026 – 10:00 horas</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t>SIN COSTO</t>
+          <t>$25.000,00</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr">
@@ -2188,12 +2180,12 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Crespo</t>
         </is>
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-b7b0120caf49d551</t>
+          <t>id-1609ce58e128c413</t>
         </is>
       </c>
     </row>
@@ -2203,19 +2195,19 @@
           <t>17/09/2026</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE URDINARRAIN</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2225,18 +2217,22 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>08/2026</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr"/>
+          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCL UIDO</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>29/09/2026</t>
+        </is>
+      </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -2244,7 +2240,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K24" s="4" t="inlineStr"/>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L24" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2262,7 +2262,7 @@
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-7a200161bcc9b02b</t>
+          <t>id-1590925c21c7e363</t>
         </is>
       </c>
     </row>
@@ -2272,19 +2272,19 @@
           <t>17/09/2026</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
+          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2294,18 +2294,22 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>10/26</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr"/>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2313,7 +2317,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K25" s="4" t="inlineStr"/>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>$ 100 (Cien)</t>
+        </is>
+      </c>
       <c r="L25" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2331,29 +2339,29 @@
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-511256e6329e386a</t>
+          <t>id-75a5c9dd5b4aa6f3</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2363,18 +2371,22 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>03/26</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
-        </is>
-      </c>
-      <c r="H26" s="4" t="inlineStr"/>
+          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2395,19 +2407,19 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-46c6d9f1f9210d1e</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>23/09/2026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2415,14 +2427,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr">
+      <c r="C27" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>MUNICIPALIDAD DE VIALE</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2432,18 +2444,18 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>02/2026</t>
+          <t>08/26</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+          <t>de asfalto 70- 16 destinado a la producción de pavimento de la Planta Asfáltica, y que a c ontinuación se detalla y</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2464,19 +2476,19 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-ef1ddb923c7e7fdb</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2484,14 +2496,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2501,18 +2513,18 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>001-2026</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2520,7 +2532,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K28" s="4" t="inlineStr"/>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L28" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2533,19 +2549,19 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-b7b0120caf49d551</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2555,12 +2571,12 @@
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Infraestructura</t>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>MUNICIPALIDAD DE URDINARRAIN</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2570,18 +2586,18 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>05/2025</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
+          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2602,19 +2618,19 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-7a200161bcc9b02b</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2622,14 +2638,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C30" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2639,18 +2655,18 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>06/2025</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2671,12 +2687,12 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
+          <t>id-511256e6329e386a</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2707,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C31" s="7" t="inlineStr">
+      <c r="C31" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2706,16 +2722,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F31" s="4" t="inlineStr"/>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>03/26</t>
+        </is>
+      </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2741,7 +2761,7 @@
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-ebeeb6a87e688d85</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
@@ -2756,7 +2776,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C32" s="7" t="inlineStr">
+      <c r="C32" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2773,18 +2793,18 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>04/2025</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2810,7 +2830,7 @@
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-34c85bcdb9b1123f</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
@@ -2825,7 +2845,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C33" s="7" t="inlineStr">
+      <c r="C33" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2842,18 +2862,18 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>03/2025</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2879,14 +2899,14 @@
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-75bfffae63b7eedc</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2894,7 +2914,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
+      <c r="C34" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2911,18 +2931,18 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>05/2025</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -2948,14 +2968,14 @@
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-07ddb93a12c5a870</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2963,7 +2983,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C35" s="7" t="inlineStr">
+      <c r="C35" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2980,18 +3000,18 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>06/2025</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>Concurso de Precio N° 02/2025</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3017,14 +3037,14 @@
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-7c1bf02160a66f67</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3032,31 +3052,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C36" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr"/>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3077,19 +3097,19 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>id-654eebef400f89cd</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3097,35 +3117,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C37" s="7" t="inlineStr">
+      <c r="C37" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Concurso</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>01/26</t>
+          <t>04/2025</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3146,19 +3166,19 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>id-9a16884dd5a64a49</t>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -3166,35 +3186,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C38" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>2026-1227</t>
+          <t>03/2025</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -3215,19 +3235,19 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>id-0691eb485d7548eb</t>
+          <t>id-75bfffae63b7eedc</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>19/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3237,33 +3257,33 @@
       </c>
       <c r="C39" s="8" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Solicitud de Cotización</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>235/26</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>Contratación de servicio para puesta en marcha de Grupo Electrógeno 30KVA, ubicado en el Edificio Tribunales de C. del Uruguay, calle San Martín Nº665.</t>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>Ver el sitio</t>
+          <t>Publicada 06/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -3284,12 +3304,12 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
-          <t>id-d3938e7b907594a8</t>
+          <t>id-07ddb93a12c5a870</t>
         </is>
       </c>
     </row>
@@ -3306,33 +3326,33 @@
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Solicitud de Cotización</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>233/26</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>Reemplazo, provisión e instalación de las barreras vehiculares automáticas en el Edificio Central de Tribunales, de Paraná (sito Laprida N°250).</t>
+          <t>Concurso de Precio N° 02/2025</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr"/>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Ver el sitio</t>
+          <t>Publicada 19/06/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
@@ -3353,12 +3373,12 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
-          <t>id-f48b8e7889aac66c</t>
+          <t>id-7c1bf02160a66f67</t>
         </is>
       </c>
     </row>
@@ -3373,35 +3393,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C41" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Concurso</t>
-        </is>
-      </c>
-      <c r="F41" s="4" t="inlineStr">
-        <is>
-          <t>04/26</t>
-        </is>
-      </c>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr"/>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>Edif. Tribunales – Chajarí, departamento de Federación. Obra “Reparaciones generales de baños e instalación eléctrica – 2° piso”</t>
+          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Ver el sitio</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
@@ -3422,17 +3438,500 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="O41" s="4" t="inlineStr">
+        <is>
+          <t>id-654eebef400f89cd</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Concurso</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>01/26</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="inlineStr"/>
+      <c r="I42" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J42" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K42" s="4" t="inlineStr"/>
+      <c r="L42" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M42" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="O42" s="4" t="inlineStr">
+        <is>
+          <t>id-9a16884dd5a64a49</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>Materiales</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>ENERSA</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Licitación</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>2026-1227</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr"/>
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K43" s="4" t="inlineStr"/>
+      <c r="L43" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M43" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>ENERSA</t>
+        </is>
+      </c>
+      <c r="O43" s="4" t="inlineStr">
+        <is>
+          <t>id-0691eb485d7548eb</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>10-2026</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
+        </is>
+      </c>
+      <c r="H44" s="4" t="inlineStr"/>
+      <c r="I44" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego — figura como Pendiente</t>
+        </is>
+      </c>
+      <c r="J44" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K44" s="4" t="inlineStr"/>
+      <c r="L44" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M44" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="O44" s="4" t="inlineStr">
+        <is>
+          <t>id-bdd0abb0374c3f42</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Licitación Privada</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>04-2026</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr"/>
+      <c r="I45" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego — figura como Pendiente</t>
+        </is>
+      </c>
+      <c r="J45" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K45" s="4" t="inlineStr"/>
+      <c r="L45" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M45" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>CAFESG (Salto Grande)</t>
+        </is>
+      </c>
+      <c r="O45" s="4" t="inlineStr">
+        <is>
+          <t>id-023b6b75e7014a9c</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>23/09/2026</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
           <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
-      <c r="O41" s="4" t="inlineStr">
-        <is>
-          <t>id-2466cef612391e08</t>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Solicitud de Cotización</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>236/26</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>Provisión y envío de materiales de pinturería para el Taller de Mantenimiento del Edificio Tribunales localidad Concordia.</t>
+        </is>
+      </c>
+      <c r="H46" s="4" t="inlineStr"/>
+      <c r="I46" s="4" t="inlineStr">
+        <is>
+          <t>Ver el sitio</t>
+        </is>
+      </c>
+      <c r="J46" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K46" s="4" t="inlineStr"/>
+      <c r="L46" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M46" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>Poder Judicial de Entre Ríos</t>
+        </is>
+      </c>
+      <c r="O46" s="4" t="inlineStr">
+        <is>
+          <t>id-d0f81989a1411fa1</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>19/09/2026</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Poder Judicial de Entre Ríos</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Solicitud de Cotización</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>235/26</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>Contratación de servicio para puesta en marcha de Grupo Electrógeno 30KVA, ubicado en el Edificio Tribunales de C. del Uruguay, calle San Martín Nº665.</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr"/>
+      <c r="I47" s="4" t="inlineStr">
+        <is>
+          <t>Ver el sitio</t>
+        </is>
+      </c>
+      <c r="J47" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K47" s="4" t="inlineStr"/>
+      <c r="L47" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M47" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>Poder Judicial de Entre Ríos</t>
+        </is>
+      </c>
+      <c r="O47" s="4" t="inlineStr">
+        <is>
+          <t>id-d3938e7b907594a8</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Poder Judicial de Entre Ríos</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Solicitud de Cotización</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>233/26</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>Reemplazo, provisión e instalación de las barreras vehiculares automáticas en el Edificio Central de Tribunales, de Paraná (sito Laprida N°250).</t>
+        </is>
+      </c>
+      <c r="H48" s="4" t="inlineStr"/>
+      <c r="I48" s="4" t="inlineStr">
+        <is>
+          <t>Ver el sitio</t>
+        </is>
+      </c>
+      <c r="J48" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K48" s="4" t="inlineStr"/>
+      <c r="L48" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M48" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>Poder Judicial de Entre Ríos</t>
+        </is>
+      </c>
+      <c r="O48" s="4" t="inlineStr">
+        <is>
+          <t>id-f48b8e7889aac66c</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O41"/>
+  <autoFilter ref="A1:O48"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -3514,6 +4013,20 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId78"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId79"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L43" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L47" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L48" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId94"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 24/09/2026 08:46
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -2699,7 +2699,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2707,14 +2707,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2724,18 +2724,18 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>03/26</t>
+          <t>10-2026</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>Ver pliego — figura como Pendiente</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2756,19 +2756,19 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-bdd0abb0374c3f42</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2776,35 +2776,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación Privada</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>02/2026</t>
+          <t>04-2026</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>Ver pliego — figura como Pendiente</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2825,19 +2825,19 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-023b6b75e7014a9c</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2845,35 +2845,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C33" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Solicitud de Cotización</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>240/26</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+          <t>Contratación del servicio de reparación prioritaria de seis (6) escalones de mármol de la escalera de acceso al entrepiso y primer piso del Edificio Tribunales de Gualeguaychú sito en calle Roque Sáenz Peña N°94.</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>Ver el sitio</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2894,19 +2894,19 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-ba80195eeddbd2bd</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>23/09/2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2914,35 +2914,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C34" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Solicitud de Cotización</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>05/2025</t>
+          <t>236/26</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
+          <t>Provisión y envío de materiales de pinturería para el Taller de Mantenimiento del Edificio Tribunales localidad Concordia.</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>Ver el sitio</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -2963,19 +2963,19 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-d0f81989a1411fa1</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>19/09/2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2983,35 +2983,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C35" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Solicitud de Cotización</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>06/2025</t>
+          <t>235/26</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>Contratación de servicio para puesta en marcha de Grupo Electrógeno 30KVA, ubicado en el Edificio Tribunales de C. del Uruguay, calle San Martín Nº665.</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Ver el sitio</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3032,12 +3032,12 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
+          <t>id-d3938e7b907594a8</t>
         </is>
       </c>
     </row>
@@ -3067,16 +3067,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F36" s="4" t="inlineStr"/>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>03/26</t>
+        </is>
+      </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3102,7 +3106,7 @@
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>id-ebeeb6a87e688d85</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
@@ -3134,18 +3138,18 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>04/2025</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3171,7 +3175,7 @@
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>id-34c85bcdb9b1123f</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
@@ -3203,18 +3207,18 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>03/2025</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -3240,14 +3244,14 @@
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>id-75bfffae63b7eedc</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3272,18 +3276,18 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>05/2025</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -3309,14 +3313,14 @@
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
-          <t>id-07ddb93a12c5a870</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3341,18 +3345,18 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>06/2025</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>Concurso de Precio N° 02/2025</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr"/>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
@@ -3378,14 +3382,14 @@
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
-          <t>id-7c1bf02160a66f67</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3393,31 +3397,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C41" s="7" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr"/>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
@@ -3438,19 +3442,19 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
-          <t>id-654eebef400f89cd</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3465,28 +3469,28 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Concurso</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>01/26</t>
+          <t>04/2025</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr"/>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr">
@@ -3507,19 +3511,19 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O42" s="4" t="inlineStr">
         <is>
-          <t>id-9a16884dd5a64a49</t>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -3527,35 +3531,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C43" s="7" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>2026-1227</t>
+          <t>03/2025</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr"/>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr">
@@ -3576,12 +3580,12 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O43" s="4" t="inlineStr">
         <is>
-          <t>id-0691eb485d7548eb</t>
+          <t>id-75bfffae63b7eedc</t>
         </is>
       </c>
     </row>
@@ -3596,14 +3600,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C44" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -3613,18 +3617,18 @@
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>10-2026</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr"/>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego — figura como Pendiente</t>
+          <t>Publicada 06/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr">
@@ -3645,12 +3649,12 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O44" s="4" t="inlineStr">
         <is>
-          <t>id-bdd0abb0374c3f42</t>
+          <t>id-07ddb93a12c5a870</t>
         </is>
       </c>
     </row>
@@ -3665,35 +3669,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C45" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Licitación Privada</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
+          <t>Concurso de Precio N° 02/2025</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr"/>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego — figura como Pendiente</t>
+          <t>Publicada 19/06/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J45" s="4" t="inlineStr">
@@ -3714,19 +3718,19 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O45" s="4" t="inlineStr">
         <is>
-          <t>id-023b6b75e7014a9c</t>
+          <t>id-7c1bf02160a66f67</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>23/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3734,35 +3738,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C46" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Solicitud de Cotización</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="inlineStr">
-        <is>
-          <t>236/26</t>
-        </is>
-      </c>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr"/>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>Provisión y envío de materiales de pinturería para el Taller de Mantenimiento del Edificio Tribunales localidad Concordia.</t>
+          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
         </is>
       </c>
       <c r="H46" s="4" t="inlineStr"/>
       <c r="I46" s="4" t="inlineStr">
         <is>
-          <t>Ver el sitio</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J46" s="4" t="inlineStr">
@@ -3783,19 +3783,19 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O46" s="4" t="inlineStr">
         <is>
-          <t>id-d0f81989a1411fa1</t>
+          <t>id-654eebef400f89cd</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>19/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3803,35 +3803,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C47" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Solicitud de Cotización</t>
+          <t>Concurso</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>235/26</t>
+          <t>01/26</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>Contratación de servicio para puesta en marcha de Grupo Electrógeno 30KVA, ubicado en el Edificio Tribunales de C. del Uruguay, calle San Martín Nº665.</t>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
         </is>
       </c>
       <c r="H47" s="4" t="inlineStr"/>
       <c r="I47" s="4" t="inlineStr">
         <is>
-          <t>Ver el sitio</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J47" s="4" t="inlineStr">
@@ -3852,12 +3852,12 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O47" s="4" t="inlineStr">
         <is>
-          <t>id-d3938e7b907594a8</t>
+          <t>id-9a16884dd5a64a49</t>
         </is>
       </c>
     </row>
@@ -3872,35 +3872,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C48" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Solicitud de Cotización</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>233/26</t>
+          <t>2026-1227</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>Reemplazo, provisión e instalación de las barreras vehiculares automáticas en el Edificio Central de Tribunales, de Paraná (sito Laprida N°250).</t>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
         </is>
       </c>
       <c r="H48" s="4" t="inlineStr"/>
       <c r="I48" s="4" t="inlineStr">
         <is>
-          <t>Ver el sitio</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J48" s="4" t="inlineStr">
@@ -3921,12 +3921,12 @@
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="O48" s="4" t="inlineStr">
         <is>
-          <t>id-f48b8e7889aac66c</t>
+          <t>id-0691eb485d7548eb</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 25/09/2026 08:10
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$45</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O48"/>
+  <dimension ref="A1:O45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1838,7 +1838,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>COLON — MUNICIPALIDAD DE COLON</t>
+          <t>MUNICIPALIDAD DE CRESPO -- ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1846,32 +1846,32 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr"/>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN DE MATERIALES PARA OBRAS COMPLEMENTARIAS Al PLAN DE PAVIMENTACIÓN URBANA”</t>
+          <t>Adquisición de 145 metros lineales de modulo canal premoldeado cajón tipo pórtico de 2,00 X 1,00 (interior) X 1,00 mts. de longitud de hormigón para canalizar calle Los Quechuas al final</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>24 de SEPTIEMBRE de 2026</t>
+          <t>28 de septiembre de 2026 10:00 Hs. Lugar: Sección Suministros, Palacio Municipal sito en 25 de mayo Nº 943, C</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K19" s="4" t="inlineStr">
-        <is>
-          <t>Sin Cargo</t>
-        </is>
-      </c>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="K19" s="4" t="inlineStr"/>
       <c r="L19" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1889,7 +1889,7 @@
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>id-bc610b64999d147d</t>
+          <t>id-61e8747a99305fe9</t>
         </is>
       </c>
     </row>
@@ -1904,47 +1904,51 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>COLON — COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>Municipalidad de Crespo</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>5/2026</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>REMODELACI ON Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE – DPTO. COLON – PROVINCIA DE ENTRE RIOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>Adquisición de 145 metros lineales de módulo canal premoldeado.</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIU</t>
+          <t>28/9/2026 – 10:00 horas</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="K20" s="4" t="inlineStr"/>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t>$25.000,00</t>
+        </is>
+      </c>
       <c r="L20" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1957,12 +1961,12 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Crespo</t>
         </is>
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>id-d97b43a99f1e1824</t>
+          <t>id-1609ce58e128c413</t>
         </is>
       </c>
     </row>
@@ -1977,14 +1981,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL DE SALTO GRANDE</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1994,30 +1998,34 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>09/2026</t>
+          <t>08/2026</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>“REFACCION, RESTAURACION Y PUESTA EN VALOR – ESCUELA N° 15 NORMAL “DOMINGO FAUSTINO SARMIENTO” – CIUDAD DE CONCORDIA – DEPARTAMENTO CONCORDIA – PROVINCIA DE ENTRE RIOS” de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCL UIDO</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 10:00 Lugar: OFICINAS CENTRALES DE LA C AFESG – CALLE SAN JUAN Nº 2097 – CI</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="K21" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L21" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2030,12 +2038,12 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos + CAFESG (Salto Grande)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-f8fab7a7b3a06a2d</t>
+          <t>id-1590925c21c7e363</t>
         </is>
       </c>
     </row>
@@ -2050,14 +2058,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE CRESPO -- ENTRE RÍOS</t>
+          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2067,30 +2075,34 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>05/2026</t>
+          <t>10/26</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 145 metros lineales de modulo canal premoldeado cajón tipo pórtico de 2,00 X 1,00 (interior) X 1,00 mts. de longitud de hormigón para canalizar calle Los Quechuas al final</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>28 de septiembre de 2026 10:00 Hs. Lugar: Sección Suministros, Palacio Municipal sito en 25 de mayo Nº 943, C</t>
+          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
-        </is>
-      </c>
-      <c r="K22" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>$ 100 (Cien)</t>
+        </is>
+      </c>
       <c r="L22" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2108,7 +2120,7 @@
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-61e8747a99305fe9</t>
+          <t>id-75a5c9dd5b4aa6f3</t>
         </is>
       </c>
     </row>
@@ -2123,51 +2135,47 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Municipalidad de Crespo</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>5/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 145 metros lineales de módulo canal premoldeado.</t>
+          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>28/9/2026 – 10:00 horas</t>
+          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
-        </is>
-      </c>
-      <c r="K23" s="4" t="inlineStr">
-        <is>
-          <t>$25.000,00</t>
-        </is>
-      </c>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K23" s="4" t="inlineStr"/>
       <c r="L23" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2180,34 +2188,34 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Municipalidad de Crespo</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-1609ce58e128c413</t>
+          <t>id-46c6d9f1f9210d1e</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+          <t>23/09/2026</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>MUNICIPALIDAD DE VIALE</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2217,22 +2225,18 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>08/2026</t>
+          <t>08/26</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCL UIDO</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>29/09/2026</t>
-        </is>
-      </c>
+          <t>de asfalto 70- 16 destinado a la producción de pavimento de la Planta Asfáltica, y que a c ontinuación se detalla y</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr"/>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>29/09/2026</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -2240,11 +2244,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K24" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K24" s="4" t="inlineStr"/>
       <c r="L24" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2262,7 +2262,7 @@
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-1590925c21c7e363</t>
+          <t>id-ef1ddb923c7e7fdb</t>
         </is>
       </c>
     </row>
@@ -2272,9 +2272,9 @@
           <t>17/09/2026</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
@@ -2284,7 +2284,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2294,22 +2294,18 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>10/26</t>
+          <t>001-2026</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>30/09/2026</t>
-        </is>
-      </c>
+          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr"/>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2319,7 +2315,7 @@
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>$ 100 (Cien)</t>
+          <t>SIN COSTO</t>
         </is>
       </c>
       <c r="L25" s="6" t="inlineStr">
@@ -2339,7 +2335,7 @@
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-75a5c9dd5b4aa6f3</t>
+          <t>id-b7b0120caf49d551</t>
         </is>
       </c>
     </row>
@@ -2349,19 +2345,19 @@
           <t>17/09/2026</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C26" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>MUNICIPALIDAD DE URDINARRAIN</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2371,22 +2367,18 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
-        </is>
-      </c>
-      <c r="H26" s="4" t="inlineStr">
-        <is>
-          <t>30/09/2026</t>
-        </is>
-      </c>
+          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2407,19 +2399,19 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-46c6d9f1f9210d1e</t>
+          <t>id-7a200161bcc9b02b</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>23/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2427,14 +2419,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C27" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE VIALE</t>
+          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2444,12 +2436,12 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>08/26</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>de asfalto 70- 16 destinado a la producción de pavimento de la Planta Asfáltica, y que a c ontinuación se detalla y</t>
+          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
@@ -2481,7 +2473,7 @@
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-ef1ddb923c7e7fdb</t>
+          <t>id-511256e6329e386a</t>
         </is>
       </c>
     </row>
@@ -2503,7 +2495,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2513,18 +2505,18 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>001-2026</t>
+          <t>10-2026</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
+          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
+          <t>Ver pliego — figura como Pendiente</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2532,11 +2524,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K28" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K28" s="4" t="inlineStr"/>
       <c r="L28" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2549,12 +2537,12 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-b7b0120caf49d551</t>
+          <t>id-bdd0abb0374c3f42</t>
         </is>
       </c>
     </row>
@@ -2569,35 +2557,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE URDINARRAIN</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación Privada</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>04-2026</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
+          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Ver pliego — figura como Pendiente</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2618,19 +2606,19 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>CAFESG (Salto Grande)</t>
         </is>
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-7a200161bcc9b02b</t>
+          <t>id-023b6b75e7014a9c</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2638,35 +2626,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Solicitud de Cotización</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>240/26</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
+          <t>Contratación del servicio de reparación prioritaria de seis (6) escalones de mármol de la escalera de acceso al entrepiso y primer piso del Edificio Tribunales de Gualeguaychú sito en calle Roque Sáenz Peña N°94.</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Ver el sitio</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2687,19 +2675,19 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-511256e6329e386a</t>
+          <t>id-ba80195eeddbd2bd</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>23/09/2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2714,28 +2702,28 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Solicitud de Cotización</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>10-2026</t>
+          <t>236/26</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
+          <t>Provisión y envío de materiales de pinturería para el Taller de Mantenimiento del Edificio Tribunales localidad Concordia.</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego — figura como Pendiente</t>
+          <t>Ver el sitio</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2756,19 +2744,19 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-bdd0abb0374c3f42</t>
+          <t>id-d0f81989a1411fa1</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>19/09/2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2783,28 +2771,28 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Licitación Privada</t>
+          <t>Solicitud de Cotización</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>235/26</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
+          <t>Contratación de servicio para puesta en marcha de Grupo Electrógeno 30KVA, ubicado en el Edificio Tribunales de C. del Uruguay, calle San Martín Nº665.</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego — figura como Pendiente</t>
+          <t>Ver el sitio</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2825,19 +2813,19 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-023b6b75e7014a9c</t>
+          <t>id-d3938e7b907594a8</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2845,35 +2833,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C33" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Solicitud de Cotización</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>240/26</t>
+          <t>03/26</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>Contratación del servicio de reparación prioritaria de seis (6) escalones de mármol de la escalera de acceso al entrepiso y primer piso del Edificio Tribunales de Gualeguaychú sito en calle Roque Sáenz Peña N°94.</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Ver el sitio</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2894,19 +2882,19 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-ba80195eeddbd2bd</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>23/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2914,35 +2902,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C34" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Solicitud de Cotización</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>236/26</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>Provisión y envío de materiales de pinturería para el Taller de Mantenimiento del Edificio Tribunales localidad Concordia.</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Ver el sitio</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -2963,19 +2951,19 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-d0f81989a1411fa1</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>19/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2983,35 +2971,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C35" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Solicitud de Cotización</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>235/26</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>Contratación de servicio para puesta en marcha de Grupo Electrógeno 30KVA, ubicado en el Edificio Tribunales de C. del Uruguay, calle San Martín Nº665.</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Ver el sitio</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3032,12 +3020,12 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-d3938e7b907594a8</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
@@ -3069,18 +3057,18 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>03/26</t>
+          <t>05/2025</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3106,7 +3094,7 @@
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
@@ -3138,18 +3126,18 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>02/2026</t>
+          <t>06/2025</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3175,7 +3163,7 @@
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
@@ -3205,20 +3193,16 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F38" s="4" t="inlineStr">
-        <is>
-          <t>01/2026</t>
-        </is>
-      </c>
+      <c r="F38" s="4" t="inlineStr"/>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -3244,7 +3228,7 @@
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
@@ -3276,18 +3260,18 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>05/2025</t>
+          <t>04/2025</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -3313,7 +3297,7 @@
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
@@ -3345,18 +3329,18 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>06/2025</t>
+          <t>03/2025</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr"/>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
@@ -3382,14 +3366,14 @@
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
+          <t>id-75bfffae63b7eedc</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3412,16 +3396,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F41" s="4" t="inlineStr"/>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>02/2025</t>
+        </is>
+      </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
+          <t>Publicada 06/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
@@ -3447,14 +3435,14 @@
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
-          <t>id-ebeeb6a87e688d85</t>
+          <t>id-07ddb93a12c5a870</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3479,18 +3467,18 @@
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>04/2025</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+          <t>Concurso de Precio N° 02/2025</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr"/>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
+          <t>Publicada 19/06/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr">
@@ -3516,14 +3504,14 @@
       </c>
       <c r="O42" s="4" t="inlineStr">
         <is>
-          <t>id-34c85bcdb9b1123f</t>
+          <t>id-7c1bf02160a66f67</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -3531,35 +3519,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F43" s="4" t="inlineStr">
-        <is>
-          <t>03/2025</t>
-        </is>
-      </c>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr"/>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr"/>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr">
@@ -3580,12 +3564,12 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O43" s="4" t="inlineStr">
         <is>
-          <t>id-75bfffae63b7eedc</t>
+          <t>id-654eebef400f89cd</t>
         </is>
       </c>
     </row>
@@ -3607,28 +3591,28 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Concurso</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>01/26</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr"/>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr">
@@ -3649,12 +3633,12 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O44" s="4" t="inlineStr">
         <is>
-          <t>id-07ddb93a12c5a870</t>
+          <t>id-9a16884dd5a64a49</t>
         </is>
       </c>
     </row>
@@ -3669,35 +3653,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>2026-1227</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>Concurso de Precio N° 02/2025</t>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr"/>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J45" s="4" t="inlineStr">
@@ -3718,220 +3702,17 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="O45" s="4" t="inlineStr">
         <is>
-          <t>id-7c1bf02160a66f67</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C46" s="7" t="inlineStr">
-        <is>
-          <t>Materiales</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="inlineStr"/>
-      <c r="G46" s="5" t="inlineStr">
-        <is>
-          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
-        </is>
-      </c>
-      <c r="H46" s="4" t="inlineStr"/>
-      <c r="I46" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J46" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K46" s="4" t="inlineStr"/>
-      <c r="L46" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M46" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
-        </is>
-      </c>
-      <c r="O46" s="4" t="inlineStr">
-        <is>
-          <t>id-654eebef400f89cd</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Concurso</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr">
-        <is>
-          <t>01/26</t>
-        </is>
-      </c>
-      <c r="G47" s="5" t="inlineStr">
-        <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
-        </is>
-      </c>
-      <c r="H47" s="4" t="inlineStr"/>
-      <c r="I47" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J47" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K47" s="4" t="inlineStr"/>
-      <c r="L47" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M47" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
-        </is>
-      </c>
-      <c r="O47" s="4" t="inlineStr">
-        <is>
-          <t>id-9a16884dd5a64a49</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C48" s="7" t="inlineStr">
-        <is>
-          <t>Materiales</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>ENERSA</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>Licitación</t>
-        </is>
-      </c>
-      <c r="F48" s="4" t="inlineStr">
-        <is>
-          <t>2026-1227</t>
-        </is>
-      </c>
-      <c r="G48" s="5" t="inlineStr">
-        <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
-        </is>
-      </c>
-      <c r="H48" s="4" t="inlineStr"/>
-      <c r="I48" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J48" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K48" s="4" t="inlineStr"/>
-      <c r="L48" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M48" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>ENERSA</t>
-        </is>
-      </c>
-      <c r="O48" s="4" t="inlineStr">
-        <is>
           <t>id-0691eb485d7548eb</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O48"/>
+  <autoFilter ref="A1:O45"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -4021,12 +3802,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId86"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId87"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L47" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L48" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId94"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 26/09/2026 08:37
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$47</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -43,7 +43,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -75,6 +75,11 @@
         <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -88,7 +93,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -101,6 +106,7 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -466,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O45"/>
+  <dimension ref="A1:O47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -793,7 +799,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>26/09/2026</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -801,29 +807,29 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE SALUD</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Licitación Publica</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>17/26</t>
+          <t>07/2026</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Adquirir Una (01) Mesa de Anestesia. Destino: Hospital “San José” de Diamante, dependiente del Ministerio de Salud de la Provincia de Entre Ríos</t>
+          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”, destinada a la obra denominada “Nueva Pileta en el Polideportivo El Aguará”,</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -833,15 +839,19 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
+          <t>06/10/2026 HORA: 11:00 HS</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
-        </is>
-      </c>
-      <c r="K5" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L5" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -859,7 +869,7 @@
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>id-3312d89e1a3e2e53</t>
+          <t>id-65d18d99bf0b2c6c</t>
         </is>
       </c>
     </row>
@@ -881,37 +891,37 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
+          <t>PARANA — MINISTERIO DE SALUD</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación Publica</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>31/2026</t>
+          <t>17/26</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>“Pavimento Rígido – 03 (tres) Cuadras Barrio San Felipe”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>Adquirir Una (01) Mesa de Anestesia. Destino: Hospital “San José” de Diamante, dependiente del Ministerio de Salud de la Provincia de Entre Ríos</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>06/10/2026</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>07 de octubre de 2026 Hora: 10:00</t>
+          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>06/10/2026</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr"/>
@@ -932,14 +942,14 @@
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>id-76d9566cb30a6df5</t>
+          <t>id-3312d89e1a3e2e53</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>23/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -947,9 +957,9 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -964,22 +974,22 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>32/2026</t>
+          <t>31/2026</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>"Adquisición de 835 m3 de Hormigón Calidad H25 para 08 cuadras de Pavimento", en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>“Pavimento Rígido – 03 (tres) Cuadras Barrio San Felipe”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>08 de octubre de 2026 Hora: 10:00</t>
+          <t>07 de octubre de 2026 Hora: 10:00</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -1005,7 +1015,7 @@
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>id-0ace7de8f16d3baf</t>
+          <t>id-76d9566cb30a6df5</t>
         </is>
       </c>
     </row>
@@ -1020,9 +1030,9 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1037,12 +1047,12 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>33/2026</t>
+          <t>32/2026</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>“Pavimento Rígido – 04 (cuatro) Cuadras Barrio San Roque y 01 (una) Cuadra Barrio Vicente Obrego”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>"Adquisición de 835 m3 de Hormigón Calidad H25 para 08 cuadras de Pavimento", en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -1052,7 +1062,7 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>08 de octubre de 2026 Hora: 11:00</t>
+          <t>08 de octubre de 2026 Hora: 10:00</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -1078,14 +1088,14 @@
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>id-fe71ac2aaf71b8d8</t>
+          <t>id-0ace7de8f16d3baf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>23/09/2026</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1093,14 +1103,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1110,22 +1120,22 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>33/2026</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>“PROVISIÓN DE UNA (1) MINICARGADORA 0 KM, CON CUCHARÓN FRONTAL DE USO GENERAL, UN (1) MARTILLO HIDRÁULICO Y UN (1) COMPACTADOR/RODILLO VIBRATORIO LISO”</t>
+          <t>“Pavimento Rígido – 04 (cuatro) Cuadras Barrio San Roque y 01 (una) Cuadra Barrio Vicente Obrego”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>09/10/2026 HORA: 10:00 HS</t>
+          <t>08 de octubre de 2026 Hora: 11:00</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1133,11 +1143,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>($ 270.000,00) PESOS DOSCIENTOS SETENTA MIL</t>
-        </is>
-      </c>
+      <c r="K9" s="4" t="inlineStr"/>
       <c r="L9" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1155,7 +1161,7 @@
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>id-779e4cd290f2e64e</t>
+          <t>id-fe71ac2aaf71b8d8</t>
         </is>
       </c>
     </row>
@@ -1177,7 +1183,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
+          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1192,7 +1198,7 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>“ Concesión de la Explotación Comercial de un (01) Camión de Comidas Rápidas (para cubrir el total de cuatro puestos) en la Zona Joven – Parque La Salamanca de la Municipalidad de Concepción del Uruguay – Entre Ríos”, en un todo de acuerdo a los Pliegos de B ases, Condiciones Particulares y demás documentación</t>
+          <t>“Concesión de la Explotación Comercial de un (01) Camión de Comidas Rápidas (para cubrir el total de cuatro puestos) en la Zona Joven – Parque La Salamanca de la Municipalidad de Concepción del Uruguay – Entre Ríos”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -1243,14 +1249,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1260,22 +1266,22 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>11/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>OBRA "PAVIMENTACION URBANA CALLE TRATADO DEL PILAR B° 3 DE FEBRERO - MUNICIPALIDAD DE SANTA ELENA" (Según Pliegos de Bases y condi ciones)</t>
+          <t>“PROVISIÓN DE UNA (1) MINICARGADORA 0 KM, CON CUCHARÓN FRONTAL DE USO GENERAL, UN (1) MARTILLO HIDRÁULICO Y UN (1) COMPACTADOR/RODILLO VIBRATORIO LISO”</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026 HORA: 10: 00 HS</t>
+          <t>09/10/2026 HORA: 10:00 HS</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1285,7 +1291,7 @@
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>$ 728.000,00 PESOS SETECIENTOS VEINTIOCHO MIL</t>
+          <t>($ 270.000,00) PESOS DOSCIENTOS SETENTA MIL</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
@@ -1305,14 +1311,14 @@
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>id-1a2561509308b1b6</t>
+          <t>id-779e4cd290f2e64e</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1320,14 +1326,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
+          <t>MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1342,7 +1348,7 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>REFACCION EN ESCUELA N° 65 “ALMIRANTE BROWN” – CIUDAD DE CONCORDIA - DEPARTAMENTO CONCORDIA - PROVINCIA DE ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>OBRA "PAVIMENTACION URBANA CALLE TRATADO DEL PILAR B° 3 DE FEBRERO - MUNICIPALIDAD DE SANTA ELENA" (Según Pliegos de Bases y condi ciones)</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -1352,15 +1358,19 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 09:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
+          <t>13/10/2026 HORA: 10: 00 HS</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
-        </is>
-      </c>
-      <c r="K12" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>$ 728.000,00 PESOS SETECIENTOS VEINTIOCHO MIL</t>
+        </is>
+      </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1378,7 +1388,7 @@
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>id-fc30d5c0b0589a79</t>
+          <t>id-1a2561509308b1b6</t>
         </is>
       </c>
     </row>
@@ -1410,12 +1420,12 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>13/2026</t>
+          <t>11/2026</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>REPARACIONES VARIAS EN C. P. E. F. Nº 3 “PROFESOR HUGO LA NASA” – CIUDAD DE CONCEPCION DEL URUGUAY - DEPARTAMENTO URUGUAY - PROVINCIA D E ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>REFACCION EN ESCUELA N° 65 “ALMIRANTE BROWN” – CIUDAD DE CONCORDIA - DEPARTAMENTO CONCORDIA - PROVINCIA DE ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
@@ -1425,7 +1435,7 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 09:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -1451,7 +1461,7 @@
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>id-9d3847fb0e2b0929</t>
+          <t>id-fc30d5c0b0589a79</t>
         </is>
       </c>
     </row>
@@ -1483,12 +1493,12 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>12/2026</t>
+          <t>13/2026</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>RECAMBIO DE CUBIERTA Y REPARACIONES VARIAS EN ESCUELA Nº 92 “CONGRESO DE TUCUMAN” – CONCEPCION DEL URUGUAY - DPTO. URUGUAY – PROVINCIA DE ENTRE RIOS de acuerdo a las c ondiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>REPARACIONES VARIAS EN C. P. E. F. Nº 3 “PROFESOR HUGO LA NASA” – CIUDAD DE CONCEPCION DEL URUGUAY - DEPARTAMENTO URUGUAY - PROVINCIA D E ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -1498,7 +1508,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 10:30 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1524,14 +1534,14 @@
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>id-059239b424b9c936</t>
+          <t>id-9d3847fb0e2b0929</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>23/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1539,14 +1549,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>VICTORIA — MUNICIPALIDAD DE VICTORIA</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1556,27 +1566,27 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>008/2026</t>
+          <t>12/2026</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Proveer a la Municipalidad de Victoria, Entre Ríos, de Veinticinco Mil (25.000) litros de Diésel 500, para movilidad de vehículos y maquinarias viales, Ocho Mil (8.000) litros de Gasoil Tipo euro o similar y Ocho (8.000) litros de nafta súper para vehículos y áreas afectadas a la Secretaria de Planeamiento y Dirección de Ambiente y Desarrollo sostenible;</t>
+          <t>RECAMBIO DE CUBIERTA Y REPARACIONES VARIAS EN ESCUELA Nº 92 “CONGRESO DE TUCUMAN” – CONCEPCION DEL URUGUAY - DPTO. URUGUAY – PROVINCIA DE ENTRE RIOS de acuerdo a las c ondiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>14/10/2026</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>14 de octubre de 2026 a las 09:00 hs., en la Oficina de Compras de la Municipalidad de Victoria, Entr</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 10:30 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>06/10/2026</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr"/>
@@ -1597,14 +1607,14 @@
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>id-a9af9f59c8c487c8</t>
+          <t>id-059239b424b9c936</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>23/09/2026</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1612,14 +1622,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>SALUD ENTRE RÍOS S.A.U</t>
+          <t>VICTORIA — MUNICIPALIDAD DE VICTORIA</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1627,20 +1637,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr"/>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>008/2026</t>
+        </is>
+      </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Contratación de Servicio de Viandas para el Hospital de la Baxada</t>
+          <t>Proveer a la Municipalidad de Victoria, Entre Ríos, de Veinticinco Mil (25.000) litros de Diésel 500, para movilidad de vehículos y maquinarias viales , Ocho Mil (8.000) litros de Gasoil Tipo euro o similar y Ocho (8.000) litros de nafta súper para vehículos y áreas afectadas a la Secretaria de Planeamiento y Dirección de Ambiente y Desarrollo sostenible;</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>14/10/2026</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Hospital de la Baxada, calle Gral. Al varado Nº 2.250 Paraná, Entre Ríos, el día 19/10/2026 a las 10:00 hs</t>
+          <t>14 de octubre de 2026 a las 09:00 hs., en la Oficina de Compras de la Municipalidad de Victoria, Entr</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -1648,11 +1662,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K16" s="4" t="inlineStr">
-        <is>
-          <t>Ninguno</t>
-        </is>
-      </c>
+      <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1670,7 +1680,7 @@
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>id-d35d5e849089d7ac</t>
+          <t>id-a9af9f59c8c487c8</t>
         </is>
       </c>
     </row>
@@ -1692,7 +1702,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>PARANA — SALUD ENTRE RÍOS S.A.U</t>
+          <t>SALUD ENTRE RÍOS S.A.U</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1703,17 +1713,17 @@
       <c r="F17" s="4" t="inlineStr"/>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Servicio de Recolección, Lavado, Desinfección, Secado, Planchado y Transporte de Ropa Hospitalaria</t>
+          <t>Contratación de Servicio de Viandas para el Hospital de la Baxada</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>21/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Hospital de la Baxada, calle Gral. Alvarado Nº 2.250 Paraná, Entre Ríos, el día 21/10/2026 a las 10:00 hs</t>
+          <t>Hospital de la Baxada, calle Gral. Al varado Nº 2.250 Paraná, Entre Ríos, el día 19/10/2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1743,14 +1753,14 @@
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>id-6b955df9d3f6241a</t>
+          <t>id-d35d5e849089d7ac</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>23/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1765,32 +1775,28 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>PARANA — SALUD ENTRE RÍOS S.A.U</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>CONCURSO DE PRECIOS</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>308/2026</t>
-        </is>
-      </c>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr"/>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>CONTRATACION DE SERVICIO DE ILUMINACION, PANTALLA LED Y SONIDO</t>
+          <t>Servicio de Recolección, Lavado, Desinfección, Secado, Planchado y Transporte de Ropa Hospitalaria</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>23/09/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>23-09-2026 10:30</t>
+          <t>Hospital de la Baxada, calle Gral. Alvarado Nº 2.250 Paraná, Entre Ríos, el día 21/10/2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1798,7 +1804,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K18" s="4" t="inlineStr"/>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
       <c r="L18" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1811,19 +1821,19 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>id-e39cbe830cc7226a</t>
+          <t>id-6b955df9d3f6241a</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>26/09/2026</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1831,14 +1841,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE CRESPO -- ENTRE RÍOS</t>
+          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1848,30 +1858,34 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>05/2026</t>
+          <t>11/26</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 145 metros lineales de modulo canal premoldeado cajón tipo pórtico de 2,00 X 1,00 (interior) X 1,00 mts. de longitud de hormigón para canalizar calle Los Quechuas al final</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “TERMINACION ESCUELA Nº 40 “JOSÉ ENRIQUE RODÓ”-SEPTIMO DISTRITO-DEPARTAMENTO GUALEGUAY.”</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>23/10/2026</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>28 de septiembre de 2026 10:00 Hs. Lugar: Sección Suministros, Palacio Municipal sito en 25 de mayo Nº 943, C</t>
+          <t>DE LAS OFERTAS: el día 23 de Octubre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
-        </is>
-      </c>
-      <c r="K19" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>$ 100 (Cien)</t>
+        </is>
+      </c>
       <c r="L19" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1889,14 +1903,14 @@
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>id-61e8747a99305fe9</t>
+          <t>id-86cc9c230734c462</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>26/09/2026</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1904,51 +1918,47 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Municipalidad de Crespo</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>5/2026</t>
+          <t>11/2026</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 145 metros lineales de módulo canal premoldeado.</t>
+          <t>Terminación Escuela N° 40 "José Enrique Rodó", Séptimo Distrito</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>23/10/2026</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>28/9/2026 – 10:00 horas</t>
+          <t>viernes, 23 de octubre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
-        </is>
-      </c>
-      <c r="K20" s="4" t="inlineStr">
-        <is>
-          <t>$25.000,00</t>
-        </is>
-      </c>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K20" s="4" t="inlineStr"/>
       <c r="L20" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1961,12 +1971,12 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Municipalidad de Crespo</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>id-1609ce58e128c413</t>
+          <t>id-322a40f5e43af35d</t>
         </is>
       </c>
     </row>
@@ -1981,14 +1991,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>MUNICIPALIDAD DE CRESPO -- ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1998,34 +2008,30 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>08/2026</t>
+          <t>05/2026</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCL UIDO</t>
+          <t>Adquisición de 145 metros lineales de modulo canal premoldeado cajón tipo pórtico de 2,00 X 1,00 (interior) X 1,00 mts. de longitud de hormigón para canalizar calle Los Quechuas al final</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>29/09/2026</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>29/09/2026</t>
+          <t>28 de septiembre de 2026 10:00 Hs. Lugar: Sección Suministros, Palacio Municipal sito en 25 de mayo Nº 943, C</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K21" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+          <t>08/09/2026</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr"/>
       <c r="L21" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2043,7 +2049,7 @@
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-1590925c21c7e363</t>
+          <t>id-61e8747a99305fe9</t>
         </is>
       </c>
     </row>
@@ -2058,49 +2064,49 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>Municipalidad de Crespo</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>10/26</t>
+          <t>5/2026</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
+          <t>Adquisición de 145 metros lineales de módulo canal premoldeado.</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>28/9/2026 – 10:00 horas</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
-          <t>$ 100 (Cien)</t>
+          <t>$25.000,00</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr">
@@ -2115,12 +2121,12 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Crespo</t>
         </is>
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-75a5c9dd5b4aa6f3</t>
+          <t>id-1609ce58e128c413</t>
         </is>
       </c>
     </row>
@@ -2135,14 +2141,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2152,22 +2158,22 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>08/2026</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
+          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCL UIDO</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2175,7 +2181,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K23" s="4" t="inlineStr"/>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L23" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2188,34 +2198,34 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-46c6d9f1f9210d1e</t>
+          <t>id-1590925c21c7e363</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>23/09/2026</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE VIALE</t>
+          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2225,18 +2235,22 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>08/26</t>
+          <t>10/26</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>de asfalto 70- 16 destinado a la producción de pavimento de la Planta Asfáltica, y que a c ontinuación se detalla y</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr"/>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -2244,7 +2258,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K24" s="4" t="inlineStr"/>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>$ 100 (Cien)</t>
+        </is>
+      </c>
       <c r="L24" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2262,7 +2280,7 @@
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-ef1ddb923c7e7fdb</t>
+          <t>id-75a5c9dd5b4aa6f3</t>
         </is>
       </c>
     </row>
@@ -2272,9 +2290,9 @@
           <t>17/09/2026</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
@@ -2284,7 +2302,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2294,18 +2312,22 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>001-2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr"/>
+          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>30/09/2026</t>
+        </is>
+      </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
+          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2313,11 +2335,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K25" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K25" s="4" t="inlineStr"/>
       <c r="L25" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2330,19 +2348,19 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-b7b0120caf49d551</t>
+          <t>id-46c6d9f1f9210d1e</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>26/09/2026</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2350,14 +2368,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE URDINARRAIN</t>
+          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2367,18 +2385,18 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>001/26</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
+          <t>ADQUISICIÓN de UN (1) FURGON UTILITARIO CHICO con 5 asientos 0 KM. con destino a Subsecretaria de Asistencia Directa y Emergencia</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>DE LAS PROPUESTAS: 20 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2404,14 +2422,14 @@
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-7a200161bcc9b02b</t>
+          <t>id-ca205f0874380f69</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>26/09/2026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2419,14 +2437,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
+          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2436,18 +2454,18 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>07/2026</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
+          <t>Transporte de mil doscientos cincuenta metros cúbicos (1.250 m³) de broza grillada desde Cantera “Tayreta” (Ruta Nacional N° 14 km 135) hasta juris dicción de la comuna, de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Viernes 09 de octubre del corriente año a las 10:00 hs en la Oficina de la Sede de la Comuna</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2473,14 +2491,14 @@
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-511256e6329e386a</t>
+          <t>id-24e9015ecceeff7f</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>26/09/2026</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2488,35 +2506,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C28" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>INSTITUTO CARBÓ S.R.L</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>10-2026</t>
-        </is>
-      </c>
+          <t>Licitación</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr"/>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>REMODELACION Y TERMINACION ESCUELA Nº 54 “CARLOS SOURIGUES” - BARRIO PERUCHO VERNA – SAN JOSE– DPTO. COLON – PROVINCIA DE ENTRE RIOS- Apertura: Jueves 24 DE SEPTIEMBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD DE CONCORDIA – ENTRE RIOS.-</t>
+          <t>sin internación en materia de salud, pre- hospitalarias, atención médica, domiciliaria y traslados sanitarios de alta</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego — figura como Pendiente</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2537,19 +2551,19 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-bdd0abb0374c3f42</t>
+          <t>id-6aa57c7437a30ca3</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>23/09/2026</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2557,35 +2571,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C29" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>MUNICIPALIDAD DE VIALE</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Licitación Privada</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>08/26</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>REFACCION Y AMPLIACION ESCUELA Nº 56 “HIPOLITO YRIGOYEN“– CIUDAD DE COLON - DEPARTAMENTO COLON - PROVINCIA DE ENTRE RÍOS Apertura: La apertura de las propuestas se realizará el día Viernes 11 de Septiembre de 2026 a las 10:00 horas, en las Oficinas de C.A.F.E.S.G. de la Ciudad de Concordia, sitas en Calle San Juan Nº 2097.</t>
+          <t>de asf alto 70-16 destinado a la producción de pavimento de la Planta Asfáltica, y que a continuación se detalla y</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego — figura como Pendiente</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2606,19 +2620,19 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>CAFESG (Salto Grande)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-023b6b75e7014a9c</t>
+          <t>id-ef1ddb923c7e7fdb</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2633,28 +2647,28 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Solicitud de Cotización</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>240/26</t>
+          <t>001-2026</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>Contratación del servicio de reparación prioritaria de seis (6) escalones de mármol de la escalera de acceso al entrepiso y primer piso del Edificio Tribunales de Gualeguaychú sito en calle Roque Sáenz Peña N°94.</t>
+          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Ver el sitio</t>
+          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2662,7 +2676,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K30" s="4" t="inlineStr"/>
+      <c r="K30" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L30" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2675,19 +2693,19 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-ba80195eeddbd2bd</t>
+          <t>id-b7b0120caf49d551</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>23/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2695,35 +2713,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C31" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>MUNICIPALIDAD DE URDINARRAIN</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Solicitud de Cotización</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>236/26</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>Provisión y envío de materiales de pinturería para el Taller de Mantenimiento del Edificio Tribunales localidad Concordia.</t>
+          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Ver el sitio</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2744,19 +2762,19 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-d0f81989a1411fa1</t>
+          <t>id-7a200161bcc9b02b</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>19/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2764,35 +2782,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C32" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Solicitud de Cotización</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>235/26</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>Contratación de servicio para puesta en marcha de Grupo Electrógeno 30KVA, ubicado en el Edificio Tribunales de C. del Uruguay, calle San Martín Nº665.</t>
+          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Ver el sitio</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2813,12 +2831,12 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-d3938e7b907594a8</t>
+          <t>id-511256e6329e386a</t>
         </is>
       </c>
     </row>
@@ -3711,8 +3729,146 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Poder Judicial de Entre Ríos</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>08/26</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>Obra “Readecuación del sistema de climatización –ala sur- Edificio Tribunales Gualeguay”.</t>
+        </is>
+      </c>
+      <c r="H46" s="4" t="inlineStr"/>
+      <c r="I46" s="4" t="inlineStr">
+        <is>
+          <t>Ver el sitio</t>
+        </is>
+      </c>
+      <c r="J46" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K46" s="4" t="inlineStr"/>
+      <c r="L46" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M46" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>Poder Judicial de Entre Ríos</t>
+        </is>
+      </c>
+      <c r="O46" s="4" t="inlineStr">
+        <is>
+          <t>id-9ca2387eef6d6fc1</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Poder Judicial de Entre Ríos</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Solicitud de Cotización</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>240/26</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>Contratación del servicio de reparación prioritaria de seis (6) escalones de mármol de la escalera de acceso al entrepiso y primer piso del Edificio Tribunales de Gualeguaychú sito en calle Roque Sáenz Peña N°94.</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr"/>
+      <c r="I47" s="4" t="inlineStr">
+        <is>
+          <t>Ver el sitio</t>
+        </is>
+      </c>
+      <c r="J47" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K47" s="4" t="inlineStr"/>
+      <c r="L47" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M47" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>Poder Judicial de Entre Ríos</t>
+        </is>
+      </c>
+      <c r="O47" s="4" t="inlineStr">
+        <is>
+          <t>id-ba80195eeddbd2bd</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O45"/>
+  <autoFilter ref="A1:O47"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -3802,6 +3958,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId86"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId87"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L47" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId92"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 27/09/2026 08:02
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$46</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O47"/>
+  <dimension ref="A1:O46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2774,7 +2774,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2782,14 +2782,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>GUALEGUAY — COMUNA DE SEXTO DISTRITO</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -2799,18 +2799,18 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>03/26</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN MAQUINARIA VIAL PARA COMUNA SEXTO DISTRITO – MOTONIVELADORA ARTICULADA”</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2831,12 +2831,12 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-511256e6329e386a</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
@@ -2868,18 +2868,18 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>03/26</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2905,7 +2905,7 @@
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
@@ -2937,18 +2937,18 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>02/2026</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -2974,7 +2974,7 @@
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
@@ -3006,18 +3006,18 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>05/2025</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3043,7 +3043,7 @@
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
@@ -3075,18 +3075,18 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>05/2025</t>
+          <t>06/2025</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3112,7 +3112,7 @@
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
@@ -3142,20 +3142,16 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F37" s="4" t="inlineStr">
-        <is>
-          <t>06/2025</t>
-        </is>
-      </c>
+      <c r="F37" s="4" t="inlineStr"/>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3181,7 +3177,7 @@
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
@@ -3211,16 +3207,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F38" s="4" t="inlineStr"/>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>04/2025</t>
+        </is>
+      </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -3246,7 +3246,7 @@
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>id-ebeeb6a87e688d85</t>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
@@ -3278,18 +3278,18 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>04/2025</t>
+          <t>03/2025</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -3315,14 +3315,14 @@
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
-          <t>id-34c85bcdb9b1123f</t>
+          <t>id-75bfffae63b7eedc</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3347,18 +3347,18 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>03/2025</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr"/>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
+          <t>Publicada 06/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
@@ -3384,7 +3384,7 @@
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
-          <t>id-75bfffae63b7eedc</t>
+          <t>id-07ddb93a12c5a870</t>
         </is>
       </c>
     </row>
@@ -3421,13 +3421,13 @@
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>Concurso de Precio N° 02/2025</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>Publicada 19/06/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
@@ -3453,7 +3453,7 @@
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
-          <t>id-07ddb93a12c5a870</t>
+          <t>id-7c1bf02160a66f67</t>
         </is>
       </c>
     </row>
@@ -3468,35 +3468,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="inlineStr">
-        <is>
-          <t>02/2025</t>
-        </is>
-      </c>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr"/>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>Concurso de Precio N° 02/2025</t>
+          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr"/>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr">
@@ -3517,12 +3513,12 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O42" s="4" t="inlineStr">
         <is>
-          <t>id-7c1bf02160a66f67</t>
+          <t>id-654eebef400f89cd</t>
         </is>
       </c>
     </row>
@@ -3537,9 +3533,9 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C43" s="7" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -3549,13 +3545,17 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F43" s="4" t="inlineStr"/>
+          <t>Concurso</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>01/26</t>
+        </is>
+      </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr"/>
@@ -3587,7 +3587,7 @@
       </c>
       <c r="O43" s="4" t="inlineStr">
         <is>
-          <t>id-654eebef400f89cd</t>
+          <t>id-9a16884dd5a64a49</t>
         </is>
       </c>
     </row>
@@ -3602,29 +3602,29 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Concurso</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>01/26</t>
+          <t>2026-1227</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr"/>
@@ -3651,19 +3651,19 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="O44" s="4" t="inlineStr">
         <is>
-          <t>id-9a16884dd5a64a49</t>
+          <t>id-0691eb485d7548eb</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>26/09/2026</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -3671,35 +3671,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C45" s="7" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>2026-1227</t>
+          <t>08/26</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+          <t>Obra “Readecuación del sistema de climatización –ala sur- Edificio Tribunales Gualeguay”.</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr"/>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Ver el sitio</t>
         </is>
       </c>
       <c r="J45" s="4" t="inlineStr">
@@ -3720,19 +3720,19 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="O45" s="4" t="inlineStr">
         <is>
-          <t>id-0691eb485d7548eb</t>
+          <t>id-9ca2387eef6d6fc1</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>26/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3752,17 +3752,17 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Solicitud de Cotización</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>08/26</t>
+          <t>240/26</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>Obra “Readecuación del sistema de climatización –ala sur- Edificio Tribunales Gualeguay”.</t>
+          <t>Contratación del servicio de reparación prioritaria de seis (6) escalones de mármol de la escalera de acceso al entrepiso y primer piso del Edificio Tribunales de Gualeguaychú sito en calle Roque Sáenz Peña N°94.</t>
         </is>
       </c>
       <c r="H46" s="4" t="inlineStr"/>
@@ -3794,81 +3794,12 @@
       </c>
       <c r="O46" s="4" t="inlineStr">
         <is>
-          <t>id-9ca2387eef6d6fc1</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>24/09/2026</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C47" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Poder Judicial de Entre Ríos</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Solicitud de Cotización</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr">
-        <is>
-          <t>240/26</t>
-        </is>
-      </c>
-      <c r="G47" s="5" t="inlineStr">
-        <is>
-          <t>Contratación del servicio de reparación prioritaria de seis (6) escalones de mármol de la escalera de acceso al entrepiso y primer piso del Edificio Tribunales de Gualeguaychú sito en calle Roque Sáenz Peña N°94.</t>
-        </is>
-      </c>
-      <c r="H47" s="4" t="inlineStr"/>
-      <c r="I47" s="4" t="inlineStr">
-        <is>
-          <t>Ver el sitio</t>
-        </is>
-      </c>
-      <c r="J47" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K47" s="4" t="inlineStr"/>
-      <c r="L47" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M47" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>Poder Judicial de Entre Ríos</t>
-        </is>
-      </c>
-      <c r="O47" s="4" t="inlineStr">
-        <is>
           <t>id-ba80195eeddbd2bd</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O47"/>
+  <autoFilter ref="A1:O46"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -3960,8 +3891,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId88"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId89"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L47" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId92"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 28/09/2026 08:03
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -2774,7 +2774,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2782,35 +2782,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>03/26</t>
-        </is>
-      </c>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr"/>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2831,19 +2827,19 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-654eebef400f89cd</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2858,28 +2854,28 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Concurso</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>02/2026</t>
+          <t>01/26</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2900,19 +2896,19 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-9a16884dd5a64a49</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2920,35 +2916,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C34" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>2026-1227</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -2969,19 +2965,19 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-0691eb485d7548eb</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>26/09/2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2989,14 +2985,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C35" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3006,18 +3002,18 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>05/2025</t>
+          <t>08/26</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
+          <t>Obra “Readecuación del sistema de climatización –ala sur- Edificio Tribunales Gualeguay”.</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>Ver el sitio</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3038,19 +3034,19 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-9ca2387eef6d6fc1</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3058,35 +3054,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C36" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C36" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Solicitud de Cotización</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>06/2025</t>
+          <t>240/26</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>Contratación del servicio de reparación prioritaria de seis (6) escalones de mármol de la escalera de acceso al entrepiso y primer piso del Edificio Tribunales de Gualeguaychú sito en calle Roque Sáenz Peña N°94.</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Ver el sitio</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3107,12 +3103,12 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
+          <t>id-ba80195eeddbd2bd</t>
         </is>
       </c>
     </row>
@@ -3142,16 +3138,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F37" s="4" t="inlineStr"/>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>03/26</t>
+        </is>
+      </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3177,7 +3177,7 @@
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>id-ebeeb6a87e688d85</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
@@ -3209,18 +3209,18 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>04/2025</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -3246,7 +3246,7 @@
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>id-34c85bcdb9b1123f</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
@@ -3278,18 +3278,18 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>03/2025</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -3315,14 +3315,14 @@
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
-          <t>id-75bfffae63b7eedc</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3347,18 +3347,18 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>05/2025</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr"/>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
@@ -3384,14 +3384,14 @@
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
-          <t>id-07ddb93a12c5a870</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3416,18 +3416,18 @@
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>06/2025</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>Concurso de Precio N° 02/2025</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
@@ -3453,14 +3453,14 @@
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
-          <t>id-7c1bf02160a66f67</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3468,31 +3468,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C42" s="7" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr"/>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr"/>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr">
@@ -3513,19 +3513,19 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O42" s="4" t="inlineStr">
         <is>
-          <t>id-654eebef400f89cd</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -3540,28 +3540,28 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Concurso</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>01/26</t>
+          <t>04/2025</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr"/>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr">
@@ -3582,19 +3582,19 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O43" s="4" t="inlineStr">
         <is>
-          <t>id-9a16884dd5a64a49</t>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -3602,35 +3602,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C44" s="7" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>2026-1227</t>
+          <t>03/2025</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr"/>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr">
@@ -3651,19 +3651,19 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O44" s="4" t="inlineStr">
         <is>
-          <t>id-0691eb485d7548eb</t>
+          <t>id-75bfffae63b7eedc</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>26/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -3671,14 +3671,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C45" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -3688,18 +3688,18 @@
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>08/26</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>Obra “Readecuación del sistema de climatización –ala sur- Edificio Tribunales Gualeguay”.</t>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr"/>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>Ver el sitio</t>
+          <t>Publicada 06/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J45" s="4" t="inlineStr">
@@ -3720,19 +3720,19 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O45" s="4" t="inlineStr">
         <is>
-          <t>id-9ca2387eef6d6fc1</t>
+          <t>id-07ddb93a12c5a870</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3740,35 +3740,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C46" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Solicitud de Cotización</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>240/26</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>Contratación del servicio de reparación prioritaria de seis (6) escalones de mármol de la escalera de acceso al entrepiso y primer piso del Edificio Tribunales de Gualeguaychú sito en calle Roque Sáenz Peña N°94.</t>
+          <t>Concurso de Precio N° 02/2025</t>
         </is>
       </c>
       <c r="H46" s="4" t="inlineStr"/>
       <c r="I46" s="4" t="inlineStr">
         <is>
-          <t>Ver el sitio</t>
+          <t>Publicada 19/06/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J46" s="4" t="inlineStr">
@@ -3789,12 +3789,12 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O46" s="4" t="inlineStr">
         <is>
-          <t>id-ba80195eeddbd2bd</t>
+          <t>id-7c1bf02160a66f67</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 29/09/2026 08:05
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -57,11 +57,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00E6D9F2"/>
       </patternFill>
     </fill>
@@ -73,6 +68,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O46"/>
+  <dimension ref="A1:O44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -572,7 +572,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>23/09/2026</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -582,27 +582,27 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Vehículos</t>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>COLON — MUNICIPALIDAD DE VILLA ELISA (E.R.)</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>LICITACIÓN PÚBLICA</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>004/26</t>
+          <t>86/2026</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN DE UN (1) VEHÍCULO PARA TRANSPORTE DE PASAJEROS DE (5) CINCO PLAZAS 0 KM - MODELO/AÑO 2026, PARA LA MUNICIPALIDAD DE LA CIUDAD DE VILLA ELISA, ENTRE RÍOS</t>
+          <t>ADQUISICION DE CAL VIVA AEREA</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
@@ -612,7 +612,7 @@
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>01 de OCTUBRE de 2026 a la hora 10:00 en la Oficina de Compras de la Municipalidad de Villa Elisa, Entre Ríos</t>
+          <t>01-10-2026 08:00</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
@@ -620,11 +620,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">$ 20.000,00 (Pesos Veinte mil con 00/100) el que se puede adquirir en </t>
-        </is>
-      </c>
+      <c r="K2" s="4" t="inlineStr"/>
       <c r="L2" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -637,19 +633,19 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O2" s="4" t="inlineStr">
         <is>
-          <t>id-0132097e777a3442</t>
+          <t>id-ee4153887a6e1e8d</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>23/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -659,37 +655,37 @@
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>Materiales</t>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>86/2026</t>
+          <t>016/2026</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICION DE CAL VIVA AEREA</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de mano de obra, materiales y equipamiento para ejecución de restitución de galibo y repavimentación en Avenida Belgrano y Avenida 1° de Mayo de esta ciudad de chajari</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>02/10/2026</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>01-10-2026 08:00</t>
+          <t>02 DE OCTUBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -697,7 +693,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr"/>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>$ 100.000, 00. - (PESOS CIEN MIL CON 00/100)</t>
+        </is>
+      </c>
       <c r="L3" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -710,19 +710,19 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
-          <t>id-ee4153887a6e1e8d</t>
+          <t>id-53f1430f94acb0b0</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>26/09/2026</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -732,12 +732,12 @@
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>Infraestructura</t>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -747,22 +747,22 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>016/2026</t>
+          <t>07/2026</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de mano de obra, materiales y equipamiento para ejecución de restitución de galibo y repavimentación en Avenida Belgrano y Avenida 1° de Mayo de esta ciudad de chajari</t>
+          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”, destinada a la obra denominada “Nueva Pileta en el Polideportivo El Aguará”,</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>02/10/2026</t>
+          <t>06/10/2026</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>02 DE OCTUBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>06/10/2026 HORA: 11:00 HS</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -772,7 +772,7 @@
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>$ 100.000, 00. - (PESOS CIEN MIL CON 00/100)</t>
+          <t>SIN COSTO</t>
         </is>
       </c>
       <c r="L4" s="6" t="inlineStr">
@@ -792,14 +792,14 @@
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
-          <t>id-53f1430f94acb0b0</t>
+          <t>id-65d18d99bf0b2c6c</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>26/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -807,29 +807,29 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>PARANA — MINISTERIO DE SALUD</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación Publica</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>07/2026</t>
+          <t>17/26</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”, destinada a la obra denominada “Nueva Pileta en el Polideportivo El Aguará”,</t>
+          <t>Adquirir Una (01) Mesa de Anestesia. Destino: Hospital “San José” de Diamante, dependiente del Ministerio de Salud de la Provincia de Entre Ríos</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -839,19 +839,15 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026 HORA: 11:00 HS</t>
+          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr"/>
       <c r="L5" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -869,7 +865,7 @@
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>id-65d18d99bf0b2c6c</t>
+          <t>id-3312d89e1a3e2e53</t>
         </is>
       </c>
     </row>
@@ -884,44 +880,44 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE SALUD</t>
+          <t>MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Licitación Publica</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>17/26</t>
+          <t>31/2026</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Adquirir Una (01) Mesa de Anestesia. Destino: Hospital “San José” de Diamante, dependiente del Ministerio de Salud de la Provincia de Entre Ríos</t>
+          <t>“Pavimento Rígido – 03 (tres) Cuadras Barrio San Felipe”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
+          <t>07 de octubre de 2026 Hora: 10:00</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr"/>
@@ -942,14 +938,14 @@
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>id-3312d89e1a3e2e53</t>
+          <t>id-76d9566cb30a6df5</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>23/09/2026</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -957,9 +953,9 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -974,22 +970,22 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>31/2026</t>
+          <t>32/2026</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>“Pavimento Rígido – 03 (tres) Cuadras Barrio San Felipe”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>"Adquisición de 835 m3 de Hormigón Calidad H25 para 08 cuadras de Pavimento", en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>07 de octubre de 2026 Hora: 10:00</t>
+          <t>08 de octubre de 2026 Hora: 10:00</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -1015,7 +1011,7 @@
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>id-76d9566cb30a6df5</t>
+          <t>id-0ace7de8f16d3baf</t>
         </is>
       </c>
     </row>
@@ -1032,7 +1028,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Materiales</t>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1047,12 +1043,12 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>32/2026</t>
+          <t>33/2026</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>"Adquisición de 835 m3 de Hormigón Calidad H25 para 08 cuadras de Pavimento", en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>“Pavimento Rígido – 04 (cuatro) Cuadras Barrio San Roque y 01 (una) Cuadra Barrio Vicente Obrego”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -1062,7 +1058,7 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>08 de octubre de 2026 Hora: 10:00</t>
+          <t>08 de octubre de 2026 Hora: 11:00</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -1088,7 +1084,7 @@
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>id-0ace7de8f16d3baf</t>
+          <t>id-fe71ac2aaf71b8d8</t>
         </is>
       </c>
     </row>
@@ -1103,14 +1099,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
+          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1120,22 +1116,22 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>33/2026</t>
+          <t>34/2026</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>“Pavimento Rígido – 04 (cuatro) Cuadras Barrio San Roque y 01 (una) Cuadra Barrio Vicente Obrego”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>“Concesión de la Explotación Comercial de un (01) Camión de Comidas Rápidas (para cubrir el total de cuatro puestos) en la Zona Joven – Parque La Salamanca de la Municipalidad de Concepción del Uruguay – Entre Ríos”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>08 de octubre de 2026 Hora: 11:00</t>
+          <t>09 de octubre de 2026 Hora: 10:00</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1161,14 +1157,14 @@
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>id-fe71ac2aaf71b8d8</t>
+          <t>id-b147fbd9d3081bfc</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>23/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1176,14 +1172,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>Vehículos</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1193,12 +1189,12 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>34/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>“Concesión de la Explotación Comercial de un (01) Camión de Comidas Rápidas (para cubrir el total de cuatro puestos) en la Zona Joven – Parque La Salamanca de la Municipalidad de Concepción del Uruguay – Entre Ríos”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>“PROVISIÓN DE UNA (1) MINICARGADORA 0 KM, CON CUCHARÓN FRONTAL DE USO GENERAL, UN (1) MARTILLO HIDRÁULICO Y UN (1) COMPACTADOR/RODILLO VIBRATORIO LISO”</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -1208,7 +1204,7 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>09 de octubre de 2026 Hora: 10:00</t>
+          <t>09/10/2026 HORA: 10:00 HS</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1216,7 +1212,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr"/>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>($ 270.000,00) PESOS DOSCIENTOS SETENTA MIL</t>
+        </is>
+      </c>
       <c r="L10" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1234,7 +1234,7 @@
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>id-b147fbd9d3081bfc</t>
+          <t>id-779e4cd290f2e64e</t>
         </is>
       </c>
     </row>
@@ -1249,14 +1249,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1266,22 +1266,22 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>11/2026</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>“PROVISIÓN DE UNA (1) MINICARGADORA 0 KM, CON CUCHARÓN FRONTAL DE USO GENERAL, UN (1) MARTILLO HIDRÁULICO Y UN (1) COMPACTADOR/RODILLO VIBRATORIO LISO”</t>
+          <t>OBRA "PAVIMENTACION URBANA CALLE TRATADO DEL PILAR B° 3 DE FEBRERO - MUNICIPALIDAD DE SANTA ELENA" (Según Pliegos de Bases y condi ciones)</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>09/10/2026 HORA: 10:00 HS</t>
+          <t>13/10/2026 HORA: 10: 00 HS</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>($ 270.000,00) PESOS DOSCIENTOS SETENTA MIL</t>
+          <t>$ 728.000,00 PESOS SETECIENTOS VEINTIOCHO MIL</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
@@ -1311,14 +1311,14 @@
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>id-779e4cd290f2e64e</t>
+          <t>id-1a2561509308b1b6</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1328,12 +1328,12 @@
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Infraestructura</t>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>OBRA "PAVIMENTACION URBANA CALLE TRATADO DEL PILAR B° 3 DE FEBRERO - MUNICIPALIDAD DE SANTA ELENA" (Según Pliegos de Bases y condi ciones)</t>
+          <t>REFACCION EN ESCUELA N° 65 “ALMIRANTE BROWN” – CIUDAD DE CONCORDIA - DEPARTAMENTO CONCORDIA - PROVINCIA DE ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -1358,19 +1358,15 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026 HORA: 10: 00 HS</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 09:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K12" s="4" t="inlineStr">
-        <is>
-          <t>$ 728.000,00 PESOS SETECIENTOS VEINTIOCHO MIL</t>
-        </is>
-      </c>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr"/>
       <c r="L12" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1388,7 +1384,7 @@
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>id-1a2561509308b1b6</t>
+          <t>id-fc30d5c0b0589a79</t>
         </is>
       </c>
     </row>
@@ -1403,7 +1399,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
@@ -1420,12 +1416,12 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>11/2026</t>
+          <t>13/2026</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>REFACCION EN ESCUELA N° 65 “ALMIRANTE BROWN” – CIUDAD DE CONCORDIA - DEPARTAMENTO CONCORDIA - PROVINCIA DE ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>REPARACIONES VARIAS EN C. P. E. F. Nº 3 “PROFESOR HUGO LA NASA” – CIUDAD DE CONCEPCION DEL URUGUAY - DEPARTAMENTO URUGUAY - PROVINCIA D E ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
@@ -1435,7 +1431,7 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 09:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -1461,7 +1457,7 @@
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>id-fc30d5c0b0589a79</t>
+          <t>id-9d3847fb0e2b0929</t>
         </is>
       </c>
     </row>
@@ -1476,7 +1472,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
@@ -1493,12 +1489,12 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>13/2026</t>
+          <t>12/2026</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>REPARACIONES VARIAS EN C. P. E. F. Nº 3 “PROFESOR HUGO LA NASA” – CIUDAD DE CONCEPCION DEL URUGUAY - DEPARTAMENTO URUGUAY - PROVINCIA D E ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>RECAMBIO DE CUBIERTA Y REPARACIONES VARIAS EN ESCUELA Nº 92 “CONGRESO DE TUCUMAN” – CONCEPCION DEL URUGUAY - DPTO. URUGUAY – PROVINCIA DE ENTRE RIOS de acuerdo a las c ondiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -1508,7 +1504,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 10:30 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1534,14 +1530,14 @@
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>id-9d3847fb0e2b0929</t>
+          <t>id-059239b424b9c936</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>23/09/2026</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1551,12 +1547,12 @@
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
+          <t>VICTORIA — MUNICIPALIDAD DE VICTORIA</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1566,27 +1562,27 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>12/2026</t>
+          <t>008/2026</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>RECAMBIO DE CUBIERTA Y REPARACIONES VARIAS EN ESCUELA Nº 92 “CONGRESO DE TUCUMAN” – CONCEPCION DEL URUGUAY - DPTO. URUGUAY – PROVINCIA DE ENTRE RIOS de acuerdo a las c ondiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>Proveer a la Municipalidad de Victoria, Entre Ríos, de Veinticinco Mil (25.000) litros de Diésel 500, para movilidad de vehículos y maquinarias viales , Ocho Mil (8.000) litros de Gasoil Tipo euro o similar y Ocho (8.000) litros de nafta súper para vehículos y áreas afectadas a la Secretaria de Planeamiento y Dirección de Ambiente y Desarrollo sostenible;</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026</t>
+          <t>14/10/2026</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 10:30 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
+          <t>14 de octubre de 2026 a las 09:00 hs., en la Oficina de Compras de la Municipalidad de Victoria, Entr</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr"/>
@@ -1607,14 +1603,14 @@
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>id-059239b424b9c936</t>
+          <t>id-a9af9f59c8c487c8</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>23/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1622,14 +1618,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>VICTORIA — MUNICIPALIDAD DE VICTORIA</t>
+          <t>SALUD ENTRE RÍOS S.A.U</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1637,24 +1633,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>008/2026</t>
-        </is>
-      </c>
+      <c r="F16" s="4" t="inlineStr"/>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Proveer a la Municipalidad de Victoria, Entre Ríos, de Veinticinco Mil (25.000) litros de Diésel 500, para movilidad de vehículos y maquinarias viales , Ocho Mil (8.000) litros de Gasoil Tipo euro o similar y Ocho (8.000) litros de nafta súper para vehículos y áreas afectadas a la Secretaria de Planeamiento y Dirección de Ambiente y Desarrollo sostenible;</t>
+          <t>Contratación de Servicio de Viandas para el Hospital de la Baxada</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>14/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>14 de octubre de 2026 a las 09:00 hs., en la Oficina de Compras de la Municipalidad de Victoria, Entr</t>
+          <t>Hospital de la Baxada, calle Gral. Al varado Nº 2.250 Paraná, Entre Ríos, el día 19/10/2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -1662,7 +1654,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K16" s="4" t="inlineStr"/>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
       <c r="L16" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1680,7 +1676,7 @@
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>id-a9af9f59c8c487c8</t>
+          <t>id-d35d5e849089d7ac</t>
         </is>
       </c>
     </row>
@@ -1695,14 +1691,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>SALUD ENTRE RÍOS S.A.U</t>
+          <t>PARANA — SALUD ENTRE RÍOS S.A.U</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1713,17 +1709,17 @@
       <c r="F17" s="4" t="inlineStr"/>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Contratación de Servicio de Viandas para el Hospital de la Baxada</t>
+          <t>Servicio de Recolección, Lavado, Desinfección, Secado, Planchado y Transporte de Ropa Hospitalaria</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Hospital de la Baxada, calle Gral. Al varado Nº 2.250 Paraná, Entre Ríos, el día 19/10/2026 a las 10:00 hs</t>
+          <t>Hospital de la Baxada, calle Gral. Alvarado Nº 2.250 Paraná, Entre Ríos, el día 21/10/2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1753,14 +1749,14 @@
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>id-d35d5e849089d7ac</t>
+          <t>id-6b955df9d3f6241a</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>26/09/2026</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1770,12 +1766,12 @@
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>Infraestructura</t>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>PARANA — SALUD ENTRE RÍOS S.A.U</t>
+          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1783,20 +1779,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr"/>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>11/26</t>
+        </is>
+      </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Servicio de Recolección, Lavado, Desinfección, Secado, Planchado y Transporte de Ropa Hospitalaria</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “TERMINACION ESCUELA Nº 40 “JOSÉ ENRIQUE RODÓ”-SEPTIMO DISTRITO-DEPARTAMENTO GUALEGUAY.”</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>21/10/2026</t>
+          <t>23/10/2026</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>Hospital de la Baxada, calle Gral. Alvarado Nº 2.250 Paraná, Entre Ríos, el día 21/10/2026 a las 10:00 hs</t>
+          <t>DE LAS OFERTAS: el día 23 de Octubre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1806,7 +1806,7 @@
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>$ 100 (Cien)</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>id-6b955df9d3f6241a</t>
+          <t>id-86cc9c230734c462</t>
         </is>
       </c>
     </row>
@@ -1841,14 +1841,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1858,12 +1858,12 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>11/26</t>
+          <t>11/2026</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “TERMINACION ESCUELA Nº 40 “JOSÉ ENRIQUE RODÓ”-SEPTIMO DISTRITO-DEPARTAMENTO GUALEGUAY.”</t>
+          <t>Terminación Escuela N° 40 "José Enrique Rodó", Séptimo Distrito</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1873,7 +1873,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 23 de Octubre de 2026 a las 10:00 hs</t>
+          <t>viernes, 23 de octubre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1881,11 +1881,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K19" s="4" t="inlineStr">
-        <is>
-          <t>$ 100 (Cien)</t>
-        </is>
-      </c>
+      <c r="K19" s="4" t="inlineStr"/>
       <c r="L19" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1898,19 +1894,19 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>id-86cc9c230734c462</t>
+          <t>id-322a40f5e43af35d</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>26/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1918,47 +1914,51 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>Municipalidad de Crespo</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>11/2026</t>
+          <t>5/2026</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Terminación Escuela N° 40 "José Enrique Rodó", Séptimo Distrito</t>
+          <t>Adquisición de 145 metros lineales de módulo canal premoldeado.</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>23/10/2026</t>
+          <t>28/09/2026</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>viernes, 23 de octubre de 2026 - 10:00hs</t>
+          <t>28/9/2026 – 10:00 horas</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K20" s="4" t="inlineStr"/>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t>$25.000,00</t>
+        </is>
+      </c>
       <c r="L20" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1971,12 +1971,12 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Municipalidad de Crespo</t>
         </is>
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>id-322a40f5e43af35d</t>
+          <t>id-1609ce58e128c413</t>
         </is>
       </c>
     </row>
@@ -1991,14 +1991,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE CRESPO -- ENTRE RÍOS</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2008,30 +2008,34 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>05/2026</t>
+          <t>08/2026</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 145 metros lineales de modulo canal premoldeado cajón tipo pórtico de 2,00 X 1,00 (interior) X 1,00 mts. de longitud de hormigón para canalizar calle Los Quechuas al final</t>
+          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCL UIDO</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>28 de septiembre de 2026 10:00 Hs. Lugar: Sección Suministros, Palacio Municipal sito en 25 de mayo Nº 943, C</t>
+          <t>29/09/2026</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>08/09/2026</t>
-        </is>
-      </c>
-      <c r="K21" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L21" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2049,7 +2053,7 @@
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-61e8747a99305fe9</t>
+          <t>id-1590925c21c7e363</t>
         </is>
       </c>
     </row>
@@ -2064,49 +2068,49 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Municipalidad de Crespo</t>
+          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>5/2026</t>
+          <t>10/26</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 145 metros lineales de módulo canal premoldeado.</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>28/9/2026 – 10:00 horas</t>
+          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
-          <t>$25.000,00</t>
+          <t>$ 100 (Cien)</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr">
@@ -2121,12 +2125,12 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Municipalidad de Crespo</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-1609ce58e128c413</t>
+          <t>id-75a5c9dd5b4aa6f3</t>
         </is>
       </c>
     </row>
@@ -2141,14 +2145,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2158,22 +2162,22 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>08/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCL UIDO</t>
+          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>29/09/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>29/09/2026</t>
+          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2181,11 +2185,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K23" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K23" s="4" t="inlineStr"/>
       <c r="L23" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2198,34 +2198,34 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-1590925c21c7e363</t>
+          <t>id-46c6d9f1f9210d1e</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2235,22 +2235,18 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>10/26</t>
+          <t>001/26</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>30/09/2026</t>
-        </is>
-      </c>
+          <t>ADQUISICIÓN de UN (1) FURGON UTILITARIO CHICO con 5 asientos 0 KM. con destino a Subsecretaria de Asistencia Directa y Emergencia</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr"/>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>DE LAS PROPUESTAS: 20 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -2258,11 +2254,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K24" s="4" t="inlineStr">
-        <is>
-          <t>$ 100 (Cien)</t>
-        </is>
-      </c>
+      <c r="K24" s="4" t="inlineStr"/>
       <c r="L24" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2280,29 +2272,29 @@
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-75a5c9dd5b4aa6f3</t>
+          <t>id-ca205f0874380f69</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2312,22 +2304,18 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>07/2026</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>30/09/2026</t>
-        </is>
-      </c>
+          <t>Transporte de mil doscientos cincuenta metros cúbicos (1.250 m³) de broza grillada desde Cantera “Tayreta” (Ruta Nacional N° 14 km 135) hasta juris dicción de la comuna, de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr"/>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
+          <t>Viernes 09 de octubre del corriente año a las 10:00 hs en la Oficina de la Sede de la Comuna</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2348,12 +2336,12 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-46c6d9f1f9210d1e</t>
+          <t>id-24e9015ecceeff7f</t>
         </is>
       </c>
     </row>
@@ -2368,35 +2356,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
+          <t>INSTITUTO CARBÓ S.R.L</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>001/26</t>
-        </is>
-      </c>
+          <t>Licitación</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr"/>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN de UN (1) FURGON UTILITARIO CHICO con 5 asientos 0 KM. con destino a Subsecretaria de Asistencia Directa y Emergencia</t>
+          <t>sin internación en materia de salud, pre- hospitalarias, atención médica, domiciliaria y traslados sanitarios de alta</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>DE LAS PROPUESTAS: 20 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2422,14 +2406,14 @@
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-ca205f0874380f69</t>
+          <t>id-6aa57c7437a30ca3</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>26/09/2026</t>
+          <t>23/09/2026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2437,14 +2421,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C27" s="10" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
+          <t>MUNICIPALIDAD DE VIALE</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2454,18 +2438,18 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>07/2026</t>
+          <t>08/26</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>Transporte de mil doscientos cincuenta metros cúbicos (1.250 m³) de broza grillada desde Cantera “Tayreta” (Ruta Nacional N° 14 km 135) hasta juris dicción de la comuna, de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>de asf alto 70-16 destinado a la producción de pavimento de la Planta Asfáltica, y que a continuación se detalla y</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Viernes 09 de octubre del corriente año a las 10:00 hs en la Oficina de la Sede de la Comuna</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2491,14 +2475,14 @@
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-24e9015ecceeff7f</t>
+          <t>id-ef1ddb923c7e7fdb</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>26/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2508,29 +2492,33 @@
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>Infraestructura</t>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>INSTITUTO CARBÓ S.R.L</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Licitación</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>001-2026</t>
+        </is>
+      </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>sin internación en materia de salud, pre- hospitalarias, atención médica, domiciliaria y traslados sanitarios de alta</t>
+          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2538,7 +2526,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K28" s="4" t="inlineStr"/>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L28" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2556,14 +2548,14 @@
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-6aa57c7437a30ca3</t>
+          <t>id-b7b0120caf49d551</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>23/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2571,14 +2563,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C29" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE VIALE</t>
+          <t>MUNICIPALIDAD DE URDINARRAIN</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2588,12 +2580,12 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>08/26</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>de asf alto 70-16 destinado a la producción de pavimento de la Planta Asfáltica, y que a continuación se detalla y</t>
+          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
@@ -2625,14 +2617,14 @@
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-ef1ddb923c7e7fdb</t>
+          <t>id-7a200161bcc9b02b</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>26/09/2026</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2640,14 +2632,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C30" s="9" t="inlineStr">
+      <c r="C30" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2657,18 +2649,18 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>001-2026</t>
+          <t>08/26</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
+          <t>Obra “Readecuación del sistema de climatización –ala sur- Edificio Tribunales Gualeguay”.</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
+          <t>Ver el sitio</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2676,11 +2668,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K30" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K30" s="4" t="inlineStr"/>
       <c r="L30" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2693,19 +2681,19 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-b7b0120caf49d551</t>
+          <t>id-9ca2387eef6d6fc1</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2713,35 +2701,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C31" s="7" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE URDINARRAIN</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Solicitud de Cotización</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>240/26</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
+          <t>Contratación del servicio de reparación prioritaria de seis (6) escalones de mármol de la escalera de acceso al entrepiso y primer piso del Edificio Tribunales de Gualeguaychú sito en calle Roque Sáenz Peña N°94.</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Ver el sitio</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2762,12 +2750,12 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-7a200161bcc9b02b</t>
+          <t>id-ba80195eeddbd2bd</t>
         </is>
       </c>
     </row>
@@ -2782,7 +2770,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C32" s="7" t="inlineStr">
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>Materiales</t>
         </is>
@@ -2847,7 +2835,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C33" s="8" t="inlineStr">
+      <c r="C33" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2916,7 +2904,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>Materiales</t>
         </is>
@@ -2977,7 +2965,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>26/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2985,14 +2973,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C35" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3002,18 +2990,18 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>08/26</t>
+          <t>03/26</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>Obra “Readecuación del sistema de climatización –ala sur- Edificio Tribunales Gualeguay”.</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Ver el sitio</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3034,19 +3022,19 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-9ca2387eef6d6fc1</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3054,35 +3042,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C36" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Solicitud de Cotización</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>240/26</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>Contratación del servicio de reparación prioritaria de seis (6) escalones de mármol de la escalera de acceso al entrepiso y primer piso del Edificio Tribunales de Gualeguaychú sito en calle Roque Sáenz Peña N°94.</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Ver el sitio</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3103,12 +3091,12 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>id-ba80195eeddbd2bd</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
@@ -3123,7 +3111,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C37" s="8" t="inlineStr">
+      <c r="C37" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -3140,18 +3128,18 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>03/26</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3177,7 +3165,7 @@
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
@@ -3192,7 +3180,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C38" s="8" t="inlineStr">
+      <c r="C38" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -3209,18 +3197,18 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>02/2026</t>
+          <t>05/2025</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -3246,7 +3234,7 @@
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
@@ -3261,7 +3249,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C39" s="8" t="inlineStr">
+      <c r="C39" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -3278,18 +3266,18 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>06/2025</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -3315,7 +3303,7 @@
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
@@ -3330,7 +3318,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C40" s="8" t="inlineStr">
+      <c r="C40" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -3345,20 +3333,16 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F40" s="4" t="inlineStr">
-        <is>
-          <t>05/2025</t>
-        </is>
-      </c>
+      <c r="F40" s="4" t="inlineStr"/>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr"/>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
@@ -3384,7 +3368,7 @@
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
@@ -3399,7 +3383,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C41" s="8" t="inlineStr">
+      <c r="C41" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -3416,18 +3400,18 @@
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>06/2025</t>
+          <t>04/2025</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
@@ -3453,7 +3437,7 @@
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
@@ -3468,7 +3452,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C42" s="8" t="inlineStr">
+      <c r="C42" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -3483,16 +3467,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F42" s="4" t="inlineStr"/>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>03/2025</t>
+        </is>
+      </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr"/>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr">
@@ -3518,14 +3506,14 @@
       </c>
       <c r="O42" s="4" t="inlineStr">
         <is>
-          <t>id-ebeeb6a87e688d85</t>
+          <t>id-75bfffae63b7eedc</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -3533,7 +3521,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C43" s="8" t="inlineStr">
+      <c r="C43" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -3550,18 +3538,18 @@
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>04/2025</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr"/>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
+          <t>Publicada 06/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr">
@@ -3587,14 +3575,14 @@
       </c>
       <c r="O43" s="4" t="inlineStr">
         <is>
-          <t>id-34c85bcdb9b1123f</t>
+          <t>id-07ddb93a12c5a870</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -3602,7 +3590,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C44" s="8" t="inlineStr">
+      <c r="C44" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -3619,18 +3607,18 @@
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>03/2025</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+          <t>Concurso de Precio N° 02/2025</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr"/>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
+          <t>Publicada 19/06/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr">
@@ -3656,150 +3644,12 @@
       </c>
       <c r="O44" s="4" t="inlineStr">
         <is>
-          <t>id-75bfffae63b7eedc</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>IAPV (Vivienda)</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="inlineStr">
-        <is>
-          <t>02/2025</t>
-        </is>
-      </c>
-      <c r="G45" s="5" t="inlineStr">
-        <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
-        </is>
-      </c>
-      <c r="H45" s="4" t="inlineStr"/>
-      <c r="I45" s="4" t="inlineStr">
-        <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
-        </is>
-      </c>
-      <c r="J45" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K45" s="4" t="inlineStr"/>
-      <c r="L45" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M45" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>IAPV — Viviendas</t>
-        </is>
-      </c>
-      <c r="O45" s="4" t="inlineStr">
-        <is>
-          <t>id-07ddb93a12c5a870</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>IAPV (Vivienda)</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="inlineStr">
-        <is>
-          <t>02/2025</t>
-        </is>
-      </c>
-      <c r="G46" s="5" t="inlineStr">
-        <is>
-          <t>Concurso de Precio N° 02/2025</t>
-        </is>
-      </c>
-      <c r="H46" s="4" t="inlineStr"/>
-      <c r="I46" s="4" t="inlineStr">
-        <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
-        </is>
-      </c>
-      <c r="J46" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K46" s="4" t="inlineStr"/>
-      <c r="L46" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M46" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>IAPV — Viviendas</t>
-        </is>
-      </c>
-      <c r="O46" s="4" t="inlineStr">
-        <is>
           <t>id-7c1bf02160a66f67</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O46"/>
+  <autoFilter ref="A1:O44"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -3887,10 +3737,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId84"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId85"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId90"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 30/09/2026 08:03
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$43</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O44"/>
+  <dimension ref="A1:O43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1991,14 +1991,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2008,22 +2008,22 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>08/2026</t>
+          <t>10/26</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>“PROVISION DE “UN (1) CAMIÓN CON CAJA VOLCADORA 0 KM”. -PRESUPUESTO: ($ 129.000.000,00), PESOS CIENTO VEINTINUEVE MILLONES IVA INCL UIDO</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>29/09/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>29/09/2026</t>
+          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -2033,7 +2033,7 @@
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>SIN COSTO</t>
+          <t>$ 100 (Cien)</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr">
@@ -2053,7 +2053,7 @@
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-1590925c21c7e363</t>
+          <t>id-75a5c9dd5b4aa6f3</t>
         </is>
       </c>
     </row>
@@ -2075,7 +2075,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2085,12 +2085,12 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>10/26</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
+          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -2100,7 +2100,7 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -2108,11 +2108,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K22" s="4" t="inlineStr">
-        <is>
-          <t>$ 100 (Cien)</t>
-        </is>
-      </c>
+      <c r="K22" s="4" t="inlineStr"/>
       <c r="L22" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2125,34 +2121,34 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-75a5c9dd5b4aa6f3</t>
+          <t>id-46c6d9f1f9210d1e</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2162,22 +2158,18 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>001/26</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t>30/09/2026</t>
-        </is>
-      </c>
+          <t>ADQUISICIÓN de UN (1) FURGON UTILITARIO CHICO con 5 asientos 0 KM. con destino a Subsecretaria de Asistencia Directa y Emergencia</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr"/>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
+          <t>DE LAS PROPUESTAS: 20 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2198,12 +2190,12 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-46c6d9f1f9210d1e</t>
+          <t>id-ca205f0874380f69</t>
         </is>
       </c>
     </row>
@@ -2218,14 +2210,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
+          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2235,18 +2227,18 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>001/26</t>
+          <t>07/2026</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN de UN (1) FURGON UTILITARIO CHICO con 5 asientos 0 KM. con destino a Subsecretaria de Asistencia Directa y Emergencia</t>
+          <t>Transporte de mil doscientos cincuenta metros cúbicos (1.250 m³) de broza grillada desde Cantera “Tayreta” (Ruta Nacional N° 14 km 135) hasta juris dicción de la comuna, de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr"/>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>DE LAS PROPUESTAS: 20 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
+          <t>Viernes 09 de octubre del corriente año a las 10:00 hs en la Oficina de la Sede de la Comuna</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -2272,7 +2264,7 @@
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-ca205f0874380f69</t>
+          <t>id-24e9015ecceeff7f</t>
         </is>
       </c>
     </row>
@@ -2287,35 +2279,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C25" s="10" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
+          <t>INSTITUTO CARBÓ S.R.L</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>07/2026</t>
-        </is>
-      </c>
+          <t>Licitación</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr"/>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>Transporte de mil doscientos cincuenta metros cúbicos (1.250 m³) de broza grillada desde Cantera “Tayreta” (Ruta Nacional N° 14 km 135) hasta juris dicción de la comuna, de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>sin internación en materia de salud, pre- hospitalarias, atención médica, domiciliaria y traslados sanitarios de alta</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr"/>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Viernes 09 de octubre del corriente año a las 10:00 hs en la Oficina de la Sede de la Comuna</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2341,14 +2329,14 @@
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-24e9015ecceeff7f</t>
+          <t>id-6aa57c7437a30ca3</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>26/09/2026</t>
+          <t>23/09/2026</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2363,18 +2351,22 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>INSTITUTO CARBÓ S.R.L</t>
+          <t>MUNICIPALIDAD DE VIALE</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Licitación</t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>08/26</t>
+        </is>
+      </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>sin internación en materia de salud, pre- hospitalarias, atención médica, domiciliaria y traslados sanitarios de alta</t>
+          <t>de asf alto 70-16 destinado a la producción de pavimento de la Planta Asfáltica, y que a continuación se detalla y</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
@@ -2406,14 +2398,14 @@
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-6aa57c7437a30ca3</t>
+          <t>id-ef1ddb923c7e7fdb</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>23/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2421,14 +2413,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE VIALE</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2438,18 +2430,18 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>08/26</t>
+          <t>001-2026</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>de asf alto 70-16 destinado a la producción de pavimento de la Planta Asfáltica, y que a continuación se detalla y</t>
+          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2457,7 +2449,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K27" s="4" t="inlineStr"/>
+      <c r="K27" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L27" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2475,7 +2471,7 @@
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-ef1ddb923c7e7fdb</t>
+          <t>id-b7b0120caf49d551</t>
         </is>
       </c>
     </row>
@@ -2490,14 +2486,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
+          <t>MUNICIPALIDAD DE URDINARRAIN</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2507,18 +2503,18 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>001-2026</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
+          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2526,11 +2522,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K28" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K28" s="4" t="inlineStr"/>
       <c r="L28" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2548,14 +2540,14 @@
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-b7b0120caf49d551</t>
+          <t>id-7a200161bcc9b02b</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>26/09/2026</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2563,14 +2555,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE URDINARRAIN</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2580,18 +2572,18 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>08/26</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
+          <t>Obra “Readecuación del sistema de climatización –ala sur- Edificio Tribunales Gualeguay”.</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Ver el sitio</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2612,19 +2604,19 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-7a200161bcc9b02b</t>
+          <t>id-9ca2387eef6d6fc1</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>26/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2644,17 +2636,17 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Solicitud de Cotización</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>08/26</t>
+          <t>240/26</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>Obra “Readecuación del sistema de climatización –ala sur- Edificio Tribunales Gualeguay”.</t>
+          <t>Contratación del servicio de reparación prioritaria de seis (6) escalones de mármol de la escalera de acceso al entrepiso y primer piso del Edificio Tribunales de Gualeguaychú sito en calle Roque Sáenz Peña N°94.</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
@@ -2686,14 +2678,14 @@
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-9ca2387eef6d6fc1</t>
+          <t>id-ba80195eeddbd2bd</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2701,35 +2693,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Solicitud de Cotización</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>240/26</t>
-        </is>
-      </c>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr"/>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>Contratación del servicio de reparación prioritaria de seis (6) escalones de mármol de la escalera de acceso al entrepiso y primer piso del Edificio Tribunales de Gualeguaychú sito en calle Roque Sáenz Peña N°94.</t>
+          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Ver el sitio</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2750,12 +2738,12 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-ba80195eeddbd2bd</t>
+          <t>id-654eebef400f89cd</t>
         </is>
       </c>
     </row>
@@ -2770,9 +2758,9 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2782,13 +2770,17 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr"/>
+          <t>Concurso</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>01/26</t>
+        </is>
+      </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
@@ -2820,7 +2812,7 @@
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-654eebef400f89cd</t>
+          <t>id-9a16884dd5a64a49</t>
         </is>
       </c>
     </row>
@@ -2835,29 +2827,29 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C33" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Concurso</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>01/26</t>
+          <t>2026-1227</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
@@ -2884,19 +2876,19 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-9a16884dd5a64a49</t>
+          <t>id-0691eb485d7548eb</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2904,35 +2896,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>2026-1227</t>
+          <t>03/26</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -2953,12 +2945,12 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-0691eb485d7548eb</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
@@ -2990,18 +2982,18 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>03/26</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3027,7 +3019,7 @@
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
@@ -3059,18 +3051,18 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>02/2026</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3096,7 +3088,7 @@
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
@@ -3128,18 +3120,18 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>05/2025</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3165,7 +3157,7 @@
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
@@ -3197,18 +3189,18 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>05/2025</t>
+          <t>06/2025</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -3234,7 +3226,7 @@
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
@@ -3264,20 +3256,16 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F39" s="4" t="inlineStr">
-        <is>
-          <t>06/2025</t>
-        </is>
-      </c>
+      <c r="F39" s="4" t="inlineStr"/>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -3303,7 +3291,7 @@
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
@@ -3333,16 +3321,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F40" s="4" t="inlineStr"/>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>04/2025</t>
+        </is>
+      </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr"/>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
@@ -3368,7 +3360,7 @@
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
-          <t>id-ebeeb6a87e688d85</t>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
@@ -3400,18 +3392,18 @@
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>04/2025</t>
+          <t>03/2025</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
@@ -3437,14 +3429,14 @@
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
-          <t>id-34c85bcdb9b1123f</t>
+          <t>id-75bfffae63b7eedc</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3469,18 +3461,18 @@
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>03/2025</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr"/>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
+          <t>Publicada 06/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr">
@@ -3506,7 +3498,7 @@
       </c>
       <c r="O42" s="4" t="inlineStr">
         <is>
-          <t>id-75bfffae63b7eedc</t>
+          <t>id-07ddb93a12c5a870</t>
         </is>
       </c>
     </row>
@@ -3543,13 +3535,13 @@
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>Concurso de Precio N° 02/2025</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr"/>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>Publicada 19/06/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr">
@@ -3575,81 +3567,12 @@
       </c>
       <c r="O43" s="4" t="inlineStr">
         <is>
-          <t>id-07ddb93a12c5a870</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C44" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>IAPV (Vivienda)</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t>02/2025</t>
-        </is>
-      </c>
-      <c r="G44" s="5" t="inlineStr">
-        <is>
-          <t>Concurso de Precio N° 02/2025</t>
-        </is>
-      </c>
-      <c r="H44" s="4" t="inlineStr"/>
-      <c r="I44" s="4" t="inlineStr">
-        <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
-        </is>
-      </c>
-      <c r="J44" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K44" s="4" t="inlineStr"/>
-      <c r="L44" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M44" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N44" t="inlineStr">
-        <is>
-          <t>IAPV — Viviendas</t>
-        </is>
-      </c>
-      <c r="O44" s="4" t="inlineStr">
-        <is>
           <t>id-7c1bf02160a66f67</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O44"/>
+  <autoFilter ref="A1:O43"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -3735,8 +3658,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId82"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L43" r:id="rId83"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId86"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 01/10/2026 08:22
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O43"/>
+  <dimension ref="A1:O42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1998,7 +1998,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2008,12 +2008,12 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>10/26</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “ IMPERMEABILIZACION CUBIERTA DE TECHOS, REPARACION DE MAMPOSTERIAS Y PINTURA ESCUELA Nº 2 “ALVAREZ CONDARCO”-CHAJARI-DEPARTAME NTO FEDERACION.”</t>
+          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -2023,7 +2023,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 30 de Septiembre de 2026 a las 10:00 hs</t>
+          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -2031,11 +2031,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K21" s="4" t="inlineStr">
-        <is>
-          <t>$ 100 (Cien)</t>
-        </is>
-      </c>
+      <c r="K21" s="4" t="inlineStr"/>
       <c r="L21" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2048,34 +2044,34 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-75a5c9dd5b4aa6f3</t>
+          <t>id-46c6d9f1f9210d1e</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2085,22 +2081,18 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>001/26</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr">
-        <is>
-          <t>30/09/2026</t>
-        </is>
-      </c>
+          <t>ADQUISICIÓN de UN (1) FURGON UTILITARIO CHICO con 5 asientos 0 KM. con destino a Subsecretaria de Asistencia Directa y Emergencia</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr"/>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
+          <t>DE LAS PROPUESTAS: 20 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -2121,12 +2113,12 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-46c6d9f1f9210d1e</t>
+          <t>id-ca205f0874380f69</t>
         </is>
       </c>
     </row>
@@ -2141,14 +2133,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
+          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2158,18 +2150,18 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>001/26</t>
+          <t>07/2026</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN de UN (1) FURGON UTILITARIO CHICO con 5 asientos 0 KM. con destino a Subsecretaria de Asistencia Directa y Emergencia</t>
+          <t>Transporte de mil doscientos cincuenta metros cúbicos (1.250 m³) de broza grillada desde Cantera “Tayreta” (Ruta Nacional N° 14 km 135) hasta juris dicción de la comuna, de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr"/>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>DE LAS PROPUESTAS: 20 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
+          <t>Viernes 09 de octubre del corriente año a las 10:00 hs en la Oficina de la Sede de la Comuna</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2195,7 +2187,7 @@
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-ca205f0874380f69</t>
+          <t>id-24e9015ecceeff7f</t>
         </is>
       </c>
     </row>
@@ -2210,35 +2202,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C24" s="10" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
+          <t>INSTITUTO CARBÓ S.R.L</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>07/2026</t>
-        </is>
-      </c>
+          <t>Licitación</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr"/>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Transporte de mil doscientos cincuenta metros cúbicos (1.250 m³) de broza grillada desde Cantera “Tayreta” (Ruta Nacional N° 14 km 135) hasta juris dicción de la comuna, de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>sin internación en materia de salud, pre- hospitalarias, atención médica, domiciliaria y traslados sanitarios de alta</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr"/>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>Viernes 09 de octubre del corriente año a las 10:00 hs en la Oficina de la Sede de la Comuna</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -2264,14 +2252,14 @@
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-24e9015ecceeff7f</t>
+          <t>id-6aa57c7437a30ca3</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>26/09/2026</t>
+          <t>23/09/2026</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2286,18 +2274,22 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>INSTITUTO CARBÓ S.R.L</t>
+          <t>MUNICIPALIDAD DE VIALE</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Licitación</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>08/26</t>
+        </is>
+      </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>sin internación en materia de salud, pre- hospitalarias, atención médica, domiciliaria y traslados sanitarios de alta</t>
+          <t>de asf alto 70-16 destinado a la producción de pavimento de la Planta Asfáltica, y que a continuación se detalla y</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr"/>
@@ -2329,14 +2321,14 @@
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-6aa57c7437a30ca3</t>
+          <t>id-ef1ddb923c7e7fdb</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>23/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2344,14 +2336,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE VIALE</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2361,18 +2353,18 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>08/26</t>
+          <t>001-2026</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>de asf alto 70-16 destinado a la producción de pavimento de la Planta Asfáltica, y que a continuación se detalla y</t>
+          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2380,7 +2372,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K26" s="4" t="inlineStr"/>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L26" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2398,7 +2394,7 @@
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-ef1ddb923c7e7fdb</t>
+          <t>id-b7b0120caf49d551</t>
         </is>
       </c>
     </row>
@@ -2413,14 +2409,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C27" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
+          <t>MUNICIPALIDAD DE URDINARRAIN</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2430,18 +2426,18 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>001-2026</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
+          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2449,11 +2445,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K27" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K27" s="4" t="inlineStr"/>
       <c r="L27" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2471,14 +2463,14 @@
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-b7b0120caf49d551</t>
+          <t>id-7a200161bcc9b02b</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>26/09/2026</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2486,14 +2478,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE URDINARRAIN</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2503,18 +2495,18 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>08/26</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
+          <t>Obra “Readecuación del sistema de climatización –ala sur- Edificio Tribunales Gualeguay”.</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Ver el sitio</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2535,19 +2527,19 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-7a200161bcc9b02b</t>
+          <t>id-9ca2387eef6d6fc1</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>26/09/2026</t>
+          <t>24/09/2026</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2567,17 +2559,17 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Solicitud de Cotización</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>08/26</t>
+          <t>240/26</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Obra “Readecuación del sistema de climatización –ala sur- Edificio Tribunales Gualeguay”.</t>
+          <t>Contratación del servicio de reparación prioritaria de seis (6) escalones de mármol de la escalera de acceso al entrepiso y primer piso del Edificio Tribunales de Gualeguaychú sito en calle Roque Sáenz Peña N°94.</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
@@ -2609,14 +2601,14 @@
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-9ca2387eef6d6fc1</t>
+          <t>id-ba80195eeddbd2bd</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2624,35 +2616,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C30" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Solicitud de Cotización</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>240/26</t>
-        </is>
-      </c>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr"/>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>Contratación del servicio de reparación prioritaria de seis (6) escalones de mármol de la escalera de acceso al entrepiso y primer piso del Edificio Tribunales de Gualeguaychú sito en calle Roque Sáenz Peña N°94.</t>
+          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Ver el sitio</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2673,12 +2661,12 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-ba80195eeddbd2bd</t>
+          <t>id-654eebef400f89cd</t>
         </is>
       </c>
     </row>
@@ -2693,9 +2681,9 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2705,13 +2693,17 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr"/>
+          <t>Concurso</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>01/26</t>
+        </is>
+      </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
@@ -2743,7 +2735,7 @@
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-654eebef400f89cd</t>
+          <t>id-9a16884dd5a64a49</t>
         </is>
       </c>
     </row>
@@ -2758,29 +2750,29 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C32" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Concurso</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>01/26</t>
+          <t>2026-1227</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
@@ -2807,19 +2799,19 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-9a16884dd5a64a49</t>
+          <t>id-0691eb485d7548eb</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2827,35 +2819,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>2026-1227</t>
+          <t>03/26</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2876,12 +2868,12 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-0691eb485d7548eb</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
@@ -2913,18 +2905,18 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>03/26</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -2950,7 +2942,7 @@
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
@@ -2982,18 +2974,18 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>02/2026</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3019,7 +3011,7 @@
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
@@ -3051,18 +3043,18 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>05/2025</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3088,7 +3080,7 @@
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
@@ -3120,18 +3112,18 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>05/2025</t>
+          <t>06/2025</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3157,7 +3149,7 @@
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
@@ -3187,20 +3179,16 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F38" s="4" t="inlineStr">
-        <is>
-          <t>06/2025</t>
-        </is>
-      </c>
+      <c r="F38" s="4" t="inlineStr"/>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -3226,7 +3214,7 @@
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
@@ -3256,16 +3244,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F39" s="4" t="inlineStr"/>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>04/2025</t>
+        </is>
+      </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -3291,7 +3283,7 @@
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
-          <t>id-ebeeb6a87e688d85</t>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
@@ -3323,18 +3315,18 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>04/2025</t>
+          <t>03/2025</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr"/>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
@@ -3360,14 +3352,14 @@
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
-          <t>id-34c85bcdb9b1123f</t>
+          <t>id-75bfffae63b7eedc</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3392,18 +3384,18 @@
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>03/2025</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
+          <t>Publicada 06/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
@@ -3429,7 +3421,7 @@
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
-          <t>id-75bfffae63b7eedc</t>
+          <t>id-07ddb93a12c5a870</t>
         </is>
       </c>
     </row>
@@ -3466,13 +3458,13 @@
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>Concurso de Precio N° 02/2025</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr"/>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>Publicada 19/06/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr">
@@ -3498,81 +3490,12 @@
       </c>
       <c r="O42" s="4" t="inlineStr">
         <is>
-          <t>id-07ddb93a12c5a870</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C43" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>IAPV (Vivienda)</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F43" s="4" t="inlineStr">
-        <is>
-          <t>02/2025</t>
-        </is>
-      </c>
-      <c r="G43" s="5" t="inlineStr">
-        <is>
-          <t>Concurso de Precio N° 02/2025</t>
-        </is>
-      </c>
-      <c r="H43" s="4" t="inlineStr"/>
-      <c r="I43" s="4" t="inlineStr">
-        <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
-        </is>
-      </c>
-      <c r="J43" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K43" s="4" t="inlineStr"/>
-      <c r="L43" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M43" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>IAPV — Viviendas</t>
-        </is>
-      </c>
-      <c r="O43" s="4" t="inlineStr">
-        <is>
           <t>id-7c1bf02160a66f67</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O43"/>
+  <autoFilter ref="A1:O42"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -3656,8 +3579,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId80"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId81"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L43" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId84"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Sumar el Boletín Oficial de la Municipalidad de Paraná
Las obras públicas grandes de Paraná (como la 87/2026, red cloacal del Colector
Noroeste por $636M) NO salen en compras.parana.gob.ar: ahí sólo hay compras
chicas. Van por el Boletín Oficial municipal, que al 01/10/2026 está fuera de
servicio ('estamos trabajando para reestablecer el servicio').

Queda cargado y activo: cuando lo restablezcan empieza a traer solo y el
Diagnóstico lo muestra en verde. Verificado que esa licitación tampoco aparece
en el Boletín provincial.
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$37</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -57,7 +57,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E6D9F2"/>
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -67,12 +72,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00E6D9F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O42"/>
+  <dimension ref="A1:O37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -572,7 +572,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>23/09/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -582,7 +582,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Materiales</t>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -592,17 +592,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA</t>
+          <t>CONCURSO DE PRECIOS</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>86/2026</t>
+          <t>311/2026</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICION DE CAL VIVA AEREA</t>
+          <t>ADQUISICION DE LAMPARAS PARA VEHICULOS</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
@@ -612,7 +612,7 @@
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>01-10-2026 08:00</t>
+          <t>01-10-2026 10:30</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
@@ -638,14 +638,14 @@
       </c>
       <c r="O2" s="4" t="inlineStr">
         <is>
-          <t>id-ee4153887a6e1e8d</t>
+          <t>id-5824d400c85d33c6</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -655,37 +655,37 @@
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>Infraestructura</t>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>CONCURSO DE PRECIOS</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>016/2026</t>
+          <t>321/2026</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de mano de obra, materiales y equipamiento para ejecución de restitución de galibo y repavimentación en Avenida Belgrano y Avenida 1° de Mayo de esta ciudad de chajari</t>
+          <t>ALQUILER DE CARPAS, BAÑOS QUIMICOS Y DISPENSER</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>02/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>02 DE OCTUBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>01-10-2026 11:30</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -693,11 +693,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>$ 100.000, 00. - (PESOS CIEN MIL CON 00/100)</t>
-        </is>
-      </c>
+      <c r="K3" s="4" t="inlineStr"/>
       <c r="L3" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -710,19 +706,19 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
-          <t>id-53f1430f94acb0b0</t>
+          <t>id-ee8fe54e83fd3889</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>26/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -732,12 +728,12 @@
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -747,22 +743,22 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>07/2026</t>
+          <t>016/2026</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”, destinada a la obra denominada “Nueva Pileta en el Polideportivo El Aguará”,</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de mano de obra, materiales y equipamiento para ejecución de restitución de galibo y repavimentación en Avenida Belgrano y Avenida 1° de Mayo de esta ciudad de chajari</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
+          <t>02/10/2026</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026 HORA: 11:00 HS</t>
+          <t>02 DE OCTUBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -772,7 +768,7 @@
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>SIN COSTO</t>
+          <t>$ 100.000, 00. - (PESOS CIEN MIL CON 00/100)</t>
         </is>
       </c>
       <c r="L4" s="6" t="inlineStr">
@@ -792,14 +788,14 @@
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
-          <t>id-65d18d99bf0b2c6c</t>
+          <t>id-53f1430f94acb0b0</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>26/09/2026</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -809,27 +805,27 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Infraestructura</t>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE SALUD</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Licitación Publica</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>17/26</t>
+          <t>07/2026</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Adquirir Una (01) Mesa de Anestesia. Destino: Hospital “San José” de Diamante, dependiente del Ministerio de Salud de la Provincia de Entre Ríos</t>
+          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”, destinada a la obra denominada “Nueva Pileta en el Polideportivo El Aguará”,</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -839,15 +835,19 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
+          <t>06/10/2026 HORA: 11:00 HS</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
-        </is>
-      </c>
-      <c r="K5" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L5" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -865,7 +865,7 @@
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>id-3312d89e1a3e2e53</t>
+          <t>id-65d18d99bf0b2c6c</t>
         </is>
       </c>
     </row>
@@ -880,44 +880,44 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
+          <t>PARANA — MINISTERIO DE SALUD</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación Publica</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>31/2026</t>
+          <t>17/26</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>“Pavimento Rígido – 03 (tres) Cuadras Barrio San Felipe”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>Adquirir Una (01) Mesa de Anestesia. Destino: Hospital “San José” de Diamante, dependiente del Ministerio de Salud de la Provincia de Entre Ríos</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>06/10/2026</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>07 de octubre de 2026 Hora: 10:00</t>
+          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>06/10/2026</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr"/>
@@ -938,14 +938,14 @@
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>id-76d9566cb30a6df5</t>
+          <t>id-3312d89e1a3e2e53</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>23/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -953,9 +953,9 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -970,22 +970,22 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>32/2026</t>
+          <t>31/2026</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>"Adquisición de 835 m3 de Hormigón Calidad H25 para 08 cuadras de Pavimento", en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>“Pavimento Rígido – 03 (tres) Cuadras Barrio San Felipe”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>08 de octubre de 2026 Hora: 10:00</t>
+          <t>07 de octubre de 2026 Hora: 10:00</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -1011,7 +1011,7 @@
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>id-0ace7de8f16d3baf</t>
+          <t>id-76d9566cb30a6df5</t>
         </is>
       </c>
     </row>
@@ -1026,9 +1026,9 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1043,12 +1043,12 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>33/2026</t>
+          <t>32/2026</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>“Pavimento Rígido – 04 (cuatro) Cuadras Barrio San Roque y 01 (una) Cuadra Barrio Vicente Obrego”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>"Adquisición de 835 m3 de Hormigón Calidad H25 para 08 cuadras de Pavimento", en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>08 de octubre de 2026 Hora: 11:00</t>
+          <t>08 de octubre de 2026 Hora: 10:00</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -1084,7 +1084,7 @@
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>id-fe71ac2aaf71b8d8</t>
+          <t>id-0ace7de8f16d3baf</t>
         </is>
       </c>
     </row>
@@ -1099,14 +1099,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
+          <t>MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1116,22 +1116,22 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>34/2026</t>
+          <t>33/2026</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>“Concesión de la Explotación Comercial de un (01) Camión de Comidas Rápidas (para cubrir el total de cuatro puestos) en la Zona Joven – Parque La Salamanca de la Municipalidad de Concepción del Uruguay – Entre Ríos”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>“Pavimento Rígido – 04 (cuatro) Cuadras Barrio San Roque y 01 (una) Cuadra Barrio Vicente Obrego”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>09 de octubre de 2026 Hora: 10:00</t>
+          <t>08 de octubre de 2026 Hora: 11:00</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1157,14 +1157,14 @@
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>id-b147fbd9d3081bfc</t>
+          <t>id-fe71ac2aaf71b8d8</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>23/09/2026</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1172,14 +1172,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Vehículos</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1189,12 +1189,12 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>34/2026</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>“PROVISIÓN DE UNA (1) MINICARGADORA 0 KM, CON CUCHARÓN FRONTAL DE USO GENERAL, UN (1) MARTILLO HIDRÁULICO Y UN (1) COMPACTADOR/RODILLO VIBRATORIO LISO”</t>
+          <t>“Concesión de la Explotación Comercial de un (01) Camión de Comidas Rápidas (para cubrir el total de cuatro puestos) en la Zona Joven – Parque La Salamanca de la Municipalidad de Concepción del Uruguay – Entre Ríos”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -1204,7 +1204,7 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>09/10/2026 HORA: 10:00 HS</t>
+          <t>09 de octubre de 2026 Hora: 10:00</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1212,11 +1212,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr">
-        <is>
-          <t>($ 270.000,00) PESOS DOSCIENTOS SETENTA MIL</t>
-        </is>
-      </c>
+      <c r="K10" s="4" t="inlineStr"/>
       <c r="L10" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1234,7 +1230,7 @@
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>id-779e4cd290f2e64e</t>
+          <t>id-b147fbd9d3081bfc</t>
         </is>
       </c>
     </row>
@@ -1249,14 +1245,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1266,22 +1262,22 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>11/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>OBRA "PAVIMENTACION URBANA CALLE TRATADO DEL PILAR B° 3 DE FEBRERO - MUNICIPALIDAD DE SANTA ELENA" (Según Pliegos de Bases y condi ciones)</t>
+          <t>“PROVISIÓN DE UNA (1) MINICARGADORA 0 KM, CON CUCHARÓN FRONTAL DE USO GENERAL, UN (1) MARTILLO HIDRÁULICO Y UN (1) COMPACTADOR/RODILLO VIBRATORIO LISO”</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026 HORA: 10: 00 HS</t>
+          <t>09/10/2026 HORA: 10:00 HS</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1291,7 +1287,7 @@
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>$ 728.000,00 PESOS SETECIENTOS VEINTIOCHO MIL</t>
+          <t>($ 270.000,00) PESOS DOSCIENTOS SETENTA MIL</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
@@ -1311,14 +1307,14 @@
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>id-1a2561509308b1b6</t>
+          <t>id-779e4cd290f2e64e</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>20/09/2026</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1328,12 +1324,12 @@
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
+          <t>MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1348,7 +1344,7 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>REFACCION EN ESCUELA N° 65 “ALMIRANTE BROWN” – CIUDAD DE CONCORDIA - DEPARTAMENTO CONCORDIA - PROVINCIA DE ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>OBRA "PAVIMENTACION URBANA CALLE TRATADO DEL PILAR B° 3 DE FEBRERO - MUNICIPALIDAD DE SANTA ELENA" (Según Pliegos de Bases y condi ciones)</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -1358,15 +1354,19 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 09:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
+          <t>13/10/2026 HORA: 10: 00 HS</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
-        </is>
-      </c>
-      <c r="K12" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>$ 728.000,00 PESOS SETECIENTOS VEINTIOCHO MIL</t>
+        </is>
+      </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1384,7 +1384,7 @@
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>id-fc30d5c0b0589a79</t>
+          <t>id-1a2561509308b1b6</t>
         </is>
       </c>
     </row>
@@ -1399,7 +1399,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
@@ -1416,12 +1416,12 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>13/2026</t>
+          <t>11/2026</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>REPARACIONES VARIAS EN C. P. E. F. Nº 3 “PROFESOR HUGO LA NASA” – CIUDAD DE CONCEPCION DEL URUGUAY - DEPARTAMENTO URUGUAY - PROVINCIA D E ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>REFACCION EN ESCUELA N° 65 “ALMIRANTE BROWN” – CIUDAD DE CONCORDIA - DEPARTAMENTO CONCORDIA - PROVINCIA DE ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 09:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -1457,7 +1457,7 @@
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>id-9d3847fb0e2b0929</t>
+          <t>id-fc30d5c0b0589a79</t>
         </is>
       </c>
     </row>
@@ -1472,7 +1472,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
@@ -1489,12 +1489,12 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>12/2026</t>
+          <t>13/2026</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>RECAMBIO DE CUBIERTA Y REPARACIONES VARIAS EN ESCUELA Nº 92 “CONGRESO DE TUCUMAN” – CONCEPCION DEL URUGUAY - DPTO. URUGUAY – PROVINCIA DE ENTRE RIOS de acuerdo a las c ondiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>REPARACIONES VARIAS EN C. P. E. F. Nº 3 “PROFESOR HUGO LA NASA” – CIUDAD DE CONCEPCION DEL URUGUAY - DEPARTAMENTO URUGUAY - PROVINCIA D E ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 10:30 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1530,14 +1530,14 @@
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>id-059239b424b9c936</t>
+          <t>id-9d3847fb0e2b0929</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>23/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1545,14 +1545,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>VICTORIA — MUNICIPALIDAD DE VICTORIA</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1562,27 +1562,27 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>008/2026</t>
+          <t>12/2026</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Proveer a la Municipalidad de Victoria, Entre Ríos, de Veinticinco Mil (25.000) litros de Diésel 500, para movilidad de vehículos y maquinarias viales , Ocho Mil (8.000) litros de Gasoil Tipo euro o similar y Ocho (8.000) litros de nafta súper para vehículos y áreas afectadas a la Secretaria de Planeamiento y Dirección de Ambiente y Desarrollo sostenible;</t>
+          <t>RECAMBIO DE CUBIERTA Y REPARACIONES VARIAS EN ESCUELA Nº 92 “CONGRESO DE TUCUMAN” – CONCEPCION DEL URUGUAY - DPTO. URUGUAY – PROVINCIA DE ENTRE RIOS de acuerdo a las c ondiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>14/10/2026</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>14 de octubre de 2026 a las 09:00 hs., en la Oficina de Compras de la Municipalidad de Victoria, Entr</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 10:30 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>06/10/2026</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr"/>
@@ -1603,14 +1603,14 @@
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>id-a9af9f59c8c487c8</t>
+          <t>id-059239b424b9c936</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1618,14 +1618,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>SALUD ENTRE RÍOS S.A.U</t>
+          <t>MUNICIPALIDAD DE COLON</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1636,17 +1636,17 @@
       <c r="F16" s="4" t="inlineStr"/>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Contratación de Servicio de Viandas para el Hospital de la Baxada</t>
+          <t>“ADQUISICIÓN DE MATERIALES ELÉCTRICOS PARA EJECUCIÓN DEL PROYECTO DE RECONVERSIÓN Y OPTIMIZACIÓN DEL ALUMBRADO PÚBLICO DE LA CIUDAD DE COLÓN”</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>14/10/2026</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Hospital de la Baxada, calle Gral. Al varado Nº 2.250 Paraná, Entre Ríos, el día 19/10/2026 a las 10:00 hs</t>
+          <t>14 de OCTUBRE de 2026</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -1656,7 +1656,7 @@
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>Sin Cargo</t>
         </is>
       </c>
       <c r="L16" s="6" t="inlineStr">
@@ -1676,14 +1676,14 @@
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>id-d35d5e849089d7ac</t>
+          <t>id-9e122d52de12ffef</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1691,14 +1691,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>PARANA — SALUD ENTRE RÍOS S.A.U</t>
+          <t>DIAMANTE — COMUNA ALDEA PROTESTANTE -- DIAMANTE -- ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1706,20 +1706,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr"/>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>03/2026</t>
+        </is>
+      </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Servicio de Recolección, Lavado, Desinfección, Secado, Planchado y Transporte de Ropa Hospitalaria</t>
+          <t>Conforme a lo autorizado por decreto Nº 290/26 llámese a licitación pública Nº 03/26 con el objeto de comprar 10 toneladas de emulsión catiónica súper estable (asfalto de imprimación), puesto en Aldea Protestante</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>21/10/2026</t>
+          <t>14/10/2026</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Hospital de la Baxada, calle Gral. Alvarado Nº 2.250 Paraná, Entre Ríos, el día 21/10/2026 a las 10:00 hs</t>
+          <t>miércoles 14 de octubre de 2026 – Hora nueve (09:00) Lugar de presentación de la oferta: Sede Comuna Aldea Protestan</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1727,11 +1731,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K17" s="4" t="inlineStr">
-        <is>
-          <t>Ninguno</t>
-        </is>
-      </c>
+      <c r="K17" s="4" t="inlineStr"/>
       <c r="L17" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1749,14 +1749,14 @@
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>id-6b955df9d3f6241a</t>
+          <t>id-c2f3a25cfb37fd38</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>26/09/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1764,14 +1764,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1781,22 +1781,22 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>11/26</t>
+          <t>017/2026</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “TERMINACION ESCUELA Nº 40 “JOSÉ ENRIQUE RODÓ”-SEPTIMO DISTRITO-DEPARTAMENTO GUALEGUAY.”</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de UNA (1) MOTONIVELADORA, nueva, sin uso, cero km, con una potencia entre 220/240 HP, con opción a implementos, que será utilizada para el área del corralón municipal</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>23/10/2026</t>
+          <t>14/10/2026</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 23 de Octubre de 2026 a las 10:00 hs</t>
+          <t>14 DE OCTUBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1806,7 +1806,7 @@
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>$ 100 (Cien)</t>
+          <t>$100.000,00. - (PESOS CIEN MIL CON 00/100) PRESUPUESTO OFICIAL ESTIMAD</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr">
@@ -1826,14 +1826,14 @@
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>id-86cc9c230734c462</t>
+          <t>id-4c3b33859e596759</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>26/09/2026</t>
+          <t>23/09/2026</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1841,14 +1841,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>VICTORIA — MUNICIPALIDAD DE VICTORIA</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1858,22 +1858,22 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>11/2026</t>
+          <t>008/2026</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Terminación Escuela N° 40 "José Enrique Rodó", Séptimo Distrito</t>
+          <t>Proveer a la Municipalidad de Victoria, Entre Ríos, de Veinticinco Mil (25.000) litros de Diésel 500, para movilidad de vehículos y maquinarias viales , Ocho Mil (8.000) litros de Gasoil Tipo euro o similar y Ocho (8.000) litros de nafta súper para vehículos y áreas afectadas a la Secretaria de Planeamiento y Dirección de Ambiente y Desarrollo sostenible;</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>23/10/2026</t>
+          <t>14/10/2026</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>viernes, 23 de octubre de 2026 - 10:00hs</t>
+          <t>14 de octubre de 2026 a las 09:00 hs., en la Oficina de Compras de la Municipalidad de Victoria, Entr</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1894,19 +1894,19 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>id-322a40f5e43af35d</t>
+          <t>id-a9af9f59c8c487c8</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1914,49 +1914,49 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C20" s="9" t="inlineStr">
         <is>
           <t>Materiales</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Municipalidad de Crespo</t>
+          <t>MINISTERIO DE SALUD — GOBIERNO DE ENTRE RIOS</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>5/2026</t>
+          <t>18/26</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 145 metros lineales de módulo canal premoldeado.</t>
+          <t>Adquirir Sesenta Mil (60.000) Kilogramos de Leche Entera en Polvo Instantánea, Fortificada con Hierro, Zinc y Ácido Ascórbico</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>16/10/2026</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>28/9/2026 – 10:00 horas</t>
+          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>28/09/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>$25.000,00</t>
+          <t>PESOS TRES MIL QUINIENTOS ($ 3.500,00)</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
@@ -1971,19 +1971,19 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Municipalidad de Crespo</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>id-1609ce58e128c413</t>
+          <t>id-04a917d50ccab2e3</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1993,12 +1993,12 @@
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>VILLAGUAY — MUNICIPALIDAD DE VILLAGUAY</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2006,24 +2006,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>10/2026</t>
-        </is>
-      </c>
+      <c r="F21" s="4" t="inlineStr"/>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Impermeabilización cubierta de techos, reparación de mamposterías y pintura Escuela N° 2 "Alvarez Condarco", Chajarí</t>
+          <t>Contratación, ejecución, liquidación, pago y recepción de la obra destinada a la elaboración del Proyecto Ejecutivo, provisión de materiales, mano de obra, equipos, ejecución, ensayos, habilitación y puesta en servicio de la instalación de gas natural para la Planta Municipal de Elaboración de Mezcla Asfáltica en Caliente, ubicada en el Lote N.º 4 de la Chacra N.º 263 del Parque Industrial de Villaguay, Provincia de Entre Ríos. La contratación comprenderá una solución i ntegral bajo modalidad “llave en mano”, incluyendo todos los trabajos, provisiones, trámites, representaciones técnicas, insp</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>16/10/2026</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 30 de septiembre de 2026 - 10:00hs</t>
+          <t>16 de octubre del año 2026 a las 10:00 Horas, la que se realizara en la Ofici na de suministros de la Municipalidad de V</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -2031,7 +2027,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K21" s="4" t="inlineStr"/>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>$ 50.000,00</t>
+        </is>
+      </c>
       <c r="L21" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2044,34 +2044,34 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-46c6d9f1f9210d1e</t>
+          <t>id-55f1e5ca423a9262</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>26/09/2026</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+          <t>20/09/2026</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
+          <t>SALUD ENTRE RÍOS S.A.U</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2079,20 +2079,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>001/26</t>
-        </is>
-      </c>
+      <c r="F22" s="4" t="inlineStr"/>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN de UN (1) FURGON UTILITARIO CHICO con 5 asientos 0 KM. con destino a Subsecretaria de Asistencia Directa y Emergencia</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr"/>
+          <t>Contratación de Servicio de Viandas para el Hospital de la Baxada</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>19/10/2026</t>
+        </is>
+      </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>DE LAS PROPUESTAS: 20 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
+          <t>Hospital de la Baxada, calle Gral. Al varado Nº 2.250 Paraná, Entre Ríos, el día 19/10/2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -2100,7 +2100,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K22" s="4" t="inlineStr"/>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
       <c r="L22" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2118,29 +2122,29 @@
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-ca205f0874380f69</t>
+          <t>id-d35d5e849089d7ac</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>26/09/2026</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C23" s="10" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+          <t>20/09/2026</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
+          <t>PARANA — SALUD ENTRE RÍOS S.A.U</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2148,20 +2152,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>07/2026</t>
-        </is>
-      </c>
+      <c r="F23" s="4" t="inlineStr"/>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Transporte de mil doscientos cincuenta metros cúbicos (1.250 m³) de broza grillada desde Cantera “Tayreta” (Ruta Nacional N° 14 km 135) hasta juris dicción de la comuna, de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr"/>
+          <t>Servicio de Recolección, Lavado, Desinfección, Secado, Planchado y Transporte de Ropa Hospitalaria</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>21/10/2026</t>
+        </is>
+      </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Viernes 09 de octubre del corriente año a las 10:00 hs en la Oficina de la Sede de la Comuna</t>
+          <t>Hospital de la Baxada, calle Gral. Alvarado Nº 2.250 Paraná, Entre Ríos, el día 21/10/2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2169,7 +2173,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K23" s="4" t="inlineStr"/>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
       <c r="L23" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2187,7 +2195,7 @@
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-24e9015ecceeff7f</t>
+          <t>id-6b955df9d3f6241a</t>
         </is>
       </c>
     </row>
@@ -2197,36 +2205,44 @@
           <t>26/09/2026</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Infraestructura</t>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>INSTITUTO CARBÓ S.R.L</t>
+          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Licitación</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>11/26</t>
+        </is>
+      </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>sin internación en materia de salud, pre- hospitalarias, atención médica, domiciliaria y traslados sanitarios de alta</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr"/>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “TERMINACION ESCUELA Nº 40 “JOSÉ ENRIQUE RODÓ”-SEPTIMO DISTRITO-DEPARTAMENTO GUALEGUAY.”</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>DE LAS OFERTAS: el día 23 de Octubre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -2234,7 +2250,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K24" s="4" t="inlineStr"/>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>$ 100 (Cien)</t>
+        </is>
+      </c>
       <c r="L24" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2252,29 +2272,29 @@
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-6aa57c7437a30ca3</t>
+          <t>id-86cc9c230734c462</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>23/09/2026</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Infraestructura</t>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE VIALE</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2284,18 +2304,22 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>08/26</t>
+          <t>11/2026</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>de asf alto 70-16 destinado a la producción de pavimento de la Planta Asfáltica, y que a continuación se detalla y</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr"/>
+          <t>Terminación Escuela N° 40 "José Enrique Rodó", Séptimo Distrito</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>viernes, 23 de octubre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2316,19 +2340,19 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-ef1ddb923c7e7fdb</t>
+          <t>id-322a40f5e43af35d</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>26/09/2026</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2336,14 +2360,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C26" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
+          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2353,18 +2377,18 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>001-2026</t>
+          <t>001/26</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
+          <t>ADQUISICIÓN de UN (1) FURGON UTILITARIO CHICO con 5 asientos 0 KM. con destino a Subsecretaria de Asistencia Directa y Emergencia</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
+          <t>DE LAS PROPUESTAS: 20 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2372,11 +2396,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K26" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K26" s="4" t="inlineStr"/>
       <c r="L26" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2394,14 +2414,14 @@
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-b7b0120caf49d551</t>
+          <t>id-ca205f0874380f69</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>17/09/2026</t>
+          <t>26/09/2026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2409,14 +2429,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE URDINARRAIN</t>
+          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2426,18 +2446,18 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>07/2026</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
+          <t>Transporte de mil doscientos cincuenta metros cúbicos (1.250 m³) de broza grillada desde Cantera “Tayreta” (Ruta Nacional N° 14 km 135) hasta jurisdicción de la comuna, de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Viernes 09 de octubre del corriente año a las 10:00 hs en la Oficina de la Sede de la Comuna</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2463,7 +2483,7 @@
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-7a200161bcc9b02b</t>
+          <t>id-24e9015ecceeff7f</t>
         </is>
       </c>
     </row>
@@ -2480,33 +2500,29 @@
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>INSTITUTO CARBÓ S.R.L</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>08/26</t>
-        </is>
-      </c>
+          <t>Licitación</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr"/>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Obra “Readecuación del sistema de climatización –ala sur- Edificio Tribunales Gualeguay”.</t>
+          <t>sin internación en materia de salud, pre- hospitalarias, atención médica, domiciliaria y traslados sanitarios de alta</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Ver el sitio</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2527,19 +2543,19 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-9ca2387eef6d6fc1</t>
+          <t>id-6aa57c7437a30ca3</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>24/09/2026</t>
+          <t>23/09/2026</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2549,33 +2565,33 @@
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>MUNICIPALIDAD DE VIALE</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Solicitud de Cotización</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>240/26</t>
+          <t>08/26</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Contratación del servicio de reparación prioritaria de seis (6) escalones de mármol de la escalera de acceso al entrepiso y primer piso del Edificio Tribunales de Gualeguaychú sito en calle Roque Sáenz Peña N°94.</t>
+          <t>de asf alto 70-16 destinado a la producción de pavimento de la Planta Asfáltica, y que a continuación se detalla y</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Ver el sitio</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2596,12 +2612,12 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-ba80195eeddbd2bd</t>
+          <t>id-ef1ddb923c7e7fdb</t>
         </is>
       </c>
     </row>
@@ -2616,31 +2632,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>001-2026</t>
+        </is>
+      </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
+          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2648,7 +2668,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K30" s="4" t="inlineStr"/>
+      <c r="K30" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L30" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2661,12 +2685,12 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-654eebef400f89cd</t>
+          <t>id-b7b0120caf49d551</t>
         </is>
       </c>
     </row>
@@ -2681,35 +2705,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C31" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>MUNICIPALIDAD DE URDINARRAIN</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Concurso</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>01/26</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2730,12 +2754,12 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-9a16884dd5a64a49</t>
+          <t>id-7a200161bcc9b02b</t>
         </is>
       </c>
     </row>
@@ -2750,35 +2774,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>2026-1227</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 06/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2786,7 +2810,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K32" s="4" t="inlineStr"/>
+      <c r="K32" s="4" t="inlineStr">
+        <is>
+          <t>$ 120.976,01</t>
+        </is>
+      </c>
       <c r="L32" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2799,19 +2827,19 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-0691eb485d7548eb</t>
+          <t>id-07ddb93a12c5a870</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2819,7 +2847,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C33" s="7" t="inlineStr">
+      <c r="C33" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2836,18 +2864,18 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>03/26</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+          <t>Concurso de Precio N° 02/2025</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>Publicada 19/06/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2873,14 +2901,14 @@
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-7c1bf02160a66f67</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2888,35 +2916,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t>02/2026</t>
-        </is>
-      </c>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr"/>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -2937,19 +2961,19 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-654eebef400f89cd</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2957,35 +2981,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C35" s="7" t="inlineStr">
+      <c r="C35" s="8" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Concurso</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>01/26</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3006,19 +3030,19 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-9a16884dd5a64a49</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>17/09/2026</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3026,35 +3050,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C36" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C36" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>05/2025</t>
+          <t>2026-1227</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3075,19 +3099,19 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-0691eb485d7548eb</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>20/09/2026</t>
+          <t>26/09/2026</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3097,12 +3121,12 @@
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>Infraestructura</t>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3112,18 +3136,18 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>06/2025</t>
+          <t>08/26</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>Obra “Readecuación del sistema de climatización –ala sur- Edificio Tribunales Gualeguay”.</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Ver el sitio</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3144,358 +3168,17 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Poder Judicial de Entre Ríos</t>
         </is>
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>20/09/2026</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C38" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>IAPV (Vivienda)</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F38" s="4" t="inlineStr"/>
-      <c r="G38" s="5" t="inlineStr">
-        <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
-        </is>
-      </c>
-      <c r="H38" s="4" t="inlineStr"/>
-      <c r="I38" s="4" t="inlineStr">
-        <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
-        </is>
-      </c>
-      <c r="J38" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K38" s="4" t="inlineStr"/>
-      <c r="L38" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M38" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N38" t="inlineStr">
-        <is>
-          <t>IAPV — Viviendas</t>
-        </is>
-      </c>
-      <c r="O38" s="4" t="inlineStr">
-        <is>
-          <t>id-ebeeb6a87e688d85</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>20/09/2026</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C39" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>IAPV (Vivienda)</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F39" s="4" t="inlineStr">
-        <is>
-          <t>04/2025</t>
-        </is>
-      </c>
-      <c r="G39" s="5" t="inlineStr">
-        <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
-        </is>
-      </c>
-      <c r="H39" s="4" t="inlineStr"/>
-      <c r="I39" s="4" t="inlineStr">
-        <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
-        </is>
-      </c>
-      <c r="J39" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K39" s="4" t="inlineStr"/>
-      <c r="L39" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M39" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>IAPV — Viviendas</t>
-        </is>
-      </c>
-      <c r="O39" s="4" t="inlineStr">
-        <is>
-          <t>id-34c85bcdb9b1123f</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>20/09/2026</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C40" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>IAPV (Vivienda)</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F40" s="4" t="inlineStr">
-        <is>
-          <t>03/2025</t>
-        </is>
-      </c>
-      <c r="G40" s="5" t="inlineStr">
-        <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
-        </is>
-      </c>
-      <c r="H40" s="4" t="inlineStr"/>
-      <c r="I40" s="4" t="inlineStr">
-        <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
-        </is>
-      </c>
-      <c r="J40" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K40" s="4" t="inlineStr"/>
-      <c r="L40" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M40" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N40" t="inlineStr">
-        <is>
-          <t>IAPV — Viviendas</t>
-        </is>
-      </c>
-      <c r="O40" s="4" t="inlineStr">
-        <is>
-          <t>id-75bfffae63b7eedc</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C41" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>IAPV (Vivienda)</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F41" s="4" t="inlineStr">
-        <is>
-          <t>02/2025</t>
-        </is>
-      </c>
-      <c r="G41" s="5" t="inlineStr">
-        <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
-        </is>
-      </c>
-      <c r="H41" s="4" t="inlineStr"/>
-      <c r="I41" s="4" t="inlineStr">
-        <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
-        </is>
-      </c>
-      <c r="J41" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K41" s="4" t="inlineStr"/>
-      <c r="L41" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M41" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>IAPV — Viviendas</t>
-        </is>
-      </c>
-      <c r="O41" s="4" t="inlineStr">
-        <is>
-          <t>id-07ddb93a12c5a870</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>17/09/2026</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C42" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>IAPV (Vivienda)</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="inlineStr">
-        <is>
-          <t>02/2025</t>
-        </is>
-      </c>
-      <c r="G42" s="5" t="inlineStr">
-        <is>
-          <t>Concurso de Precio N° 02/2025</t>
-        </is>
-      </c>
-      <c r="H42" s="4" t="inlineStr"/>
-      <c r="I42" s="4" t="inlineStr">
-        <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
-        </is>
-      </c>
-      <c r="J42" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K42" s="4" t="inlineStr"/>
-      <c r="L42" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M42" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>IAPV — Viviendas</t>
-        </is>
-      </c>
-      <c r="O42" s="4" t="inlineStr">
-        <is>
-          <t>id-7c1bf02160a66f67</t>
+          <t>id-9ca2387eef6d6fc1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O42"/>
+  <autoFilter ref="A1:O37"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -3569,16 +3252,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId70"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L38" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId82"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 02/10/2026 08:06
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$36</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -62,7 +62,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -72,7 +72,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O35"/>
+  <dimension ref="A1:O36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -572,7 +572,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -587,7 +587,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA — INSTITUTO AUTÁRQUICO DE PLANEAMIENTO YY VI</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -597,22 +597,22 @@
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>05/2026</t>
+          <t>016/2026</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>COMPLEJO HABITACIONAL SAN AGUSTIN (P.P.) PARANÁ 24 VIVIENDAS, 7 LOCALES COMERCIALES Y 27 ESPACIOS DE ESTACIONAMIENTOS DEPARTAMENTO: PARANÁ Para ná , mi ércoles 7 de octubre de 20</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de mano de obra, materiales y equipamiento para ejecución de restitución de galibo y repavimentación en Avenida Belgrano y Avenida 1° de Mayo de esta ciudad de chajari</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>01/12/2026</t>
+          <t>02/10/2026</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>DÍA: 01 /12 /2026 HORA: 10:30 hs</t>
+          <t>02 DE OCTUBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
@@ -622,7 +622,7 @@
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>$ 299.794,33</t>
+          <t>$ 100.000, 00. - (PESOS CIEN MIL CON 00/100)</t>
         </is>
       </c>
       <c r="L2" s="6" t="inlineStr">
@@ -642,54 +642,54 @@
       </c>
       <c r="O2" s="4" t="inlineStr">
         <is>
-          <t>id-be1efacbe31d4a09</t>
+          <t>id-53f1430f94acb0b0</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>07/2026</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”, destinada a la obra denominada “Nueva Pileta en el Polideportivo El Aguará”,</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
           <t>06/10/2026</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>IAPV (Vivienda)</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>05/2026</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>COMPLEJO HABITACIONAL SAN AGUSTÍN (P</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>01/12/2026</t>
-        </is>
-      </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>01/12/2026 (leído del aviso)</t>
+          <t>06/10/2026 HORA: 11:00 HS</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -699,7 +699,7 @@
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>$ 299.794,33</t>
+          <t>SIN COSTO</t>
         </is>
       </c>
       <c r="L3" s="6" t="inlineStr">
@@ -714,19 +714,19 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
-          <t>id-ccb22bcad9356438</t>
+          <t>id-65d18d99bf0b2c6c</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>14/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -741,7 +741,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE SANTA ANA</t>
+          <t>PARANA — MINISTERIO DE SALUD</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -751,34 +751,30 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>06/2026</t>
+          <t>17/26</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Provisión de mano de obra, materiales, maquinarias y herramientas para pavimento asfáltico en Santa Ana</t>
+          <t>Adquirir Una (01) Mesa de Anestesia. Destino: Hospital “San José” de Diamante, dependiente del Ministerio de Salud de la Provincia de Entre Ríos</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>06/11/2026</t>
+          <t>06/10/2026</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>Viernes 06 de Noviembre de 2026, 10 hs</t>
+          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>$ 150.000, 00.- (Pesos Ciento Cincuenta Mil)</t>
-        </is>
-      </c>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr"/>
       <c r="L4" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -796,54 +792,54 @@
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
-          <t>id-270211eda8d9288f</t>
+          <t>id-3312d89e1a3e2e53</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>31/2026</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>“Pavimento Rígido – 03 (tres) Cuadras Barrio San Felipe”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
           <t>07/10/2026</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>COLON — MUNICIPALIDAD DE VILLA ELISA (E.R.)</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>004/26</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>ADQUISICIÓN DE UN (1) VEHÍCULO PARA TRANSPORTE DE PASAJEROS DE (5) CINCO PLAZAS 0 KM - MODELO/AÑO 2026, PARA LA MUNICIPALIDAD DE LA CIUDAD DE VILLA ELISA, ENTRE RÍOS</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>12/11/2026</t>
-        </is>
-      </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>12 de NOVIEMBRE de 2026 a la hora 10:00 en la Oficina de Compras de la Municipalidad de Villa Elisa, Entre Ríos</t>
+          <t>07 de octubre de 2026 Hora: 10:00</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -851,11 +847,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">$ 20.000,00 (Pesos Veinte mil con 00/100) el que se puede adquirir en </t>
-        </is>
-      </c>
+      <c r="K5" s="4" t="inlineStr"/>
       <c r="L5" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -873,7 +865,7 @@
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>id-bb3703ff360c8c43</t>
+          <t>id-76d9566cb30a6df5</t>
         </is>
       </c>
     </row>
@@ -888,14 +880,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -905,22 +897,22 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>87/2026</t>
+          <t>32/2026</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Contratar la ejecución de la obra denominada “Construcción de Red Cloacal Subsidiaria del Colector Noroeste Barrio Ciudad Paisaje”</t>
+          <t>"Adquisición de 835 m3 de Hormigón Calidad H25 para 08 cuadras de Pavimento", en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>martes, 13 de octubre de 2026 a las 10:00</t>
+          <t>08 de octubre de 2026 Hora: 10:00</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -928,11 +920,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t>$ 10.000 (pesos diez mil)</t>
-        </is>
-      </c>
+      <c r="K6" s="4" t="inlineStr"/>
       <c r="L6" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -945,12 +933,12 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Boletín Oficial Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>id-ceeb594e8bcc4ff7</t>
+          <t>id-0ace7de8f16d3baf</t>
         </is>
       </c>
     </row>
@@ -972,7 +960,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>COLON — MUNICIPALIDAD DE COLON</t>
+          <t>MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -980,20 +968,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr"/>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>33/2026</t>
+        </is>
+      </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN DE MATERIALES ELÉCTRICOS PARA EJECUCIÓN DEL PROYECTO DE RECONVERSIÓN Y OPTIMIZACIÓN DEL ALUMBRADO PÚBLICO DE LA CIUDAD DE COLÓN”</t>
+          <t>“Pavimento Rígido – 04 (cuatro) Cuadras Barrio San Roque y 01 (una) Cuadra Barrio Vicente Obrego”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>14/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>14 de OCTUBRE de 2026</t>
+          <t>08 de octubre de 2026 Hora: 11:00</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -1001,11 +993,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr">
-        <is>
-          <t>Sin Cargo</t>
-        </is>
-      </c>
+      <c r="K7" s="4" t="inlineStr"/>
       <c r="L7" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1023,7 +1011,7 @@
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>id-9e122d52de12ffef</t>
+          <t>id-fe71ac2aaf71b8d8</t>
         </is>
       </c>
     </row>
@@ -1038,14 +1026,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>DIAMANTE — COMUNA ALDEA PROTESTANTE -- DIAMANTE -- ENTRE RÍOS</t>
+          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1055,22 +1043,22 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>03/2026</t>
+          <t>34/2026</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Conforme a lo autorizado por decreto Nº 290/26 llámese a licitación pública Nº 03/26 con el objeto de comprar 10 toneladas de emulsión catiónica súper estable (asfalto de imprimación), puesto en Aldea Protestante</t>
+          <t>“Concesión de la Explotación Comercial de un (01) Camión de Comidas Rápidas (para cubrir el total de cuatro puestos) en la Zona Joven – Parque La Salamanca de la Municipalidad de Concepción del Uruguay – Entre Ríos”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>14/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>miércoles 14 de octubre de 2026 – Hora nueve (09:00) Lugar de presentación de la oferta: Sede Comuna Aldea Protestan</t>
+          <t>09 de octubre de 2026 Hora: 10:00</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -1096,7 +1084,7 @@
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>id-c2f3a25cfb37fd38</t>
+          <t>id-b147fbd9d3081bfc</t>
         </is>
       </c>
     </row>
@@ -1111,14 +1099,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>Vehículos</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1128,22 +1116,22 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>017/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de UNA (1) MOTONIVELADORA, nueva, sin uso, cero km, con una potencia entre 220/240 HP, con opción a implementos, que será utilizada para el área del corralón municipal</t>
+          <t>“PROVISIÓN DE UNA (1) MINICARGADORA 0 KM, CON CUCHARÓN FRONTAL DE USO GENERAL, UN (1) MARTILLO HIDRÁULICO Y UN (1) COMPACTADOR/RODILLO VIBRATORIO LISO”</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>14/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>14 DE OCTUBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>09/10/2026 HORA: 10:00 HS</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1153,7 +1141,7 @@
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>$100.000,00. - (PESOS CIEN MIL CON 00/100) PRESUPUESTO OFICIAL ESTIMAD</t>
+          <t>($ 270.000,00) PESOS DOSCIENTOS SETENTA MIL</t>
         </is>
       </c>
       <c r="L9" s="6" t="inlineStr">
@@ -1173,7 +1161,7 @@
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>id-4c3b33859e596759</t>
+          <t>id-779e4cd290f2e64e</t>
         </is>
       </c>
     </row>
@@ -1188,14 +1176,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>VICTORIA — MUNICIPALIDAD DE VICTORIA</t>
+          <t>MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1205,22 +1193,22 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>008/2026</t>
+          <t>11/2026</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Proveer a la Municipalidad de Victoria, Entre Ríos, de Veinticinco Mil (25.000) litros de Diésel 500, para movilidad de vehículos y maquinarias viales , Ocho Mil (8.000) litros de Gasoil Tipo euro o similar y Ocho (8.000) litros de nafta súper para vehículos y áreas afectadas a la Secretaria de Planeamiento y Dirección de Ambiente y Desarrollo sostenible;</t>
+          <t>OBRA "PAVIMENTACION URBANA CALLE TRATADO DEL PILAR B° 3 DE FEBRERO - MUNICIPALIDAD DE SANTA ELENA" (Según Pliegos de Bases y condi ciones)</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>14/10/2026</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>14 de octubre de 2026 a las 09:00 hs., en la Oficina de Compras de la Municipalidad de Victoria, Entr</t>
+          <t>13/10/2026 HORA: 10: 00 HS</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1228,7 +1216,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr"/>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>$ 728.000,00 PESOS SETECIENTOS VEINTIOCHO MIL</t>
+        </is>
+      </c>
       <c r="L10" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1246,66 +1238,62 @@
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>id-a9af9f59c8c487c8</t>
+          <t>id-1a2561509308b1b6</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>11/2026</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>REFACCION EN ESCUELA N° 65 “ALMIRANTE BROWN” – CIUDAD DE CONCORDIA - DEPARTAMENTO CONCORDIA - PROVINCIA DE ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>13/10/2026</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 09:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
           <t>06/10/2026</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE ALDEA SAN ANTONIO</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>002/2026</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>ADQUISICIÓN DE UNA MÁQUINA MOTONIVELADORA PARA INCORPORAR AL PARQUE AUTOMOTOR DE LA MUNICIPALIDAD DE ALDEA SAN ANTONIO</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>15/10/2026</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>15 de octubre de 2026, a las 08:00 horas, en el Edificio Municipal</t>
-        </is>
-      </c>
-      <c r="J11" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K11" s="4" t="inlineStr">
-        <is>
-          <t>PESOS CIEN MIL con 00/100 ($ 100.000,00. -)</t>
-        </is>
-      </c>
+      <c r="K11" s="4" t="inlineStr"/>
       <c r="L11" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1323,7 +1311,7 @@
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>id-95a507b67b7b1450</t>
+          <t>id-fc30d5c0b0589a79</t>
         </is>
       </c>
     </row>
@@ -1338,14 +1326,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>MINISTERIO DE SALUD — GOBIERNO DE ENTRE RIOS</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1355,34 +1343,30 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>18/26</t>
+          <t>13/2026</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Adquirir Sesenta Mil (60.000) Kilogramos de Leche Entera en Polvo Instantánea, Fortificada con Hierro, Zinc y Ácido Ascórbico</t>
+          <t>REPARACIONES VARIAS EN C. P. E. F. Nº 3 “PROFESOR HUGO LA NASA” – CIUDAD DE CONCEPCION DEL URUGUAY - DEPARTAMENTO URUGUAY - PROVINCIA D E ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>16/10/2026</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K12" s="4" t="inlineStr">
-        <is>
-          <t>PESOS TRES MIL QUINIENTOS ($ 3.500,00)</t>
-        </is>
-      </c>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr"/>
       <c r="L12" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1400,7 +1384,7 @@
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>id-04a917d50ccab2e3</t>
+          <t>id-9d3847fb0e2b0929</t>
         </is>
       </c>
     </row>
@@ -1415,14 +1399,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>VILLAGUAY — MUNICIPALIDAD DE VILLAGUAY</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1430,32 +1414,32 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr"/>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>12/2026</t>
+        </is>
+      </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Contratación, ejecución, liquidación, pago y recepción de la obra destinada a la elaboración del Proyecto Ejecutivo, provisión de materiales, mano de obra, equipos, ejecución, ensayos, habilitación y puesta en servicio de la instalación de gas natural para la Planta Municipal de Elaboración de Mezcla Asfáltica en Caliente, ubicada en el Lote N.º 4 de la Chacra N.º 263 del Parque Industrial de Villaguay, Provincia de Entre Ríos. La contratación comprender á una solución integral bajo modalidad “llave en mano”, incluyendo todos los trabajos, provisiones, trámites, representaciones técnicas, insp</t>
+          <t>RECAMBIO DE CUBIERTA Y REPARACIONES VARIAS EN ESCUELA Nº 92 “CONGRESO DE TUCUMAN” – CONCEPCION DEL URUGUAY - DPTO. URUGUAY – PROVINCIA DE ENTRE RIOS de acuerdo a las c ondiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>16/10/2026</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>16 de octubre del año 2026 a las 10:00 Horas, la que se reali zara en la Oficina de suministros de la Municipalidad de V</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 10:30 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K13" s="4" t="inlineStr">
-        <is>
-          <t>$ 50.000,00</t>
-        </is>
-      </c>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="inlineStr"/>
       <c r="L13" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1473,14 +1457,14 @@
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>id-55f1e5ca423a9262</t>
+          <t>id-059239b424b9c936</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1495,7 +1479,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1505,22 +1489,22 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>87/2026</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN CONCEPCIÓN DEL URUGUAY 63 VIV</t>
+          <t>Contratar la ejecución de la obra denominada “Construcción de Red Cloacal Subsidiaria del Colector Noroeste Barrio Ciudad Paisaje”</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>17/11/2026</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>17/11/2026 (leído del aviso)</t>
+          <t>martes, 13 de octubre de 2026 a las 10:00</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1530,7 +1514,7 @@
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
-          <t>$138.748,07</t>
+          <t>$ 10.000 (pesos diez mil)</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr">
@@ -1545,12 +1529,12 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>id-1a3c1f8e036ac91e</t>
+          <t>id-ceeb594e8bcc4ff7</t>
         </is>
       </c>
     </row>
@@ -1572,7 +1556,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>SALUD ENTRE RÍOS S.A.U</t>
+          <t>MUNICIPALIDAD DE COLON</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1583,17 +1567,17 @@
       <c r="F15" s="4" t="inlineStr"/>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Contratación de Servicio de Viandas para el Hospital de la Baxada</t>
+          <t>“ADQUISICIÓN DE MATERIALES ELÉCTRICOS PARA EJECUCIÓN DEL PROYECTO DE RECONVERSIÓN Y OPTIMIZACIÓN DEL ALUMBRADO PÚBLICO DE LA CIUDAD DE COLÓN”</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>14/10/2026</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>Hospital de la Baxada, calle Gral. Al varado Nº 2.250 Paraná, Entre Ríos, el día 19/10/2026 a las 10:00 hs</t>
+          <t>14 de OCTUBRE de 2026</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1603,7 +1587,7 @@
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>Sin Cargo</t>
         </is>
       </c>
       <c r="L15" s="6" t="inlineStr">
@@ -1623,14 +1607,14 @@
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>id-d35d5e849089d7ac</t>
+          <t>id-9e122d52de12ffef</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1638,14 +1622,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>VILLAGUAY — MUNICIPALIDAD DE VILLAGUAY</t>
+          <t>DIAMANTE — COMUNA ALDEA PROTESTANTE -- DIAMANTE -- ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1653,20 +1637,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr"/>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>03/2026</t>
+        </is>
+      </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Provisión de una (1) camioneta usada destinada al Parque Automotor Municipal</t>
+          <t>Conforme a lo autorizado por decreto Nº 290/26 llámese a licitación pública Nº 03/26 con el objeto de comprar 10 toneladas de emulsión catiónica súper estable (asfalto de imprimación), puesto en Aldea Protestante</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>21/10/2026</t>
+          <t>14/10/2026</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>21 de octubre del año 2026 a las 10:00 Horas, la que se realizara en la Oficina de suministros de la Municipalidad de Vi</t>
+          <t>miércoles 14 de octubre de 2026 – Hora nueve (09:00) Lugar de presentación de la oferta: Sede Comuna Aldea Protestan</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -1674,11 +1662,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K16" s="4" t="inlineStr">
-        <is>
-          <t>$10.000,00</t>
-        </is>
-      </c>
+      <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1696,7 +1680,7 @@
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>id-2d3dded56e6c6f6a</t>
+          <t>id-c2f3a25cfb37fd38</t>
         </is>
       </c>
     </row>
@@ -1711,14 +1695,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>PARANA — SALUD ENTRE RÍOS S.A.U</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1726,20 +1710,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr"/>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>017/2026</t>
+        </is>
+      </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Servicio de Recolección, Lavado, Desinfección, Secado, Planchado y Transporte de Ropa Hospitalaria</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de UNA (1) MOTONIVELADORA, nueva, sin uso, cero km, con una potencia entre 220/240 HP, con opción a implementos, que será utilizada para el área del corralón municipal</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>21/10/2026</t>
+          <t>14/10/2026</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Hospital de la Baxada, calle Gral. Alvarado Nº 2.250 Paraná, Entre Ríos, el día 21/10/2026 a las 10:00 hs</t>
+          <t>14 DE OCTUBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1749,7 +1737,7 @@
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>$100.000,00. - (PESOS CIEN MIL CON 00/100) PRESUPUESTO OFICIAL ESTIMAD</t>
         </is>
       </c>
       <c r="L17" s="6" t="inlineStr">
@@ -1769,54 +1757,54 @@
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>id-6b955df9d3f6241a</t>
+          <t>id-4c3b33859e596759</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>VICTORIA — MUNICIPALIDAD DE VICTORIA</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>008/2026</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>Proveer a la Municipalidad de Victoria, Entre Ríos, de Veinticinco Mil (25.000) litros de Diésel 500, para movilidad de vehículos y maquinarias viales , Ocho Mil (8.000) litros de Gasoil Tipo euro o similar y Ocho (8.000) litros de nafta súper para vehículos y áreas afectadas a la Secretaria de Planeamiento y Dirección de Ambiente y Desarrollo sostenible;</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
           <t>14/10/2026</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>GUALEGUAYCHU — MUNICIPALIDAD DE GUALEGUAYCHÚ</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>23/2026</t>
-        </is>
-      </c>
-      <c r="G18" s="5" t="inlineStr">
-        <is>
-          <t>ADQUISICIÓN de TRESCIENTOS (300) METROS CÚBICOS de HORMIGÓN ELABORADO, tipo H- 21, puesto en obra, destinado a los trabajos de bacheo en diferentes sectores de esta ciudad, debiendo ajustarse a los Pliegos de Condiciones Particulares</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>23/10/2026</t>
-        </is>
-      </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>23 de octubre del año 2026 a las 11: 00 horas</t>
+          <t>14 de octubre de 2026 a las 09:00 hs., en la Oficina de Compras de la Municipalidad de Victoria, Entr</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1842,7 +1830,7 @@
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>id-0297d8a28266a5af</t>
+          <t>id-a9af9f59c8c487c8</t>
         </is>
       </c>
     </row>
@@ -1857,14 +1845,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>MINISTERIO DE SALUD — GOBIERNO DE ENTRE RIOS</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1874,22 +1862,22 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>11/26</t>
+          <t>18/26</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “TERMINACION ESCUELA Nº 40 “JOSÉ ENRIQUE RODÓ”-SEPTIMO DISTRITO-DEPARTAMENTO GUALEGUAY.”</t>
+          <t>Adquirir Sesenta Mil (60.000) Kilogramos de Leche Entera en Polvo Instantánea, Fortificada con Hierro, Zinc y Ácido Ascórbico</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>23/10/2026</t>
+          <t>16/10/2026</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 23 de Octubre de 2026 a las 10:00 hs</t>
+          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1899,7 +1887,7 @@
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>$ 100 (Cien)</t>
+          <t>PESOS TRES MIL QUINIENTOS ($ 3.500,00)</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr">
@@ -1919,7 +1907,7 @@
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>id-86cc9c230734c462</t>
+          <t>id-04a917d50ccab2e3</t>
         </is>
       </c>
     </row>
@@ -1934,14 +1922,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>VILLAGUAY — MUNICIPALIDAD DE VILLAGUAY</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1949,24 +1937,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>11/2026</t>
-        </is>
-      </c>
+      <c r="F20" s="4" t="inlineStr"/>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Terminación Escuela N° 40 "José Enrique Rodó", Séptimo Distrito</t>
+          <t>Contratación, ejecución, liquidación, pago y recepción de la obra destinada a la elaboración del Proyecto Ejecutivo, provisión de materiales, mano de obra, equipos, ejecución, ensayos, habilitación y puesta en servicio de la instalación de gas natural para la Planta Municipal de Elaboración de Mezcla Asfáltica en Caliente, ubicada en el Lote N.º 4 de la Chacra N.º 263 del Parque Industrial de Villaguay, Provincia de Entre Ríos. La contratación comprender á una solución integral bajo modalidad “llave en mano”, incluyendo todos los trabajos, provisiones, trámites, representaciones técnicas, insp</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>23/10/2026</t>
+          <t>16/10/2026</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>viernes, 23 de octubre de 2026 - 10:00hs</t>
+          <t>16 de octubre del año 2026 a las 10:00 Horas, la que se reali zara en la Oficina de suministros de la Municipalidad de V</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1974,7 +1958,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K20" s="4" t="inlineStr"/>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t>$ 50.000,00</t>
+        </is>
+      </c>
       <c r="L20" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1987,19 +1975,19 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>id-322a40f5e43af35d</t>
+          <t>id-55f1e5ca423a9262</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>02/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -2007,14 +1995,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>COMUNA DE EL PALENQUE</t>
+          <t>SALUD ENTRE RÍOS S.A.U</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2022,24 +2010,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>06/26</t>
-        </is>
-      </c>
+      <c r="F21" s="4" t="inlineStr"/>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de UNA (1) PALA CARGADORA 0 KM destinada a trabajos en la Comuna</t>
+          <t>Contratación de Servicio de Viandas para el Hospital de la Baxada</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>26/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>26/10/2026, 12:30 horas, Lugar: Sede Administrativa de la Comuna de El Palenque, sito en calle San Martín sin número, El</t>
+          <t>Hospital de la Baxada, calle Gral. Al varado Nº 2.250 Paraná, Entre Ríos, el día 19/10/2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -2049,7 +2033,7 @@
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>pesos cero ($0,00)</t>
+          <t>Ninguno</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr">
@@ -2069,14 +2053,14 @@
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-4b7dfe1bdd0c2ac6</t>
+          <t>id-d35d5e849089d7ac</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -2084,14 +2068,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>COMUNA DE EL PALENQUE</t>
+          <t>PARANA — SALUD ENTRE RÍOS S.A.U</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2099,24 +2083,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>07/26</t>
-        </is>
-      </c>
+      <c r="F22" s="4" t="inlineStr"/>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de UN (1) TRACTOR AGRÍCOLA 0 KM DE HASTA 90 HP, CABINADO 4 x4, CON PALA FRONTAL destinado a trabajos en la Comuna</t>
+          <t>Servicio de Recolección, Lavado, Desinfección, Secado, Planchado y Transporte de Ropa Hospitalaria</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>28/10/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>28/10/2026, 12:40 horas, Lugar: Sede Administrativa de la Comuna de El Palenque, sito en calle San Martín sin número, El</t>
+          <t>Hospital de la Baxada, calle Gral. Alvarado Nº 2.250 Paraná, Entre Ríos, el día 21/10/2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -2126,7 +2106,7 @@
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
-          <t>pesos cero ($ 0,00)</t>
+          <t>Ninguno</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr">
@@ -2146,14 +2126,14 @@
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-54e2b94544e5c76f</t>
+          <t>id-6b955df9d3f6241a</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -2163,12 +2143,12 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Vehículos</t>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>VILLAGUAY — COMUNA DE MOJONES SUD YY PARAJE LOS ALGARROBOS</t>
+          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2176,20 +2156,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr"/>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>11/26</t>
+        </is>
+      </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN DE MOTONIVELADORA USADA</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “TERMINACION ESCUELA Nº 40 “JOSÉ ENRIQUE RODÓ”-SEPTIMO DISTRITO-DEPARTAMENTO GUALEGUAY.”</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>29/10/2026</t>
+          <t>23/10/2026</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>29/10/2026 a las 16:30 hs</t>
+          <t>DE LAS OFERTAS: el día 23 de Octubre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2199,7 +2183,7 @@
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t>$ 10.000 (PESOS DIEZ MIL)</t>
+          <t>$ 100 (Cien)</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr">
@@ -2219,29 +2203,29 @@
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-2aa97e0762afa9ea</t>
+          <t>id-86cc9c230734c462</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Vehículos</t>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2251,18 +2235,22 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>002/26</t>
+          <t>11/2026</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN de UN (1) TRACTOR 4 x4 C/CABINA DE 90 А 100 НР - 0 Km. con destino a Secretaria de Obras y Servicios Publicos</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr"/>
+          <t>Terminación Escuela N° 40 "José Enrique Rodó", Séptimo Distrito</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>DE LAS PROPUESTAS: 28 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
+          <t>viernes, 23 de octubre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -2283,12 +2271,12 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-da43a5f725393cbf</t>
+          <t>id-322a40f5e43af35d</t>
         </is>
       </c>
     </row>
@@ -2325,7 +2313,7 @@
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>Transporte de mil doscientos cincuenta metros cúbicos (1.250 m³) de broza grillada desde Cantera “Tayreta” (Ruta Nacional N° 14 km 135) hasta jurisdicción de la comuna, de acuerdo a los Pliegos de Bases, Condiciones Part iculares y demás documentación</t>
+          <t>Transporte de mil doscientos cincuenta metros cúbicos (1.250 m³) de broza grillada desde Cantera “Tayreta” (Ruta Nacional N° 14 km 135) hasta jurisdicción de la comuna, de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr"/>
@@ -2364,7 +2352,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>02/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2372,14 +2360,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>DIAMANTE — MUNICIPALIDAD DE DIAMANTE -- ENTRE RÍOS</t>
+          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2387,16 +2375,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr"/>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>001/26</t>
+        </is>
+      </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Solicitar Contratación de una empresa para la Obra de “22 (veintidós) cuadras de pavimento urbano” – Grupo 1- según Expte. Letra “D” Nº 2196</t>
+          <t>ADQUISICIÓN de UN (1) FURGON UTILITARIO CHICO con 5 asientos 0 KM. con destino a Subsecretaria de Asistencia Directa y Emergencia</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>viernes 23 de octubre de 2.026, a la hora diez (10.00)</t>
+          <t>DE LAS PROPUESTAS: 20 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2422,14 +2414,14 @@
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-4f207bef5c709ad6</t>
+          <t>id-ca205f0874380f69</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2444,7 +2436,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>CONCORDIA — APEX S.A.S</t>
+          <t>INSTITUTO CARBÓ S.R.L</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2455,7 +2447,7 @@
       <c r="F27" s="4" t="inlineStr"/>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>instalaciones eléctricas, sanitarias, hidráulicas, mecánicas o de cualquier otra naturaleza relacionada con el sector</t>
+          <t>sin internación en materia de salud, pre- hospitalarias, atención médica, domiciliaria y traslados sanitarios de alta</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
@@ -2487,14 +2479,14 @@
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-a20c6b2b6fcf36a2</t>
+          <t>id-6aa57c7437a30ca3</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2502,25 +2494,29 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Boletín Oficial</t>
+          <t>MUNICIPALIDAD DE VIALE</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Remate</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>08/26</t>
+        </is>
+      </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>los vehículos se encuentran en exhibición por lo cuál la información registral, de rentas y de infracciones puede ser</t>
+          <t>de asf alto 70-16 destinado a la producción de pavimento de la Planta Asfáltica, y que a continuación se detalla y</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
@@ -2552,7 +2548,7 @@
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-fb8d7dc09e202fea</t>
+          <t>id-ef1ddb923c7e7fdb</t>
         </is>
       </c>
     </row>
@@ -2569,12 +2565,12 @@
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Vehículos</t>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2584,18 +2580,18 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>001/26</t>
+          <t>001-2026</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN de UN (1) FURGON UTILITARIO CHICO con 5 asientos 0 KM. con destino a Subsecretaria de Asistencia Directa y Emergencia</t>
+          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>DE LAS PROPUESTAS: 20 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
+          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2603,7 +2599,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K29" s="4" t="inlineStr"/>
+      <c r="K29" s="4" t="inlineStr">
+        <is>
+          <t>SIN COSTO</t>
+        </is>
+      </c>
       <c r="L29" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2621,7 +2621,7 @@
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-ca205f0874380f69</t>
+          <t>id-b7b0120caf49d551</t>
         </is>
       </c>
     </row>
@@ -2636,25 +2636,29 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>INSTITUTO CARBÓ S.R.L</t>
+          <t>MUNICIPALIDAD DE URDINARRAIN</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Licitación</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>sin internación en materia de salud, pre- hospitalarias, atención médica, domiciliaria y traslados sanitarios de alta</t>
+          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
@@ -2686,7 +2690,7 @@
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-6aa57c7437a30ca3</t>
+          <t>id-7a200161bcc9b02b</t>
         </is>
       </c>
     </row>
@@ -2708,7 +2712,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE VIALE</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2718,18 +2722,18 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>08/26</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>de asf alto 70-16 destinado a la producción de pavimento de la Planta Asfáltica, y que a continuación se detalla y</t>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Publicada 06/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2737,7 +2741,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K31" s="4" t="inlineStr"/>
+      <c r="K31" s="4" t="inlineStr">
+        <is>
+          <t>$ 120.976,01</t>
+        </is>
+      </c>
       <c r="L31" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2750,19 +2758,19 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-ef1ddb923c7e7fdb</t>
+          <t>id-07ddb93a12c5a870</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>02/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2777,24 +2785,28 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>02/2025</t>
+        </is>
+      </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>CONSTRUCCIÓN DE OBRAS DE ARTE EN EL DEPARTAMENTO LA PAZ. 1) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE EN R.P. S/Nº SOBRE Aº ESTACAS – “CAMINO SAUCECITO” – TRAMO: R.P.Nº 1 – ESCUELA Nº 62 – DISTRITO ESTACAS – DEPARTAMENTO LA PAZ – 2) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE SOBRE Aº ESTACAS SAN GUSTAVO – TRAMO: […]</t>
+          <t>Concurso de Precio N° 02/2025</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 19/06/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2815,12 +2827,12 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-3d7728874996f284</t>
+          <t>id-7c1bf02160a66f67</t>
         </is>
       </c>
     </row>
@@ -3027,8 +3039,77 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Poder Judicial de Entre Ríos</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>08/26</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>Obra “Readecuación del sistema de climatización –ala sur- Edificio Tribunales Gualeguay”.</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr"/>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>Ver el sitio</t>
+        </is>
+      </c>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K36" s="4" t="inlineStr"/>
+      <c r="L36" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M36" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>Poder Judicial de Entre Ríos</t>
+        </is>
+      </c>
+      <c r="O36" s="4" t="inlineStr">
+        <is>
+          <t>id-9ca2387eef6d6fc1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O35"/>
+  <autoFilter ref="A1:O36"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -3098,6 +3179,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M34" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId67"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId70"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 03/10/2026 08:54
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$46</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -57,12 +57,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O36"/>
+  <dimension ref="A1:O46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -582,12 +582,12 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Infraestructura</t>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARÍ</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -597,22 +597,22 @@
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>016/2026</t>
+          <t>07/2026</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de mano de obra, materiales y equipamiento para ejecución de restitución de galibo y repavimentación en Avenida Belgrano y Avenida 1° de Mayo de esta ciudad de chajari</t>
+          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”, destinada a la obra denominada “Nueva Pileta en el Polideportivo El Aguará”,</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>02/10/2026</t>
+          <t>06/10/2026</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>02 DE OCTUBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>06/10/2026 HORA: 11:00 HS</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
@@ -622,7 +622,7 @@
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>$ 100.000, 00. - (PESOS CIEN MIL CON 00/100)</t>
+          <t>SIN COSTO</t>
         </is>
       </c>
       <c r="L2" s="6" t="inlineStr">
@@ -642,7 +642,7 @@
       </c>
       <c r="O2" s="4" t="inlineStr">
         <is>
-          <t>id-53f1430f94acb0b0</t>
+          <t>id-65d18d99bf0b2c6c</t>
         </is>
       </c>
     </row>
@@ -659,27 +659,27 @@
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>PARANA — MINISTERIO DE SALUD</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación Publica</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>07/2026</t>
+          <t>17/26</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”, destinada a la obra denominada “Nueva Pileta en el Polideportivo El Aguará”,</t>
+          <t>Adquirir Una (01) Mesa de Anestesia. Destino: Hospital “San José” de Diamante, dependiente del Ministerio de Salud de la Provincia de Entre Ríos</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
@@ -689,19 +689,15 @@
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026 HORA: 11:00 HS</t>
+          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr"/>
       <c r="L3" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -719,7 +715,7 @@
       </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
-          <t>id-65d18d99bf0b2c6c</t>
+          <t>id-3312d89e1a3e2e53</t>
         </is>
       </c>
     </row>
@@ -734,44 +730,44 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE SALUD</t>
+          <t>MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Licitación Publica</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>17/26</t>
+          <t>31/2026</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Adquirir Una (01) Mesa de Anestesia. Destino: Hospital “San José” de Diamante, dependiente del Ministerio de Salud de la Provincia de Entre Ríos</t>
+          <t>“Pavimento Rígido – 03 (tres) Cuadras Barrio San Felipe”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
+          <t>07 de octubre de 2026 Hora: 10:00</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr"/>
@@ -792,7 +788,7 @@
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
-          <t>id-3312d89e1a3e2e53</t>
+          <t>id-76d9566cb30a6df5</t>
         </is>
       </c>
     </row>
@@ -807,9 +803,9 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -824,22 +820,22 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>31/2026</t>
+          <t>32/2026</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>“Pavimento Rígido – 03 (tres) Cuadras Barrio San Felipe”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>"Adquisición de 835 m3 de Hormigón Calidad H25 para 08 cuadras de Pavimento", en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>07 de octubre de 2026 Hora: 10:00</t>
+          <t>08 de octubre de 2026 Hora: 10:00</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -865,7 +861,7 @@
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>id-76d9566cb30a6df5</t>
+          <t>id-0ace7de8f16d3baf</t>
         </is>
       </c>
     </row>
@@ -880,9 +876,9 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -897,12 +893,12 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>32/2026</t>
+          <t>33/2026</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>"Adquisición de 835 m3 de Hormigón Calidad H25 para 08 cuadras de Pavimento", en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>“Pavimento Rígido – 04 (cuatro) Cuadras Barrio San Roque y 01 (una) Cuadra Barrio Vicente Obrego”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -912,7 +908,7 @@
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>08 de octubre de 2026 Hora: 10:00</t>
+          <t>08 de octubre de 2026 Hora: 11:00</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -938,7 +934,7 @@
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>id-0ace7de8f16d3baf</t>
+          <t>id-fe71ac2aaf71b8d8</t>
         </is>
       </c>
     </row>
@@ -953,14 +949,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
+          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -970,22 +966,22 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>33/2026</t>
+          <t>34/2026</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>“Pavimento Rígido – 04 (cuatro) Cuadras Barrio San Roque y 01 (una) Cuadra Barrio Vicente Obrego”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>“Concesión de la Explotación Comercial de un (01) Camión de Comidas Rápidas (para cubrir el total de cuatro puestos) en la Zona Joven – Parque La Salamanca de la Municipalidad de Concepción del Uruguay – Entre Ríos”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>08 de octubre de 2026 Hora: 11:00</t>
+          <t>09 de octubre de 2026 Hora: 10:00</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -1011,7 +1007,7 @@
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>id-fe71ac2aaf71b8d8</t>
+          <t>id-b147fbd9d3081bfc</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1029,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1043,12 +1039,12 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>34/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>“Concesión de la Explotación Comercial de un (01) Camión de Comidas Rápidas (para cubrir el total de cuatro puestos) en la Zona Joven – Parque La Salamanca de la Municipalidad de Concepción del Uruguay – Entre Ríos”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>“PROVISIÓN DE UNA (1) MINICARGADORA 0 KM, CON CUCHARÓN FRONTAL DE USO GENERAL, UN (1) MARTILLO HIDRÁULICO Y UN (1) COMPACTADOR/RODILLO VIBRATORIO LISO”</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -1058,7 +1054,7 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>09 de octubre de 2026 Hora: 10:00</t>
+          <t>09/10/2026 HORA: 10:00 HS</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -1066,7 +1062,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr"/>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>($ 270.000,00) PESOS DOSCIENTOS SETENTA MIL</t>
+        </is>
+      </c>
       <c r="L8" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1084,7 +1084,7 @@
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>id-b147fbd9d3081bfc</t>
+          <t>id-779e4cd290f2e64e</t>
         </is>
       </c>
     </row>
@@ -1099,14 +1099,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1116,22 +1116,22 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>11/2026</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>“PROVISIÓN DE UNA (1) MINICARGADORA 0 KM, CON CUCHARÓN FRONTAL DE USO GENERAL, UN (1) MARTILLO HIDRÁULICO Y UN (1) COMPACTADOR/RODILLO VIBRATORIO LISO”</t>
+          <t>OBRA "PAVIMENTACION URBANA CALLE TRATADO DEL PILAR B° 3 DE FEBRERO - MUNICIPALIDAD DE SANTA ELENA" (Según Pliegos de Bases y condi ciones)</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>09/10/2026 HORA: 10:00 HS</t>
+          <t>13/10/2026 HORA: 10: 00 HS</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1141,7 +1141,7 @@
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>($ 270.000,00) PESOS DOSCIENTOS SETENTA MIL</t>
+          <t>$ 728.000,00 PESOS SETECIENTOS VEINTIOCHO MIL</t>
         </is>
       </c>
       <c r="L9" s="6" t="inlineStr">
@@ -1161,7 +1161,7 @@
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>id-779e4cd290f2e64e</t>
+          <t>id-1a2561509308b1b6</t>
         </is>
       </c>
     </row>
@@ -1178,12 +1178,12 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Infraestructura</t>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1198,7 +1198,7 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>OBRA "PAVIMENTACION URBANA CALLE TRATADO DEL PILAR B° 3 DE FEBRERO - MUNICIPALIDAD DE SANTA ELENA" (Según Pliegos de Bases y condi ciones)</t>
+          <t>REFACCION EN ESCUELA N° 65 “ALMIRANTE BROWN” – CIUDAD DE CONCORDIA - DEPARTAMENTO CONCORDIA - PROVINCIA DE ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -1208,19 +1208,15 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026 HORA: 10: 00 HS</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 09:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K10" s="4" t="inlineStr">
-        <is>
-          <t>$ 728.000,00 PESOS SETECIENTOS VEINTIOCHO MIL</t>
-        </is>
-      </c>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr"/>
       <c r="L10" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1238,7 +1234,7 @@
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>id-1a2561509308b1b6</t>
+          <t>id-fc30d5c0b0589a79</t>
         </is>
       </c>
     </row>
@@ -1253,7 +1249,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
@@ -1270,12 +1266,12 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>11/2026</t>
+          <t>13/2026</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>REFACCION EN ESCUELA N° 65 “ALMIRANTE BROWN” – CIUDAD DE CONCORDIA - DEPARTAMENTO CONCORDIA - PROVINCIA DE ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>REPARACIONES VARIAS EN C. P. E. F. Nº 3 “PROFESOR HUGO LA NASA” – CIUDAD DE CONCEPCION DEL URUGUAY - DEPARTAMENTO URUGUAY - PROVINCIA D E ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1285,7 +1281,7 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 09:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1311,7 +1307,7 @@
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>id-fc30d5c0b0589a79</t>
+          <t>id-9d3847fb0e2b0929</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1322,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
@@ -1343,12 +1339,12 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>13/2026</t>
+          <t>12/2026</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>REPARACIONES VARIAS EN C. P. E. F. Nº 3 “PROFESOR HUGO LA NASA” – CIUDAD DE CONCEPCION DEL URUGUAY - DEPARTAMENTO URUGUAY - PROVINCIA D E ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>RECAMBIO DE CUBIERTA Y REPARACIONES VARIAS EN ESCUELA Nº 92 “CONGRESO DE TUCUMAN” – CONCEPCION DEL URUGUAY - DPTO. URUGUAY – PROVINCIA DE ENTRE RIOS de acuerdo a las c ondiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -1358,7 +1354,7 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 10:30 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
@@ -1384,7 +1380,7 @@
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>id-9d3847fb0e2b0929</t>
+          <t>id-059239b424b9c936</t>
         </is>
       </c>
     </row>
@@ -1401,12 +1397,12 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1416,12 +1412,12 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>12/2026</t>
+          <t>87/2026</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>RECAMBIO DE CUBIERTA Y REPARACIONES VARIAS EN ESCUELA Nº 92 “CONGRESO DE TUCUMAN” – CONCEPCION DEL URUGUAY - DPTO. URUGUAY – PROVINCIA DE ENTRE RIOS de acuerdo a las c ondiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>Contratar la ejecución de la obra denominada “Construcción de Red Cloacal Subsidiaria del Colector Noroeste Barrio Ciudad Paisaje”</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
@@ -1431,15 +1427,19 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 10:30 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
+          <t>martes, 13 de octubre de 2026 a las 10:00</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
-        </is>
-      </c>
-      <c r="K13" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>$ 10.000 (pesos diez mil)</t>
+        </is>
+      </c>
       <c r="L13" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1452,12 +1452,12 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Boletín Oficial Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>id-059239b424b9c936</t>
+          <t>id-ceeb594e8bcc4ff7</t>
         </is>
       </c>
     </row>
@@ -1472,14 +1472,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>COLON — MUNICIPALIDAD DE COLON</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1487,24 +1487,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>87/2026</t>
-        </is>
-      </c>
+      <c r="F14" s="4" t="inlineStr"/>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Contratar la ejecución de la obra denominada “Construcción de Red Cloacal Subsidiaria del Colector Noroeste Barrio Ciudad Paisaje”</t>
+          <t>“ADQUISICIÓN DE MATERIALES ELÉCTRICOS PARA EJECUCIÓN DEL PROYECTO DE RECONVERSIÓN Y OPTIMIZACIÓN DEL ALUMBRADO PÚBLICO DE LA CIUDAD DE COLÓN”</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026</t>
+          <t>14/10/2026</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>martes, 13 de octubre de 2026 a las 10:00</t>
+          <t>14 de OCTUBRE de 2026</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1514,7 +1510,7 @@
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
-          <t>$ 10.000 (pesos diez mil)</t>
+          <t>Sin Cargo</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr">
@@ -1529,12 +1525,12 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Boletín Oficial Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>id-ceeb594e8bcc4ff7</t>
+          <t>id-9e122d52de12ffef</t>
         </is>
       </c>
     </row>
@@ -1549,14 +1545,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE COLON</t>
+          <t>DIAMANTE — COMUNA ALDEA PROTESTANTE -- DIAMANTE -- ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1564,10 +1560,14 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr"/>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>03/2026</t>
+        </is>
+      </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN DE MATERIALES ELÉCTRICOS PARA EJECUCIÓN DEL PROYECTO DE RECONVERSIÓN Y OPTIMIZACIÓN DEL ALUMBRADO PÚBLICO DE LA CIUDAD DE COLÓN”</t>
+          <t>Conforme a lo autorizado por decreto Nº 290/26 llámese a licitación pública Nº 03/26 con el objeto de comprar 10 toneladas de emulsión catiónica súper estable (asfalto de imprimación), puesto en Aldea Protestante</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
@@ -1577,7 +1577,7 @@
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>14 de OCTUBRE de 2026</t>
+          <t>miércoles 14 de octubre de 2026 – Hora nueve (09:00) Lugar de presentación de la oferta: Sede Comuna Aldea Protestan</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1585,11 +1585,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K15" s="4" t="inlineStr">
-        <is>
-          <t>Sin Cargo</t>
-        </is>
-      </c>
+      <c r="K15" s="4" t="inlineStr"/>
       <c r="L15" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1607,7 +1603,7 @@
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>id-9e122d52de12ffef</t>
+          <t>id-c2f3a25cfb37fd38</t>
         </is>
       </c>
     </row>
@@ -1622,14 +1618,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>DIAMANTE — COMUNA ALDEA PROTESTANTE -- DIAMANTE -- ENTRE RÍOS</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1639,12 +1635,12 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>03/2026</t>
+          <t>017/2026</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Conforme a lo autorizado por decreto Nº 290/26 llámese a licitación pública Nº 03/26 con el objeto de comprar 10 toneladas de emulsión catiónica súper estable (asfalto de imprimación), puesto en Aldea Protestante</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de UNA (1) MOTONIVELADORA, nueva, sin uso, cero km, con una potencia entre 220/240 HP, con opción a implementos, que será utilizada para el área del corralón municipal</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
@@ -1654,7 +1650,7 @@
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>miércoles 14 de octubre de 2026 – Hora nueve (09:00) Lugar de presentación de la oferta: Sede Comuna Aldea Protestan</t>
+          <t>14 DE OCTUBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -1662,7 +1658,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K16" s="4" t="inlineStr"/>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>$100.000,00. - (PESOS CIEN MIL CON 00/100) PRESUPUESTO OFICIAL ESTIMAD</t>
+        </is>
+      </c>
       <c r="L16" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1680,7 +1680,7 @@
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>id-c2f3a25cfb37fd38</t>
+          <t>id-4c3b33859e596759</t>
         </is>
       </c>
     </row>
@@ -1702,7 +1702,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
+          <t>VICTORIA — MUNICIPALIDAD DE VICTORIA</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1712,12 +1712,12 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>017/2026</t>
+          <t>008/2026</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de UNA (1) MOTONIVELADORA, nueva, sin uso, cero km, con una potencia entre 220/240 HP, con opción a implementos, que será utilizada para el área del corralón municipal</t>
+          <t>Proveer a la Municipalidad de Victoria, Entre Ríos, de Veinticinco Mil (25.000) litros de Diésel 500, para movilidad de vehículos y maquinarias viales , Ocho Mil (8.000) litros de Gasoil Tipo euro o similar y Ocho (8.000) litros de nafta súper para vehículos y áreas afectadas a la Secretaria de Planeamiento y Dirección de Ambiente y Desarrollo sostenible;</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -1727,7 +1727,7 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>14 DE OCTUBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>14 de octubre de 2026 a las 09:00 hs., en la Oficina de Compras de la Municipalidad de Victoria, Entr</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1735,11 +1735,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K17" s="4" t="inlineStr">
-        <is>
-          <t>$100.000,00. - (PESOS CIEN MIL CON 00/100) PRESUPUESTO OFICIAL ESTIMAD</t>
-        </is>
-      </c>
+      <c r="K17" s="4" t="inlineStr"/>
       <c r="L17" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1757,14 +1753,14 @@
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>id-4c3b33859e596759</t>
+          <t>id-a9af9f59c8c487c8</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1779,7 +1775,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>VICTORIA — MUNICIPALIDAD DE VICTORIA</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1789,12 +1785,12 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>008/2026</t>
+          <t>89/2026</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Proveer a la Municipalidad de Victoria, Entre Ríos, de Veinticinco Mil (25.000) litros de Diésel 500, para movilidad de vehículos y maquinarias viales , Ocho Mil (8.000) litros de Gasoil Tipo euro o similar y Ocho (8.000) litros de nafta súper para vehículos y áreas afectadas a la Secretaria de Planeamiento y Dirección de Ambiente y Desarrollo sostenible;</t>
+          <t>Adquisición de balanzas básculas para pesaje de ejes de camiones</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1804,7 +1800,7 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>14 de octubre de 2026 a las 09:00 hs., en la Oficina de Compras de la Municipalidad de Victoria, Entr</t>
+          <t>miércoles, 14 de octubre de 2026 a las 08:00</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1825,12 +1821,12 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Boletín Oficial Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>id-a9af9f59c8c487c8</t>
+          <t>id-d963348e34fcb0d3</t>
         </is>
       </c>
     </row>
@@ -1922,7 +1918,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -1995,7 +1991,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C21" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2068,7 +2064,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C22" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -2141,7 +2137,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
@@ -2210,7 +2206,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2218,7 +2214,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
@@ -2283,22 +2279,22 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C25" s="10" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
+          <t>COMUNA DE EL PALENQUE</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2308,18 +2304,22 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>07/2026</t>
+          <t>06/26</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>Transporte de mil doscientos cincuenta metros cúbicos (1.250 m³) de broza grillada desde Cantera “Tayreta” (Ruta Nacional N° 14 km 135) hasta jurisdicción de la comuna, de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr"/>
+          <t>Adquisición de UNA (1) PALA CARGADORA 0 KM destinada a trabajos en la Comuna</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>26/10/2026</t>
+        </is>
+      </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Viernes 09 de octubre del corriente año a las 10:00 hs en la Oficina de la Sede de la Comuna</t>
+          <t>26/10/2026, 12:30 horas, Lugar: Sede Administrativa de la Comuna de El Palenque, sito en calle San Martín sin número, El</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2327,7 +2327,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K25" s="4" t="inlineStr"/>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>pesos cero ($ 0,00)</t>
+        </is>
+      </c>
       <c r="L25" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2345,14 +2349,14 @@
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-24e9015ecceeff7f</t>
+          <t>id-4b7dfe1bdd0c2ac6</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2360,14 +2364,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C26" s="9" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
+          <t>MUNICIPALIDAD DE DIAMANTE -- ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2375,20 +2379,16 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>001/26</t>
-        </is>
-      </c>
+      <c r="F26" s="4" t="inlineStr"/>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN de UN (1) FURGON UTILITARIO CHICO con 5 asientos 0 KM. con destino a Subsecretaria de Asistencia Directa y Emergencia</t>
+          <t>Solicitar Contratación de una empresa para la Obra de “22 (veintidós) cuadras de pavimento urbano” – Grupo 1- según Expte. Letra “D” Nº 2196</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>DE LAS PROPUESTAS: 20 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
+          <t>viernes 23 de octubre de 2.026, a la hora diez (10.00)</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2414,7 +2414,7 @@
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-ca205f0874380f69</t>
+          <t>id-4f207bef5c709ad6</t>
         </is>
       </c>
     </row>
@@ -2429,31 +2429,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>INSTITUTO CARBÓ S.R.L</t>
+          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Licitación</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>07/2026</t>
+        </is>
+      </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>sin internación en materia de salud, pre- hospitalarias, atención médica, domiciliaria y traslados sanitarios de alta</t>
+          <t>Transporte de mil doscientos cincuenta metros cúbicos (1.250 m³) de broza grillada desde Cantera “Tayreta” (Ruta Nacional N° 14 km 135) hasta jurisdicción de la comuna, de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Viernes 09 de octubre del corriente año a las 10:00 hs en la Of icina de la Sede de la Comuna</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2479,7 +2483,7 @@
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-6aa57c7437a30ca3</t>
+          <t>id-24e9015ecceeff7f</t>
         </is>
       </c>
     </row>
@@ -2494,14 +2498,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE VIALE</t>
+          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2511,18 +2515,18 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>08/26</t>
+          <t>001/26</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>de asf alto 70-16 destinado a la producción de pavimento de la Planta Asfáltica, y que a continuación se detalla y</t>
+          <t>ADQUISICIÓN de UN (1) FURGON UTILITARIO CHICO con 5 asientos 0 KM. con destino a Subsecretaria de Asistencia Directa y Emergencia</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>DE LAS PROPUESTAS: 20 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2548,7 +2552,7 @@
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-ef1ddb923c7e7fdb</t>
+          <t>id-ca205f0874380f69</t>
         </is>
       </c>
     </row>
@@ -2565,33 +2569,29 @@
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
+          <t>INSTITUTO CARBÓ S.R.L</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>001-2026</t>
-        </is>
-      </c>
+          <t>Licitación</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr"/>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
+          <t>sin internación en materia de salud, pre- hospitalarias, atención médica, domiciliaria y traslados sanitarios de alta</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2599,11 +2599,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K29" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K29" s="4" t="inlineStr"/>
       <c r="L29" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2621,7 +2617,7 @@
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-b7b0120caf49d551</t>
+          <t>id-6aa57c7437a30ca3</t>
         </is>
       </c>
     </row>
@@ -2636,14 +2632,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C30" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE URDINARRAIN</t>
+          <t>MUNICIPALIDAD DE VIALE</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2653,12 +2649,12 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>08/26</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
+          <t>de asf alto 70-16 destinado a la producción de pavimento de la Planta Asfáltica, y que a continuación se detalla y</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
@@ -2690,7 +2686,7 @@
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-7a200161bcc9b02b</t>
+          <t>id-ef1ddb923c7e7fdb</t>
         </is>
       </c>
     </row>
@@ -2707,12 +2703,12 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Infraestructura</t>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2722,18 +2718,18 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>001-2026</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2743,7 +2739,7 @@
       </c>
       <c r="K31" s="4" t="inlineStr">
         <is>
-          <t>$ 120.976,01</t>
+          <t>SIN COSTO</t>
         </is>
       </c>
       <c r="L31" s="6" t="inlineStr">
@@ -2758,12 +2754,12 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-07ddb93a12c5a870</t>
+          <t>id-b7b0120caf49d551</t>
         </is>
       </c>
     </row>
@@ -2778,14 +2774,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>MUNICIPALIDAD DE URDINARRAIN</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -2795,18 +2791,18 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>Concurso de Precio N° 02/2025</t>
+          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2827,19 +2823,19 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-7c1bf02160a66f67</t>
+          <t>id-7a200161bcc9b02b</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2847,31 +2843,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C33" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>03/26</t>
+        </is>
+      </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2892,19 +2892,19 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-654eebef400f89cd</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2912,35 +2912,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C34" s="3" t="inlineStr">
+      <c r="C34" s="7" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Concurso</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>01/26</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -2961,19 +2961,19 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-9a16884dd5a64a49</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2981,35 +2981,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C35" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>2026-1227</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3030,19 +3030,19 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-0691eb485d7548eb</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3052,12 +3052,12 @@
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3067,18 +3067,18 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>08/26</t>
+          <t>05/2025</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>Obra “Readecuación del sistema de climatización –ala sur- Edificio Tribunales Gualeguay”.</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Ver el sitio</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3099,17 +3099,695 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>Poder Judicial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>id-9ca2387eef6d6fc1</t>
+          <t>id-22811eab8859abaf</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>IAPV (Vivienda)</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>06/2025</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr"/>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>Publicada 18/11/2025 — ver pliego</t>
+        </is>
+      </c>
+      <c r="J37" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K37" s="4" t="inlineStr"/>
+      <c r="L37" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M37" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>IAPV — Viviendas</t>
+        </is>
+      </c>
+      <c r="O37" s="4" t="inlineStr">
+        <is>
+          <t>id-c019bf4a08989c09</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>IAPV (Vivienda)</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr"/>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="inlineStr"/>
+      <c r="I38" s="4" t="inlineStr">
+        <is>
+          <t>Publicada 11/11/2025 — ver pliego</t>
+        </is>
+      </c>
+      <c r="J38" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K38" s="4" t="inlineStr"/>
+      <c r="L38" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M38" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>IAPV — Viviendas</t>
+        </is>
+      </c>
+      <c r="O38" s="4" t="inlineStr">
+        <is>
+          <t>id-ebeeb6a87e688d85</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>IAPV (Vivienda)</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>04/2025</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr"/>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>Publicada 23/10/2025 — ver pliego</t>
+        </is>
+      </c>
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K39" s="4" t="inlineStr"/>
+      <c r="L39" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M39" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>IAPV — Viviendas</t>
+        </is>
+      </c>
+      <c r="O39" s="4" t="inlineStr">
+        <is>
+          <t>id-34c85bcdb9b1123f</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>IAPV (Vivienda)</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>03/2025</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="inlineStr"/>
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>Publicada 08/10/2025 — ver pliego</t>
+        </is>
+      </c>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K40" s="4" t="inlineStr"/>
+      <c r="L40" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M40" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>IAPV — Viviendas</t>
+        </is>
+      </c>
+      <c r="O40" s="4" t="inlineStr">
+        <is>
+          <t>id-75bfffae63b7eedc</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>IAPV (Vivienda)</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>02/2025</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr"/>
+      <c r="I41" s="4" t="inlineStr">
+        <is>
+          <t>Publicada 06/10/2025 — ver pliego</t>
+        </is>
+      </c>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K41" s="4" t="inlineStr"/>
+      <c r="L41" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M41" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>IAPV — Viviendas</t>
+        </is>
+      </c>
+      <c r="O41" s="4" t="inlineStr">
+        <is>
+          <t>id-07ddb93a12c5a870</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>IAPV (Vivienda)</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>02/2025</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>Concurso de Precio N° 02/2025</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="inlineStr"/>
+      <c r="I42" s="4" t="inlineStr">
+        <is>
+          <t>Publicada 19/06/2025 — ver pliego</t>
+        </is>
+      </c>
+      <c r="J42" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K42" s="4" t="inlineStr"/>
+      <c r="L42" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M42" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>IAPV — Viviendas</t>
+        </is>
+      </c>
+      <c r="O42" s="4" t="inlineStr">
+        <is>
+          <t>id-7c1bf02160a66f67</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr"/>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>CONSTRUCCIÓN DE OBRAS DE ARTE EN EL DEPARTAMENTO LA PAZ. 1) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE EN R.P. S/Nº SOBRE Aº ESTACAS – “CAMINO SAUCECITO” – TRAMO: R.P.Nº 1 – ESCUELA Nº 62 – DISTRITO ESTACAS – DEPARTAMENTO LA PAZ – 2) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE SOBRE Aº ESTACAS SAN GUSTAVO – TRAMO: […]</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr"/>
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K43" s="4" t="inlineStr"/>
+      <c r="L43" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M43" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="O43" s="4" t="inlineStr">
+        <is>
+          <t>id-3d7728874996f284</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>Materiales</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr"/>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
+        </is>
+      </c>
+      <c r="H44" s="4" t="inlineStr"/>
+      <c r="I44" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J44" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K44" s="4" t="inlineStr"/>
+      <c r="L44" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M44" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="O44" s="4" t="inlineStr">
+        <is>
+          <t>id-654eebef400f89cd</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Concurso</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>01/26</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr"/>
+      <c r="I45" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J45" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K45" s="4" t="inlineStr"/>
+      <c r="L45" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M45" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="O45" s="4" t="inlineStr">
+        <is>
+          <t>id-9a16884dd5a64a49</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>Materiales</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>ENERSA</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Licitación</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>2026-1227</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+        </is>
+      </c>
+      <c r="H46" s="4" t="inlineStr"/>
+      <c r="I46" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J46" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K46" s="4" t="inlineStr"/>
+      <c r="L46" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M46" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>ENERSA</t>
+        </is>
+      </c>
+      <c r="O46" s="4" t="inlineStr">
+        <is>
+          <t>id-0691eb485d7548eb</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O36"/>
+  <autoFilter ref="A1:O46"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -3181,6 +3859,26 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M35" r:id="rId68"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId69"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M36" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M37" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L38" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M38" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M39" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L43" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId90"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 04/10/2026 08:19
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$45</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O46"/>
+  <dimension ref="A1:O45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2766,7 +2766,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2774,14 +2774,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE URDINARRAIN</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -2791,18 +2791,18 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>03/26</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de 300 M³ de hormigón elaborado H -21 (puesto en obra)</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2823,12 +2823,12 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-7a200161bcc9b02b</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
@@ -2860,18 +2860,18 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>03/26</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2897,7 +2897,7 @@
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
@@ -2929,18 +2929,18 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>02/2026</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -2966,7 +2966,7 @@
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
@@ -2998,18 +2998,18 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>05/2025</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3035,7 +3035,7 @@
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
@@ -3067,18 +3067,18 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>05/2025</t>
+          <t>06/2025</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3104,7 +3104,7 @@
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
@@ -3134,20 +3134,16 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F37" s="4" t="inlineStr">
-        <is>
-          <t>06/2025</t>
-        </is>
-      </c>
+      <c r="F37" s="4" t="inlineStr"/>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3173,7 +3169,7 @@
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
@@ -3203,16 +3199,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F38" s="4" t="inlineStr"/>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>04/2025</t>
+        </is>
+      </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -3238,7 +3238,7 @@
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>id-ebeeb6a87e688d85</t>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
@@ -3270,18 +3270,18 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>04/2025</t>
+          <t>03/2025</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -3307,14 +3307,14 @@
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
-          <t>id-34c85bcdb9b1123f</t>
+          <t>id-75bfffae63b7eedc</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3339,18 +3339,18 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>03/2025</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr"/>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
+          <t>Publicada 06/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
@@ -3376,7 +3376,7 @@
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
-          <t>id-75bfffae63b7eedc</t>
+          <t>id-07ddb93a12c5a870</t>
         </is>
       </c>
     </row>
@@ -3413,13 +3413,13 @@
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>Concurso de Precio N° 02/2025</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>Publicada 19/06/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
@@ -3445,14 +3445,14 @@
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
-          <t>id-07ddb93a12c5a870</t>
+          <t>id-7c1bf02160a66f67</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3467,28 +3467,24 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="inlineStr">
-        <is>
-          <t>02/2025</t>
-        </is>
-      </c>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr"/>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>Concurso de Precio N° 02/2025</t>
+          <t>CONSTRUCCIÓN DE OBRAS DE ARTE EN EL DEPARTAMENTO LA PAZ. 1) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE EN R.P. S/Nº SOBRE Aº ESTACAS – “CAMINO SAUCECITO” – TRAMO: R.P.Nº 1 – ESCUELA Nº 62 – DISTRITO ESTACAS – DEPARTAMENTO LA PAZ – 2) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE SOBRE Aº ESTACAS SAN GUSTAVO – TRAMO: […]</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr"/>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr">
@@ -3509,19 +3505,19 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O42" s="4" t="inlineStr">
         <is>
-          <t>id-7c1bf02160a66f67</t>
+          <t>id-3d7728874996f284</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -3529,9 +3525,9 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C43" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -3547,7 +3543,7 @@
       <c r="F43" s="4" t="inlineStr"/>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>CONSTRUCCIÓN DE OBRAS DE ARTE EN EL DEPARTAMENTO LA PAZ. 1) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE EN R.P. S/Nº SOBRE Aº ESTACAS – “CAMINO SAUCECITO” – TRAMO: R.P.Nº 1 – ESCUELA Nº 62 – DISTRITO ESTACAS – DEPARTAMENTO LA PAZ – 2) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE SOBRE Aº ESTACAS SAN GUSTAVO – TRAMO: […]</t>
+          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr"/>
@@ -3579,7 +3575,7 @@
       </c>
       <c r="O43" s="4" t="inlineStr">
         <is>
-          <t>id-3d7728874996f284</t>
+          <t>id-654eebef400f89cd</t>
         </is>
       </c>
     </row>
@@ -3594,9 +3590,9 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -3606,13 +3602,17 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F44" s="4" t="inlineStr"/>
+          <t>Concurso</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>01/26</t>
+        </is>
+      </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr"/>
@@ -3644,7 +3644,7 @@
       </c>
       <c r="O44" s="4" t="inlineStr">
         <is>
-          <t>id-654eebef400f89cd</t>
+          <t>id-9a16884dd5a64a49</t>
         </is>
       </c>
     </row>
@@ -3659,29 +3659,29 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C45" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Concurso</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>01/26</t>
+          <t>2026-1227</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr"/>
@@ -3708,86 +3708,17 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="O45" s="4" t="inlineStr">
         <is>
-          <t>id-9a16884dd5a64a49</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>ENERSA</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Licitación</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="inlineStr">
-        <is>
-          <t>2026-1227</t>
-        </is>
-      </c>
-      <c r="G46" s="5" t="inlineStr">
-        <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
-        </is>
-      </c>
-      <c r="H46" s="4" t="inlineStr"/>
-      <c r="I46" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J46" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K46" s="4" t="inlineStr"/>
-      <c r="L46" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M46" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>ENERSA</t>
-        </is>
-      </c>
-      <c r="O46" s="4" t="inlineStr">
-        <is>
           <t>id-0691eb485d7548eb</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O46"/>
+  <autoFilter ref="A1:O45"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -3877,8 +3808,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId86"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId87"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId90"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 06/10/2026 08:08
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O45"/>
+  <dimension ref="A1:O44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2693,7 +2693,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2701,14 +2701,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE GILBERT</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2718,18 +2718,18 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>001-2026</t>
+          <t>03/26</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>LLAMADO A LICITACIÓN PÚBLICA Nº 001 -2026 – DECRETO N° 134/2026 DEPARTAMENTO EJECUTIVO. “CONTRATACION DE MANO DE OBRA PARA LA CONSTRUCCION DE UNA PILETA SEMI - OLIMPICA Y OBRAS COMPLEMENTARIAS EN EL MARCO DEL PLIEGO DE BASES Y CONDICIONES GENERALES Y PLIEGO DE CONDICIONES PARTICULARES Y ESPECIFICACIONES TECNICAS”</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Miércoles Treinta (30) de septiembre de 2026 a las 09:30 horas, en el Honorable Concejo Deliberante del M</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2737,11 +2737,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K31" s="4" t="inlineStr">
-        <is>
-          <t>SIN COSTO</t>
-        </is>
-      </c>
+      <c r="K31" s="4" t="inlineStr"/>
       <c r="L31" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2754,12 +2750,12 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-b7b0120caf49d551</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
@@ -2791,18 +2787,18 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>03/26</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2828,7 +2824,7 @@
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
@@ -2860,18 +2856,18 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>02/2026</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2897,7 +2893,7 @@
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
@@ -2929,18 +2925,18 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>05/2025</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -2966,7 +2962,7 @@
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
@@ -2998,18 +2994,18 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>05/2025</t>
+          <t>06/2025</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3035,7 +3031,7 @@
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
@@ -3065,20 +3061,16 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>06/2025</t>
-        </is>
-      </c>
+      <c r="F36" s="4" t="inlineStr"/>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3104,7 +3096,7 @@
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
@@ -3134,16 +3126,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F37" s="4" t="inlineStr"/>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>04/2025</t>
+        </is>
+      </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3169,7 +3165,7 @@
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>id-ebeeb6a87e688d85</t>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
@@ -3201,18 +3197,18 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>04/2025</t>
+          <t>03/2025</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -3238,14 +3234,14 @@
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>id-34c85bcdb9b1123f</t>
+          <t>id-75bfffae63b7eedc</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3270,18 +3266,18 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>03/2025</t>
+          <t>02/2025</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
+          <t>Publicada 06/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -3307,7 +3303,7 @@
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
-          <t>id-75bfffae63b7eedc</t>
+          <t>id-07ddb93a12c5a870</t>
         </is>
       </c>
     </row>
@@ -3344,13 +3340,13 @@
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>Concurso de Precio N° 02/2025</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr"/>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>Publicada 19/06/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
@@ -3376,14 +3372,14 @@
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
-          <t>id-07ddb93a12c5a870</t>
+          <t>id-7c1bf02160a66f67</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3398,28 +3394,24 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F41" s="4" t="inlineStr">
-        <is>
-          <t>02/2025</t>
-        </is>
-      </c>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr"/>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>Concurso de Precio N° 02/2025</t>
+          <t>CONSTRUCCIÓN DE OBRAS DE ARTE EN EL DEPARTAMENTO LA PAZ. 1) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE EN R.P. S/Nº SOBRE Aº ESTACAS – “CAMINO SAUCECITO” – TRAMO: R.P.Nº 1 – ESCUELA Nº 62 – DISTRITO ESTACAS – DEPARTAMENTO LA PAZ – 2) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE SOBRE Aº ESTACAS SAN GUSTAVO – TRAMO: […]</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
@@ -3440,19 +3432,19 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
-          <t>id-7c1bf02160a66f67</t>
+          <t>id-3d7728874996f284</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3460,9 +3452,9 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C42" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -3478,7 +3470,7 @@
       <c r="F42" s="4" t="inlineStr"/>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>CONSTRUCCIÓN DE OBRAS DE ARTE EN EL DEPARTAMENTO LA PAZ. 1) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE EN R.P. S/Nº SOBRE Aº ESTACAS – “CAMINO SAUCECITO” – TRAMO: R.P.Nº 1 – ESCUELA Nº 62 – DISTRITO ESTACAS – DEPARTAMENTO LA PAZ – 2) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE SOBRE Aº ESTACAS SAN GUSTAVO – TRAMO: […]</t>
+          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr"/>
@@ -3510,7 +3502,7 @@
       </c>
       <c r="O42" s="4" t="inlineStr">
         <is>
-          <t>id-3d7728874996f284</t>
+          <t>id-654eebef400f89cd</t>
         </is>
       </c>
     </row>
@@ -3525,9 +3517,9 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -3537,13 +3529,17 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F43" s="4" t="inlineStr"/>
+          <t>Concurso</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>01/26</t>
+        </is>
+      </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr"/>
@@ -3575,7 +3571,7 @@
       </c>
       <c r="O43" s="4" t="inlineStr">
         <is>
-          <t>id-654eebef400f89cd</t>
+          <t>id-9a16884dd5a64a49</t>
         </is>
       </c>
     </row>
@@ -3590,29 +3586,29 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C44" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Concurso</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>01/26</t>
+          <t>2026-1227</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr"/>
@@ -3639,86 +3635,17 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="O44" s="4" t="inlineStr">
         <is>
-          <t>id-9a16884dd5a64a49</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>ENERSA</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Licitación</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="inlineStr">
-        <is>
-          <t>2026-1227</t>
-        </is>
-      </c>
-      <c r="G45" s="5" t="inlineStr">
-        <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
-        </is>
-      </c>
-      <c r="H45" s="4" t="inlineStr"/>
-      <c r="I45" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J45" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K45" s="4" t="inlineStr"/>
-      <c r="L45" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M45" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>ENERSA</t>
-        </is>
-      </c>
-      <c r="O45" s="4" t="inlineStr">
-        <is>
           <t>id-0691eb485d7548eb</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O45"/>
+  <autoFilter ref="A1:O44"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -3806,8 +3733,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId84"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId85"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId88"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 07/10/2026 08:21
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$49</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -57,17 +57,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E6D9F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O44"/>
+  <dimension ref="A1:O49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -572,7 +572,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -582,12 +582,12 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA — INSTITUTO AUTÁRQUICO DE PLANEAMIENTO YY VI</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -597,22 +597,22 @@
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>07/2026</t>
+          <t>05/2026</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>“PROVISIÓN, TRASLADO, EXCAVACIÓN, PREPARACIÓN DEL TERRENO, INSTALACIÓN Y PUESTA EN FUNCIONAMIENTO DE UNA (1) PISCINA INFANTIL, CON EQUIPAMIENTO Y ACCESORIOS”, destinada a la obra denominada “Nueva Pileta en el Polideportivo El Aguará”,</t>
+          <t>COMPLEJO HABITACIONAL SAN AGUSTIN (P.P.) PARANÁ 24 VIVIENDAS, 7 LOCALES COMERCIALES Y 27 ESPACIOS DE ESTACIONAMIENTOS DEPARTAMENTO: PARANÁ</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
+          <t>01/12/2026</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026 HORA: 11:00 HS</t>
+          <t>DÍA: 01 /12/2026 HORA: 10:30 hs</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
@@ -622,7 +622,7 @@
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>SIN COSTO</t>
+          <t>$ 299.794,33</t>
         </is>
       </c>
       <c r="L2" s="6" t="inlineStr">
@@ -642,7 +642,7 @@
       </c>
       <c r="O2" s="4" t="inlineStr">
         <is>
-          <t>id-65d18d99bf0b2c6c</t>
+          <t>id-be1efacbe31d4a09</t>
         </is>
       </c>
     </row>
@@ -657,44 +657,44 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE SALUD</t>
+          <t>MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Licitación Publica</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>17/26</t>
+          <t>31/2026</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>Adquirir Una (01) Mesa de Anestesia. Destino: Hospital “San José” de Diamante, dependiente del Ministerio de Salud de la Provincia de Entre Ríos</t>
+          <t>“Pavimento Rígido – 03 (tres) Cuadras Barrio San Felipe”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
+          <t>07 de octubre de 2026 Hora: 10:00</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr"/>
@@ -715,7 +715,7 @@
       </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
-          <t>id-3312d89e1a3e2e53</t>
+          <t>id-76d9566cb30a6df5</t>
         </is>
       </c>
     </row>
@@ -732,7 +732,7 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Infraestructura</t>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -747,22 +747,22 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>31/2026</t>
+          <t>32/2026</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>“Pavimento Rígido – 03 (tres) Cuadras Barrio San Felipe”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>"Adquisición de 835 m3 de Hormigón Calidad H25 para 08 cuadras de Pavimento", en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>07 de octubre de 2026 Hora: 10:00</t>
+          <t>08 de octubre de 2026 Hora: 10:00</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
-          <t>id-76d9566cb30a6df5</t>
+          <t>id-0ace7de8f16d3baf</t>
         </is>
       </c>
     </row>
@@ -803,9 +803,9 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -820,12 +820,12 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>32/2026</t>
+          <t>33/2026</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>"Adquisición de 835 m3 de Hormigón Calidad H25 para 08 cuadras de Pavimento", en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>“Pavimento Rígido – 04 (cuatro) Cuadras Barrio San Roque y 01 (una) Cuadra Barrio Vicente Obrego”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -835,7 +835,7 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>08 de octubre de 2026 Hora: 10:00</t>
+          <t>08 de octubre de 2026 Hora: 11:00</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -861,14 +861,14 @@
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>id-0ace7de8f16d3baf</t>
+          <t>id-fe71ac2aaf71b8d8</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -876,29 +876,29 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>CONCURSO DE PRECIOS</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>33/2026</t>
+          <t>302/2026</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>“Pavimento Rígido – 04 (cuatro) Cuadras Barrio San Roque y 01 (una) Cuadra Barrio Vicente Obrego”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>ADQUISICION DE MAT. PARA LA CONSTRUCCION, ARTICULOS DE FERRETERIA , PINTURERUA Y MAT. ELECTRICOS</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>08 de octubre de 2026 Hora: 11:00</t>
+          <t>08-10-2026 08:30</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -929,12 +929,12 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>id-fe71ac2aaf71b8d8</t>
+          <t>id-2d3ee6d70e7e432c</t>
         </is>
       </c>
     </row>
@@ -1099,7 +1099,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -1176,7 +1176,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
@@ -1249,7 +1249,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
@@ -1322,7 +1322,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
@@ -1395,7 +1395,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -1472,7 +1472,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -1545,7 +1545,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>Materiales</t>
         </is>
@@ -1760,7 +1760,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1780,7 +1780,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>LICITACIÓN PÚBLICA</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -1790,7 +1790,7 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de balanzas básculas para pesaje de ejes de camiones</t>
+          <t>ADQUISICION DE BALANZA BASCULA PARA PESAJE DE EJESDE CAMIONES</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1800,7 +1800,7 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 14 de octubre de 2026 a las 08:00</t>
+          <t>14-10-2026 08:00</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1821,19 +1821,19 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Boletín Oficial Municipalidad de Paraná</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>id-d963348e34fcb0d3</t>
+          <t>id-4ee814ba6420f0cc</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1841,14 +1841,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>MINISTERIO DE SALUD — GOBIERNO DE ENTRE RIOS</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1858,22 +1858,22 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>18/26</t>
+          <t>89/2026</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Adquirir Sesenta Mil (60.000) Kilogramos de Leche Entera en Polvo Instantánea, Fortificada con Hierro, Zinc y Ácido Ascórbico</t>
+          <t>Adquisición de balanzas básculas para pesaje de ejes de camiones</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>16/10/2026</t>
+          <t>14/10/2026</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
+          <t>miércoles, 14 de octubre de 2026 a las 08:00</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1881,11 +1881,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K19" s="4" t="inlineStr">
-        <is>
-          <t>PESOS TRES MIL QUINIENTOS ($ 3.500,00)</t>
-        </is>
-      </c>
+      <c r="K19" s="4" t="inlineStr"/>
       <c r="L19" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1898,19 +1894,19 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Boletín Oficial Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>id-04a917d50ccab2e3</t>
+          <t>id-d963348e34fcb0d3</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1918,14 +1914,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>VILLAGUAY — MUNICIPALIDAD DE VILLAGUAY</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE ALDEA SAN ANTONIO</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1933,20 +1929,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr"/>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>002/2026</t>
+        </is>
+      </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Contratación, ejecución, liquidación, pago y recepción de la obra destinada a la elaboración del Proyecto Ejecutivo, provisión de materiales, mano de obra, equipos, ejecución, ensayos, habilitación y puesta en servicio de la instalación de gas natural para la Planta Municipal de Elaboración de Mezcla Asfáltica en Caliente, ubicada en el Lote N.º 4 de la Chacra N.º 263 del Parque Industrial de Villaguay, Provincia de Entre Ríos. La contratación comprender á una solución integral bajo modalidad “llave en mano”, incluyendo todos los trabajos, provisiones, trámites, representaciones técnicas, insp</t>
+          <t>ADQUISICIÓN DE UNA MÁQUINA MOTONIVELADORA PARA INCORPORAR AL PARQUE AUTOMOTOR DE LA MUNICIPALIDAD DE ALDEA SAN ANTONIO</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>16/10/2026</t>
+          <t>15/10/2026</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>16 de octubre del año 2026 a las 10:00 Horas, la que se reali zara en la Oficina de suministros de la Municipalidad de V</t>
+          <t>15 de octubre de 2026, a las 08:00 horas, en el Edificio Municipal</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>$ 50.000,00</t>
+          <t>PESOS CIEN MIL con 00/ 100 ($ 100.000,00.-)</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
@@ -1976,7 +1976,7 @@
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>id-55f1e5ca423a9262</t>
+          <t>id-95a507b67b7b1450</t>
         </is>
       </c>
     </row>
@@ -1993,12 +1993,12 @@
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Infraestructura</t>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>SALUD ENTRE RÍOS S.A.U</t>
+          <t>MINISTERIO DE SALUD — GOBIERNO DE ENTRE RIOS</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2006,20 +2006,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr"/>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>18/26</t>
+        </is>
+      </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Contratación de Servicio de Viandas para el Hospital de la Baxada</t>
+          <t>Adquirir Sesenta Mil (60.000) Kilogramos de Leche Entera en Polvo Instantánea, Fortificada con Hierro, Zinc y Ácido Ascórbico</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>16/10/2026</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>Hospital de la Baxada, calle Gral. Al varado Nº 2.250 Paraná, Entre Ríos, el día 19/10/2026 a las 10:00 hs</t>
+          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -2029,7 +2033,7 @@
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>PESOS TRES MIL QUINIENTOS ($ 3.500,00)</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr">
@@ -2049,7 +2053,7 @@
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-d35d5e849089d7ac</t>
+          <t>id-04a917d50ccab2e3</t>
         </is>
       </c>
     </row>
@@ -2064,14 +2068,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>PARANA — SALUD ENTRE RÍOS S.A.U</t>
+          <t>VILLAGUAY — MUNICIPALIDAD DE VILLAGUAY</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2082,17 +2086,17 @@
       <c r="F22" s="4" t="inlineStr"/>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Servicio de Recolección, Lavado, Desinfección, Secado, Planchado y Transporte de Ropa Hospitalaria</t>
+          <t>Contratación, ejecución, liquidación, pago y recepción de la obra destinada a la elaboración del Proyecto Ejecutivo, provisión de materiales, mano de obra, equipos, ejecución, ensayos, habilitación y puesta en servicio de la instalación de gas natural para la Planta Municipal de Elaboración de Mezcla Asfáltica en Caliente, ubicada en el Lote N.º 4 de la Chacra N.º 263 del Parque Industrial de Villaguay, Provincia de Entre Ríos. La contratación comprender á una solución integral bajo modalidad “llave en mano”, incluyendo todos los trabajos, provisiones, trámites, representaciones técnicas, insp</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>21/10/2026</t>
+          <t>16/10/2026</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Hospital de la Baxada, calle Gral. Alvarado Nº 2.250 Paraná, Entre Ríos, el día 21/10/2026 a las 10:00 hs</t>
+          <t>16 de octubre del año 2026 a las 10:00 Horas, la que se reali zara en la Oficina de suministros de la Municipalidad de V</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -2102,7 +2106,7 @@
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>$ 50.000,00</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr">
@@ -2122,7 +2126,7 @@
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-6b955df9d3f6241a</t>
+          <t>id-55f1e5ca423a9262</t>
         </is>
       </c>
     </row>
@@ -2139,12 +2143,12 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>SALUD ENTRE RÍOS S.A.U</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2152,24 +2156,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>11/26</t>
-        </is>
-      </c>
+      <c r="F23" s="4" t="inlineStr"/>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “TERMINACION ESCUELA Nº 40 “JOSÉ ENRIQUE RODÓ”-SEPTIMO DISTRITO-DEPARTAMENTO GUALEGUAY.”</t>
+          <t>Contratación de Servicio de Viandas para el Hospital de la Baxada</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>23/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 23 de Octubre de 2026 a las 10:00 hs</t>
+          <t>Hospital de la Baxada, calle Gral. Al varado Nº 2.250 Paraná, Entre Ríos, el día 19/10/2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2179,7 +2179,7 @@
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t>$ 100 (Cien)</t>
+          <t>Ninguno</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr">
@@ -2199,14 +2199,14 @@
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-86cc9c230734c462</t>
+          <t>id-d35d5e849089d7ac</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2214,14 +2214,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>MUNICIPALIDAD DE VILLAGUAY</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2229,24 +2229,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>11/2026</t>
-        </is>
-      </c>
+      <c r="F24" s="4" t="inlineStr"/>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Terminación Escuela N° 40 "José Enrique Rodó", Séptimo Distrito</t>
+          <t>Provisión de una (1) camioneta usada destinada al Parque Automotor Municipal</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>23/10/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>viernes, 23 de octubre de 2026 - 10:00hs</t>
+          <t>21 de octubre del año 2026 a las 10:00 Horas, la que se realizara en la Oficina de suministros de la Municipalidad de Vi</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -2254,7 +2250,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K24" s="4" t="inlineStr"/>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>$10.000,00</t>
+        </is>
+      </c>
       <c r="L24" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2267,19 +2267,19 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-322a40f5e43af35d</t>
+          <t>id-2d3dded56e6c6f6a</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -2287,14 +2287,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>COMUNA DE EL PALENQUE</t>
+          <t>PARANA — SALUD ENTRE RÍOS S.A.U</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2302,24 +2302,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>06/26</t>
-        </is>
-      </c>
+      <c r="F25" s="4" t="inlineStr"/>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de UNA (1) PALA CARGADORA 0 KM destinada a trabajos en la Comuna</t>
+          <t>Servicio de Recolección, Lavado, Desinfección, Secado, Planchado y Transporte de Ropa Hospitalaria</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>26/10/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>26/10/2026, 12:30 horas, Lugar: Sede Administrativa de la Comuna de El Palenque, sito en calle San Martín sin número, El</t>
+          <t>Hospital de la Baxada, calle Gral. Alvarado Nº 2.250 Paraná, Entre Ríos, el día 21/10/2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2329,7 +2325,7 @@
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>pesos cero ($ 0,00)</t>
+          <t>Ninguno</t>
         </is>
       </c>
       <c r="L25" s="6" t="inlineStr">
@@ -2349,29 +2345,29 @@
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-4b7dfe1bdd0c2ac6</t>
+          <t>id-6b955df9d3f6241a</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE DIAMANTE -- ENTRE RÍOS</t>
+          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2379,16 +2375,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr"/>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>11/26</t>
+        </is>
+      </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Solicitar Contratación de una empresa para la Obra de “22 (veintidós) cuadras de pavimento urbano” – Grupo 1- según Expte. Letra “D” Nº 2196</t>
-        </is>
-      </c>
-      <c r="H26" s="4" t="inlineStr"/>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “TERMINACION ESCUELA Nº 40 “JOSÉ ENRIQUE RODÓ”-SEPTIMO DISTRITO-DEPARTAMENTO GUALEGUAY.”</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>viernes 23 de octubre de 2.026, a la hora diez (10.00)</t>
+          <t>DE LAS OFERTAS: el día 23 de Octubre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2396,7 +2400,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K26" s="4" t="inlineStr"/>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>$ 100 (Cien)</t>
+        </is>
+      </c>
       <c r="L26" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2414,29 +2422,29 @@
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-4f207bef5c709ad6</t>
+          <t>id-86cc9c230734c462</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C27" s="10" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2446,18 +2454,22 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>07/2026</t>
+          <t>11/2026</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>Transporte de mil doscientos cincuenta metros cúbicos (1.250 m³) de broza grillada desde Cantera “Tayreta” (Ruta Nacional N° 14 km 135) hasta jurisdicción de la comuna, de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="inlineStr"/>
+          <t>Terminación Escuela N° 40 "José Enrique Rodó", Séptimo Distrito</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>23/10/2026</t>
+        </is>
+      </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Viernes 09 de octubre del corriente año a las 10:00 hs en la Of icina de la Sede de la Comuna</t>
+          <t>viernes, 23 de octubre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2478,24 +2490,24 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-24e9015ecceeff7f</t>
+          <t>id-322a40f5e43af35d</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
@@ -2505,7 +2517,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
+          <t>COMUNA DE EL PALENQUE</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2515,18 +2527,22 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>001/26</t>
+          <t>06/26</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN de UN (1) FURGON UTILITARIO CHICO con 5 asientos 0 KM. con destino a Subsecretaria de Asistencia Directa y Emergencia</t>
-        </is>
-      </c>
-      <c r="H28" s="4" t="inlineStr"/>
+          <t>Adquisición de UNA (1) PALA CARGADORA 0 KM destinada a trabajos en la Comuna</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>26/10/2026</t>
+        </is>
+      </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>DE LAS PROPUESTAS: 20 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
+          <t>26/10/2026, 12:30 horas, Lugar: Sede Administrativa de la Comuna de El Palenque, sito en calle San Martín sin número, El</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2534,7 +2550,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K28" s="4" t="inlineStr"/>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>pesos cero ($0,00)</t>
+        </is>
+      </c>
       <c r="L28" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2552,14 +2572,14 @@
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-ca205f0874380f69</t>
+          <t>id-4b7dfe1bdd0c2ac6</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2567,31 +2587,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>INSTITUTO CARBÓ S.R.L</t>
+          <t>DIAMANTE — MUNICIPALIDAD DE DIAMANTE -- ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr"/>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>sin internación en materia de salud, pre- hospitalarias, atención médica, domiciliaria y traslados sanitarios de alta</t>
+          <t>Solicitar Contratación de una empresa para la Obra de “22 (veintidós) cuadras de pavimento urbano” – Grupo 1- según Expte. Letra “D” Nº 2196</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>viernes 23 de octubre de 2.026, a la hora diez (10.00)</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2617,7 +2637,7 @@
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-6aa57c7437a30ca3</t>
+          <t>id-4f207bef5c709ad6</t>
         </is>
       </c>
     </row>
@@ -2632,14 +2652,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C30" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE VIALE</t>
+          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2649,18 +2669,18 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>08/26</t>
+          <t>07/2026</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>de asf alto 70-16 destinado a la producción de pavimento de la Planta Asfáltica, y que a continuación se detalla y</t>
+          <t>Transporte de mil doscientos cincuenta metros cúbicos (1.250 m³) de broza grillada desde Cantera “Tayreta” (Ruta Nacional N ° 14 km 135) hasta jurisdicción de la comuna, de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Viernes 09 de octubre del corriente año a las 10:00 hs en la Oficina de la Sede de la Comuna</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2686,14 +2706,14 @@
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-ef1ddb923c7e7fdb</t>
+          <t>id-24e9015ecceeff7f</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2701,35 +2721,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C31" s="7" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>CONCORDIA — APEX S.A.S</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>03/26</t>
-        </is>
-      </c>
+          <t>Licitación</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr"/>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+          <t>instalaciones eléctricas, sanitarias, hidráulicas, mecánicas o de cualquier otra naturaleza relacionada con el sector</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2750,19 +2766,19 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-a20c6b2b6fcf36a2</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2770,35 +2786,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C32" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Boletín Oficial</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>02/2026</t>
-        </is>
-      </c>
+          <t>Remate</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr"/>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+          <t>los vehículos se encuentran en exhibición por lo cuál la información registral, de rentas y de infracciones puede ser</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2819,19 +2831,19 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-fb8d7dc09e202fea</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2839,14 +2851,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C33" s="7" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2856,18 +2868,18 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>001/26</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+          <t>ADQUISICIÓN de UN (1) FURGON UTILITARIO CHICO con 5 asientos 0 KM. con destino a Subsecretaria de Asistencia Directa y Emergencia</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>DE LAS PROPUESTAS: 20 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2888,19 +2900,19 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-ca205f0874380f69</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2908,35 +2920,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>INSTITUTO CARBÓ S.R.L</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t>05/2025</t>
-        </is>
-      </c>
+          <t>Licitación</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr"/>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
+          <t>sin internación en materia de salud, pre- hospitalarias, atención médica, domiciliaria y traslados sanitarios de alta</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -2957,19 +2965,19 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-6aa57c7437a30ca3</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2977,14 +2985,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C35" s="7" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>MUNICIPALIDAD DE VIALE</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -2994,18 +3002,18 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>06/2025</t>
+          <t>08/26</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>de asf alto 70-16 destinado a la producción de pavimento de la Planta Asfáltica, y que a continuación se detalla y</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3026,19 +3034,19 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
+          <t>id-ef1ddb923c7e7fdb</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3046,7 +3054,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C36" s="7" t="inlineStr">
+      <c r="C36" s="3" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -3061,16 +3069,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F36" s="4" t="inlineStr"/>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+          <t>TERMINACIÓN CONCEPCIÓN DEL URUGUAY 63 VIV</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
+          <t>Publicada 06/10/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3096,14 +3108,14 @@
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>id-ebeeb6a87e688d85</t>
+          <t>id-1a3c1f8e036ac91e</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3111,7 +3123,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C37" s="7" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -3128,18 +3140,18 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>04/2025</t>
+          <t>05/2026</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+          <t>COMPLEJO HABITACIONAL SAN AGUSTÍN (P</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
+          <t>Publicada 05/10/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3165,7 +3177,7 @@
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>id-34c85bcdb9b1123f</t>
+          <t>id-ccb22bcad9356438</t>
         </is>
       </c>
     </row>
@@ -3180,7 +3192,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C38" s="7" t="inlineStr">
+      <c r="C38" s="3" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -3197,18 +3209,18 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>03/2025</t>
+          <t>03/26</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -3234,14 +3246,14 @@
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>id-75bfffae63b7eedc</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3249,7 +3261,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C39" s="7" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -3266,18 +3278,18 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>CONCORDIA 18 VIVIENDAS EN DUPLEX</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2025 — ver pliego</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -3303,14 +3315,14 @@
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
-          <t>id-07ddb93a12c5a870</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3318,7 +3330,7 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C40" s="7" t="inlineStr">
+      <c r="C40" s="3" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
@@ -3335,18 +3347,18 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>02/2025</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>Concurso de Precio N° 02/2025</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr"/>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Publicada 19/06/2025 — ver pliego</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
@@ -3372,7 +3384,7 @@
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
-          <t>id-7c1bf02160a66f67</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
@@ -3387,31 +3399,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C41" s="7" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F41" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>05/2025</t>
+        </is>
+      </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>CONSTRUCCIÓN DE OBRAS DE ARTE EN EL DEPARTAMENTO LA PAZ. 1) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE EN R.P. S/Nº SOBRE Aº ESTACAS – “CAMINO SAUCECITO” – TRAMO: R.P.Nº 1 – ESCUELA Nº 62 – DISTRITO ESTACAS – DEPARTAMENTO LA PAZ – 2) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE SOBRE Aº ESTACAS SAN GUSTAVO – TRAMO: […]</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
@@ -3432,19 +3448,19 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
-          <t>id-3d7728874996f284</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3452,31 +3468,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>06/2025</t>
+        </is>
+      </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr"/>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr">
@@ -3497,19 +3517,19 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O42" s="4" t="inlineStr">
         <is>
-          <t>id-654eebef400f89cd</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -3517,35 +3537,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C43" s="7" t="inlineStr">
+      <c r="C43" s="3" t="inlineStr">
         <is>
           <t>Infraestructura</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Concurso</t>
-        </is>
-      </c>
-      <c r="F43" s="4" t="inlineStr">
-        <is>
-          <t>01/26</t>
-        </is>
-      </c>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr"/>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr"/>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr">
@@ -3566,19 +3582,19 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O43" s="4" t="inlineStr">
         <is>
-          <t>id-9a16884dd5a64a49</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -3586,35 +3602,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>2026-1227</t>
+          <t>04/2025</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr"/>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr">
@@ -3635,17 +3651,354 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
+          <t>IAPV — Viviendas</t>
+        </is>
+      </c>
+      <c r="O44" s="4" t="inlineStr">
+        <is>
+          <t>id-34c85bcdb9b1123f</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>IAPV (Vivienda)</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>03/2025</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr"/>
+      <c r="I45" s="4" t="inlineStr">
+        <is>
+          <t>Publicada 08/10/2025 — ver pliego</t>
+        </is>
+      </c>
+      <c r="J45" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K45" s="4" t="inlineStr"/>
+      <c r="L45" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M45" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>IAPV — Viviendas</t>
+        </is>
+      </c>
+      <c r="O45" s="4" t="inlineStr">
+        <is>
+          <t>id-75bfffae63b7eedc</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr"/>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>CONSTRUCCIÓN DE OBRAS DE ARTE EN EL DEPARTAMENTO LA PAZ. 1) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE EN R.P. S/Nº SOBRE Aº ESTACAS – “CAMINO SAUCECITO” – TRAMO: R.P.Nº 1 – ESCUELA Nº 62 – DISTRITO ESTACAS – DEPARTAMENTO LA PAZ – 2) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE SOBRE Aº ESTACAS SAN GUSTAVO – TRAMO: […]</t>
+        </is>
+      </c>
+      <c r="H46" s="4" t="inlineStr"/>
+      <c r="I46" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J46" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K46" s="4" t="inlineStr"/>
+      <c r="L46" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M46" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="O46" s="4" t="inlineStr">
+        <is>
+          <t>id-3d7728874996f284</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>Materiales</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr"/>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr"/>
+      <c r="I47" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J47" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K47" s="4" t="inlineStr"/>
+      <c r="L47" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M47" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="O47" s="4" t="inlineStr">
+        <is>
+          <t>id-654eebef400f89cd</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Concurso</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>01/26</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+        </is>
+      </c>
+      <c r="H48" s="4" t="inlineStr"/>
+      <c r="I48" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J48" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K48" s="4" t="inlineStr"/>
+      <c r="L48" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M48" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="O48" s="4" t="inlineStr">
+        <is>
+          <t>id-9a16884dd5a64a49</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>Materiales</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
           <t>ENERSA</t>
         </is>
       </c>
-      <c r="O44" s="4" t="inlineStr">
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Licitación</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>2026-1227</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="inlineStr"/>
+      <c r="I49" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J49" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K49" s="4" t="inlineStr"/>
+      <c r="L49" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M49" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>ENERSA</t>
+        </is>
+      </c>
+      <c r="O49" s="4" t="inlineStr">
         <is>
           <t>id-0691eb485d7548eb</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O44"/>
+  <autoFilter ref="A1:O49"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -3733,6 +4086,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId84"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId85"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L47" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L48" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L49" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M49" r:id="rId96"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 08/10/2026 08:13
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$51</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O49"/>
+  <dimension ref="A1:O51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -602,7 +602,7 @@
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>COMPLEJO HABITACIONAL SAN AGUSTIN (P.P.) PARANÁ 24 VIVIENDAS, 7 LOCALES COMERCIALES Y 27 ESPACIOS DE ESTACIONAMIENTOS DEPARTAMENTO: PARANÁ</t>
+          <t>COMPLEJO HABITACIONAL SAN AGUSTIN (P.P.) PARANÁ 24 VIVIENDAS, 7 LOCALES COMERCIALES Y 27 ESPACIOS DE ESTACIONAMIENTOS DEPARTAMENTO: PARANÁ Para ná , mi ércoles 7 de octubre de 20</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
@@ -612,7 +612,7 @@
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>DÍA: 01 /12/2026 HORA: 10:30 hs</t>
+          <t>DÍA: 01 /12 /2026 HORA: 10:30 hs</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
@@ -657,9 +657,9 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -674,22 +674,22 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>31/2026</t>
+          <t>32/2026</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>“Pavimento Rígido – 03 (tres) Cuadras Barrio San Felipe”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>"Adquisición de 835 m3 de Hormigón Calidad H25 para 08 cuadras de Pavimento", en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>07 de octubre de 2026 Hora: 10:00</t>
+          <t>08 de octubre de 2026 Hora: 10:00</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -715,7 +715,7 @@
       </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
-          <t>id-76d9566cb30a6df5</t>
+          <t>id-0ace7de8f16d3baf</t>
         </is>
       </c>
     </row>
@@ -730,9 +730,9 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -747,12 +747,12 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>32/2026</t>
+          <t>33/2026</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>"Adquisición de 835 m3 de Hormigón Calidad H25 para 08 cuadras de Pavimento", en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>“Pavimento Rígido – 04 (cuatro) Cuadras Barrio San Roque y 01 (una) Cuadra Barrio Vicente Obrego”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
@@ -762,7 +762,7 @@
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>08 de octubre de 2026 Hora: 10:00</t>
+          <t>08 de octubre de 2026 Hora: 11:00</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -788,14 +788,14 @@
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
-          <t>id-0ace7de8f16d3baf</t>
+          <t>id-fe71ac2aaf71b8d8</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -803,29 +803,29 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>CONCURSO DE PRECIOS</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>33/2026</t>
+          <t>302/2026</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>“Pavimento Rígido – 04 (cuatro) Cuadras Barrio San Roque y 01 (una) Cuadra Barrio Vicente Obrego”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>ADQUISICION DE MAT. PARA LA CONSTRUCCION, ARTICULOS DE FERRETERIA , PINTURERUA Y MAT. ELECTRICOS</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -835,7 +835,7 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>08 de octubre de 2026 Hora: 11:00</t>
+          <t>08-10-2026 08:30</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -856,19 +856,19 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>id-fe71ac2aaf71b8d8</t>
+          <t>id-2d3ee6d70e7e432c</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -876,39 +876,39 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>CONCURSO DE PRECIOS</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>302/2026</t>
+          <t>34/2026</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICION DE MAT. PARA LA CONSTRUCCION, ARTICULOS DE FERRETERIA , PINTURERUA Y MAT. ELECTRICOS</t>
+          <t>“Concesión de la Explotación Comercial de un (01) Camión de Comidas Rápidas (para cubrir el total de cuatro puestos) en la Zona Joven – Parque La Salamanca de la Municipalidad de Concepción del Uruguay – Entre Ríos”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>08-10-2026 08:30</t>
+          <t>09 de octubre de 2026 Hora: 10:00</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -929,12 +929,12 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>id-2d3ee6d70e7e432c</t>
+          <t>id-b147fbd9d3081bfc</t>
         </is>
       </c>
     </row>
@@ -956,7 +956,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -966,12 +966,12 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>34/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>“Concesión de la Explotación Comercial de un (01) Camión de Comidas Rápidas (para cubrir el total de cuatro puestos) en la Zona Joven – Parque La Salamanca de la Municipalidad de Concepción del Uruguay – Entre Ríos”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>“PROVISIÓN DE UNA (1) MINICARGADORA 0 KM, CON CUCHARÓN FRONTAL DE USO GENERAL, UN (1) MARTILLO HIDRÁULICO Y UN (1) COMPACTADOR/RODILLO VIBRATORIO LISO”</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -981,7 +981,7 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>09 de octubre de 2026 Hora: 10:00</t>
+          <t>09/10/2026 HORA: 10:00 HS</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -989,7 +989,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr"/>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>($ 270.000,00) PESOS DOSCIENTOS SETENTA MIL</t>
+        </is>
+      </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1007,14 +1011,14 @@
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>id-b147fbd9d3081bfc</t>
+          <t>id-779e4cd290f2e64e</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1029,7 +1033,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>COLON — MUNICIPALIDAD DE VILLA ELISA (E.R.)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1039,22 +1043,22 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>004/26</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>“PROVISIÓN DE UNA (1) MINICARGADORA 0 KM, CON CUCHARÓN FRONTAL DE USO GENERAL, UN (1) MARTILLO HIDRÁULICO Y UN (1) COMPACTADOR/RODILLO VIBRATORIO LISO”</t>
+          <t>ADQUISICIÓN DE UN (1) VEHÍCULO PARA TRANSPORTE DE PASAJEROS DE (5) CINCO PLAZAS 0 KM - MODELO/AÑO 2026, PARA LA MUNICIPALIDAD DE LA CIUDAD DE VILLA ELISA, ENTRE RÍOS</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>12/11/2026</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>09/10/2026 HORA: 10:00 HS</t>
+          <t>12 de NOVIEMBRE de 2026 a la hora 10:00 en la Oficina de Compras de la Municipalidad de Villa Elisa, Entre Ríos</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -1064,7 +1068,7 @@
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>($ 270.000,00) PESOS DOSCIENTOS SETENTA MIL</t>
+          <t>$ 20.000,00 (Pesos Veint e mil con 00/100) el que se puede adquirir en</t>
         </is>
       </c>
       <c r="L8" s="6" t="inlineStr">
@@ -1084,7 +1088,7 @@
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>id-779e4cd290f2e64e</t>
+          <t>id-bb3703ff360c8c43</t>
         </is>
       </c>
     </row>
@@ -1936,7 +1940,7 @@
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN DE UNA MÁQUINA MOTONIVELADORA PARA INCORPORAR AL PARQUE AUTOMOTOR DE LA MUNICIPALIDAD DE ALDEA SAN ANTONIO</t>
+          <t>ADQUISICIÓN DE UNA MÁQUINA MOTONIVELADORA PARA INCORPORAR AL PARQUE AUTOMOTOR DE LA MUNICIP ALIDAD DE ALDEA SAN ANTONIO</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1956,7 +1960,7 @@
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>PESOS CIEN MIL con 00/ 100 ($ 100.000,00.-)</t>
+          <t>PESOS CIEN MIL con 00/100 ($ 100.000,00. -)</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
@@ -2133,7 +2137,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -2148,7 +2152,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>SALUD ENTRE RÍOS S.A.U</t>
+          <t>INSTITUTO AUTÁRQUICO DE PLANEAMIENTO YY VIVIENDA — URUGUAY</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2156,20 +2160,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr"/>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Contratación de Servicio de Viandas para el Hospital de la Baxada</t>
+          <t>TERMINACIÓN CONCEPCIÓN DEL URUGUAY 63 VIV. ETAPA I 17 VIV. (P. P.) DEPARTAMENTO: URUGUAY PRESUPUESTO OFICIAL Obras de Viviendas y Complem entarias: $ 1.042.925.971,90 y su equivalente UVIs 693.301,14 Obras de Infraestructuras y Nexos $ 344.554.736,26 y su equivalente UVIs 229.048,08</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>17/11/2026</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Hospital de la Baxada, calle Gral. Al varado Nº 2.250 Paraná, Entre Ríos, el día 19/10/2026 a las 10:00 hs</t>
+          <t>DÍA: 17/11/2026 HOR A: 10:00 HS</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2179,7 +2187,7 @@
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>$ 138.748,07</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr">
@@ -2199,14 +2207,14 @@
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-d35d5e849089d7ac</t>
+          <t>id-b0fe9ebcdc39e73a</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2214,14 +2222,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE VILLAGUAY</t>
+          <t>SALUD ENTRE RÍOS S.A.U</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2232,17 +2240,17 @@
       <c r="F24" s="4" t="inlineStr"/>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Provisión de una (1) camioneta usada destinada al Parque Automotor Municipal</t>
+          <t>Contratación de Servicio de Viandas para el Hospital de la Baxada</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>21/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>21 de octubre del año 2026 a las 10:00 Horas, la que se realizara en la Oficina de suministros de la Municipalidad de Vi</t>
+          <t>Hospital de la Baxada, calle Gral. Al varado Nº 2.250 Paraná, Entre Ríos, el día 19/10/2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -2252,7 +2260,7 @@
       </c>
       <c r="K24" s="4" t="inlineStr">
         <is>
-          <t>$10.000,00</t>
+          <t>Ninguno</t>
         </is>
       </c>
       <c r="L24" s="6" t="inlineStr">
@@ -2272,14 +2280,14 @@
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-2d3dded56e6c6f6a</t>
+          <t>id-d35d5e849089d7ac</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -2287,14 +2295,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>PARANA — SALUD ENTRE RÍOS S.A.U</t>
+          <t>VILLAGUAY — MUNICIPALIDAD DE VILLAGUAY</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2305,7 +2313,7 @@
       <c r="F25" s="4" t="inlineStr"/>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>Servicio de Recolección, Lavado, Desinfección, Secado, Planchado y Transporte de Ropa Hospitalaria</t>
+          <t>Provisión de una (1) camioneta usada destinada al Parque Automotor Municipal</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
@@ -2315,7 +2323,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Hospital de la Baxada, calle Gral. Alvarado Nº 2.250 Paraná, Entre Ríos, el día 21/10/2026 a las 10:00 hs</t>
+          <t>21 de octubre del año 2026 a las 10:00 Horas, la que se realizara en la Oficina de suministros de la Municipalidad de Vi</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2325,7 +2333,7 @@
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>$10.000,00</t>
         </is>
       </c>
       <c r="L25" s="6" t="inlineStr">
@@ -2345,7 +2353,7 @@
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-6b955df9d3f6241a</t>
+          <t>id-2d3dded56e6c6f6a</t>
         </is>
       </c>
     </row>
@@ -2360,14 +2368,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C26" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>PARANA — SALUD ENTRE RÍOS S.A.U</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2375,24 +2383,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>11/26</t>
-        </is>
-      </c>
+      <c r="F26" s="4" t="inlineStr"/>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “TERMINACION ESCUELA Nº 40 “JOSÉ ENRIQUE RODÓ”-SEPTIMO DISTRITO-DEPARTAMENTO GUALEGUAY.”</t>
+          <t>Servicio de Recolección, Lavado, Desinfección, Secado, Planchado y Transporte de Ropa Hospitalaria</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>23/10/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 23 de Octubre de 2026 a las 10:00 hs</t>
+          <t>Hospital de la Baxada, calle Gral. Alvarado Nº 2.250 Paraná, Entre Ríos, el día 21/10/2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2402,7 +2406,7 @@
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>$ 100 (Cien)</t>
+          <t>Ninguno</t>
         </is>
       </c>
       <c r="L26" s="6" t="inlineStr">
@@ -2422,14 +2426,14 @@
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-86cc9c230734c462</t>
+          <t>id-6b955df9d3f6241a</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -2444,7 +2448,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2454,12 +2458,12 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>11/2026</t>
+          <t>11/26</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>Terminación Escuela N° 40 "José Enrique Rodó", Séptimo Distrito</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “TERMINACION ESCUELA Nº 40 “JOSÉ ENRIQUE RODÓ”-SEPTIMO DISTRITO-DEPARTAMENTO GUALEGUAY.”</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
@@ -2469,7 +2473,7 @@
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>viernes, 23 de octubre de 2026 - 10:00hs</t>
+          <t>DE LAS OFERTAS: el día 23 de Octubre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2477,7 +2481,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K27" s="4" t="inlineStr"/>
+      <c r="K27" s="4" t="inlineStr">
+        <is>
+          <t>$ 100 (Cien)</t>
+        </is>
+      </c>
       <c r="L27" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2490,12 +2498,12 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-322a40f5e43af35d</t>
+          <t>id-86cc9c230734c462</t>
         </is>
       </c>
     </row>
@@ -2510,14 +2518,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C28" s="9" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>COMUNA DE EL PALENQUE</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2527,22 +2535,22 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>06/26</t>
+          <t>11/2026</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de UNA (1) PALA CARGADORA 0 KM destinada a trabajos en la Comuna</t>
+          <t>Terminación Escuela N° 40 "José Enrique Rodó", Séptimo Distrito</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>26/10/2026</t>
+          <t>23/10/2026</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>26/10/2026, 12:30 horas, Lugar: Sede Administrativa de la Comuna de El Palenque, sito en calle San Martín sin número, El</t>
+          <t>viernes, 23 de octubre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2550,11 +2558,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K28" s="4" t="inlineStr">
-        <is>
-          <t>pesos cero ($0,00)</t>
-        </is>
-      </c>
+      <c r="K28" s="4" t="inlineStr"/>
       <c r="L28" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2567,12 +2571,12 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-4b7dfe1bdd0c2ac6</t>
+          <t>id-322a40f5e43af35d</t>
         </is>
       </c>
     </row>
@@ -2582,19 +2586,19 @@
           <t>03/10/2026</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>DIAMANTE — MUNICIPALIDAD DE DIAMANTE -- ENTRE RÍOS</t>
+          <t>COMUNA DE EL PALENQUE</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2602,16 +2606,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr"/>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>06/26</t>
+        </is>
+      </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Solicitar Contratación de una empresa para la Obra de “22 (veintidós) cuadras de pavimento urbano” – Grupo 1- según Expte. Letra “D” Nº 2196</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr"/>
+          <t>Adquisición de UNA (1) PALA CARGADORA 0 KM destinada a trabajos en la Comuna</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>26/10/2026</t>
+        </is>
+      </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>viernes 23 de octubre de 2.026, a la hora diez (10.00)</t>
+          <t>26/10/2026, 12:30 horas, Lugar: Sede Administrativa de la Comuna de El Palenque, sito en calle San Martín sin número, El</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2619,7 +2631,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K29" s="4" t="inlineStr"/>
+      <c r="K29" s="4" t="inlineStr">
+        <is>
+          <t>pesos cero ($0,00)</t>
+        </is>
+      </c>
       <c r="L29" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2637,29 +2653,29 @@
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-4f207bef5c709ad6</t>
+          <t>id-4b7dfe1bdd0c2ac6</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C30" s="10" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+          <t>08/10/2026</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
+          <t>COMUNA DE EL PALENQUE</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2669,18 +2685,22 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>07/2026</t>
+          <t>07/26</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>Transporte de mil doscientos cincuenta metros cúbicos (1.250 m³) de broza grillada desde Cantera “Tayreta” (Ruta Nacional N ° 14 km 135) hasta jurisdicción de la comuna, de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
-        </is>
-      </c>
-      <c r="H30" s="4" t="inlineStr"/>
+          <t>Adquisición de UN (1) TRACTOR AGRÍCOLA 0 KM DE HASTA 9 0 HP, CABINADO 4 x4, CON PALA FRONTAL destinado a trabajos en la Comuna</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>28/10/2026</t>
+        </is>
+      </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Viernes 09 de octubre del corriente año a las 10:00 hs en la Oficina de la Sede de la Comuna</t>
+          <t>28/10/2026, 12:40 horas, Lugar: Sede Administrativa de la Comuna de El Palenque, sito en calle San Martín sin número, El</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2688,7 +2708,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K30" s="4" t="inlineStr"/>
+      <c r="K30" s="4" t="inlineStr">
+        <is>
+          <t>pesos cero ($ 0,00)</t>
+        </is>
+      </c>
       <c r="L30" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2706,14 +2730,14 @@
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-24e9015ecceeff7f</t>
+          <t>id-54e2b94544e5c76f</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2721,31 +2745,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>CONCORDIA — APEX S.A.S</t>
+          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Licitación</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>07/2026</t>
+        </is>
+      </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>instalaciones eléctricas, sanitarias, hidráulicas, mecánicas o de cualquier otra naturaleza relacionada con el sector</t>
+          <t>Transporte de mil doscientos cincuenta metros cúbicos (1.250 m³) de broza grillada desde Cantera “Tayreta” (Ruta Nacional N° 14 km 135) hasta jurisdicción de la comuna, de acuerdo a los Pliegos de Bases, Condiciones Part iculares y demás documentación</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Viernes 09 de octubre del corriente año a las 10:00 hs en la Oficina de la Sede de la Comuna</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2771,14 +2799,14 @@
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-a20c6b2b6fcf36a2</t>
+          <t>id-24e9015ecceeff7f</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2786,31 +2814,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C32" s="9" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Boletín Oficial</t>
+          <t>DIAMANTE — MUNICIPALIDAD DE DIAMANTE -- ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Remate</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr"/>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>los vehículos se encuentran en exhibición por lo cuál la información registral, de rentas y de infracciones puede ser</t>
+          <t>Solicitar Contratación de una empresa para la Obra de “22 (veintidós) cuadras de pavimento urbano” – Grupo 1- según Expte. Letra “D” Nº 2196</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>viernes 23 de octubre de 2.026, a la hora diez (10.00)</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2836,14 +2864,14 @@
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-fb8d7dc09e202fea</t>
+          <t>id-4f207bef5c709ad6</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2851,35 +2879,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C33" s="9" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
+          <t>CONCORDIA — APEX S.A.S</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>001/26</t>
-        </is>
-      </c>
+          <t>Licitación</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr"/>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN de UN (1) FURGON UTILITARIO CHICO con 5 asientos 0 KM. con destino a Subsecretaria de Asistencia Directa y Emergencia</t>
+          <t>instalaciones eléctricas, sanitarias, hidráulicas, mecánicas o de cualquier otra naturaleza relacionada con el sector</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>DE LAS PROPUESTAS: 20 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2905,14 +2929,14 @@
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-ca205f0874380f69</t>
+          <t>id-a20c6b2b6fcf36a2</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2920,25 +2944,25 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>INSTITUTO CARBÓ S.R.L</t>
+          <t>Boletín Oficial</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Remate</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr"/>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>sin internación en materia de salud, pre- hospitalarias, atención médica, domiciliaria y traslados sanitarios de alta</t>
+          <t>los vehículos se encuentran en exhibición por lo cuál la información registral, de rentas y de infracciones puede ser</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
@@ -2970,7 +2994,7 @@
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-6aa57c7437a30ca3</t>
+          <t>id-fb8d7dc09e202fea</t>
         </is>
       </c>
     </row>
@@ -2985,14 +3009,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE VIALE</t>
+          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3002,18 +3026,18 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>08/26</t>
+          <t>001/26</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>de asf alto 70-16 destinado a la producción de pavimento de la Planta Asfáltica, y que a continuación se detalla y</t>
+          <t>ADQUISICIÓN de UN (1) FURGON UTILITARIO CHICO con 5 asientos 0 KM. con destino a Subsecretaria de Asistencia Directa y Emergencia</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>DE LAS PROPUESTAS: 20 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3039,14 +3063,14 @@
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-ef1ddb923c7e7fdb</t>
+          <t>id-ca205f0874380f69</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3061,28 +3085,24 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>INSTITUTO CARBÓ S.R.L</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>04/2026</t>
-        </is>
-      </c>
+          <t>Licitación</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr"/>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN CONCEPCIÓN DEL URUGUAY 63 VIV</t>
+          <t>sin internación en materia de salud, pre- hospitalarias, atención médica, domiciliaria y traslados sanitarios de alta</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2026 — ver pliego</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3103,19 +3123,19 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>id-1a3c1f8e036ac91e</t>
+          <t>id-6aa57c7437a30ca3</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3130,7 +3150,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>MUNICIPALIDAD DE VIALE</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3140,18 +3160,18 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>05/2026</t>
+          <t>08/26</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>COMPLEJO HABITACIONAL SAN AGUSTÍN (P</t>
+          <t>de asf alto 70-16 destinado a la producción de pavimento de la Planta Asfáltica, y que a continuación se detalla y</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/10/2026 — ver pliego</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3172,19 +3192,19 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>id-ccb22bcad9356438</t>
+          <t>id-ef1ddb923c7e7fdb</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -3209,18 +3229,18 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>03/26</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+          <t>TERMINACIÓN CONCEPCIÓN DEL URUGUAY 63 VIV</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>Publicada 06/10/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -3246,14 +3266,14 @@
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-1a3c1f8e036ac91e</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3278,18 +3298,18 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>02/2026</t>
+          <t>05/2026</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+          <t>COMPLEJO HABITACIONAL SAN AGUSTÍN (P</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>Publicada 05/10/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -3315,7 +3335,7 @@
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-ccb22bcad9356438</t>
         </is>
       </c>
     </row>
@@ -3347,18 +3367,18 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>03/26</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr"/>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
@@ -3384,7 +3404,7 @@
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
@@ -3416,18 +3436,18 @@
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>05/2025</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
@@ -3453,7 +3473,7 @@
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
@@ -3485,18 +3505,18 @@
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>06/2025</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr"/>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr">
@@ -3522,7 +3542,7 @@
       </c>
       <c r="O42" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
@@ -3552,16 +3572,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F43" s="4" t="inlineStr"/>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>05/2025</t>
+        </is>
+      </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr"/>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr">
@@ -3587,7 +3611,7 @@
       </c>
       <c r="O43" s="4" t="inlineStr">
         <is>
-          <t>id-ebeeb6a87e688d85</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
@@ -3619,18 +3643,18 @@
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>04/2025</t>
+          <t>06/2025</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr"/>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr">
@@ -3656,7 +3680,7 @@
       </c>
       <c r="O44" s="4" t="inlineStr">
         <is>
-          <t>id-34c85bcdb9b1123f</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
@@ -3686,20 +3710,16 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F45" s="4" t="inlineStr">
-        <is>
-          <t>03/2025</t>
-        </is>
-      </c>
+      <c r="F45" s="4" t="inlineStr"/>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr"/>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J45" s="4" t="inlineStr">
@@ -3725,7 +3745,7 @@
       </c>
       <c r="O45" s="4" t="inlineStr">
         <is>
-          <t>id-75bfffae63b7eedc</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
@@ -3747,24 +3767,28 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>04/2025</t>
+        </is>
+      </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>CONSTRUCCIÓN DE OBRAS DE ARTE EN EL DEPARTAMENTO LA PAZ. 1) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE EN R.P. S/Nº SOBRE Aº ESTACAS – “CAMINO SAUCECITO” – TRAMO: R.P.Nº 1 – ESCUELA Nº 62 – DISTRITO ESTACAS – DEPARTAMENTO LA PAZ – 2) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE SOBRE Aº ESTACAS SAN GUSTAVO – TRAMO: […]</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H46" s="4" t="inlineStr"/>
       <c r="I46" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J46" s="4" t="inlineStr">
@@ -3785,19 +3809,19 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O46" s="4" t="inlineStr">
         <is>
-          <t>id-3d7728874996f284</t>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3805,31 +3829,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C47" s="7" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>03/2025</t>
+        </is>
+      </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
         </is>
       </c>
       <c r="H47" s="4" t="inlineStr"/>
       <c r="I47" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J47" s="4" t="inlineStr">
@@ -3850,19 +3878,19 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O47" s="4" t="inlineStr">
         <is>
-          <t>id-654eebef400f89cd</t>
+          <t>id-75bfffae63b7eedc</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -3882,17 +3910,13 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Concurso</t>
-        </is>
-      </c>
-      <c r="F48" s="4" t="inlineStr">
-        <is>
-          <t>01/26</t>
-        </is>
-      </c>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr"/>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>CONSTRUCCIÓN DE OBRAS DE ARTE EN EL DEPARTAMENTO LA PAZ. 1) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE EN R.P. S/Nº SOBRE Aº ESTACAS – “CAMINO SAUCECITO” – TRAMO: R.P.Nº 1 – ESCUELA Nº 62 – DISTRITO ESTACAS – DEPARTAMENTO LA PAZ – 2) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE SOBRE Aº ESTACAS SAN GUSTAVO – TRAMO: […]</t>
         </is>
       </c>
       <c r="H48" s="4" t="inlineStr"/>
@@ -3924,7 +3948,7 @@
       </c>
       <c r="O48" s="4" t="inlineStr">
         <is>
-          <t>id-9a16884dd5a64a49</t>
+          <t>id-3d7728874996f284</t>
         </is>
       </c>
     </row>
@@ -3946,22 +3970,18 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Licitación</t>
-        </is>
-      </c>
-      <c r="F49" s="4" t="inlineStr">
-        <is>
-          <t>2026-1227</t>
-        </is>
-      </c>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr"/>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
         </is>
       </c>
       <c r="H49" s="4" t="inlineStr"/>
@@ -3988,17 +4008,155 @@
       </c>
       <c r="N49" t="inlineStr">
         <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="O49" s="4" t="inlineStr">
+        <is>
+          <t>id-654eebef400f89cd</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Concurso</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>01/26</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+        </is>
+      </c>
+      <c r="H50" s="4" t="inlineStr"/>
+      <c r="I50" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J50" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K50" s="4" t="inlineStr"/>
+      <c r="L50" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M50" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="O50" s="4" t="inlineStr">
+        <is>
+          <t>id-9a16884dd5a64a49</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>Materiales</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
           <t>ENERSA</t>
         </is>
       </c>
-      <c r="O49" s="4" t="inlineStr">
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Licitación</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>2026-1227</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="inlineStr"/>
+      <c r="I51" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J51" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K51" s="4" t="inlineStr"/>
+      <c r="L51" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M51" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>ENERSA</t>
+        </is>
+      </c>
+      <c r="O51" s="4" t="inlineStr">
         <is>
           <t>id-0691eb485d7548eb</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O49"/>
+  <autoFilter ref="A1:O51"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -4096,6 +4254,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId94"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L49" r:id="rId95"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M49" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L50" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M50" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L51" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M51" r:id="rId100"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 09/10/2026 08:22
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$49</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -62,17 +62,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E6D9F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E6D9F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O51"/>
+  <dimension ref="A1:O49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -649,7 +649,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -659,27 +659,27 @@
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>Materiales</t>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>CONCURSO DE PRECIOS</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>32/2026</t>
+          <t>302/2026</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>"Adquisición de 835 m3 de Hormigón Calidad H25 para 08 cuadras de Pavimento", en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>ADQUISICION DE MAT. PARA LA CONSTRUCCION, ARTICULOS DE FERRETERIA , PINTURERUA Y MAT. ELECTRICOS</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
@@ -689,7 +689,7 @@
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>08 de octubre de 2026 Hora: 10:00</t>
+          <t>08-10-2026 08:30</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -710,12 +710,12 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
-          <t>id-0ace7de8f16d3baf</t>
+          <t>id-2d3ee6d70e7e432c</t>
         </is>
       </c>
     </row>
@@ -730,14 +730,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
+          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -747,22 +747,22 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>33/2026</t>
+          <t>34/2026</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>“Pavimento Rígido – 04 (cuatro) Cuadras Barrio San Roque y 01 (una) Cuadra Barrio Vicente Obrego”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>“Concesión de la Explotación Comercial de un (01) Camión de Comidas Rápidas (para cubrir el total de cuatro puestos) en la Zona Joven – Parque La Salamanca de la Municipalidad de Concepción del Uruguay – Entre Ríos”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>08 de octubre de 2026 Hora: 11:00</t>
+          <t>09 de octubre de 2026 Hora: 10:00</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -788,14 +788,14 @@
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
-          <t>id-fe71ac2aaf71b8d8</t>
+          <t>id-b147fbd9d3081bfc</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -805,37 +805,37 @@
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>CONCURSO DE PRECIOS</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>302/2026</t>
+          <t>10/2026</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICION DE MAT. PARA LA CONSTRUCCION, ARTICULOS DE FERRETERIA , PINTURERUA Y MAT. ELECTRICOS</t>
+          <t>“PROVISIÓN DE UNA (1) MINICARGADORA 0 KM, CON CUCHARÓN FRONTAL DE USO GENERAL, UN (1) MARTILLO HIDRÁULICO Y UN (1) COMPACTADOR/RODILLO VIBRATORIO LISO”</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>09/10/2026</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>08-10-2026 08:30</t>
+          <t>09/10/2026 HORA: 10:00 HS</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -843,7 +843,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr"/>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>($ 270.000,00) PESOS DOSCIENTOS SETENTA MIL</t>
+        </is>
+      </c>
       <c r="L5" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -856,19 +860,19 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>id-2d3ee6d70e7e432c</t>
+          <t>id-779e4cd290f2e64e</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -876,14 +880,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>Vehículos</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
+          <t>COLON — MUNICIPALIDAD DE VILLA ELISA (E.R.)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -893,22 +897,22 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>34/2026</t>
+          <t>004/26</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>“Concesión de la Explotación Comercial de un (01) Camión de Comidas Rápidas (para cubrir el total de cuatro puestos) en la Zona Joven – Parque La Salamanca de la Municipalidad de Concepción del Uruguay – Entre Ríos”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>ADQUISICIÓN DE UN (1) VEHÍCULO PARA TRANSPORTE DE PASAJEROS DE (5) CINCO PLAZAS 0 KM - MODELO/AÑO 2026, PARA LA MUNICIPALIDAD DE LA CIUDAD DE VILLA ELISA, ENTRE RÍOS</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>12/11/2026</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>09 de octubre de 2026 Hora: 10:00</t>
+          <t>12 de NOVIEMBRE de 2026 a la hora 10:00 en la Oficina de Compras de la Municipalidad de Villa Elisa, Entre Ríos</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -916,7 +920,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr"/>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>$ 20.000,00 (Pesos Veint e mil con 00/100) el que se puede adquirir en</t>
+        </is>
+      </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -934,7 +942,7 @@
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>id-b147fbd9d3081bfc</t>
+          <t>id-bb3703ff360c8c43</t>
         </is>
       </c>
     </row>
@@ -949,14 +957,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -966,22 +974,22 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>11/2026</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>“PROVISIÓN DE UNA (1) MINICARGADORA 0 KM, CON CUCHARÓN FRONTAL DE USO GENERAL, UN (1) MARTILLO HIDRÁULICO Y UN (1) COMPACTADOR/RODILLO VIBRATORIO LISO”</t>
+          <t>OBRA "PAVIMENTACION URBANA CALLE TRATADO DEL PILAR B° 3 DE FEBRERO - MUNICIPALIDAD DE SANTA ELENA" (Según Pliegos de Bases y condi ciones)</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>09/10/2026 HORA: 10:00 HS</t>
+          <t>13/10/2026 HORA: 10: 00 HS</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -991,7 +999,7 @@
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>($ 270.000,00) PESOS DOSCIENTOS SETENTA MIL</t>
+          <t>$ 728.000,00 PESOS SETECIENTOS VEINTIOCHO MIL</t>
         </is>
       </c>
       <c r="L7" s="6" t="inlineStr">
@@ -1011,14 +1019,14 @@
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>id-779e4cd290f2e64e</t>
+          <t>id-1a2561509308b1b6</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1026,14 +1034,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>COLON — MUNICIPALIDAD DE VILLA ELISA (E.R.)</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1043,34 +1051,30 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>004/26</t>
+          <t>11/2026</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN DE UN (1) VEHÍCULO PARA TRANSPORTE DE PASAJEROS DE (5) CINCO PLAZAS 0 KM - MODELO/AÑO 2026, PARA LA MUNICIPALIDAD DE LA CIUDAD DE VILLA ELISA, ENTRE RÍOS</t>
+          <t>REFACCION EN ESCUELA N° 65 “ALMIRANTE BROWN” – CIUDAD DE CONCORDIA - DEPARTAMENTO CONCORDIA - PROVINCIA DE ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>12/11/2026</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>12 de NOVIEMBRE de 2026 a la hora 10:00 en la Oficina de Compras de la Municipalidad de Villa Elisa, Entre Ríos</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 09:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K8" s="4" t="inlineStr">
-        <is>
-          <t>$ 20.000,00 (Pesos Veint e mil con 00/100) el que se puede adquirir en</t>
-        </is>
-      </c>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr"/>
       <c r="L8" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1088,7 +1092,7 @@
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>id-bb3703ff360c8c43</t>
+          <t>id-fc30d5c0b0589a79</t>
         </is>
       </c>
     </row>
@@ -1103,14 +1107,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1120,12 +1124,12 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>11/2026</t>
+          <t>13/2026</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>OBRA "PAVIMENTACION URBANA CALLE TRATADO DEL PILAR B° 3 DE FEBRERO - MUNICIPALIDAD DE SANTA ELENA" (Según Pliegos de Bases y condi ciones)</t>
+          <t>REPARACIONES VARIAS EN C. P. E. F. Nº 3 “PROFESOR HUGO LA NASA” – CIUDAD DE CONCEPCION DEL URUGUAY - DEPARTAMENTO URUGUAY - PROVINCIA D E ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -1135,19 +1139,15 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026 HORA: 10: 00 HS</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>$ 728.000,00 PESOS SETECIENTOS VEINTIOCHO MIL</t>
-        </is>
-      </c>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr"/>
       <c r="L9" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1165,7 +1165,7 @@
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>id-1a2561509308b1b6</t>
+          <t>id-9d3847fb0e2b0929</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1180,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
@@ -1197,12 +1197,12 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>11/2026</t>
+          <t>12/2026</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>REFACCION EN ESCUELA N° 65 “ALMIRANTE BROWN” – CIUDAD DE CONCORDIA - DEPARTAMENTO CONCORDIA - PROVINCIA DE ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>RECAMBIO DE CUBIERTA Y REPARACIONES VARIAS EN ESCUELA Nº 92 “CONGRESO DE TUCUMAN” – CONCEPCION DEL URUGUAY - DPTO. URUGUAY – PROVINCIA DE ENTRE RIOS de acuerdo a las c ondiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -1212,7 +1212,7 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 09:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 10:30 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>id-fc30d5c0b0589a79</t>
+          <t>id-059239b424b9c936</t>
         </is>
       </c>
     </row>
@@ -1253,14 +1253,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1270,12 +1270,12 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>13/2026</t>
+          <t>87/2026</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>REPARACIONES VARIAS EN C. P. E. F. Nº 3 “PROFESOR HUGO LA NASA” – CIUDAD DE CONCEPCION DEL URUGUAY - DEPARTAMENTO URUGUAY - PROVINCIA D E ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>Contratar la ejecución de la obra denominada “Construcción de Red Cloacal Subsidiaria del Colector Noroeste Barrio Ciudad Paisaje”</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1285,15 +1285,19 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
+          <t>martes, 13 de octubre de 2026 a las 10:00</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
-        </is>
-      </c>
-      <c r="K11" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>$ 10.000 (pesos diez mil)</t>
+        </is>
+      </c>
       <c r="L11" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1306,12 +1310,12 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Boletín Oficial Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>id-9d3847fb0e2b0929</t>
+          <t>id-ceeb594e8bcc4ff7</t>
         </is>
       </c>
     </row>
@@ -1326,14 +1330,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
+          <t>COLON — MUNICIPALIDAD DE COLON</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1341,32 +1345,32 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>12/2026</t>
-        </is>
-      </c>
+      <c r="F12" s="4" t="inlineStr"/>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>RECAMBIO DE CUBIERTA Y REPARACIONES VARIAS EN ESCUELA Nº 92 “CONGRESO DE TUCUMAN” – CONCEPCION DEL URUGUAY - DPTO. URUGUAY – PROVINCIA DE ENTRE RIOS de acuerdo a las c ondiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>“ADQUISICIÓN DE MATERIALES ELÉCTRICOS PARA EJECUCIÓN DEL PROYECTO DE RECONVERSIÓN Y OPTIMIZACIÓN DEL ALUMBRADO PÚBLICO DE LA CIUDAD DE COLÓN”</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026</t>
+          <t>14/10/2026</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 10:30 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
+          <t>14 de OCTUBRE de 2026</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
-        </is>
-      </c>
-      <c r="K12" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>Sin Cargo</t>
+        </is>
+      </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1384,7 +1388,7 @@
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>id-059239b424b9c936</t>
+          <t>id-9e122d52de12ffef</t>
         </is>
       </c>
     </row>
@@ -1399,14 +1403,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>DIAMANTE — COMUNA ALDEA PROTESTANTE -- DIAMANTE -- ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1416,22 +1420,22 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>87/2026</t>
+          <t>03/2026</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Contratar la ejecución de la obra denominada “Construcción de Red Cloacal Subsidiaria del Colector Noroeste Barrio Ciudad Paisaje”</t>
+          <t>Conforme a lo autorizado por decreto Nº 290/26 llámese a licitación pública Nº 03/26 con el objeto de comprar 10 toneladas de emulsión catiónica súper estable (asfalto de imprimación), puesto en Aldea Protestante</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026</t>
+          <t>14/10/2026</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>martes, 13 de octubre de 2026 a las 10:00</t>
+          <t>miércoles 14 de octubre de 2026 – Hora nueve (09:00) Lugar de presentación de la oferta: Sede Comuna Aldea Protestan</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -1439,11 +1443,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K13" s="4" t="inlineStr">
-        <is>
-          <t>$ 10.000 (pesos diez mil)</t>
-        </is>
-      </c>
+      <c r="K13" s="4" t="inlineStr"/>
       <c r="L13" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1456,12 +1456,12 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Boletín Oficial Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>id-ceeb594e8bcc4ff7</t>
+          <t>id-c2f3a25cfb37fd38</t>
         </is>
       </c>
     </row>
@@ -1476,14 +1476,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>COLON — MUNICIPALIDAD DE COLON</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1491,10 +1491,14 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr"/>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>017/2026</t>
+        </is>
+      </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN DE MATERIALES ELÉCTRICOS PARA EJECUCIÓN DEL PROYECTO DE RECONVERSIÓN Y OPTIMIZACIÓN DEL ALUMBRADO PÚBLICO DE LA CIUDAD DE COLÓN”</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de UNA (1) MOTONIVELADORA, nueva, sin uso, cero km, con una potencia entre 220/240 HP, con opción a implementos, que será utilizada para el área del corralón municipal</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -1504,7 +1508,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>14 de OCTUBRE de 2026</t>
+          <t>14 DE OCTUBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1514,7 +1518,7 @@
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
-          <t>Sin Cargo</t>
+          <t>$100.000,00. - (PESOS CIEN MIL CON 00/100) PRESUPUESTO OFICIAL ESTIMAD</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr">
@@ -1534,7 +1538,7 @@
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>id-9e122d52de12ffef</t>
+          <t>id-4c3b33859e596759</t>
         </is>
       </c>
     </row>
@@ -1549,14 +1553,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>DIAMANTE — COMUNA ALDEA PROTESTANTE -- DIAMANTE -- ENTRE RÍOS</t>
+          <t>VICTORIA — MUNICIPALIDAD DE VICTORIA</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1566,12 +1570,12 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>03/2026</t>
+          <t>008/2026</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Conforme a lo autorizado por decreto Nº 290/26 llámese a licitación pública Nº 03/26 con el objeto de comprar 10 toneladas de emulsión catiónica súper estable (asfalto de imprimación), puesto en Aldea Protestante</t>
+          <t>Proveer a la Municipalidad de Victoria, Entre Ríos, de Veinticinco Mil (25.000) litros de Diésel 500, para movilidad de vehículos y maquinarias viales , Ocho Mil (8.000) litros de Gasoil Tipo euro o similar y Ocho (8.000) litros de nafta súper para vehículos y áreas afectadas a la Secretaria de Planeamiento y Dirección de Ambiente y Desarrollo sostenible;</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
@@ -1581,7 +1585,7 @@
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>miércoles 14 de octubre de 2026 – Hora nueve (09:00) Lugar de presentación de la oferta: Sede Comuna Aldea Protestan</t>
+          <t>14 de octubre de 2026 a las 09:00 hs., en la Oficina de Compras de la Municipalidad de Victoria, Entr</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1607,14 +1611,14 @@
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>id-c2f3a25cfb37fd38</t>
+          <t>id-a9af9f59c8c487c8</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1622,29 +1626,29 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>Vehículos</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>LICITACIÓN PÚBLICA</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>017/2026</t>
+          <t>89/2026</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de UNA (1) MOTONIVELADORA, nueva, sin uso, cero km, con una potencia entre 220/240 HP, con opción a implementos, que será utilizada para el área del corralón municipal</t>
+          <t>ADQUISICION DE BALANZA BASCULA PARA PESAJE DE EJESDE CAMIONES</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
@@ -1654,7 +1658,7 @@
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>14 DE OCTUBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>14-10-2026 08:00</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -1662,11 +1666,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K16" s="4" t="inlineStr">
-        <is>
-          <t>$100.000,00. - (PESOS CIEN MIL CON 00/100) PRESUPUESTO OFICIAL ESTIMAD</t>
-        </is>
-      </c>
+      <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1679,19 +1679,19 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>id-4c3b33859e596759</t>
+          <t>id-4ee814ba6420f0cc</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1699,14 +1699,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>Vehículos</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>VICTORIA — MUNICIPALIDAD DE VICTORIA</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1716,12 +1716,12 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>008/2026</t>
+          <t>89/2026</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Proveer a la Municipalidad de Victoria, Entre Ríos, de Veinticinco Mil (25.000) litros de Diésel 500, para movilidad de vehículos y maquinarias viales , Ocho Mil (8.000) litros de Gasoil Tipo euro o similar y Ocho (8.000) litros de nafta súper para vehículos y áreas afectadas a la Secretaria de Planeamiento y Dirección de Ambiente y Desarrollo sostenible;</t>
+          <t>Adquisición de balanzas básculas para pesaje de ejes de camiones</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>14 de octubre de 2026 a las 09:00 hs., en la Oficina de Compras de la Municipalidad de Victoria, Entr</t>
+          <t>miércoles, 14 de octubre de 2026 a las 08:00</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1752,12 +1752,12 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Boletín Oficial Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>id-a9af9f59c8c487c8</t>
+          <t>id-d963348e34fcb0d3</t>
         </is>
       </c>
     </row>
@@ -1772,39 +1772,39 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>Vehículos</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE ALDEA SAN ANTONIO</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>89/2026</t>
+          <t>002/2026</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICION DE BALANZA BASCULA PARA PESAJE DE EJESDE CAMIONES</t>
+          <t>ADQUISICIÓN DE UNA MÁQUINA MOTONIVELADORA PARA INCORPORAR AL PARQUE AUTOMOTOR DE LA MUNICIP ALIDAD DE ALDEA SAN ANTONIO</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>14/10/2026</t>
+          <t>15/10/2026</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>14-10-2026 08:00</t>
+          <t>15 de octubre de 2026, a las 08:00 horas, en el Edificio Municipal</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1812,7 +1812,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K18" s="4" t="inlineStr"/>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t>PESOS CIEN MIL con 00/100 ($ 100.000,00. -)</t>
+        </is>
+      </c>
       <c r="L18" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1825,19 +1829,19 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>id-4ee814ba6420f0cc</t>
+          <t>id-95a507b67b7b1450</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1847,12 +1851,12 @@
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>Vehículos</t>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>MINISTERIO DE SALUD — GOBIERNO DE ENTRE RIOS</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1862,22 +1866,22 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>89/2026</t>
+          <t>18/26</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de balanzas básculas para pesaje de ejes de camiones</t>
+          <t>Adquirir Sesenta Mil (60.000) Kilogramos de Leche Entera en Polvo Instantánea, Fortificada con Hierro, Zinc y Ácido Ascórbico</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>14/10/2026</t>
+          <t>16/10/2026</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 14 de octubre de 2026 a las 08:00</t>
+          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1885,7 +1889,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K19" s="4" t="inlineStr"/>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>PESOS TRES MIL QUINIENTOS ($ 3.500,00)</t>
+        </is>
+      </c>
       <c r="L19" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1898,19 +1906,19 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Boletín Oficial Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>id-d963348e34fcb0d3</t>
+          <t>id-04a917d50ccab2e3</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1918,14 +1926,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE ALDEA SAN ANTONIO</t>
+          <t>VILLAGUAY — MUNICIPALIDAD DE VILLAGUAY</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1933,24 +1941,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>002/2026</t>
-        </is>
-      </c>
+      <c r="F20" s="4" t="inlineStr"/>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN DE UNA MÁQUINA MOTONIVELADORA PARA INCORPORAR AL PARQUE AUTOMOTOR DE LA MUNICIP ALIDAD DE ALDEA SAN ANTONIO</t>
+          <t>Contratación, ejecución, liquidación, pago y recepción de la obra destinada a la elaboración del Proyecto Ejecutivo, provisión de materiales, mano de obra, equipos, ejecución, ensayos, habilitación y puesta en servicio de la instalación de gas natural para la Planta Municipal de Elaboración de Mezcla Asfáltica en Caliente, ubicada en el Lote N.º 4 de la Chacra N.º 263 del Parque Industrial de Villaguay, Provincia de Entre Ríos. La contratación comprender á una solución integral bajo modalidad “llave en mano”, incluyendo todos los trabajos, provisiones, trámites, representaciones técnicas, insp</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>15/10/2026</t>
+          <t>16/10/2026</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>15 de octubre de 2026, a las 08:00 horas, en el Edificio Municipal</t>
+          <t>16 de octubre del año 2026 a las 10:00 Horas, la que se reali zara en la Oficina de suministros de la Municipalidad de V</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1960,7 +1964,7 @@
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>PESOS CIEN MIL con 00/100 ($ 100.000,00. -)</t>
+          <t>$ 50.000,00</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
@@ -1980,14 +1984,14 @@
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>id-95a507b67b7b1450</t>
+          <t>id-55f1e5ca423a9262</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1995,14 +1999,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>MINISTERIO DE SALUD — GOBIERNO DE ENTRE RIOS</t>
+          <t>INSTITUTO AUTÁRQUICO DE PLANEAMIENTO YY VIVIENDA — URUGUAY</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2012,22 +2016,22 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>18/26</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Adquirir Sesenta Mil (60.000) Kilogramos de Leche Entera en Polvo Instantánea, Fortificada con Hierro, Zinc y Ácido Ascórbico</t>
+          <t>TERMINACIÓN CONCEPCIÓN DEL URUGUAY 63 VIV. ETAPA I 17 VIV. (P. P.) DEPARTAMENTO: URUGUAY PRESUPUESTO OFICIAL Obras de Viviendas y Complem entarias: $ 1.042.925.971,90 y su equivalente UVIs 693.301,14 Obras de Infraestructuras y Nexos $ 344.554.736,26 y su equivalente UVIs 229.048,08</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>16/10/2026</t>
+          <t>17/11/2026</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
+          <t>DÍA: 17/11/2026 HOR A: 10:00 HS</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -2037,7 +2041,7 @@
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>PESOS TRES MIL QUINIENTOS ($ 3.500,00)</t>
+          <t>$ 138.748,07</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr">
@@ -2057,7 +2061,7 @@
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-04a917d50ccab2e3</t>
+          <t>id-b0fe9ebcdc39e73a</t>
         </is>
       </c>
     </row>
@@ -2079,7 +2083,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>VILLAGUAY — MUNICIPALIDAD DE VILLAGUAY</t>
+          <t>SALUD ENTRE RÍOS S.A.U</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2090,17 +2094,17 @@
       <c r="F22" s="4" t="inlineStr"/>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Contratación, ejecución, liquidación, pago y recepción de la obra destinada a la elaboración del Proyecto Ejecutivo, provisión de materiales, mano de obra, equipos, ejecución, ensayos, habilitación y puesta en servicio de la instalación de gas natural para la Planta Municipal de Elaboración de Mezcla Asfáltica en Caliente, ubicada en el Lote N.º 4 de la Chacra N.º 263 del Parque Industrial de Villaguay, Provincia de Entre Ríos. La contratación comprender á una solución integral bajo modalidad “llave en mano”, incluyendo todos los trabajos, provisiones, trámites, representaciones técnicas, insp</t>
+          <t>Contratación de Servicio de Viandas para el Hospital de la Baxada</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>16/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>16 de octubre del año 2026 a las 10:00 Horas, la que se reali zara en la Oficina de suministros de la Municipalidad de V</t>
+          <t>Hospital de la Baxada, calle Gral. Al varado Nº 2.250 Paraná, Entre Ríos, el día 19/10/2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -2110,7 +2114,7 @@
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
-          <t>$ 50.000,00</t>
+          <t>Ninguno</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr">
@@ -2130,14 +2134,14 @@
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-55f1e5ca423a9262</t>
+          <t>id-d35d5e849089d7ac</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -2145,14 +2149,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>INSTITUTO AUTÁRQUICO DE PLANEAMIENTO YY VIVIENDA — URUGUAY</t>
+          <t>VILLAGUAY — MUNICIPALIDAD DE VILLAGUAY</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2160,24 +2164,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>04/2026</t>
-        </is>
-      </c>
+      <c r="F23" s="4" t="inlineStr"/>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN CONCEPCIÓN DEL URUGUAY 63 VIV. ETAPA I 17 VIV. (P. P.) DEPARTAMENTO: URUGUAY PRESUPUESTO OFICIAL Obras de Viviendas y Complem entarias: $ 1.042.925.971,90 y su equivalente UVIs 693.301,14 Obras de Infraestructuras y Nexos $ 344.554.736,26 y su equivalente UVIs 229.048,08</t>
+          <t>Provisión de una (1) camioneta usada destinada al Parque Automotor Municipal</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>17/11/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>DÍA: 17/11/2026 HOR A: 10:00 HS</t>
+          <t>21 de octubre del año 2026 a las 10:00 Horas, la que se realizara en la Oficina de suministros de la Municipalidad de Vi</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t>$ 138.748,07</t>
+          <t>$10.000,00</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr">
@@ -2207,7 +2207,7 @@
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-b0fe9ebcdc39e73a</t>
+          <t>id-2d3dded56e6c6f6a</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>SALUD ENTRE RÍOS S.A.U</t>
+          <t>PARANA — SALUD ENTRE RÍOS S.A.U</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2240,17 +2240,17 @@
       <c r="F24" s="4" t="inlineStr"/>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Contratación de Servicio de Viandas para el Hospital de la Baxada</t>
+          <t>Servicio de Recolección, Lavado, Desinfección, Secado, Planchado y Transporte de Ropa Hospitalaria</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>Hospital de la Baxada, calle Gral. Al varado Nº 2.250 Paraná, Entre Ríos, el día 19/10/2026 a las 10:00 hs</t>
+          <t>Hospital de la Baxada, calle Gral. Alvarado Nº 2.250 Paraná, Entre Ríos, el día 21/10/2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -2280,14 +2280,14 @@
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-d35d5e849089d7ac</t>
+          <t>id-6b955df9d3f6241a</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -2295,14 +2295,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>VILLAGUAY — MUNICIPALIDAD DE VILLAGUAY</t>
+          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2310,20 +2310,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr"/>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>11/26</t>
+        </is>
+      </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>Provisión de una (1) camioneta usada destinada al Parque Automotor Municipal</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “TERMINACION ESCUELA Nº 40 “JOSÉ ENRIQUE RODÓ”-SEPTIMO DISTRITO-DEPARTAMENTO GUALEGUAY.”</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>21/10/2026</t>
+          <t>23/10/2026</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>21 de octubre del año 2026 a las 10:00 Horas, la que se realizara en la Oficina de suministros de la Municipalidad de Vi</t>
+          <t>DE LAS OFERTAS: el día 23 de Octubre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2333,7 +2337,7 @@
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>$10.000,00</t>
+          <t>$ 100 (Cien)</t>
         </is>
       </c>
       <c r="L25" s="6" t="inlineStr">
@@ -2353,14 +2357,14 @@
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-2d3dded56e6c6f6a</t>
+          <t>id-86cc9c230734c462</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2368,14 +2372,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>PARANA — SALUD ENTRE RÍOS S.A.U</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2383,20 +2387,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr"/>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>11/2026</t>
+        </is>
+      </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Servicio de Recolección, Lavado, Desinfección, Secado, Planchado y Transporte de Ropa Hospitalaria</t>
+          <t>Terminación Escuela N° 40 "José Enrique Rodó", Séptimo Distrito</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>21/10/2026</t>
+          <t>23/10/2026</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Hospital de la Baxada, calle Gral. Alvarado Nº 2.250 Paraná, Entre Ríos, el día 21/10/2026 a las 10:00 hs</t>
+          <t>viernes, 23 de octubre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2404,11 +2412,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K26" s="4" t="inlineStr">
-        <is>
-          <t>Ninguno</t>
-        </is>
-      </c>
+      <c r="K26" s="4" t="inlineStr"/>
       <c r="L26" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2421,19 +2425,19 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-6b955df9d3f6241a</t>
+          <t>id-322a40f5e43af35d</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -2443,12 +2447,12 @@
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>COMUNA DE EL PALENQUE</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2458,22 +2462,22 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>11/26</t>
+          <t>06/26</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “TERMINACION ESCUELA Nº 40 “JOSÉ ENRIQUE RODÓ”-SEPTIMO DISTRITO-DEPARTAMENTO GUALEGUAY.”</t>
+          <t>Adquisición de UNA (1) PALA CARGADORA 0 KM destinada a trabajos en la Comuna</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>23/10/2026</t>
+          <t>26/10/2026</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 23 de Octubre de 2026 a las 10:00 hs</t>
+          <t>26/10/2026, 12:30 horas, Lugar: Sede Administrativa de la Comuna de El Palenque, sito en calle San Martín sin número, El</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2483,7 +2487,7 @@
       </c>
       <c r="K27" s="4" t="inlineStr">
         <is>
-          <t>$ 100 (Cien)</t>
+          <t>pesos cero ($0,00)</t>
         </is>
       </c>
       <c r="L27" s="6" t="inlineStr">
@@ -2503,14 +2507,14 @@
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-86cc9c230734c462</t>
+          <t>id-4b7dfe1bdd0c2ac6</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -2520,12 +2524,12 @@
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>COMUNA DE EL PALENQUE</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2535,22 +2539,22 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>11/2026</t>
+          <t>07/26</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Terminación Escuela N° 40 "José Enrique Rodó", Séptimo Distrito</t>
+          <t>Adquisición de UN (1) TRACTOR AGRÍCOLA 0 KM DE HASTA 9 0 HP, CABINADO 4 x4, CON PALA FRONTAL destinado a trabajos en la Comuna</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>23/10/2026</t>
+          <t>28/10/2026</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>viernes, 23 de octubre de 2026 - 10:00hs</t>
+          <t>28/10/2026, 12:40 horas, Lugar: Sede Administrativa de la Comuna de El Palenque, sito en calle San Martín sin número, El</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2558,7 +2562,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K28" s="4" t="inlineStr"/>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>pesos cero ($ 0,00)</t>
+        </is>
+      </c>
       <c r="L28" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2571,34 +2579,34 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-322a40f5e43af35d</t>
+          <t>id-54e2b94544e5c76f</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C29" s="9" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>COMUNA DE EL PALENQUE</t>
+          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2608,22 +2616,18 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>06/26</t>
+          <t>07/2026</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de UNA (1) PALA CARGADORA 0 KM destinada a trabajos en la Comuna</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t>26/10/2026</t>
-        </is>
-      </c>
+          <t>Transporte de mil doscientos cincuenta metros cúbicos (1.250 m³) de broza grillada desde Cantera “Tayreta” (Ruta Nacional N° 14 km 135) hasta jurisdicción de la comuna, de acuerdo a los Pliegos de Bases, Condiciones Part iculares y demás documentación</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>26/10/2026, 12:30 horas, Lugar: Sede Administrativa de la Comuna de El Palenque, sito en calle San Martín sin número, El</t>
+          <t>Viernes 09 de octubre del corriente año a las 10:00 hs en la Oficina de la Sede de la Comuna</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2631,11 +2635,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K29" s="4" t="inlineStr">
-        <is>
-          <t>pesos cero ($0,00)</t>
-        </is>
-      </c>
+      <c r="K29" s="4" t="inlineStr"/>
       <c r="L29" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2653,29 +2653,29 @@
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-4b7dfe1bdd0c2ac6</t>
+          <t>id-24e9015ecceeff7f</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C30" s="9" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>COMUNA DE EL PALENQUE</t>
+          <t>DIAMANTE — MUNICIPALIDAD DE DIAMANTE -- ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2683,24 +2683,16 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>07/26</t>
-        </is>
-      </c>
+      <c r="F30" s="4" t="inlineStr"/>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de UN (1) TRACTOR AGRÍCOLA 0 KM DE HASTA 9 0 HP, CABINADO 4 x4, CON PALA FRONTAL destinado a trabajos en la Comuna</t>
-        </is>
-      </c>
-      <c r="H30" s="4" t="inlineStr">
-        <is>
-          <t>28/10/2026</t>
-        </is>
-      </c>
+          <t>Solicitar Contratación de una empresa para la Obra de “22 (veintidós) cuadras de pavimento urbano” – Grupo 1- según Expte. Letra “D” Nº 2196</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>28/10/2026, 12:40 horas, Lugar: Sede Administrativa de la Comuna de El Palenque, sito en calle San Martín sin número, El</t>
+          <t>viernes 23 de octubre de 2.026, a la hora diez (10.00)</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2708,11 +2700,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K30" s="4" t="inlineStr">
-        <is>
-          <t>pesos cero ($ 0,00)</t>
-        </is>
-      </c>
+      <c r="K30" s="4" t="inlineStr"/>
       <c r="L30" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2730,14 +2718,14 @@
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-54e2b94544e5c76f</t>
+          <t>id-4f207bef5c709ad6</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2745,35 +2733,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C31" s="10" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
+          <t>CONCORDIA — APEX S.A.S</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>07/2026</t>
-        </is>
-      </c>
+          <t>Licitación</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr"/>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>Transporte de mil doscientos cincuenta metros cúbicos (1.250 m³) de broza grillada desde Cantera “Tayreta” (Ruta Nacional N° 14 km 135) hasta jurisdicción de la comuna, de acuerdo a los Pliegos de Bases, Condiciones Part iculares y demás documentación</t>
+          <t>instalaciones eléctricas, sanitarias, hidráulicas, mecánicas o de cualquier otra naturaleza relacionada con el sector</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Viernes 09 de octubre del corriente año a las 10:00 hs en la Oficina de la Sede de la Comuna</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2799,14 +2783,14 @@
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-24e9015ecceeff7f</t>
+          <t>id-a20c6b2b6fcf36a2</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2814,31 +2798,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>DIAMANTE — MUNICIPALIDAD DE DIAMANTE -- ENTRE RÍOS</t>
+          <t>Boletín Oficial</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Remate</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr"/>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>Solicitar Contratación de una empresa para la Obra de “22 (veintidós) cuadras de pavimento urbano” – Grupo 1- según Expte. Letra “D” Nº 2196</t>
+          <t>los vehículos se encuentran en exhibición por lo cuál la información registral, de rentas y de infracciones puede ser</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>viernes 23 de octubre de 2.026, a la hora diez (10.00)</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2864,14 +2848,14 @@
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-4f207bef5c709ad6</t>
+          <t>id-fb8d7dc09e202fea</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2879,31 +2863,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>CONCORDIA — APEX S.A.S</t>
+          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Licitación</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>001/26</t>
+        </is>
+      </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>instalaciones eléctricas, sanitarias, hidráulicas, mecánicas o de cualquier otra naturaleza relacionada con el sector</t>
+          <t>ADQUISICIÓN de UN (1) FURGON UTILITARIO CHICO con 5 asientos 0 KM. con destino a Subsecretaria de Asistencia Directa y Emergencia</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>DE LAS PROPUESTAS: 20 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2929,14 +2917,14 @@
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-a20c6b2b6fcf36a2</t>
+          <t>id-ca205f0874380f69</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2944,25 +2932,25 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C34" s="9" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Boletín Oficial</t>
+          <t>INSTITUTO CARBÓ S.R.L</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Remate</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr"/>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>los vehículos se encuentran en exhibición por lo cuál la información registral, de rentas y de infracciones puede ser</t>
+          <t>sin internación en materia de salud, pre- hospitalarias, atención médica, domiciliaria y traslados sanitarios de alta</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
@@ -2994,7 +2982,7 @@
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-fb8d7dc09e202fea</t>
+          <t>id-6aa57c7437a30ca3</t>
         </is>
       </c>
     </row>
@@ -3009,14 +2997,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C35" s="9" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
+          <t>MUNICIPALIDAD DE VIALE</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3026,18 +3014,18 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>001/26</t>
+          <t>08/26</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN de UN (1) FURGON UTILITARIO CHICO con 5 asientos 0 KM. con destino a Subsecretaria de Asistencia Directa y Emergencia</t>
+          <t>de asf alto 70-16 destinado a la producción de pavimento de la Planta Asfáltica, y que a continuación se detalla y</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>DE LAS PROPUESTAS: 20 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3063,14 +3051,14 @@
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-ca205f0874380f69</t>
+          <t>id-ef1ddb923c7e7fdb</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3085,24 +3073,28 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>INSTITUTO CARBÓ S.R.L</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Licitación</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>sin internación en materia de salud, pre- hospitalarias, atención médica, domiciliaria y traslados sanitarios de alta</t>
+          <t>TERMINACIÓN CONCEPCIÓN DEL URUGUAY 63 VIV</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Publicada 06/10/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3123,19 +3115,19 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>id-6aa57c7437a30ca3</t>
+          <t>id-1a3c1f8e036ac91e</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3150,7 +3142,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE VIALE</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3160,18 +3152,18 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>08/26</t>
+          <t>05/2026</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>de asf alto 70-16 destinado a la producción de pavimento de la Planta Asfáltica, y que a continuación se detalla y</t>
+          <t>COMPLEJO HABITACIONAL SAN AGUSTÍN (P</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Publicada 05/10/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3192,19 +3184,19 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>id-ef1ddb923c7e7fdb</t>
+          <t>id-ccb22bcad9356438</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -3229,18 +3221,18 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>03/26</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN CONCEPCIÓN DEL URUGUAY 63 VIV</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2026 — ver pliego</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -3266,14 +3258,14 @@
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>id-1a3c1f8e036ac91e</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3298,18 +3290,18 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>05/2026</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>COMPLEJO HABITACIONAL SAN AGUSTÍN (P</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/10/2026 — ver pliego</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -3335,7 +3327,7 @@
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
-          <t>id-ccb22bcad9356438</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
@@ -3367,18 +3359,18 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>03/26</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr"/>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
@@ -3404,7 +3396,7 @@
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
@@ -3436,18 +3428,18 @@
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>02/2026</t>
+          <t>05/2025</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
@@ -3473,7 +3465,7 @@
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
@@ -3505,18 +3497,18 @@
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>06/2025</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr"/>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr">
@@ -3542,7 +3534,7 @@
       </c>
       <c r="O42" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
@@ -3572,20 +3564,16 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F43" s="4" t="inlineStr">
-        <is>
-          <t>05/2025</t>
-        </is>
-      </c>
+      <c r="F43" s="4" t="inlineStr"/>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr"/>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr">
@@ -3611,7 +3599,7 @@
       </c>
       <c r="O43" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
@@ -3643,18 +3631,18 @@
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>06/2025</t>
+          <t>04/2025</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr"/>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr">
@@ -3680,7 +3668,7 @@
       </c>
       <c r="O44" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
@@ -3710,16 +3698,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F45" s="4" t="inlineStr"/>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>03/2025</t>
+        </is>
+      </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr"/>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J45" s="4" t="inlineStr">
@@ -3745,7 +3737,7 @@
       </c>
       <c r="O45" s="4" t="inlineStr">
         <is>
-          <t>id-ebeeb6a87e688d85</t>
+          <t>id-75bfffae63b7eedc</t>
         </is>
       </c>
     </row>
@@ -3767,28 +3759,24 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="inlineStr">
-        <is>
-          <t>04/2025</t>
-        </is>
-      </c>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr"/>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+          <t>CONSTRUCCIÓN DE OBRAS DE ARTE EN EL DEPARTAMENTO LA PAZ. 1) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE EN R.P. S/Nº SOBRE Aº ESTACAS – “CAMINO SAUCECITO” – TRAMO: R.P.Nº 1 – ESCUELA Nº 62 – DISTRITO ESTACAS – DEPARTAMENTO LA PAZ – 2) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE SOBRE Aº ESTACAS SAN GUSTAVO – TRAMO: […]</t>
         </is>
       </c>
       <c r="H46" s="4" t="inlineStr"/>
       <c r="I46" s="4" t="inlineStr">
         <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J46" s="4" t="inlineStr">
@@ -3809,19 +3797,19 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O46" s="4" t="inlineStr">
         <is>
-          <t>id-34c85bcdb9b1123f</t>
+          <t>id-3d7728874996f284</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3829,35 +3817,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C47" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr">
-        <is>
-          <t>03/2025</t>
-        </is>
-      </c>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr"/>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
         </is>
       </c>
       <c r="H47" s="4" t="inlineStr"/>
       <c r="I47" s="4" t="inlineStr">
         <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J47" s="4" t="inlineStr">
@@ -3878,19 +3862,19 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O47" s="4" t="inlineStr">
         <is>
-          <t>id-75bfffae63b7eedc</t>
+          <t>id-654eebef400f89cd</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -3910,13 +3894,17 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F48" s="4" t="inlineStr"/>
+          <t>Concurso</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>01/26</t>
+        </is>
+      </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>CONSTRUCCIÓN DE OBRAS DE ARTE EN EL DEPARTAMENTO LA PAZ. 1) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE EN R.P. S/Nº SOBRE Aº ESTACAS – “CAMINO SAUCECITO” – TRAMO: R.P.Nº 1 – ESCUELA Nº 62 – DISTRITO ESTACAS – DEPARTAMENTO LA PAZ – 2) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE SOBRE Aº ESTACAS SAN GUSTAVO – TRAMO: […]</t>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
         </is>
       </c>
       <c r="H48" s="4" t="inlineStr"/>
@@ -3948,7 +3936,7 @@
       </c>
       <c r="O48" s="4" t="inlineStr">
         <is>
-          <t>id-3d7728874996f284</t>
+          <t>id-9a16884dd5a64a49</t>
         </is>
       </c>
     </row>
@@ -3963,25 +3951,29 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C49" s="7" t="inlineStr">
+      <c r="C49" s="9" t="inlineStr">
         <is>
           <t>Materiales</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F49" s="4" t="inlineStr"/>
+          <t>Licitación</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>2026-1227</t>
+        </is>
+      </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
         </is>
       </c>
       <c r="H49" s="4" t="inlineStr"/>
@@ -4008,155 +4000,17 @@
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="O49" s="4" t="inlineStr">
         <is>
-          <t>id-654eebef400f89cd</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C50" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>Concurso</t>
-        </is>
-      </c>
-      <c r="F50" s="4" t="inlineStr">
-        <is>
-          <t>01/26</t>
-        </is>
-      </c>
-      <c r="G50" s="5" t="inlineStr">
-        <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
-        </is>
-      </c>
-      <c r="H50" s="4" t="inlineStr"/>
-      <c r="I50" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J50" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K50" s="4" t="inlineStr"/>
-      <c r="L50" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M50" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N50" t="inlineStr">
-        <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
-        </is>
-      </c>
-      <c r="O50" s="4" t="inlineStr">
-        <is>
-          <t>id-9a16884dd5a64a49</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C51" s="7" t="inlineStr">
-        <is>
-          <t>Materiales</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>ENERSA</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Licitación</t>
-        </is>
-      </c>
-      <c r="F51" s="4" t="inlineStr">
-        <is>
-          <t>2026-1227</t>
-        </is>
-      </c>
-      <c r="G51" s="5" t="inlineStr">
-        <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
-        </is>
-      </c>
-      <c r="H51" s="4" t="inlineStr"/>
-      <c r="I51" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J51" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K51" s="4" t="inlineStr"/>
-      <c r="L51" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M51" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N51" t="inlineStr">
-        <is>
-          <t>ENERSA</t>
-        </is>
-      </c>
-      <c r="O51" s="4" t="inlineStr">
-        <is>
           <t>id-0691eb485d7548eb</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O51"/>
+  <autoFilter ref="A1:O49"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -4254,10 +4108,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId94"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L49" r:id="rId95"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M49" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L50" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M50" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L51" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M51" r:id="rId100"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 10/10/2026 08:42
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$47</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O49"/>
+  <dimension ref="A1:O47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -722,7 +722,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -737,7 +737,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>URUGUAY — MUNICIPALIDAD DE CONCEPCION DEL URUGUAY</t>
+          <t>COLON — MUNICIPALIDAD DE VILLA ELISA (E.R.)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -747,22 +747,22 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>34/2026</t>
+          <t>004/26</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>“Concesión de la Explotación Comercial de un (01) Camión de Comidas Rápidas (para cubrir el total de cuatro puestos) en la Zona Joven – Parque La Salamanca de la Municipalidad de Concepción del Uruguay – Entre Ríos”, en un todo de acuerdo a los Pliegos de Bases, Condiciones Particulares y demás documentación</t>
+          <t>ADQUISICIÓN DE UN (1) VEHÍCULO PARA TRANSPORTE DE PASAJEROS DE (5) CINCO PLAZAS 0 KM - MODELO/AÑO 2026, PARA LA MUNICIPALIDAD DE LA CIUDAD DE VILLA ELISA, ENTRE RÍOS</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>12/11/2026</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>09 de octubre de 2026 Hora: 10:00</t>
+          <t>12 de NOVIEMBRE de 2026 a la hora 10:00 en la Oficina de Compras de la Municipalidad de Villa Elisa, Entre Ríos</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -770,7 +770,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr"/>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>$ 20.000,00 (Pesos Veint e mil con 00/100) el que se puede adquirir en</t>
+        </is>
+      </c>
       <c r="L4" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -788,7 +792,7 @@
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
-          <t>id-b147fbd9d3081bfc</t>
+          <t>id-bb3703ff360c8c43</t>
         </is>
       </c>
     </row>
@@ -803,14 +807,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>LA PAZ — MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -820,22 +824,22 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>10/2026</t>
+          <t>11/2026</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>“PROVISIÓN DE UNA (1) MINICARGADORA 0 KM, CON CUCHARÓN FRONTAL DE USO GENERAL, UN (1) MARTILLO HIDRÁULICO Y UN (1) COMPACTADOR/RODILLO VIBRATORIO LISO”</t>
+          <t>OBRA "PAVIMENTACION URBANA CALLE TRATADO DEL PILAR B° 3 DE FEBRERO - MUNICIPALIDAD DE SANTA ELENA" (Según Pliegos de Bases y condi ciones)</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>09/10/2026</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>09/10/2026 HORA: 10:00 HS</t>
+          <t>13/10/2026 HORA: 10: 00 HS</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -845,7 +849,7 @@
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>($ 270.000,00) PESOS DOSCIENTOS SETENTA MIL</t>
+          <t>$ 728.000,00 PESOS SETECIENTOS VEINTIOCHO MIL</t>
         </is>
       </c>
       <c r="L5" s="6" t="inlineStr">
@@ -865,14 +869,14 @@
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>id-779e4cd290f2e64e</t>
+          <t>id-1a2561509308b1b6</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -880,14 +884,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>COLON — MUNICIPALIDAD DE VILLA ELISA (E.R.)</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -897,34 +901,30 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>004/26</t>
+          <t>11/2026</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN DE UN (1) VEHÍCULO PARA TRANSPORTE DE PASAJEROS DE (5) CINCO PLAZAS 0 KM - MODELO/AÑO 2026, PARA LA MUNICIPALIDAD DE LA CIUDAD DE VILLA ELISA, ENTRE RÍOS</t>
+          <t>REFACCION EN ESCUELA N° 65 “ALMIRANTE BROWN” – CIUDAD DE CONCORDIA - DEPARTAMENTO CONCORDIA - PROVINCIA DE ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>12/11/2026</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>12 de NOVIEMBRE de 2026 a la hora 10:00 en la Oficina de Compras de la Municipalidad de Villa Elisa, Entre Ríos</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 09:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t>$ 20.000,00 (Pesos Veint e mil con 00/100) el que se puede adquirir en</t>
-        </is>
-      </c>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr"/>
       <c r="L6" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -942,7 +942,7 @@
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>id-bb3703ff360c8c43</t>
+          <t>id-fc30d5c0b0589a79</t>
         </is>
       </c>
     </row>
@@ -957,14 +957,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -974,12 +974,12 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>11/2026</t>
+          <t>13/2026</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>OBRA "PAVIMENTACION URBANA CALLE TRATADO DEL PILAR B° 3 DE FEBRERO - MUNICIPALIDAD DE SANTA ELENA" (Según Pliegos de Bases y condi ciones)</t>
+          <t>REPARACIONES VARIAS EN C. P. E. F. Nº 3 “PROFESOR HUGO LA NASA” – CIUDAD DE CONCEPCION DEL URUGUAY - DEPARTAMENTO URUGUAY - PROVINCIA D E ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -989,19 +989,15 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026 HORA: 10: 00 HS</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K7" s="4" t="inlineStr">
-        <is>
-          <t>$ 728.000,00 PESOS SETECIENTOS VEINTIOCHO MIL</t>
-        </is>
-      </c>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr"/>
       <c r="L7" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1019,7 +1015,7 @@
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>id-1a2561509308b1b6</t>
+          <t>id-9d3847fb0e2b0929</t>
         </is>
       </c>
     </row>
@@ -1051,12 +1047,12 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>11/2026</t>
+          <t>12/2026</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>REFACCION EN ESCUELA N° 65 “ALMIRANTE BROWN” – CIUDAD DE CONCORDIA - DEPARTAMENTO CONCORDIA - PROVINCIA DE ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>RECAMBIO DE CUBIERTA Y REPARACIONES VARIAS EN ESCUELA Nº 92 “CONGRESO DE TUCUMAN” – CONCEPCION DEL URUGUAY - DPTO. URUGUAY – PROVINCIA DE ENTRE RIOS de acuerdo a las c ondiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -1066,7 +1062,7 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 09:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 10:30 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -1092,7 +1088,7 @@
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>id-fc30d5c0b0589a79</t>
+          <t>id-059239b424b9c936</t>
         </is>
       </c>
     </row>
@@ -1107,14 +1103,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1124,12 +1120,12 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>13/2026</t>
+          <t>87/2026</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>REPARACIONES VARIAS EN C. P. E. F. Nº 3 “PROFESOR HUGO LA NASA” – CIUDAD DE CONCEPCION DEL URUGUAY - DEPARTAMENTO URUGUAY - PROVINCIA D E ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>Contratar la ejecución de la obra denominada “Construcción de Red Cloacal Subsidiaria del Colector Noroeste Barrio Ciudad Paisaje”</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -1139,15 +1135,19 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
+          <t>martes, 13 de octubre de 2026 a las 10:00</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
-        </is>
-      </c>
-      <c r="K9" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>$ 10.000 (pesos diez mil)</t>
+        </is>
+      </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1160,12 +1160,12 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Boletín Oficial Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>id-9d3847fb0e2b0929</t>
+          <t>id-ceeb594e8bcc4ff7</t>
         </is>
       </c>
     </row>
@@ -1180,14 +1180,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
+          <t>COLON — MUNICIPALIDAD DE COLON</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1195,32 +1195,32 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>12/2026</t>
-        </is>
-      </c>
+      <c r="F10" s="4" t="inlineStr"/>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>RECAMBIO DE CUBIERTA Y REPARACIONES VARIAS EN ESCUELA Nº 92 “CONGRESO DE TUCUMAN” – CONCEPCION DEL URUGUAY - DPTO. URUGUAY – PROVINCIA DE ENTRE RIOS de acuerdo a las c ondiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>“ADQUISICIÓN DE MATERIALES ELÉCTRICOS PARA EJECUCIÓN DEL PROYECTO DE RECONVERSIÓN Y OPTIMIZACIÓN DEL ALUMBRADO PÚBLICO DE LA CIUDAD DE COLÓN”</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026</t>
+          <t>14/10/2026</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 10:30 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
+          <t>14 de OCTUBRE de 2026</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
-        </is>
-      </c>
-      <c r="K10" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>Sin Cargo</t>
+        </is>
+      </c>
       <c r="L10" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>id-059239b424b9c936</t>
+          <t>id-9e122d52de12ffef</t>
         </is>
       </c>
     </row>
@@ -1253,14 +1253,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>DIAMANTE — COMUNA ALDEA PROTESTANTE -- DIAMANTE -- ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1270,22 +1270,22 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>87/2026</t>
+          <t>03/2026</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Contratar la ejecución de la obra denominada “Construcción de Red Cloacal Subsidiaria del Colector Noroeste Barrio Ciudad Paisaje”</t>
+          <t>Conforme a lo autorizado por decreto Nº 290/26 llámese a licitación pública Nº 03/26 con el objeto de comprar 10 toneladas de emulsión catiónica súper estable (asfalto de imprimación), puesto en Aldea Protestante</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026</t>
+          <t>14/10/2026</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>martes, 13 de octubre de 2026 a las 10:00</t>
+          <t>miércoles 14 de octubre de 2026 – Hora nueve (09:00) Lugar de presentación de la oferta: Sede Comuna Aldea Protestan</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1293,11 +1293,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K11" s="4" t="inlineStr">
-        <is>
-          <t>$ 10.000 (pesos diez mil)</t>
-        </is>
-      </c>
+      <c r="K11" s="4" t="inlineStr"/>
       <c r="L11" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1310,12 +1306,12 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Boletín Oficial Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>id-ceeb594e8bcc4ff7</t>
+          <t>id-c2f3a25cfb37fd38</t>
         </is>
       </c>
     </row>
@@ -1330,14 +1326,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>COLON — MUNICIPALIDAD DE COLON</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1345,10 +1341,14 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr"/>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>017/2026</t>
+        </is>
+      </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN DE MATERIALES ELÉCTRICOS PARA EJECUCIÓN DEL PROYECTO DE RECONVERSIÓN Y OPTIMIZACIÓN DEL ALUMBRADO PÚBLICO DE LA CIUDAD DE COLÓN”</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de UNA (1) MOTONIVELADORA, nueva, sin uso, cero km, con una potencia entre 220/240 HP, con opción a implementos, que será utilizada para el área del corralón municipal</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -1358,7 +1358,7 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>14 de OCTUBRE de 2026</t>
+          <t>14 DE OCTUBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>Sin Cargo</t>
+          <t>$100.000,00. - (PESOS CIEN MIL CON 00/100) PRESUPUESTO OFICIAL ESTIMAD</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
@@ -1388,7 +1388,7 @@
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>id-9e122d52de12ffef</t>
+          <t>id-4c3b33859e596759</t>
         </is>
       </c>
     </row>
@@ -1403,14 +1403,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>DIAMANTE — COMUNA ALDEA PROTESTANTE -- DIAMANTE -- ENTRE RÍOS</t>
+          <t>VICTORIA — MUNICIPALIDAD DE VICTORIA</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1420,12 +1420,12 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>03/2026</t>
+          <t>008/2026</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Conforme a lo autorizado por decreto Nº 290/26 llámese a licitación pública Nº 03/26 con el objeto de comprar 10 toneladas de emulsión catiónica súper estable (asfalto de imprimación), puesto en Aldea Protestante</t>
+          <t>Proveer a la Municipalidad de Victoria, Entre Ríos, de Veinticinco Mil (25.000) litros de Diésel 500, para movilidad de vehículos y maquinarias viales , Ocho Mil (8.000) litros de Gasoil Tipo euro o similar y Ocho (8.000) litros de nafta súper para vehículos y áreas afectadas a la Secretaria de Planeamiento y Dirección de Ambiente y Desarrollo sostenible;</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
@@ -1435,7 +1435,7 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>miércoles 14 de octubre de 2026 – Hora nueve (09:00) Lugar de presentación de la oferta: Sede Comuna Aldea Protestan</t>
+          <t>14 de octubre de 2026 a las 09:00 hs., en la Oficina de Compras de la Municipalidad de Victoria, Entr</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -1461,14 +1461,14 @@
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>id-c2f3a25cfb37fd38</t>
+          <t>id-a9af9f59c8c487c8</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1483,22 +1483,22 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>LICITACIÓN PÚBLICA</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>017/2026</t>
+          <t>89/2026</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de UNA (1) MOTONIVELADORA, nueva, sin uso, cero km, con una potencia entre 220/240 HP, con opción a implementos, que será utilizada para el área del corralón municipal</t>
+          <t>ADQUISICION DE BALANZA BASCULA PARA PESAJE DE EJESDE CAMIONES</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>14 DE OCTUBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>14-10-2026 08:00</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1516,11 +1516,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K14" s="4" t="inlineStr">
-        <is>
-          <t>$100.000,00. - (PESOS CIEN MIL CON 00/100) PRESUPUESTO OFICIAL ESTIMAD</t>
-        </is>
-      </c>
+      <c r="K14" s="4" t="inlineStr"/>
       <c r="L14" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1533,19 +1529,19 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>id-4c3b33859e596759</t>
+          <t>id-4ee814ba6420f0cc</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1560,7 +1556,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>VICTORIA — MUNICIPALIDAD DE VICTORIA</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1570,12 +1566,12 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>008/2026</t>
+          <t>89/2026</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Proveer a la Municipalidad de Victoria, Entre Ríos, de Veinticinco Mil (25.000) litros de Diésel 500, para movilidad de vehículos y maquinarias viales , Ocho Mil (8.000) litros de Gasoil Tipo euro o similar y Ocho (8.000) litros de nafta súper para vehículos y áreas afectadas a la Secretaria de Planeamiento y Dirección de Ambiente y Desarrollo sostenible;</t>
+          <t>Adquisición de balanzas básculas para pesaje de ejes de camiones</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
@@ -1585,7 +1581,7 @@
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>14 de octubre de 2026 a las 09:00 hs., en la Oficina de Compras de la Municipalidad de Victoria, Entr</t>
+          <t>miércoles, 14 de octubre de 2026 a las 08:00</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1606,12 +1602,12 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Boletín Oficial Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>id-a9af9f59c8c487c8</t>
+          <t>id-d963348e34fcb0d3</t>
         </is>
       </c>
     </row>
@@ -1633,32 +1629,32 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE ALDEA SAN ANTONIO</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>89/2026</t>
+          <t>002/2026</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICION DE BALANZA BASCULA PARA PESAJE DE EJESDE CAMIONES</t>
+          <t>ADQUISICIÓN DE UNA MÁQUINA MOTONIVELADORA PARA INCORPORAR AL PARQUE AUTOMOTOR DE LA MUNICIP ALIDAD DE ALDEA SAN ANTONIO</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>14/10/2026</t>
+          <t>15/10/2026</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>14-10-2026 08:00</t>
+          <t>15 de octubre de 2026, a las 08:00 horas, en el Edificio Municipal</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -1666,7 +1662,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K16" s="4" t="inlineStr"/>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>PESOS CIEN MIL con 00/100 ($ 100.000,00. -)</t>
+        </is>
+      </c>
       <c r="L16" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1679,19 +1679,19 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>id-4ee814ba6420f0cc</t>
+          <t>id-95a507b67b7b1450</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1699,14 +1699,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>MINISTERIO DE SALUD — GOBIERNO DE ENTRE RIOS</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1716,22 +1716,22 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>89/2026</t>
+          <t>18/26</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de balanzas básculas para pesaje de ejes de camiones</t>
+          <t>Adquirir Sesenta Mil (60.000) Kilogramos de Leche Entera en Polvo Instantánea, Fortificada con Hierro, Zinc y Ácido Ascórbico</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>14/10/2026</t>
+          <t>16/10/2026</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 14 de octubre de 2026 a las 08:00</t>
+          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1739,7 +1739,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K17" s="4" t="inlineStr"/>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>PESOS TRES MIL QUINIENTOS ($ 3.500,00)</t>
+        </is>
+      </c>
       <c r="L17" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1752,19 +1756,19 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Boletín Oficial Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>id-d963348e34fcb0d3</t>
+          <t>id-04a917d50ccab2e3</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1772,14 +1776,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE ALDEA SAN ANTONIO</t>
+          <t>VILLAGUAY — MUNICIPALIDAD DE VILLAGUAY</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1787,24 +1791,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>002/2026</t>
-        </is>
-      </c>
+      <c r="F18" s="4" t="inlineStr"/>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN DE UNA MÁQUINA MOTONIVELADORA PARA INCORPORAR AL PARQUE AUTOMOTOR DE LA MUNICIP ALIDAD DE ALDEA SAN ANTONIO</t>
+          <t>Contratación, ejecución, liquidación, pago y recepción de la obra destinada a la elaboración del Proyecto Ejecutivo, provisión de materiales, mano de obra, equipos, ejecución, ensayos, habilitación y puesta en servicio de la instalación de gas natural para la Planta Municipal de Elaboración de Mezcla Asfáltica en Caliente, ubicada en el Lote N.º 4 de la Chacra N.º 263 del Parque Industrial de Villaguay, Provincia de Entre Ríos. La contratación comprender á una solución integral bajo modalidad “llave en mano”, incluyendo todos los trabajos, provisiones, trámites, representaciones técnicas, insp</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>15/10/2026</t>
+          <t>16/10/2026</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>15 de octubre de 2026, a las 08:00 horas, en el Edificio Municipal</t>
+          <t>16 de octubre del año 2026 a las 10:00 Horas, la que se reali zara en la Oficina de suministros de la Municipalidad de V</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>PESOS CIEN MIL con 00/100 ($ 100.000,00. -)</t>
+          <t>$ 50.000,00</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr">
@@ -1834,14 +1834,14 @@
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>id-95a507b67b7b1450</t>
+          <t>id-55f1e5ca423a9262</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1849,14 +1849,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>MINISTERIO DE SALUD — GOBIERNO DE ENTRE RIOS</t>
+          <t>INSTITUTO AUTÁRQUICO DE PLANEAMIENTO YY VIVIENDA — URUGUAY</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1866,22 +1866,22 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>18/26</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Adquirir Sesenta Mil (60.000) Kilogramos de Leche Entera en Polvo Instantánea, Fortificada con Hierro, Zinc y Ácido Ascórbico</t>
+          <t>TERMINACIÓN CONCEPCIÓN DEL URUGUAY 63 VIV. ETAPA I 17 VIV. (P. P.) DEPARTAMENTO: URUGUAY PRESUPUESTO OFICIAL Obras de Viviendas y Complem entarias: $ 1.042.925.971,90 y su equivalente UVIs 693.301,14 Obras de Infraestructuras y Nexos $ 344.554.736,26 y su equivalente UVIs 229.048,08</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>16/10/2026</t>
+          <t>17/11/2026</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
+          <t>DÍA: 17/11/2026 HOR A: 10:00 HS</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1891,7 +1891,7 @@
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>PESOS TRES MIL QUINIENTOS ($ 3.500,00)</t>
+          <t>$ 138.748,07</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr">
@@ -1911,7 +1911,7 @@
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>id-04a917d50ccab2e3</t>
+          <t>id-b0fe9ebcdc39e73a</t>
         </is>
       </c>
     </row>
@@ -1933,7 +1933,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>VILLAGUAY — MUNICIPALIDAD DE VILLAGUAY</t>
+          <t>SALUD ENTRE RÍOS S.A.U</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1944,17 +1944,17 @@
       <c r="F20" s="4" t="inlineStr"/>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Contratación, ejecución, liquidación, pago y recepción de la obra destinada a la elaboración del Proyecto Ejecutivo, provisión de materiales, mano de obra, equipos, ejecución, ensayos, habilitación y puesta en servicio de la instalación de gas natural para la Planta Municipal de Elaboración de Mezcla Asfáltica en Caliente, ubicada en el Lote N.º 4 de la Chacra N.º 263 del Parque Industrial de Villaguay, Provincia de Entre Ríos. La contratación comprender á una solución integral bajo modalidad “llave en mano”, incluyendo todos los trabajos, provisiones, trámites, representaciones técnicas, insp</t>
+          <t>Contratación de Servicio de Viandas para el Hospital de la Baxada</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>16/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>16 de octubre del año 2026 a las 10:00 Horas, la que se reali zara en la Oficina de suministros de la Municipalidad de V</t>
+          <t>Hospital de la Baxada, calle Gral. Al varado Nº 2.250 Paraná, Entre Ríos, el día 19/10/2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>$ 50.000,00</t>
+          <t>Ninguno</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
@@ -1984,14 +1984,14 @@
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>id-55f1e5ca423a9262</t>
+          <t>id-d35d5e849089d7ac</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1999,14 +1999,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>INSTITUTO AUTÁRQUICO DE PLANEAMIENTO YY VIVIENDA — URUGUAY</t>
+          <t>VILLAGUAY — MUNICIPALIDAD DE VILLAGUAY</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2014,24 +2014,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>04/2026</t>
-        </is>
-      </c>
+      <c r="F21" s="4" t="inlineStr"/>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN CONCEPCIÓN DEL URUGUAY 63 VIV. ETAPA I 17 VIV. (P. P.) DEPARTAMENTO: URUGUAY PRESUPUESTO OFICIAL Obras de Viviendas y Complem entarias: $ 1.042.925.971,90 y su equivalente UVIs 693.301,14 Obras de Infraestructuras y Nexos $ 344.554.736,26 y su equivalente UVIs 229.048,08</t>
+          <t>Provisión de una (1) camioneta usada destinada al Parque Automotor Municipal</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>17/11/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>DÍA: 17/11/2026 HOR A: 10:00 HS</t>
+          <t>21 de octubre del año 2026 a las 10:00 Horas, la que se realizara en la Oficina de suministros de la Municipalidad de Vi</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -2041,7 +2037,7 @@
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>$ 138.748,07</t>
+          <t>$10.000,00</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr">
@@ -2061,7 +2057,7 @@
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-b0fe9ebcdc39e73a</t>
+          <t>id-2d3dded56e6c6f6a</t>
         </is>
       </c>
     </row>
@@ -2083,7 +2079,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>SALUD ENTRE RÍOS S.A.U</t>
+          <t>PARANA — SALUD ENTRE RÍOS S.A.U</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2094,17 +2090,17 @@
       <c r="F22" s="4" t="inlineStr"/>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Contratación de Servicio de Viandas para el Hospital de la Baxada</t>
+          <t>Servicio de Recolección, Lavado, Desinfección, Secado, Planchado y Transporte de Ropa Hospitalaria</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Hospital de la Baxada, calle Gral. Al varado Nº 2.250 Paraná, Entre Ríos, el día 19/10/2026 a las 10:00 hs</t>
+          <t>Hospital de la Baxada, calle Gral. Alvarado Nº 2.250 Paraná, Entre Ríos, el día 21/10/2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -2134,14 +2130,14 @@
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-d35d5e849089d7ac</t>
+          <t>id-6b955df9d3f6241a</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -2149,14 +2145,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>VILLAGUAY — MUNICIPALIDAD DE VILLAGUAY</t>
+          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2164,20 +2160,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr"/>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>11/26</t>
+        </is>
+      </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Provisión de una (1) camioneta usada destinada al Parque Automotor Municipal</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “TERMINACION ESCUELA Nº 40 “JOSÉ ENRIQUE RODÓ”-SEPTIMO DISTRITO-DEPARTAMENTO GUALEGUAY.”</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>21/10/2026</t>
+          <t>23/10/2026</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>21 de octubre del año 2026 a las 10:00 Horas, la que se realizara en la Oficina de suministros de la Municipalidad de Vi</t>
+          <t>DE LAS OFERTAS: el día 23 de Octubre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t>$10.000,00</t>
+          <t>$ 100 (Cien)</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr">
@@ -2207,14 +2207,14 @@
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-2d3dded56e6c6f6a</t>
+          <t>id-86cc9c230734c462</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2222,14 +2222,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>PARANA — SALUD ENTRE RÍOS S.A.U</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2237,20 +2237,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr"/>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>11/2026</t>
+        </is>
+      </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Servicio de Recolección, Lavado, Desinfección, Secado, Planchado y Transporte de Ropa Hospitalaria</t>
+          <t>Terminación Escuela N° 40 "José Enrique Rodó", Séptimo Distrito</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>21/10/2026</t>
+          <t>23/10/2026</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>Hospital de la Baxada, calle Gral. Alvarado Nº 2.250 Paraná, Entre Ríos, el día 21/10/2026 a las 10:00 hs</t>
+          <t>viernes, 23 de octubre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -2258,11 +2262,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K24" s="4" t="inlineStr">
-        <is>
-          <t>Ninguno</t>
-        </is>
-      </c>
+      <c r="K24" s="4" t="inlineStr"/>
       <c r="L24" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2275,19 +2275,19 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-6b955df9d3f6241a</t>
+          <t>id-322a40f5e43af35d</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -2295,14 +2295,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>COMUNA DE EL PALENQUE</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2312,22 +2312,22 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>11/26</t>
+          <t>06/26</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “TERMINACION ESCUELA Nº 40 “JOSÉ ENRIQUE RODÓ”-SEPTIMO DISTRITO-DEPARTAMENTO GUALEGUAY.”</t>
+          <t>Adquisición de UNA (1) PALA CARGADORA 0 KM destinada a trabajos en la Comuna</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>23/10/2026</t>
+          <t>26/10/2026</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 23 de Octubre de 2026 a las 10:00 hs</t>
+          <t>26/10/2026, 12:30 horas, Lugar: Sede Administrativa de la Comuna de El Palenque, sito en calle San Martín sin número, El</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2337,7 +2337,7 @@
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>$ 100 (Cien)</t>
+          <t>pesos cero ($0,00)</t>
         </is>
       </c>
       <c r="L25" s="6" t="inlineStr">
@@ -2357,14 +2357,14 @@
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-86cc9c230734c462</t>
+          <t>id-4b7dfe1bdd0c2ac6</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -2372,14 +2372,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>COMUNA DE EL PALENQUE</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2389,22 +2389,22 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>11/2026</t>
+          <t>07/26</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Terminación Escuela N° 40 "José Enrique Rodó", Séptimo Distrito</t>
+          <t>Adquisición de UN (1) TRACTOR AGRÍCOLA 0 KM DE HASTA 9 0 HP, CABINADO 4 x4, CON PALA FRONTAL destinado a trabajos en la Comuna</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>23/10/2026</t>
+          <t>28/10/2026</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>viernes, 23 de octubre de 2026 - 10:00hs</t>
+          <t>28/10/2026, 12:40 horas, Lugar: Sede Administrativa de la Comuna de El Palenque, sito en calle San Martín sin número, El</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2412,7 +2412,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K26" s="4" t="inlineStr"/>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>pesos cero ($ 0,00)</t>
+        </is>
+      </c>
       <c r="L26" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2425,34 +2429,34 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-322a40f5e43af35d</t>
+          <t>id-54e2b94544e5c76f</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C27" s="8" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>COMUNA DE EL PALENQUE</t>
+          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2462,22 +2466,18 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>06/26</t>
+          <t>07/2026</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de UNA (1) PALA CARGADORA 0 KM destinada a trabajos en la Comuna</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="inlineStr">
-        <is>
-          <t>26/10/2026</t>
-        </is>
-      </c>
+          <t>Transporte de mil doscientos cincuenta metros cúbicos (1.250 m³) de broza grillada desde Cantera “Tayreta” (Ruta Nacional N° 14 km 135) hasta jurisdicción de la comuna, de acuerdo a los Pliegos de Bases, Condiciones Part iculares y demás documentación</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>26/10/2026, 12:30 horas, Lugar: Sede Administrativa de la Comuna de El Palenque, sito en calle San Martín sin número, El</t>
+          <t>Viernes 09 de octubre del corriente año a las 10:00 hs en la Oficina de la Sede de la Comuna</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2485,11 +2485,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K27" s="4" t="inlineStr">
-        <is>
-          <t>pesos cero ($0,00)</t>
-        </is>
-      </c>
+      <c r="K27" s="4" t="inlineStr"/>
       <c r="L27" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2507,29 +2503,29 @@
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-4b7dfe1bdd0c2ac6</t>
+          <t>id-24e9015ecceeff7f</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>COMUNA DE EL PALENQUE</t>
+          <t>DIAMANTE — MUNICIPALIDAD DE DIAMANTE -- ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2537,24 +2533,16 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>07/26</t>
-        </is>
-      </c>
+      <c r="F28" s="4" t="inlineStr"/>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de UN (1) TRACTOR AGRÍCOLA 0 KM DE HASTA 9 0 HP, CABINADO 4 x4, CON PALA FRONTAL destinado a trabajos en la Comuna</t>
-        </is>
-      </c>
-      <c r="H28" s="4" t="inlineStr">
-        <is>
-          <t>28/10/2026</t>
-        </is>
-      </c>
+          <t>Solicitar Contratación de una empresa para la Obra de “22 (veintidós) cuadras de pavimento urbano” – Grupo 1- según Expte. Letra “D” Nº 2196</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>28/10/2026, 12:40 horas, Lugar: Sede Administrativa de la Comuna de El Palenque, sito en calle San Martín sin número, El</t>
+          <t>viernes 23 de octubre de 2.026, a la hora diez (10.00)</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2562,11 +2550,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K28" s="4" t="inlineStr">
-        <is>
-          <t>pesos cero ($ 0,00)</t>
-        </is>
-      </c>
+      <c r="K28" s="4" t="inlineStr"/>
       <c r="L28" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2584,14 +2568,14 @@
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-54e2b94544e5c76f</t>
+          <t>id-4f207bef5c709ad6</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2599,35 +2583,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C29" s="10" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
+          <t>CONCORDIA — APEX S.A.S</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>07/2026</t>
-        </is>
-      </c>
+          <t>Licitación</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr"/>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Transporte de mil doscientos cincuenta metros cúbicos (1.250 m³) de broza grillada desde Cantera “Tayreta” (Ruta Nacional N° 14 km 135) hasta jurisdicción de la comuna, de acuerdo a los Pliegos de Bases, Condiciones Part iculares y demás documentación</t>
+          <t>instalaciones eléctricas, sanitarias, hidráulicas, mecánicas o de cualquier otra naturaleza relacionada con el sector</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Viernes 09 de octubre del corriente año a las 10:00 hs en la Oficina de la Sede de la Comuna</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2653,14 +2633,14 @@
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-24e9015ecceeff7f</t>
+          <t>id-a20c6b2b6fcf36a2</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2668,31 +2648,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>DIAMANTE — MUNICIPALIDAD DE DIAMANTE -- ENTRE RÍOS</t>
+          <t>Boletín Oficial</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Remate</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr"/>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>Solicitar Contratación de una empresa para la Obra de “22 (veintidós) cuadras de pavimento urbano” – Grupo 1- según Expte. Letra “D” Nº 2196</t>
+          <t>los vehículos se encuentran en exhibición por lo cuál la información registral, de rentas y de infracciones puede ser</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>viernes 23 de octubre de 2.026, a la hora diez (10.00)</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2718,14 +2698,14 @@
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-4f207bef5c709ad6</t>
+          <t>id-fb8d7dc09e202fea</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2733,31 +2713,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>CONCORDIA — APEX S.A.S</t>
+          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Licitación</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>001/26</t>
+        </is>
+      </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>instalaciones eléctricas, sanitarias, hidráulicas, mecánicas o de cualquier otra naturaleza relacionada con el sector</t>
+          <t>ADQUISICIÓN de UN (1) FURGON UTILITARIO CHICO con 5 asientos 0 KM. con destino a Subsecretaria de Asistencia Directa y Emergencia</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>DE LAS PROPUESTAS: 20 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2783,14 +2767,14 @@
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-a20c6b2b6fcf36a2</t>
+          <t>id-ca205f0874380f69</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2798,25 +2782,25 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Boletín Oficial</t>
+          <t>INSTITUTO CARBÓ S.R.L</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Remate</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr"/>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>los vehículos se encuentran en exhibición por lo cuál la información registral, de rentas y de infracciones puede ser</t>
+          <t>sin internación en materia de salud, pre- hospitalarias, atención médica, domiciliaria y traslados sanitarios de alta</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
@@ -2848,7 +2832,7 @@
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-fb8d7dc09e202fea</t>
+          <t>id-6aa57c7437a30ca3</t>
         </is>
       </c>
     </row>
@@ -2863,14 +2847,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C33" s="8" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
+          <t>MUNICIPALIDAD DE VIALE</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2880,18 +2864,18 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>001/26</t>
+          <t>08/26</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN de UN (1) FURGON UTILITARIO CHICO con 5 asientos 0 KM. con destino a Subsecretaria de Asistencia Directa y Emergencia</t>
+          <t>de asf alto 70-16 destinado a la producción de pavimento de la Planta Asfáltica, y que a continuación se detalla y</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>DE LAS PROPUESTAS: 20 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2917,14 +2901,14 @@
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-ca205f0874380f69</t>
+          <t>id-ef1ddb923c7e7fdb</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2939,24 +2923,28 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>INSTITUTO CARBÓ S.R.L</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Licitación</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>sin internación en materia de salud, pre- hospitalarias, atención médica, domiciliaria y traslados sanitarios de alta</t>
+          <t>TERMINACIÓN CONCEPCIÓN DEL URUGUAY 63 VIV</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Publicada 06/10/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -2977,19 +2965,19 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-6aa57c7437a30ca3</t>
+          <t>id-1a3c1f8e036ac91e</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3004,7 +2992,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE VIALE</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3014,18 +3002,18 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>08/26</t>
+          <t>05/2026</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>de asf alto 70-16 destinado a la producción de pavimento de la Planta Asfáltica, y que a continuación se detalla y</t>
+          <t>COMPLEJO HABITACIONAL SAN AGUSTÍN (P</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Publicada 05/10/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3046,19 +3034,19 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-ef1ddb923c7e7fdb</t>
+          <t>id-ccb22bcad9356438</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3083,18 +3071,18 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>03/26</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN CONCEPCIÓN DEL URUGUAY 63 VIV</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2026 — ver pliego</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3120,14 +3108,14 @@
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>id-1a3c1f8e036ac91e</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3152,18 +3140,18 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>05/2026</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>COMPLEJO HABITACIONAL SAN AGUSTÍN (P</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/10/2026 — ver pliego</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3189,7 +3177,7 @@
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>id-ccb22bcad9356438</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
@@ -3221,18 +3209,18 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>03/26</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -3258,7 +3246,7 @@
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
@@ -3290,18 +3278,18 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>02/2026</t>
+          <t>05/2025</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -3327,7 +3315,7 @@
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
@@ -3359,18 +3347,18 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>06/2025</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr"/>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
@@ -3396,7 +3384,7 @@
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
@@ -3426,20 +3414,16 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F41" s="4" t="inlineStr">
-        <is>
-          <t>05/2025</t>
-        </is>
-      </c>
+      <c r="F41" s="4" t="inlineStr"/>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
@@ -3465,7 +3449,7 @@
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
@@ -3497,18 +3481,18 @@
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>06/2025</t>
+          <t>04/2025</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr"/>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr">
@@ -3534,7 +3518,7 @@
       </c>
       <c r="O42" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
@@ -3564,16 +3548,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F43" s="4" t="inlineStr"/>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>03/2025</t>
+        </is>
+      </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr"/>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr">
@@ -3599,7 +3587,7 @@
       </c>
       <c r="O43" s="4" t="inlineStr">
         <is>
-          <t>id-ebeeb6a87e688d85</t>
+          <t>id-75bfffae63b7eedc</t>
         </is>
       </c>
     </row>
@@ -3621,28 +3609,24 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t>04/2025</t>
-        </is>
-      </c>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr"/>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+          <t>CONSTRUCCIÓN DE OBRAS DE ARTE EN EL DEPARTAMENTO LA PAZ. 1) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE EN R.P. S/Nº SOBRE Aº ESTACAS – “CAMINO SAUCECITO” – TRAMO: R.P.Nº 1 – ESCUELA Nº 62 – DISTRITO ESTACAS – DEPARTAMENTO LA PAZ – 2) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE SOBRE Aº ESTACAS SAN GUSTAVO – TRAMO: […]</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr"/>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr">
@@ -3663,19 +3647,19 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O44" s="4" t="inlineStr">
         <is>
-          <t>id-34c85bcdb9b1123f</t>
+          <t>id-3d7728874996f284</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -3683,35 +3667,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="inlineStr">
-        <is>
-          <t>03/2025</t>
-        </is>
-      </c>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr"/>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr"/>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J45" s="4" t="inlineStr">
@@ -3732,19 +3712,19 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O45" s="4" t="inlineStr">
         <is>
-          <t>id-75bfffae63b7eedc</t>
+          <t>id-654eebef400f89cd</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3764,13 +3744,17 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="inlineStr"/>
+          <t>Concurso</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>01/26</t>
+        </is>
+      </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>CONSTRUCCIÓN DE OBRAS DE ARTE EN EL DEPARTAMENTO LA PAZ. 1) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE EN R.P. S/Nº SOBRE Aº ESTACAS – “CAMINO SAUCECITO” – TRAMO: R.P.Nº 1 – ESCUELA Nº 62 – DISTRITO ESTACAS – DEPARTAMENTO LA PAZ – 2) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE SOBRE Aº ESTACAS SAN GUSTAVO – TRAMO: […]</t>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
         </is>
       </c>
       <c r="H46" s="4" t="inlineStr"/>
@@ -3802,7 +3786,7 @@
       </c>
       <c r="O46" s="4" t="inlineStr">
         <is>
-          <t>id-3d7728874996f284</t>
+          <t>id-9a16884dd5a64a49</t>
         </is>
       </c>
     </row>
@@ -3824,18 +3808,22 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr"/>
+          <t>Licitación</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>2026-1227</t>
+        </is>
+      </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
         </is>
       </c>
       <c r="H47" s="4" t="inlineStr"/>
@@ -3862,155 +3850,17 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="O47" s="4" t="inlineStr">
         <is>
-          <t>id-654eebef400f89cd</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C48" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>Concurso</t>
-        </is>
-      </c>
-      <c r="F48" s="4" t="inlineStr">
-        <is>
-          <t>01/26</t>
-        </is>
-      </c>
-      <c r="G48" s="5" t="inlineStr">
-        <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
-        </is>
-      </c>
-      <c r="H48" s="4" t="inlineStr"/>
-      <c r="I48" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J48" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K48" s="4" t="inlineStr"/>
-      <c r="L48" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M48" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
-        </is>
-      </c>
-      <c r="O48" s="4" t="inlineStr">
-        <is>
-          <t>id-9a16884dd5a64a49</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C49" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>ENERSA</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Licitación</t>
-        </is>
-      </c>
-      <c r="F49" s="4" t="inlineStr">
-        <is>
-          <t>2026-1227</t>
-        </is>
-      </c>
-      <c r="G49" s="5" t="inlineStr">
-        <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
-        </is>
-      </c>
-      <c r="H49" s="4" t="inlineStr"/>
-      <c r="I49" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J49" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K49" s="4" t="inlineStr"/>
-      <c r="L49" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M49" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N49" t="inlineStr">
-        <is>
-          <t>ENERSA</t>
-        </is>
-      </c>
-      <c r="O49" s="4" t="inlineStr">
-        <is>
           <t>id-0691eb485d7548eb</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O49"/>
+  <autoFilter ref="A1:O47"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -4104,10 +3954,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId90"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L47" r:id="rId91"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L48" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L49" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M49" r:id="rId96"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 12/10/2026 08:11
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$49</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -62,12 +62,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O47"/>
+  <dimension ref="A1:O49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -649,7 +649,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -659,37 +659,37 @@
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>COLON — MUNICIPALIDAD DE VILLA ELISA (E.R.)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>CONCURSO DE PRECIOS</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>302/2026</t>
+          <t>004/26</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICION DE MAT. PARA LA CONSTRUCCION, ARTICULOS DE FERRETERIA , PINTURERUA Y MAT. ELECTRICOS</t>
+          <t>ADQUISICIÓN DE UN (1) VEHÍCULO PARA TRANSPORTE DE PASAJEROS DE (5) CINCO PLAZAS 0 KM - MODELO/AÑO 2026, PARA LA MUNICIPALIDAD DE LA CIUDAD DE VILLA ELISA, ENTRE RÍOS</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>12/11/2026</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>08-10-2026 08:30</t>
+          <t>12 de NOVIEMBRE de 2026 a la hora 10:00 en la Oficina de Compras de la Municipalidad de Villa Elisa, Entre Ríos</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -697,7 +697,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr"/>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$ 20.000,00 (Pesos Veinte mil con 00/100) el que se puede adquirir en </t>
+        </is>
+      </c>
       <c r="L3" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -710,19 +714,19 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
-          <t>id-2d3ee6d70e7e432c</t>
+          <t>id-bb3703ff360c8c43</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -730,14 +734,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>COLON — MUNICIPALIDAD DE VILLA ELISA (E.R.)</t>
+          <t>MUNICIPALIDAD DE SANTA ELENA</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -747,22 +751,22 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>004/26</t>
+          <t>11/2026</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN DE UN (1) VEHÍCULO PARA TRANSPORTE DE PASAJEROS DE (5) CINCO PLAZAS 0 KM - MODELO/AÑO 2026, PARA LA MUNICIPALIDAD DE LA CIUDAD DE VILLA ELISA, ENTRE RÍOS</t>
+          <t>OBRA "PAVIMENTACION URBANA CALLE TRATADO DEL PILAR B° 3 DE FEBRERO - MUNICIPALIDAD DE SANTA ELENA" (Según Pliegos de Bases y condi ciones)</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>12/11/2026</t>
+          <t>13/10/2026</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>12 de NOVIEMBRE de 2026 a la hora 10:00 en la Oficina de Compras de la Municipalidad de Villa Elisa, Entre Ríos</t>
+          <t>13/10/2026 HORA: 10: 00 HS</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -772,7 +776,7 @@
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>$ 20.000,00 (Pesos Veint e mil con 00/100) el que se puede adquirir en</t>
+          <t>$ 728.000,00 PESOS SETECIENTOS VEINTIOCHO MIL</t>
         </is>
       </c>
       <c r="L4" s="6" t="inlineStr">
@@ -792,7 +796,7 @@
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
-          <t>id-bb3703ff360c8c43</t>
+          <t>id-1a2561509308b1b6</t>
         </is>
       </c>
     </row>
@@ -807,14 +811,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -829,7 +833,7 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>OBRA "PAVIMENTACION URBANA CALLE TRATADO DEL PILAR B° 3 DE FEBRERO - MUNICIPALIDAD DE SANTA ELENA" (Según Pliegos de Bases y condi ciones)</t>
+          <t>REFACCION EN ESCUELA N° 65 “ALMIRANTE BROWN” – CIUDAD DE CONCORDIA - DEPARTAMENTO CONCORDIA - PROVINCIA DE ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -839,19 +843,15 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026 HORA: 10: 00 HS</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 09:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t>$ 728.000,00 PESOS SETECIENTOS VEINTIOCHO MIL</t>
-        </is>
-      </c>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr"/>
       <c r="L5" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -869,7 +869,7 @@
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>id-1a2561509308b1b6</t>
+          <t>id-fc30d5c0b0589a79</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
@@ -901,12 +901,12 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>11/2026</t>
+          <t>13/2026</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>REFACCION EN ESCUELA N° 65 “ALMIRANTE BROWN” – CIUDAD DE CONCORDIA - DEPARTAMENTO CONCORDIA - PROVINCIA DE ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>REPARACIONES VARIAS EN C. P. E. F. Nº 3 “PROFESOR HUGO LA NASA” – CIUDAD DE CONCEPCION DEL URUGUAY - DEPARTAMENTO URUGUAY - PROVINCIA D E ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 09:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -942,7 +942,7 @@
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>id-fc30d5c0b0589a79</t>
+          <t>id-9d3847fb0e2b0929</t>
         </is>
       </c>
     </row>
@@ -957,7 +957,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
@@ -974,12 +974,12 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>13/2026</t>
+          <t>12/2026</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>REPARACIONES VARIAS EN C. P. E. F. Nº 3 “PROFESOR HUGO LA NASA” – CIUDAD DE CONCEPCION DEL URUGUAY - DEPARTAMENTO URUGUAY - PROVINCIA D E ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>RECAMBIO DE CUBIERTA Y REPARACIONES VARIAS EN ESCUELA Nº 92 “CONGRESO DE TUCUMAN” – CONCEPCION DEL URUGUAY - DPTO. URUGUAY – PROVINCIA DE ENTRE RIOS de acuerdo a las c ondiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -989,7 +989,7 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
+          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 10:30 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -1015,7 +1015,7 @@
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>id-9d3847fb0e2b0929</t>
+          <t>id-059239b424b9c936</t>
         </is>
       </c>
     </row>
@@ -1030,14 +1030,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1047,12 +1047,12 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>12/2026</t>
+          <t>87/2026</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>RECAMBIO DE CUBIERTA Y REPARACIONES VARIAS EN ESCUELA Nº 92 “CONGRESO DE TUCUMAN” – CONCEPCION DEL URUGUAY - DPTO. URUGUAY – PROVINCIA DE ENTRE RIOS de acuerdo a las c ondiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>Contratar la ejecución de la obra denominada “Construcción de Red Cloacal Subsidiaria del Colector Noroeste Barrio Ciudad Paisaje”</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -1062,15 +1062,19 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 10:30 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
+          <t>martes, 13 de octubre de 2026 a las 10:00</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
-        </is>
-      </c>
-      <c r="K8" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>$ 10.000 (pesos diez mil)</t>
+        </is>
+      </c>
       <c r="L8" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1083,12 +1087,12 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Boletín Oficial Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>id-059239b424b9c936</t>
+          <t>id-ceeb594e8bcc4ff7</t>
         </is>
       </c>
     </row>
@@ -1110,7 +1114,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>COLON — MUNICIPALIDAD DE COLON</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1118,24 +1122,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>87/2026</t>
-        </is>
-      </c>
+      <c r="F9" s="4" t="inlineStr"/>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Contratar la ejecución de la obra denominada “Construcción de Red Cloacal Subsidiaria del Colector Noroeste Barrio Ciudad Paisaje”</t>
+          <t>“ADQUISICIÓN DE MATERIALES ELÉCTRICOS PARA EJECUCIÓN DEL PROYECTO DE RECONVERSIÓN Y OPTIMIZACIÓN DEL ALUMBRADO PÚBLICO DE LA CIUDAD DE COLÓN”</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026</t>
+          <t>14/10/2026</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>martes, 13 de octubre de 2026 a las 10:00</t>
+          <t>14 de OCTUBRE de 2026</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1145,7 +1145,7 @@
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>$ 10.000 (pesos diez mil)</t>
+          <t>Sin Cargo</t>
         </is>
       </c>
       <c r="L9" s="6" t="inlineStr">
@@ -1160,12 +1160,12 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Boletín Oficial Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>id-ceeb594e8bcc4ff7</t>
+          <t>id-9e122d52de12ffef</t>
         </is>
       </c>
     </row>
@@ -1180,14 +1180,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>COLON — MUNICIPALIDAD DE COLON</t>
+          <t>DIAMANTE — COMUNA ALDEA PROTESTANTE -- DIAMANTE -- ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1195,10 +1195,14 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr"/>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>03/2026</t>
+        </is>
+      </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN DE MATERIALES ELÉCTRICOS PARA EJECUCIÓN DEL PROYECTO DE RECONVERSIÓN Y OPTIMIZACIÓN DEL ALUMBRADO PÚBLICO DE LA CIUDAD DE COLÓN”</t>
+          <t>Conforme a lo autorizado por decreto Nº 290/26 llámese a licitación pública Nº 03/26 con el objeto de comprar 10 toneladas de emulsión catiónica súper estable (asfalto de imprimación), puesto en Aldea Protestante</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -1208,7 +1212,7 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>14 de OCTUBRE de 2026</t>
+          <t>miércoles 14 de octubre de 2026 – Hora nueve (09:00) Lugar de presentación de la oferta: Sede Comuna Aldea Protestan</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1216,11 +1220,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr">
-        <is>
-          <t>Sin Cargo</t>
-        </is>
-      </c>
+      <c r="K10" s="4" t="inlineStr"/>
       <c r="L10" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>id-9e122d52de12ffef</t>
+          <t>id-c2f3a25cfb37fd38</t>
         </is>
       </c>
     </row>
@@ -1253,14 +1253,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>DIAMANTE — COMUNA ALDEA PROTESTANTE -- DIAMANTE -- ENTRE RÍOS</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1270,12 +1270,12 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>03/2026</t>
+          <t>017/2026</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Conforme a lo autorizado por decreto Nº 290/26 llámese a licitación pública Nº 03/26 con el objeto de comprar 10 toneladas de emulsión catiónica súper estable (asfalto de imprimación), puesto en Aldea Protestante</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de UNA (1) MOTONIVELADORA, nueva, sin uso, cero km, con una potencia entre 220/240 HP, con opción a implementos, que será utilizada para el área del corralón municipal</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1285,7 +1285,7 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>miércoles 14 de octubre de 2026 – Hora nueve (09:00) Lugar de presentación de la oferta: Sede Comuna Aldea Protestan</t>
+          <t>14 DE OCTUBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1293,7 +1293,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K11" s="4" t="inlineStr"/>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>$100.000,00. - (PESOS CIEN MIL CON 00/100) PRESUPUESTO OFICIAL ESTIMAD</t>
+        </is>
+      </c>
       <c r="L11" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1311,7 +1315,7 @@
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>id-c2f3a25cfb37fd38</t>
+          <t>id-4c3b33859e596759</t>
         </is>
       </c>
     </row>
@@ -1326,14 +1330,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>Vehículos</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
+          <t>VICTORIA — MUNICIPALIDAD DE VICTORIA</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1343,12 +1347,12 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>017/2026</t>
+          <t>008/2026</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de UNA (1) MOTONIVELADORA, nueva, sin uso, cero km, con una potencia entre 220/240 HP, con opción a implementos, que será utilizada para el área del corralón municipal</t>
+          <t>Proveer a la Municipalidad de Victoria, Entre Ríos, de Veinticinco Mil (25.000) litros de Diésel 500, para movilidad de vehículos y maquinarias viales , Ocho Mil (8.000) litros de Gasoil Tipo euro o similar y Ocho (8.000) litros de nafta súper para vehículos y áreas afectadas a la Secretaria de Planeamiento y Dirección de Ambiente y Desarrollo sostenible;</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -1358,7 +1362,7 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>14 DE OCTUBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>14 de octubre de 2026 a las 09:00 hs., en la Oficina de Compras de la Municipalidad de Victoria, Entr</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
@@ -1366,11 +1370,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr">
-        <is>
-          <t>$100.000,00. - (PESOS CIEN MIL CON 00/100) PRESUPUESTO OFICIAL ESTIMAD</t>
-        </is>
-      </c>
+      <c r="K12" s="4" t="inlineStr"/>
       <c r="L12" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1388,14 +1388,14 @@
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>id-4c3b33859e596759</t>
+          <t>id-a9af9f59c8c487c8</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1403,29 +1403,29 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>Vehículos</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>VICTORIA — MUNICIPALIDAD DE VICTORIA</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>LICITACIÓN PÚBLICA</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>008/2026</t>
+          <t>89/2026</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Proveer a la Municipalidad de Victoria, Entre Ríos, de Veinticinco Mil (25.000) litros de Diésel 500, para movilidad de vehículos y maquinarias viales , Ocho Mil (8.000) litros de Gasoil Tipo euro o similar y Ocho (8.000) litros de nafta súper para vehículos y áreas afectadas a la Secretaria de Planeamiento y Dirección de Ambiente y Desarrollo sostenible;</t>
+          <t>ADQUISICION DE BALANZA BASCULA PARA PESAJE DE EJESDE CAMIONES</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
@@ -1435,7 +1435,7 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>14 de octubre de 2026 a las 09:00 hs., en la Oficina de Compras de la Municipalidad de Victoria, Entr</t>
+          <t>14-10-2026 08:00</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -1456,19 +1456,19 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>id-a9af9f59c8c487c8</t>
+          <t>id-4ee814ba6420f0cc</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>12/10/2026</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1476,7 +1476,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>Vehículos</t>
         </is>
@@ -1488,17 +1488,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA</t>
+          <t>LICITACION PRIVADA</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>89/2026</t>
+          <t>77/2026</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICION DE BALANZA BASCULA PARA PESAJE DE EJESDE CAMIONES</t>
+          <t>SERVICIO DE ALQUILER DE RETROEXCAVADORA, MINICARGADORA, CAMION VOLCADOR Y PISON VIBRATORIO</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>14-10-2026 08:00</t>
+          <t>14-10-2026 09:00</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1534,7 +1534,7 @@
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>id-4ee814ba6420f0cc</t>
+          <t>id-12335630ae6fd191</t>
         </is>
       </c>
     </row>
@@ -1549,7 +1549,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>Vehículos</t>
         </is>
@@ -1622,7 +1622,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>Vehículos</t>
         </is>
@@ -1644,7 +1644,7 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN DE UNA MÁQUINA MOTONIVELADORA PARA INCORPORAR AL PARQUE AUTOMOTOR DE LA MUNICIP ALIDAD DE ALDEA SAN ANTONIO</t>
+          <t>ADQUISICIÓN DE UNA MÁQUINA MOTONIVELADORA PARA INCORPORAR AL PARQUE AUTOMOTOR DE LA MUNICIPALIDAD DE ALDEA SAN ANTONIO</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
@@ -1841,7 +1841,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>12/10/2026</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1849,39 +1849,39 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>INSTITUTO AUTÁRQUICO DE PLANEAMIENTO YY VIVIENDA — URUGUAY</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>CONCURSO DE PRECIOS</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>322/2026</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN CONCEPCIÓN DEL URUGUAY 63 VIV. ETAPA I 17 VIV. (P. P.) DEPARTAMENTO: URUGUAY PRESUPUESTO OFICIAL Obras de Viviendas y Complem entarias: $ 1.042.925.971,90 y su equivalente UVIs 693.301,14 Obras de Infraestructuras y Nexos $ 344.554.736,26 y su equivalente UVIs 229.048,08</t>
+          <t>REPARACION DE MOTOR COMPLETO SEGUN DETALLES</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>17/11/2026</t>
+          <t>16/10/2026</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>DÍA: 17/11/2026 HOR A: 10:00 HS</t>
+          <t>16-10-2026 08:15</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1889,11 +1889,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K19" s="4" t="inlineStr">
-        <is>
-          <t>$ 138.748,07</t>
-        </is>
-      </c>
+      <c r="K19" s="4" t="inlineStr"/>
       <c r="L19" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1906,12 +1902,12 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>id-b0fe9ebcdc39e73a</t>
+          <t>id-823d486904965498</t>
         </is>
       </c>
     </row>
@@ -1999,7 +1995,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
+      <c r="C21" s="7" t="inlineStr">
         <is>
           <t>Vehículos</t>
         </is>
@@ -2145,7 +2141,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
@@ -2222,7 +2218,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C24" s="8" t="inlineStr">
         <is>
           <t>Arquitectura</t>
         </is>
@@ -2295,7 +2291,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C25" s="8" t="inlineStr">
+      <c r="C25" s="7" t="inlineStr">
         <is>
           <t>Vehículos</t>
         </is>
@@ -2372,7 +2368,7 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C26" s="8" t="inlineStr">
+      <c r="C26" s="7" t="inlineStr">
         <is>
           <t>Vehículos</t>
         </is>
@@ -2394,7 +2390,7 @@
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de UN (1) TRACTOR AGRÍCOLA 0 KM DE HASTA 9 0 HP, CABINADO 4 x4, CON PALA FRONTAL destinado a trabajos en la Comuna</t>
+          <t>Adquisición de UN (1) TRACTOR AGRÍCOLA 0 KM DE HASTA 90 HP, CABINADO 4 x4, CON PALA FRONTAL destinado a trabajos en la Comuna</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
@@ -2441,22 +2437,22 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C27" s="10" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
+          <t>VILLAGUAY — COMUNA DE MOJONES SUD YY PARAJE LOS ALGARROBOS</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2464,20 +2460,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>07/2026</t>
-        </is>
-      </c>
+      <c r="F27" s="4" t="inlineStr"/>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>Transporte de mil doscientos cincuenta metros cúbicos (1.250 m³) de broza grillada desde Cantera “Tayreta” (Ruta Nacional N° 14 km 135) hasta jurisdicción de la comuna, de acuerdo a los Pliegos de Bases, Condiciones Part iculares y demás documentación</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="inlineStr"/>
+          <t>ADQUISICIÓN DE MOTONIVELADORA USADA</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>29/10/2026</t>
+        </is>
+      </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>Viernes 09 de octubre del corriente año a las 10:00 hs en la Oficina de la Sede de la Comuna</t>
+          <t>29/10/2026 a las 16:30 hs</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2485,7 +2481,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K27" s="4" t="inlineStr"/>
+      <c r="K27" s="4" t="inlineStr">
+        <is>
+          <t>$ 10.000 (PESOS DIEZ MIL)</t>
+        </is>
+      </c>
       <c r="L27" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2503,14 +2503,14 @@
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-24e9015ecceeff7f</t>
+          <t>id-2aa97e0762afa9ea</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>12/10/2026</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2518,14 +2518,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>DIAMANTE — MUNICIPALIDAD DE DIAMANTE -- ENTRE RÍOS</t>
+          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2533,16 +2533,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr"/>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>002/26</t>
+        </is>
+      </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Solicitar Contratación de una empresa para la Obra de “22 (veintidós) cuadras de pavimento urbano” – Grupo 1- según Expte. Letra “D” Nº 2196</t>
+          <t>ADQUISICIÓN de UN (1) TRACTOR 4 x4 C/CABINA DE 90 A 100 HP - 0 Km. con destino a Secretaria de Obras y Servicios Publicos</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>viernes 23 de octubre de 2.026, a la hora diez (10.00)</t>
+          <t>DE LAS PROPUESTAS: 28 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2568,14 +2572,14 @@
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-4f207bef5c709ad6</t>
+          <t>id-da43a5f725393cbf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2583,31 +2587,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>CONCORDIA — APEX S.A.S</t>
+          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Licitación</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>07/2026</t>
+        </is>
+      </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>instalaciones eléctricas, sanitarias, hidráulicas, mecánicas o de cualquier otra naturaleza relacionada con el sector</t>
+          <t>Transporte de mil doscientos cincuenta metros cúbicos (1.250 m³) de broza grillada desde Cantera “Tayreta” (Ruta Nacional N° 14 km 135) hasta jurisdicción de la comuna, de acuerdo a los Pliegos de Bases, Condiciones Part iculares y demás documentación</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Viernes 09 de octubre del corriente año a las 10:00 hs en la Oficina de la Sede de la Comuna</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2633,14 +2641,14 @@
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-a20c6b2b6fcf36a2</t>
+          <t>id-24e9015ecceeff7f</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2648,31 +2656,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C30" s="8" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Boletín Oficial</t>
+          <t>DIAMANTE — MUNICIPALIDAD DE DIAMANTE -- ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Remate</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr"/>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>los vehículos se encuentran en exhibición por lo cuál la información registral, de rentas y de infracciones puede ser</t>
+          <t>Solicitar Contratación de una empresa para la Obra de “22 (veintidós) cuadras de pavimento urbano” – Grupo 1- según Expte. Letra “D” Nº 2196</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>viernes 23 de octubre de 2.026, a la hora diez (10.00)</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2698,14 +2706,14 @@
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-fb8d7dc09e202fea</t>
+          <t>id-4f207bef5c709ad6</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2713,35 +2721,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C31" s="8" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
+          <t>CONCORDIA — APEX S.A.S</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>001/26</t>
-        </is>
-      </c>
+          <t>Licitación</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr"/>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN de UN (1) FURGON UTILITARIO CHICO con 5 asientos 0 KM. con destino a Subsecretaria de Asistencia Directa y Emergencia</t>
+          <t>instalaciones eléctricas, sanitarias, hidráulicas, mecánicas o de cualquier otra naturaleza relacionada con el sector</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>DE LAS PROPUESTAS: 20 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2767,14 +2771,14 @@
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-ca205f0874380f69</t>
+          <t>id-a20c6b2b6fcf36a2</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2782,25 +2786,25 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>INSTITUTO CARBÓ S.R.L</t>
+          <t>Boletín Oficial</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Remate</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr"/>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>sin internación en materia de salud, pre- hospitalarias, atención médica, domiciliaria y traslados sanitarios de alta</t>
+          <t>los vehículos se encuentran en exhibición por lo cuál la información registral, de rentas y de infracciones puede ser</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
@@ -2832,7 +2836,7 @@
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-6aa57c7437a30ca3</t>
+          <t>id-fb8d7dc09e202fea</t>
         </is>
       </c>
     </row>
@@ -2847,14 +2851,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE VIALE</t>
+          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2864,18 +2868,18 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>08/26</t>
+          <t>001/26</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>de asf alto 70-16 destinado a la producción de pavimento de la Planta Asfáltica, y que a continuación se detalla y</t>
+          <t>ADQUISICIÓN de UN (1) FURGON UTILITARIO CHICO con 5 asientos 0 KM. con destino a Subsecretaria de Asistencia Directa y Emergencia</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>DE LAS PROPUESTAS: 20 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2901,14 +2905,14 @@
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-ef1ddb923c7e7fdb</t>
+          <t>id-ca205f0874380f69</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2923,28 +2927,24 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>INSTITUTO CARBÓ S.R.L</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t>04/2026</t>
-        </is>
-      </c>
+          <t>Licitación</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr"/>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN CONCEPCIÓN DEL URUGUAY 63 VIV</t>
+          <t>sin internación en materia de salud, pre- hospitalarias, atención médica, domiciliaria y traslados sanitarios de alta</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2026 — ver pliego</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -2965,19 +2965,19 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-1a3c1f8e036ac91e</t>
+          <t>id-6aa57c7437a30ca3</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>MUNICIPALIDAD DE VIALE</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3002,18 +3002,18 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>05/2026</t>
+          <t>08/26</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>COMPLEJO HABITACIONAL SAN AGUSTÍN (P</t>
+          <t>de asf alto 70-16 destinado a la producción de pavimento de la Planta Asfáltica, y que a continuación se detalla y</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/10/2026 — ver pliego</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3034,19 +3034,19 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-ccb22bcad9356438</t>
+          <t>id-ef1ddb923c7e7fdb</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3071,18 +3071,18 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>03/26</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+          <t>TERMINACIÓN CONCEPCIÓN DEL URUGUAY 63 VIV</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>Publicada 06/10/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3108,14 +3108,14 @@
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-1a3c1f8e036ac91e</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3140,18 +3140,18 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>02/2026</t>
+          <t>05/2026</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+          <t>COMPLEJO HABITACIONAL SAN AGUSTÍN (P</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>Publicada 05/10/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3177,7 +3177,7 @@
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-ccb22bcad9356438</t>
         </is>
       </c>
     </row>
@@ -3209,18 +3209,18 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>03/26</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -3246,7 +3246,7 @@
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
@@ -3278,18 +3278,18 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>05/2025</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -3315,7 +3315,7 @@
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
@@ -3347,18 +3347,18 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>06/2025</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr"/>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
@@ -3384,7 +3384,7 @@
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
@@ -3414,16 +3414,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F41" s="4" t="inlineStr"/>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>05/2025</t>
+        </is>
+      </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
@@ -3449,7 +3453,7 @@
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
-          <t>id-ebeeb6a87e688d85</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
@@ -3481,18 +3485,18 @@
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>04/2025</t>
+          <t>06/2025</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr"/>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr">
@@ -3518,7 +3522,7 @@
       </c>
       <c r="O42" s="4" t="inlineStr">
         <is>
-          <t>id-34c85bcdb9b1123f</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
@@ -3548,20 +3552,16 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F43" s="4" t="inlineStr">
-        <is>
-          <t>03/2025</t>
-        </is>
-      </c>
+      <c r="F43" s="4" t="inlineStr"/>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr"/>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="O43" s="4" t="inlineStr">
         <is>
-          <t>id-75bfffae63b7eedc</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
@@ -3609,24 +3609,28 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F44" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>04/2025</t>
+        </is>
+      </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>CONSTRUCCIÓN DE OBRAS DE ARTE EN EL DEPARTAMENTO LA PAZ. 1) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE EN R.P. S/Nº SOBRE Aº ESTACAS – “CAMINO SAUCECITO” – TRAMO: R.P.Nº 1 – ESCUELA Nº 62 – DISTRITO ESTACAS – DEPARTAMENTO LA PAZ – 2) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE SOBRE Aº ESTACAS SAN GUSTAVO – TRAMO: […]</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr"/>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr">
@@ -3647,19 +3651,19 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O44" s="4" t="inlineStr">
         <is>
-          <t>id-3d7728874996f284</t>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -3667,31 +3671,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C45" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>03/2025</t>
+        </is>
+      </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr"/>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>Ver pliego</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J45" s="4" t="inlineStr">
@@ -3712,19 +3720,19 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O45" s="4" t="inlineStr">
         <is>
-          <t>id-654eebef400f89cd</t>
+          <t>id-75bfffae63b7eedc</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3744,17 +3752,13 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Concurso</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="inlineStr">
-        <is>
-          <t>01/26</t>
-        </is>
-      </c>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr"/>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>CONSTRUCCIÓN DE OBRAS DE ARTE EN EL DEPARTAMENTO LA PAZ. 1) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE EN R.P. S/Nº SOBRE Aº ESTACAS – “CAMINO SAUCECITO” – TRAMO: R.P.Nº 1 – ESCUELA Nº 62 – DISTRITO ESTACAS – DEPARTAMENTO LA PAZ – 2) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE SOBRE Aº ESTACAS SAN GUSTAVO – TRAMO: […]</t>
         </is>
       </c>
       <c r="H46" s="4" t="inlineStr"/>
@@ -3786,7 +3790,7 @@
       </c>
       <c r="O46" s="4" t="inlineStr">
         <is>
-          <t>id-9a16884dd5a64a49</t>
+          <t>id-3d7728874996f284</t>
         </is>
       </c>
     </row>
@@ -3808,22 +3812,18 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>ENERSA</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Licitación</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr">
-        <is>
-          <t>2026-1227</t>
-        </is>
-      </c>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr"/>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
         </is>
       </c>
       <c r="H47" s="4" t="inlineStr"/>
@@ -3850,17 +3850,155 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="O47" s="4" t="inlineStr">
+        <is>
+          <t>id-654eebef400f89cd</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Concurso</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>01/26</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+        </is>
+      </c>
+      <c r="H48" s="4" t="inlineStr"/>
+      <c r="I48" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J48" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K48" s="4" t="inlineStr"/>
+      <c r="L48" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M48" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>Vialidad Entre Ríos (DPV)</t>
+        </is>
+      </c>
+      <c r="O48" s="4" t="inlineStr">
+        <is>
+          <t>id-9a16884dd5a64a49</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C49" s="9" t="inlineStr">
+        <is>
+          <t>Materiales</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
           <t>ENERSA</t>
         </is>
       </c>
-      <c r="O47" s="4" t="inlineStr">
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Licitación</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>2026-1227</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="inlineStr"/>
+      <c r="I49" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="J49" s="4" t="inlineStr">
+        <is>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K49" s="4" t="inlineStr"/>
+      <c r="L49" s="6" t="inlineStr">
+        <is>
+          <t>ver licitación</t>
+        </is>
+      </c>
+      <c r="M49" s="6" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>ENERSA</t>
+        </is>
+      </c>
+      <c r="O49" s="4" t="inlineStr">
         <is>
           <t>id-0691eb485d7548eb</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O47"/>
+  <autoFilter ref="A1:O49"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -3954,6 +4092,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId90"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L47" r:id="rId91"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L48" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L49" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M49" r:id="rId96"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 13/10/2026 08:44
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$46</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -67,12 +67,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
+        <fgColor rgb="00E6D9F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E6D9F2"/>
+        <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O49"/>
+  <dimension ref="A1:O46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -811,14 +811,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -828,12 +828,12 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>11/2026</t>
+          <t>87/2026</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>REFACCION EN ESCUELA N° 65 “ALMIRANTE BROWN” – CIUDAD DE CONCORDIA - DEPARTAMENTO CONCORDIA - PROVINCIA DE ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>Contratar la ejecución de la obra denominada “Construcción de Red Cloacal Subsidiaria del Colector Noroeste Barrio Ciudad Paisaje”</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -843,15 +843,19 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 09:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
+          <t>martes, 13 de octubre de 2026 a las 10:00</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
-        </is>
-      </c>
-      <c r="K5" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>$ 10.000 (pesos diez mil)</t>
+        </is>
+      </c>
       <c r="L5" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -864,12 +868,12 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Boletín Oficial Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>id-fc30d5c0b0589a79</t>
+          <t>id-ceeb594e8bcc4ff7</t>
         </is>
       </c>
     </row>
@@ -884,14 +888,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
+          <t>COLON — MUNICIPALIDAD DE COLON</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -899,32 +903,32 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>13/2026</t>
-        </is>
-      </c>
+      <c r="F6" s="4" t="inlineStr"/>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>REPARACIONES VARIAS EN C. P. E. F. Nº 3 “PROFESOR HUGO LA NASA” – CIUDAD DE CONCEPCION DEL URUGUAY - DEPARTAMENTO URUGUAY - PROVINCIA D E ENTRE RÍOS de acuerdo a las condiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>“ADQUISICIÓN DE MATERIALES ELÉCTRICOS PARA EJECUCIÓN DEL PROYECTO DE RECONVERSIÓN Y OPTIMIZACIÓN DEL ALUMBRADO PÚBLICO DE LA CIUDAD DE COLÓN”</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026</t>
+          <t>14/10/2026</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 12:00 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
+          <t>14 de OCTUBRE de 2026</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="inlineStr"/>
+          <t>Ver pliego</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>Sin Cargo</t>
+        </is>
+      </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -942,7 +946,7 @@
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>id-9d3847fb0e2b0929</t>
+          <t>id-9e122d52de12ffef</t>
         </is>
       </c>
     </row>
@@ -959,12 +963,12 @@
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Arquitectura</t>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>COMISIÓN ADMINISTRADORA PARA EL FONDO ESPECIAL — DE SALTO GRANDE</t>
+          <t>DIAMANTE — COMUNA ALDEA PROTESTANTE -- DIAMANTE -- ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -974,27 +978,27 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>12/2026</t>
+          <t>03/2026</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>RECAMBIO DE CUBIERTA Y REPARACIONES VARIAS EN ESCUELA Nº 92 “CONGRESO DE TUCUMAN” – CONCEPCION DEL URUGUAY - DPTO. URUGUAY – PROVINCIA DE ENTRE RIOS de acuerdo a las c ondiciones que se detallan en los pliegos, aprobados por el Directorio de C.A.F.E.S.G</t>
+          <t>Conforme a lo autorizado por decreto Nº 290/26 llámese a licitación pública Nº 03/26 con el objeto de comprar 10 toneladas de emulsión catiónica súper estable (asfalto de imprimación), puesto en Aldea Protestante</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026</t>
+          <t>14/10/2026</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>Martes 13 DE OCTUBRE DEL AÑO 2026.- Hora: 10:30 Lugar: OFICINAS CENTRALES DE LA CAFESG – CALLE SAN JUAN Nº 2097 – CIUDAD</t>
+          <t>miércoles 14 de octubre de 2026 – Hora nueve (09:00) Lugar de presentación de la oferta: Sede Comuna Aldea Protestan</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>06/10/2026</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr"/>
@@ -1015,7 +1019,7 @@
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>id-059239b424b9c936</t>
+          <t>id-c2f3a25cfb37fd38</t>
         </is>
       </c>
     </row>
@@ -1030,14 +1034,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1047,22 +1051,22 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>87/2026</t>
+          <t>017/2026</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Contratar la ejecución de la obra denominada “Construcción de Red Cloacal Subsidiaria del Colector Noroeste Barrio Ciudad Paisaje”</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de UNA (1) MOTONIVELADORA, nueva, sin uso, cero km, con una potencia entre 220/240 HP, con opción a implementos, que será utilizada para el área del corralón municipal</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026</t>
+          <t>14/10/2026</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>martes, 13 de octubre de 2026 a las 10:00</t>
+          <t>14 DE OCTUBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -1072,7 +1076,7 @@
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>$ 10.000 (pesos diez mil)</t>
+          <t>$100.000,00. - (PESOS CIEN MIL CON 00/100) PRESUPUESTO OFICIAL ESTIMAD</t>
         </is>
       </c>
       <c r="L8" s="6" t="inlineStr">
@@ -1087,12 +1091,12 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Boletín Oficial Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>id-ceeb594e8bcc4ff7</t>
+          <t>id-4c3b33859e596759</t>
         </is>
       </c>
     </row>
@@ -1107,14 +1111,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>COLON — MUNICIPALIDAD DE COLON</t>
+          <t>VICTORIA — MUNICIPALIDAD DE VICTORIA</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1122,10 +1126,14 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr"/>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>008/2026</t>
+        </is>
+      </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN DE MATERIALES ELÉCTRICOS PARA EJECUCIÓN DEL PROYECTO DE RECONVERSIÓN Y OPTIMIZACIÓN DEL ALUMBRADO PÚBLICO DE LA CIUDAD DE COLÓN”</t>
+          <t>Proveer a la Municipalidad de Victoria, Entre Ríos, de Veinticinco Mil (25.000) litros de Diésel 500, para movilidad de vehículos y maquinarias viales , Ocho Mil (8.000) litros de Gasoil Tipo euro o similar y Ocho (8.000) litros de nafta súper para vehículos y áreas afectadas a la Secretaria de Planeamiento y Dirección de Ambiente y Desarrollo sostenible;</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -1135,7 +1143,7 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>14 de OCTUBRE de 2026</t>
+          <t>14 de octubre de 2026 a las 09:00 hs., en la Oficina de Compras de la Municipalidad de Victoria, Entr</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1143,11 +1151,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>Sin Cargo</t>
-        </is>
-      </c>
+      <c r="K9" s="4" t="inlineStr"/>
       <c r="L9" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1165,14 +1169,14 @@
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>id-9e122d52de12ffef</t>
+          <t>id-a9af9f59c8c487c8</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1180,29 +1184,29 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>DIAMANTE — COMUNA ALDEA PROTESTANTE -- DIAMANTE -- ENTRE RÍOS</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>LICITACIÓN PÚBLICA</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>03/2026</t>
+          <t>89/2026</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Conforme a lo autorizado por decreto Nº 290/26 llámese a licitación pública Nº 03/26 con el objeto de comprar 10 toneladas de emulsión catiónica súper estable (asfalto de imprimación), puesto en Aldea Protestante</t>
+          <t>ADQUISICION DE BALANZA BASCULA PARA PESAJE DE EJESDE CAMIONES</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -1212,7 +1216,7 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>miércoles 14 de octubre de 2026 – Hora nueve (09:00) Lugar de presentación de la oferta: Sede Comuna Aldea Protestan</t>
+          <t>14-10-2026 08:00</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1233,19 +1237,19 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>id-c2f3a25cfb37fd38</t>
+          <t>id-4ee814ba6420f0cc</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>12/10/2026</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1260,22 +1264,22 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>LICITACION PRIVADA</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>017/2026</t>
+          <t>77/2026</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de UNA (1) MOTONIVELADORA, nueva, sin uso, cero km, con una potencia entre 220/240 HP, con opción a implementos, que será utilizada para el área del corralón municipal</t>
+          <t>SERVICIO DE ALQUILER DE RETROEXCAVADORA, MINICARGADORA, CAMION VOLCADOR Y PISON VIBRATORIO</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1285,7 +1289,7 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>14 DE OCTUBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>14-10-2026 09:00</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1293,11 +1297,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K11" s="4" t="inlineStr">
-        <is>
-          <t>$100.000,00. - (PESOS CIEN MIL CON 00/100) PRESUPUESTO OFICIAL ESTIMAD</t>
-        </is>
-      </c>
+      <c r="K11" s="4" t="inlineStr"/>
       <c r="L11" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1310,19 +1310,19 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>id-4c3b33859e596759</t>
+          <t>id-12335630ae6fd191</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1337,7 +1337,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>VICTORIA — MUNICIPALIDAD DE VICTORIA</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1347,12 +1347,12 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>008/2026</t>
+          <t>89/2026</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Proveer a la Municipalidad de Victoria, Entre Ríos, de Veinticinco Mil (25.000) litros de Diésel 500, para movilidad de vehículos y maquinarias viales , Ocho Mil (8.000) litros de Gasoil Tipo euro o similar y Ocho (8.000) litros de nafta súper para vehículos y áreas afectadas a la Secretaria de Planeamiento y Dirección de Ambiente y Desarrollo sostenible;</t>
+          <t>Adquisición de balanzas básculas para pesaje de ejes de camiones</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -1362,7 +1362,7 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>14 de octubre de 2026 a las 09:00 hs., en la Oficina de Compras de la Municipalidad de Victoria, Entr</t>
+          <t>miércoles, 14 de octubre de 2026 a las 08:00</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
@@ -1383,12 +1383,12 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Boletín Oficial Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>id-a9af9f59c8c487c8</t>
+          <t>id-d963348e34fcb0d3</t>
         </is>
       </c>
     </row>
@@ -1410,32 +1410,32 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE ALDEA SAN ANTONIO</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>89/2026</t>
+          <t>002/2026</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICION DE BALANZA BASCULA PARA PESAJE DE EJESDE CAMIONES</t>
+          <t>ADQUISICIÓN DE UNA MÁQUINA MOTONIVELADORA PARA INCORPORAR AL PARQUE AUTOMOTOR DE LA MUNICIPALIDAD DE ALDEA SAN ANTONIO</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>14/10/2026</t>
+          <t>15/10/2026</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>14-10-2026 08:00</t>
+          <t>15 de octubre de 2026, a las 08:00 horas, en el Edificio Municipal</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -1443,7 +1443,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K13" s="4" t="inlineStr"/>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>PESOS CIEN MIL con 00/100 ($ 100.000,00. -)</t>
+        </is>
+      </c>
       <c r="L13" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1456,19 +1460,19 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>id-4ee814ba6420f0cc</t>
+          <t>id-95a507b67b7b1450</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>12/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1476,39 +1480,39 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>MINISTERIO DE SALUD — GOBIERNO DE ENTRE RIOS</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>LICITACION PRIVADA</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>77/2026</t>
+          <t>18/26</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE ALQUILER DE RETROEXCAVADORA, MINICARGADORA, CAMION VOLCADOR Y PISON VIBRATORIO</t>
+          <t>Adquirir Sesenta Mil (60.000) Kilogramos de Leche Entera en Polvo Instantánea, Fortificada con Hierro, Zinc y Ácido Ascórbico</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>14/10/2026</t>
+          <t>16/10/2026</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>14-10-2026 09:00</t>
+          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1516,7 +1520,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K14" s="4" t="inlineStr"/>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>PESOS TRES MIL QUINIENTOS ($ 3.500,00)</t>
+        </is>
+      </c>
       <c r="L14" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1529,19 +1537,19 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>id-12335630ae6fd191</t>
+          <t>id-04a917d50ccab2e3</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1549,14 +1557,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>VILLAGUAY — MUNICIPALIDAD DE VILLAGUAY</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1564,24 +1572,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>89/2026</t>
-        </is>
-      </c>
+      <c r="F15" s="4" t="inlineStr"/>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de balanzas básculas para pesaje de ejes de camiones</t>
+          <t>Contratación, ejecución, liquidación, pago y recepción de la obra destinada a la elaboración del Proyecto Ejecutivo, provisión de materiales, mano de obra, equipos, ejecución, ensayos, habilitación y puesta en servicio de la instalación de gas natural para la Planta Municipal de Elaboración de Mezcla Asfáltica en Caliente, ubicada en el Lote N.º 4 de la Chacra N.º 263 del Parque Industrial de Villaguay, Provincia de Entre Ríos. La contratación comprender á una solución integral bajo modalidad “llave en mano”, incluyendo todos los trabajos, provisiones, trámites, representaciones técnicas, insp</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>14/10/2026</t>
+          <t>16/10/2026</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 14 de octubre de 2026 a las 08:00</t>
+          <t>16 de octubre del año 2026 a las 10:00 Horas, la que se reali zara en la Oficina de suministros de la Municipalidad de V</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1589,7 +1593,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K15" s="4" t="inlineStr"/>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>$ 50.000,00</t>
+        </is>
+      </c>
       <c r="L15" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1602,19 +1610,19 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Boletín Oficial Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>id-d963348e34fcb0d3</t>
+          <t>id-55f1e5ca423a9262</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>12/10/2026</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1622,39 +1630,39 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE ALDEA SAN ANTONIO</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>CONCURSO DE PRECIOS</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>002/2026</t>
+          <t>322/2026</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN DE UNA MÁQUINA MOTONIVELADORA PARA INCORPORAR AL PARQUE AUTOMOTOR DE LA MUNICIPALIDAD DE ALDEA SAN ANTONIO</t>
+          <t>REPARACION DE MOTOR COMPLETO SEGUN DETALLES</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>15/10/2026</t>
+          <t>16/10/2026</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>15 de octubre de 2026, a las 08:00 horas, en el Edificio Municipal</t>
+          <t>16-10-2026 08:15</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -1662,11 +1670,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K16" s="4" t="inlineStr">
-        <is>
-          <t>PESOS CIEN MIL con 00/100 ($ 100.000,00. -)</t>
-        </is>
-      </c>
+      <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1679,12 +1683,12 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>id-95a507b67b7b1450</t>
+          <t>id-823d486904965498</t>
         </is>
       </c>
     </row>
@@ -1699,14 +1703,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>MINISTERIO DE SALUD — GOBIERNO DE ENTRE RIOS</t>
+          <t>SALUD ENTRE RÍOS S.A.U</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1714,24 +1718,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>18/26</t>
-        </is>
-      </c>
+      <c r="F17" s="4" t="inlineStr"/>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Adquirir Sesenta Mil (60.000) Kilogramos de Leche Entera en Polvo Instantánea, Fortificada con Hierro, Zinc y Ácido Ascórbico</t>
+          <t>Contratación de Servicio de Viandas para el Hospital de la Baxada</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>16/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
+          <t>Hospital de la Baxada, calle Gral. Al varado Nº 2.250 Paraná, Entre Ríos, el día 19/10/2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1741,7 +1741,7 @@
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t>PESOS TRES MIL QUINIENTOS ($ 3.500,00)</t>
+          <t>Ninguno</t>
         </is>
       </c>
       <c r="L17" s="6" t="inlineStr">
@@ -1761,14 +1761,14 @@
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>id-04a917d50ccab2e3</t>
+          <t>id-d35d5e849089d7ac</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1776,9 +1776,9 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1794,17 +1794,17 @@
       <c r="F18" s="4" t="inlineStr"/>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Contratación, ejecución, liquidación, pago y recepción de la obra destinada a la elaboración del Proyecto Ejecutivo, provisión de materiales, mano de obra, equipos, ejecución, ensayos, habilitación y puesta en servicio de la instalación de gas natural para la Planta Municipal de Elaboración de Mezcla Asfáltica en Caliente, ubicada en el Lote N.º 4 de la Chacra N.º 263 del Parque Industrial de Villaguay, Provincia de Entre Ríos. La contratación comprender á una solución integral bajo modalidad “llave en mano”, incluyendo todos los trabajos, provisiones, trámites, representaciones técnicas, insp</t>
+          <t>Provisión de una (1) camioneta usada destinada al Parque Automotor Municipal</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>16/10/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>16 de octubre del año 2026 a las 10:00 Horas, la que se reali zara en la Oficina de suministros de la Municipalidad de V</t>
+          <t>21 de octubre del año 2026 a las 10:00 Horas, la que se realizara en la Oficina de suministros de la Municipalidad de Vi</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>$ 50.000,00</t>
+          <t>$10.000,00</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr">
@@ -1834,14 +1834,14 @@
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>id-55f1e5ca423a9262</t>
+          <t>id-2d3dded56e6c6f6a</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>12/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1849,39 +1849,35 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>PARANA — SALUD ENTRE RÍOS S.A.U</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>CONCURSO DE PRECIOS</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>322/2026</t>
-        </is>
-      </c>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr"/>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>REPARACION DE MOTOR COMPLETO SEGUN DETALLES</t>
+          <t>Servicio de Recolección, Lavado, Desinfección, Secado, Planchado y Transporte de Ropa Hospitalaria</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>16/10/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026 08:15</t>
+          <t>Hospital de la Baxada, calle Gral. Alvarado Nº 2.250 Paraná, Entre Ríos, el día 21/10/2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1889,7 +1885,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K19" s="4" t="inlineStr"/>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
       <c r="L19" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1902,12 +1902,12 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>id-823d486904965498</t>
+          <t>id-6b955df9d3f6241a</t>
         </is>
       </c>
     </row>
@@ -1922,14 +1922,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>SALUD ENTRE RÍOS S.A.U</t>
+          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1937,20 +1937,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr"/>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>11/26</t>
+        </is>
+      </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Contratación de Servicio de Viandas para el Hospital de la Baxada</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “TERMINACION ESCUELA Nº 40 “JOSÉ ENRIQUE RODÓ”-SEPTIMO DISTRITO-DEPARTAMENTO GUALEGUAY.”</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>23/10/2026</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>Hospital de la Baxada, calle Gral. Al varado Nº 2.250 Paraná, Entre Ríos, el día 19/10/2026 a las 10:00 hs</t>
+          <t>DE LAS OFERTAS: el día 23 de Octubre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1960,7 +1964,7 @@
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>$ 100 (Cien)</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
@@ -1980,14 +1984,14 @@
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>id-d35d5e849089d7ac</t>
+          <t>id-86cc9c230734c462</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1995,14 +1999,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>VILLAGUAY — MUNICIPALIDAD DE VILLAGUAY</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2010,20 +2014,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr"/>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>11/2026</t>
+        </is>
+      </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Provisión de una (1) camioneta usada destinada al Parque Automotor Municipal</t>
+          <t>Terminación Escuela N° 40 "José Enrique Rodó", Séptimo Distrito</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>21/10/2026</t>
+          <t>23/10/2026</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>21 de octubre del año 2026 a las 10:00 Horas, la que se realizara en la Oficina de suministros de la Municipalidad de Vi</t>
+          <t>viernes, 23 de octubre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -2031,11 +2039,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K21" s="4" t="inlineStr">
-        <is>
-          <t>$10.000,00</t>
-        </is>
-      </c>
+      <c r="K21" s="4" t="inlineStr"/>
       <c r="L21" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2048,19 +2052,19 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-2d3dded56e6c6f6a</t>
+          <t>id-322a40f5e43af35d</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -2068,14 +2072,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>PARANA — SALUD ENTRE RÍOS S.A.U</t>
+          <t>COMUNA DE EL PALENQUE</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2083,20 +2087,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr"/>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>06/26</t>
+        </is>
+      </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Servicio de Recolección, Lavado, Desinfección, Secado, Planchado y Transporte de Ropa Hospitalaria</t>
+          <t>Adquisición de UNA (1) PALA CARGADORA 0 KM destinada a trabajos en la Comuna</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>21/10/2026</t>
+          <t>26/10/2026</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Hospital de la Baxada, calle Gral. Alvarado Nº 2.250 Paraná, Entre Ríos, el día 21/10/2026 a las 10:00 hs</t>
+          <t>26/10/2026, 12:30 horas, Lugar: Sede Administrativa de la Comuna de El Palenque, sito en calle San Martín sin número, El</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -2106,7 +2114,7 @@
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>pesos cero ($0,00)</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr">
@@ -2126,14 +2134,14 @@
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-6b955df9d3f6241a</t>
+          <t>id-4b7dfe1bdd0c2ac6</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -2141,14 +2149,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>COMUNA DE EL PALENQUE</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2158,22 +2166,22 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>11/26</t>
+          <t>07/26</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “TERMINACION ESCUELA Nº 40 “JOSÉ ENRIQUE RODÓ”-SEPTIMO DISTRITO-DEPARTAMENTO GUALEGUAY.”</t>
+          <t>Adquisición de UN (1) TRACTOR AGRÍCOLA 0 KM DE HASTA 90 HP, CABINADO 4 x4, CON PALA FRONTAL destinado a trabajos en la Comuna</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>23/10/2026</t>
+          <t>28/10/2026</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 23 de Octubre de 2026 a las 10:00 hs</t>
+          <t>28/10/2026, 12:40 horas, Lugar: Sede Administrativa de la Comuna de El Palenque, sito en calle San Martín sin número, El</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2183,7 +2191,7 @@
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t>$ 100 (Cien)</t>
+          <t>pesos cero ($ 0,00)</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr">
@@ -2203,14 +2211,14 @@
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-86cc9c230734c462</t>
+          <t>id-54e2b94544e5c76f</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>12/10/2026</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2218,14 +2226,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C24" s="8" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>VILLAGUAY — COMUNA DE MOJONES SUD YY PARAJE LOS ALGARROBOS</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2233,24 +2241,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>11/2026</t>
-        </is>
-      </c>
+      <c r="F24" s="4" t="inlineStr"/>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Terminación Escuela N° 40 "José Enrique Rodó", Séptimo Distrito</t>
+          <t>ADQUISICIÓN DE MOTONIVELADORA USADA</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>23/10/2026</t>
+          <t>29/10/2026</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>viernes, 23 de octubre de 2026 - 10:00hs</t>
+          <t>29/10/2026 a las 16:30 hs</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -2258,7 +2262,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K24" s="4" t="inlineStr"/>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>$ 10.000 (PESOS DIEZ MIL)</t>
+        </is>
+      </c>
       <c r="L24" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2271,24 +2279,24 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-322a40f5e43af35d</t>
+          <t>id-2aa97e0762afa9ea</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
@@ -2298,7 +2306,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>COMUNA DE EL PALENQUE</t>
+          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2308,22 +2316,18 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>06/26</t>
+          <t>002/26</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de UNA (1) PALA CARGADORA 0 KM destinada a trabajos en la Comuna</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>26/10/2026</t>
-        </is>
-      </c>
+          <t>ADQUISICIÓN de UN (1) TRACTOR 4 x4 C/CABINA DE 90 A 100 HP - 0 Km. con destino a Secretaria de Obras y Servicios Publicos</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr"/>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>26/10/2026, 12:30 horas, Lugar: Sede Administrativa de la Comuna de El Palenque, sito en calle San Martín sin número, El</t>
+          <t>DE LAS PROPUESTAS: 28 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2331,11 +2335,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K25" s="4" t="inlineStr">
-        <is>
-          <t>pesos cero ($0,00)</t>
-        </is>
-      </c>
+      <c r="K25" s="4" t="inlineStr"/>
       <c r="L25" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2353,29 +2353,29 @@
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-4b7dfe1bdd0c2ac6</t>
+          <t>id-da43a5f725393cbf</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>COMUNA DE EL PALENQUE</t>
+          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2385,22 +2385,18 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>07/26</t>
+          <t>07/2026</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de UN (1) TRACTOR AGRÍCOLA 0 KM DE HASTA 90 HP, CABINADO 4 x4, CON PALA FRONTAL destinado a trabajos en la Comuna</t>
-        </is>
-      </c>
-      <c r="H26" s="4" t="inlineStr">
-        <is>
-          <t>28/10/2026</t>
-        </is>
-      </c>
+          <t>Transporte de mil doscientos cincuenta metros cúbicos (1.250 m³) de broza grillada desde Cantera “Tayreta” (Ruta Nacional N° 14 km 135) hasta jurisdicción de la comuna, de acuerdo a los Pliegos de Bases, Condiciones Part iculares y demás documentación</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>28/10/2026, 12:40 horas, Lugar: Sede Administrativa de la Comuna de El Palenque, sito en calle San Martín sin número, El</t>
+          <t>Viernes 09 de octubre del corriente año a las 10:00 hs en la Oficina de la Sede de la Comuna</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2408,11 +2404,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K26" s="4" t="inlineStr">
-        <is>
-          <t>pesos cero ($ 0,00)</t>
-        </is>
-      </c>
+      <c r="K26" s="4" t="inlineStr"/>
       <c r="L26" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2430,29 +2422,29 @@
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-54e2b94544e5c76f</t>
+          <t>id-24e9015ecceeff7f</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>12/10/2026</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>VILLAGUAY — COMUNA DE MOJONES SUD YY PARAJE LOS ALGARROBOS</t>
+          <t>DIAMANTE — MUNICIPALIDAD DE DIAMANTE -- ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2463,17 +2455,13 @@
       <c r="F27" s="4" t="inlineStr"/>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN DE MOTONIVELADORA USADA</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="inlineStr">
-        <is>
-          <t>29/10/2026</t>
-        </is>
-      </c>
+          <t>Solicitar Contratación de una empresa para la Obra de “22 (veintidós) cuadras de pavimento urbano” – Grupo 1- según Expte. Letra “D” Nº 2196</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>29/10/2026 a las 16:30 hs</t>
+          <t>viernes 23 de octubre de 2.026, a la hora diez (10.00)</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2481,11 +2469,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K27" s="4" t="inlineStr">
-        <is>
-          <t>$ 10.000 (PESOS DIEZ MIL)</t>
-        </is>
-      </c>
+      <c r="K27" s="4" t="inlineStr"/>
       <c r="L27" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2503,14 +2487,14 @@
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-2aa97e0762afa9ea</t>
+          <t>id-4f207bef5c709ad6</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>12/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2518,35 +2502,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
+          <t>CONCORDIA — APEX S.A.S</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>002/26</t>
-        </is>
-      </c>
+          <t>Licitación</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr"/>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN de UN (1) TRACTOR 4 x4 C/CABINA DE 90 A 100 HP - 0 Km. con destino a Secretaria de Obras y Servicios Publicos</t>
+          <t>instalaciones eléctricas, sanitarias, hidráulicas, mecánicas o de cualquier otra naturaleza relacionada con el sector</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>DE LAS PROPUESTAS: 28 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2572,14 +2552,14 @@
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-da43a5f725393cbf</t>
+          <t>id-a20c6b2b6fcf36a2</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2587,35 +2567,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C29" s="10" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
+          <t>Boletín Oficial</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>07/2026</t>
-        </is>
-      </c>
+          <t>Remate</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr"/>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Transporte de mil doscientos cincuenta metros cúbicos (1.250 m³) de broza grillada desde Cantera “Tayreta” (Ruta Nacional N° 14 km 135) hasta jurisdicción de la comuna, de acuerdo a los Pliegos de Bases, Condiciones Part iculares y demás documentación</t>
+          <t>los vehículos se encuentran en exhibición por lo cuál la información registral, de rentas y de infracciones puede ser</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Viernes 09 de octubre del corriente año a las 10:00 hs en la Oficina de la Sede de la Comuna</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2641,14 +2617,14 @@
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-24e9015ecceeff7f</t>
+          <t>id-fb8d7dc09e202fea</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2656,14 +2632,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>DIAMANTE — MUNICIPALIDAD DE DIAMANTE -- ENTRE RÍOS</t>
+          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2671,16 +2647,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F30" s="4" t="inlineStr"/>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>001/26</t>
+        </is>
+      </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>Solicitar Contratación de una empresa para la Obra de “22 (veintidós) cuadras de pavimento urbano” – Grupo 1- según Expte. Letra “D” Nº 2196</t>
+          <t>ADQUISICIÓN de UN (1) FURGON UTILITARIO CHICO con 5 asientos 0 KM. con destino a Subsecretaria de Asistencia Directa y Emergencia</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>viernes 23 de octubre de 2.026, a la hora diez (10.00)</t>
+          <t>DE LAS PROPUESTAS: 20 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2706,14 +2686,14 @@
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-4f207bef5c709ad6</t>
+          <t>id-ca205f0874380f69</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2728,7 +2708,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>CONCORDIA — APEX S.A.S</t>
+          <t>INSTITUTO CARBÓ S.R.L</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2739,7 +2719,7 @@
       <c r="F31" s="4" t="inlineStr"/>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>instalaciones eléctricas, sanitarias, hidráulicas, mecánicas o de cualquier otra naturaleza relacionada con el sector</t>
+          <t>sin internación en materia de salud, pre- hospitalarias, atención médica, domiciliaria y traslados sanitarios de alta</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
@@ -2771,14 +2751,14 @@
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-a20c6b2b6fcf36a2</t>
+          <t>id-6aa57c7437a30ca3</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2786,25 +2766,29 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C32" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Boletín Oficial</t>
+          <t>MUNICIPALIDAD DE VIALE</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Remate</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>08/26</t>
+        </is>
+      </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>los vehículos se encuentran en exhibición por lo cuál la información registral, de rentas y de infracciones puede ser</t>
+          <t>de asf alto 70-16 destinado a la producción de pavimento de la Planta Asfáltica, y que a continuación se detalla y</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
@@ -2836,14 +2820,14 @@
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-fb8d7dc09e202fea</t>
+          <t>id-ef1ddb923c7e7fdb</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2851,14 +2835,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C33" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2868,18 +2852,18 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>001/26</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN de UN (1) FURGON UTILITARIO CHICO con 5 asientos 0 KM. con destino a Subsecretaria de Asistencia Directa y Emergencia</t>
+          <t>TERMINACIÓN CONCEPCIÓN DEL URUGUAY 63 VIV</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>DE LAS PROPUESTAS: 20 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
+          <t>Publicada 06/10/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2900,19 +2884,19 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-ca205f0874380f69</t>
+          <t>id-1a3c1f8e036ac91e</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2927,24 +2911,28 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>INSTITUTO CARBÓ S.R.L</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Licitación</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>sin internación en materia de salud, pre- hospitalarias, atención médica, domiciliaria y traslados sanitarios de alta</t>
+          <t>COMPLEJO HABITACIONAL SAN AGUSTÍN (P</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Publicada 05/10/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -2965,19 +2953,19 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-6aa57c7437a30ca3</t>
+          <t>id-ccb22bcad9356438</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2992,7 +2980,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE VIALE</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3002,18 +2990,18 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>08/26</t>
+          <t>03/26</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>de asf alto 70-16 destinado a la producción de pavimento de la Planta Asfáltica, y que a continuación se detalla y</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3034,19 +3022,19 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-ef1ddb923c7e7fdb</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3071,18 +3059,18 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN CONCEPCIÓN DEL URUGUAY 63 VIV</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2026 — ver pliego</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3108,14 +3096,14 @@
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>id-1a3c1f8e036ac91e</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3140,18 +3128,18 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>05/2026</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>COMPLEJO HABITACIONAL SAN AGUSTÍN (P</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/10/2026 — ver pliego</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3177,7 +3165,7 @@
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>id-ccb22bcad9356438</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
@@ -3209,18 +3197,18 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>03/26</t>
+          <t>05/2025</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -3246,7 +3234,7 @@
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
@@ -3278,18 +3266,18 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>02/2026</t>
+          <t>06/2025</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -3315,7 +3303,7 @@
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
@@ -3345,20 +3333,16 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F40" s="4" t="inlineStr">
-        <is>
-          <t>01/2026</t>
-        </is>
-      </c>
+      <c r="F40" s="4" t="inlineStr"/>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr"/>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
@@ -3384,7 +3368,7 @@
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
@@ -3416,18 +3400,18 @@
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>05/2025</t>
+          <t>04/2025</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
@@ -3453,7 +3437,7 @@
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
@@ -3485,18 +3469,18 @@
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>06/2025</t>
+          <t>03/2025</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr"/>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr">
@@ -3522,7 +3506,7 @@
       </c>
       <c r="O42" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
+          <t>id-75bfffae63b7eedc</t>
         </is>
       </c>
     </row>
@@ -3544,24 +3528,24 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Contratación Directa</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr"/>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+          <t>CONSTRUCCIÓN DE OBRAS DE ARTE EN EL DEPARTAMENTO LA PAZ. 1) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE EN R.P. S/Nº SOBRE Aº ESTACAS – “CAMINO SAUCECITO” – TRAMO: R.P.Nº 1 – ESCUELA Nº 62 – DISTRITO ESTACAS – DEPARTAMENTO LA PAZ – 2) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE SOBRE Aº ESTACAS SAN GUSTAVO – TRAMO: […]</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr"/>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr">
@@ -3582,19 +3566,19 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O43" s="4" t="inlineStr">
         <is>
-          <t>id-ebeeb6a87e688d85</t>
+          <t>id-3d7728874996f284</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -3602,35 +3586,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t>04/2025</t>
-        </is>
-      </c>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr"/>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr"/>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr">
@@ -3651,19 +3631,19 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O44" s="4" t="inlineStr">
         <is>
-          <t>id-34c85bcdb9b1123f</t>
+          <t>id-654eebef400f89cd</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -3678,28 +3658,28 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Concurso</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>03/2025</t>
+          <t>01/26</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr"/>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J45" s="4" t="inlineStr">
@@ -3720,19 +3700,19 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O45" s="4" t="inlineStr">
         <is>
-          <t>id-75bfffae63b7eedc</t>
+          <t>id-9a16884dd5a64a49</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3740,25 +3720,29 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C46" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="inlineStr"/>
+          <t>Licitación</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>2026-1227</t>
+        </is>
+      </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>CONSTRUCCIÓN DE OBRAS DE ARTE EN EL DEPARTAMENTO LA PAZ. 1) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE EN R.P. S/Nº SOBRE Aº ESTACAS – “CAMINO SAUCECITO” – TRAMO: R.P.Nº 1 – ESCUELA Nº 62 – DISTRITO ESTACAS – DEPARTAMENTO LA PAZ – 2) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE SOBRE Aº ESTACAS SAN GUSTAVO – TRAMO: […]</t>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
         </is>
       </c>
       <c r="H46" s="4" t="inlineStr"/>
@@ -3785,220 +3769,17 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="O46" s="4" t="inlineStr">
         <is>
-          <t>id-3d7728874996f284</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C47" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr"/>
-      <c r="G47" s="5" t="inlineStr">
-        <is>
-          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
-        </is>
-      </c>
-      <c r="H47" s="4" t="inlineStr"/>
-      <c r="I47" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J47" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K47" s="4" t="inlineStr"/>
-      <c r="L47" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M47" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
-        </is>
-      </c>
-      <c r="O47" s="4" t="inlineStr">
-        <is>
-          <t>id-654eebef400f89cd</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C48" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>Concurso</t>
-        </is>
-      </c>
-      <c r="F48" s="4" t="inlineStr">
-        <is>
-          <t>01/26</t>
-        </is>
-      </c>
-      <c r="G48" s="5" t="inlineStr">
-        <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
-        </is>
-      </c>
-      <c r="H48" s="4" t="inlineStr"/>
-      <c r="I48" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J48" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K48" s="4" t="inlineStr"/>
-      <c r="L48" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M48" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
-        </is>
-      </c>
-      <c r="O48" s="4" t="inlineStr">
-        <is>
-          <t>id-9a16884dd5a64a49</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C49" s="9" t="inlineStr">
-        <is>
-          <t>Materiales</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>ENERSA</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Licitación</t>
-        </is>
-      </c>
-      <c r="F49" s="4" t="inlineStr">
-        <is>
-          <t>2026-1227</t>
-        </is>
-      </c>
-      <c r="G49" s="5" t="inlineStr">
-        <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
-        </is>
-      </c>
-      <c r="H49" s="4" t="inlineStr"/>
-      <c r="I49" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J49" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K49" s="4" t="inlineStr"/>
-      <c r="L49" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M49" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N49" t="inlineStr">
-        <is>
-          <t>ENERSA</t>
-        </is>
-      </c>
-      <c r="O49" s="4" t="inlineStr">
-        <is>
           <t>id-0691eb485d7548eb</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O49"/>
+  <autoFilter ref="A1:O46"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -4090,12 +3871,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId88"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId89"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L47" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L48" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L49" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M49" r:id="rId96"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 14/10/2026 08:03
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$45</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O46"/>
+  <dimension ref="A1:O45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -741,7 +741,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE SANTA ELENA</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -751,12 +751,12 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>11/2026</t>
+          <t>87/2026</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>OBRA "PAVIMENTACION URBANA CALLE TRATADO DEL PILAR B° 3 DE FEBRERO - MUNICIPALIDAD DE SANTA ELENA" (Según Pliegos de Bases y condi ciones)</t>
+          <t>Contratar la ejecución de la obra denominada “Construcción de Red Cloacal Subsidiaria del Colector Noroeste Barrio Ciudad Paisaje”</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
@@ -766,7 +766,7 @@
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026 HORA: 10: 00 HS</t>
+          <t>martes, 13 de octubre de 2026 a las 10:00</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>$ 728.000,00 PESOS SETECIENTOS VEINTIOCHO MIL</t>
+          <t>$ 10.000 (pesos diez mil)</t>
         </is>
       </c>
       <c r="L4" s="6" t="inlineStr">
@@ -791,12 +791,12 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Boletín Oficial Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
-          <t>id-1a2561509308b1b6</t>
+          <t>id-ceeb594e8bcc4ff7</t>
         </is>
       </c>
     </row>
@@ -818,7 +818,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>COLON — MUNICIPALIDAD DE COLON</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -826,24 +826,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>87/2026</t>
-        </is>
-      </c>
+      <c r="F5" s="4" t="inlineStr"/>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Contratar la ejecución de la obra denominada “Construcción de Red Cloacal Subsidiaria del Colector Noroeste Barrio Ciudad Paisaje”</t>
+          <t>“ADQUISICIÓN DE MATERIALES ELÉCTRICOS PARA EJECUCIÓN DEL PROYECTO DE RECONVERSIÓN Y OPTIMIZACIÓN DEL ALUMBRADO PÚBLICO DE LA CIUDAD DE COLÓN”</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026</t>
+          <t>14/10/2026</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>martes, 13 de octubre de 2026 a las 10:00</t>
+          <t>14 de OCTUBRE de 2026</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -853,7 +849,7 @@
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>$ 10.000 (pesos diez mil)</t>
+          <t>Sin Cargo</t>
         </is>
       </c>
       <c r="L5" s="6" t="inlineStr">
@@ -868,12 +864,12 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Boletín Oficial Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>id-ceeb594e8bcc4ff7</t>
+          <t>id-9e122d52de12ffef</t>
         </is>
       </c>
     </row>
@@ -888,14 +884,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>COLON — MUNICIPALIDAD DE COLON</t>
+          <t>DIAMANTE — COMUNA ALDEA PROTESTANTE -- DIAMANTE -- ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -903,10 +899,14 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr"/>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>03/2026</t>
+        </is>
+      </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN DE MATERIALES ELÉCTRICOS PARA EJECUCIÓN DEL PROYECTO DE RECONVERSIÓN Y OPTIMIZACIÓN DEL ALUMBRADO PÚBLICO DE LA CIUDAD DE COLÓN”</t>
+          <t>Conforme a lo autorizado por decreto Nº 290/26 llámese a licitación pública Nº 03/26 con el objeto de comprar 10 toneladas de emulsión catiónica súper estable (asfalto de imprimación), puesto en Aldea Protestante</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>14 de OCTUBRE de 2026</t>
+          <t>miércoles 14 de octubre de 2026 – Hora nueve (09:00) Lugar de presentación de la oferta: Sede Comuna Aldea Protestan</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -924,11 +924,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t>Sin Cargo</t>
-        </is>
-      </c>
+      <c r="K6" s="4" t="inlineStr"/>
       <c r="L6" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -946,7 +942,7 @@
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>id-9e122d52de12ffef</t>
+          <t>id-c2f3a25cfb37fd38</t>
         </is>
       </c>
     </row>
@@ -961,14 +957,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>DIAMANTE — COMUNA ALDEA PROTESTANTE -- DIAMANTE -- ENTRE RÍOS</t>
+          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -978,12 +974,12 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>03/2026</t>
+          <t>017/2026</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Conforme a lo autorizado por decreto Nº 290/26 llámese a licitación pública Nº 03/26 con el objeto de comprar 10 toneladas de emulsión catiónica súper estable (asfalto de imprimación), puesto en Aldea Protestante</t>
+          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de UNA (1) MOTONIVELADORA, nueva, sin uso, cero km, con una potencia entre 220/240 HP, con opción a implementos, que será utilizada para el área del corralón municipal</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -993,7 +989,7 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>miércoles 14 de octubre de 2026 – Hora nueve (09:00) Lugar de presentación de la oferta: Sede Comuna Aldea Protestan</t>
+          <t>14 DE OCTUBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -1001,7 +997,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr"/>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>$100.000,00. - (PESOS CIEN MIL CON 00/100) PRESUPUESTO OFICIAL ESTIMAD</t>
+        </is>
+      </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1019,7 +1019,7 @@
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>id-c2f3a25cfb37fd38</t>
+          <t>id-4c3b33859e596759</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
+          <t>VICTORIA — MUNICIPALIDAD DE VICTORIA</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1051,12 +1051,12 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>017/2026</t>
+          <t>008/2026</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de UNA (1) MOTONIVELADORA, nueva, sin uso, cero km, con una potencia entre 220/240 HP, con opción a implementos, que será utilizada para el área del corralón municipal</t>
+          <t>Proveer a la Municipalidad de Victoria, Entre Ríos, de Veinticinco Mil (25.000) litros de Diésel 500, para movilidad de vehículos y maquinarias viales , Ocho Mil (8.000) litros de Gasoil Tipo euro o similar y Ocho (8.000) litros de nafta súper para vehículos y áreas afectadas a la Secretaria de Planeamiento y Dirección de Ambiente y Desarrollo sostenible;</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>14 DE OCTUBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>14 de octubre de 2026 a las 09:00 hs., en la Oficina de Compras de la Municipalidad de Victoria, Entr</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -1074,11 +1074,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr">
-        <is>
-          <t>$100.000,00. - (PESOS CIEN MIL CON 00/100) PRESUPUESTO OFICIAL ESTIMAD</t>
-        </is>
-      </c>
+      <c r="K8" s="4" t="inlineStr"/>
       <c r="L8" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1096,14 +1092,14 @@
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>id-4c3b33859e596759</t>
+          <t>id-a9af9f59c8c487c8</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1118,22 +1114,22 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>VICTORIA — MUNICIPALIDAD DE VICTORIA</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>LICITACIÓN PÚBLICA</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>008/2026</t>
+          <t>89/2026</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Proveer a la Municipalidad de Victoria, Entre Ríos, de Veinticinco Mil (25.000) litros de Diésel 500, para movilidad de vehículos y maquinarias viales , Ocho Mil (8.000) litros de Gasoil Tipo euro o similar y Ocho (8.000) litros de nafta súper para vehículos y áreas afectadas a la Secretaria de Planeamiento y Dirección de Ambiente y Desarrollo sostenible;</t>
+          <t>ADQUISICION DE BALANZA BASCULA PARA PESAJE DE EJESDE CAMIONES</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -1143,7 +1139,7 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>14 de octubre de 2026 a las 09:00 hs., en la Oficina de Compras de la Municipalidad de Victoria, Entr</t>
+          <t>14-10-2026 08:00</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1164,19 +1160,19 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>id-a9af9f59c8c487c8</t>
+          <t>id-4ee814ba6420f0cc</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>12/10/2026</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1196,17 +1192,17 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA</t>
+          <t>LICITACION PRIVADA</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>89/2026</t>
+          <t>77/2026</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICION DE BALANZA BASCULA PARA PESAJE DE EJESDE CAMIONES</t>
+          <t>SERVICIO DE ALQUILER DE RETROEXCAVADORA, MINICARGADORA, CAMION VOLCADOR Y PISON VIBRATORIO</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -1216,7 +1212,7 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>14-10-2026 08:00</t>
+          <t>14-10-2026 09:00</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1242,14 +1238,14 @@
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>id-4ee814ba6420f0cc</t>
+          <t>id-12335630ae6fd191</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>12/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1269,17 +1265,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>LICITACION PRIVADA</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>77/2026</t>
+          <t>89/2026</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE ALQUILER DE RETROEXCAVADORA, MINICARGADORA, CAMION VOLCADOR Y PISON VIBRATORIO</t>
+          <t>Adquisición de balanzas básculas para pesaje de ejes de camiones</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1289,7 +1285,7 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>14-10-2026 09:00</t>
+          <t>miércoles, 14 de octubre de 2026 a las 08:00</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1310,19 +1306,19 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>id-12335630ae6fd191</t>
+          <t>id-d963348e34fcb0d3</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1337,7 +1333,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE ALDEA SAN ANTONIO</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1347,22 +1343,22 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>89/2026</t>
+          <t>002/2026</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de balanzas básculas para pesaje de ejes de camiones</t>
+          <t>ADQUISICIÓN DE UNA MÁQUINA MOTONIVELADORA PARA INCORPORAR AL PARQUE AUTOMOTOR DE LA MUNICIPALIDAD DE ALDEA SAN ANTONIO</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>14/10/2026</t>
+          <t>15/10/2026</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 14 de octubre de 2026 a las 08:00</t>
+          <t>15 de octubre de 2026, a las 08:00 horas, en el Edificio Municipal</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
@@ -1370,7 +1366,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr"/>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>PESOS CIEN MIL con 00/100 ($ 100.000,00. -)</t>
+        </is>
+      </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1383,19 +1383,19 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Boletín Oficial Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>id-d963348e34fcb0d3</t>
+          <t>id-95a507b67b7b1450</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1403,14 +1403,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE ALDEA SAN ANTONIO</t>
+          <t>MINISTERIO DE SALUD — GOBIERNO DE ENTRE RIOS</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1420,22 +1420,22 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>002/2026</t>
+          <t>18/26</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN DE UNA MÁQUINA MOTONIVELADORA PARA INCORPORAR AL PARQUE AUTOMOTOR DE LA MUNICIPALIDAD DE ALDEA SAN ANTONIO</t>
+          <t>Adquirir Sesenta Mil (60.000) Kilogramos de Leche Entera en Polvo Instantánea, Fortificada con Hierro, Zinc y Ácido Ascórbico</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>15/10/2026</t>
+          <t>16/10/2026</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>15 de octubre de 2026, a las 08:00 horas, en el Edificio Municipal</t>
+          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>PESOS CIEN MIL con 00/100 ($ 100.000,00. -)</t>
+          <t>PESOS TRES MIL QUINIENTOS ($ 3.500,00)</t>
         </is>
       </c>
       <c r="L13" s="6" t="inlineStr">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>id-95a507b67b7b1450</t>
+          <t>id-04a917d50ccab2e3</t>
         </is>
       </c>
     </row>
@@ -1480,14 +1480,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>MINISTERIO DE SALUD — GOBIERNO DE ENTRE RIOS</t>
+          <t>VILLAGUAY — MUNICIPALIDAD DE VILLAGUAY</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1495,14 +1495,10 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>18/26</t>
-        </is>
-      </c>
+      <c r="F14" s="4" t="inlineStr"/>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Adquirir Sesenta Mil (60.000) Kilogramos de Leche Entera en Polvo Instantánea, Fortificada con Hierro, Zinc y Ácido Ascórbico</t>
+          <t>Contratación, ejecución, liquidación, pago y recepción de la obra destinada a la elaboración del Proyecto Ejecutivo, provisión de materiales, mano de obra, equipos, ejecución, ensayos, habilitación y puesta en servicio de la instalación de gas natural para la Planta Municipal de Elaboración de Mezcla Asfáltica en Caliente, ubicada en el Lote N.º 4 de la Chacra N.º 263 del Parque Industrial de Villaguay, Provincia de Entre Ríos. La contratación comprender á una solución integral bajo modalidad “llave en mano”, incluyendo todos los trabajos, provisiones, trámites, representaciones técnicas, insp</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -1512,7 +1508,7 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
+          <t>16 de octubre del año 2026 a las 10:00 Horas, la que se reali zara en la Oficina de suministros de la Municipalidad de V</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1522,7 +1518,7 @@
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
-          <t>PESOS TRES MIL QUINIENTOS ($ 3.500,00)</t>
+          <t>$ 50.000,00</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr">
@@ -1542,14 +1538,14 @@
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>id-04a917d50ccab2e3</t>
+          <t>id-55f1e5ca423a9262</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>12/10/2026</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1557,25 +1553,29 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>VILLAGUAY — MUNICIPALIDAD DE VILLAGUAY</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr"/>
+          <t>CONCURSO DE PRECIOS</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>322/2026</t>
+        </is>
+      </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Contratación, ejecución, liquidación, pago y recepción de la obra destinada a la elaboración del Proyecto Ejecutivo, provisión de materiales, mano de obra, equipos, ejecución, ensayos, habilitación y puesta en servicio de la instalación de gas natural para la Planta Municipal de Elaboración de Mezcla Asfáltica en Caliente, ubicada en el Lote N.º 4 de la Chacra N.º 263 del Parque Industrial de Villaguay, Provincia de Entre Ríos. La contratación comprender á una solución integral bajo modalidad “llave en mano”, incluyendo todos los trabajos, provisiones, trámites, representaciones técnicas, insp</t>
+          <t>REPARACION DE MOTOR COMPLETO SEGUN DETALLES</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
@@ -1585,7 +1585,7 @@
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>16 de octubre del año 2026 a las 10:00 Horas, la que se reali zara en la Oficina de suministros de la Municipalidad de V</t>
+          <t>16-10-2026 08:15</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1593,11 +1593,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K15" s="4" t="inlineStr">
-        <is>
-          <t>$ 50.000,00</t>
-        </is>
-      </c>
+      <c r="K15" s="4" t="inlineStr"/>
       <c r="L15" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1610,19 +1606,19 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>id-55f1e5ca423a9262</t>
+          <t>id-823d486904965498</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>12/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1630,39 +1626,35 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>SALUD ENTRE RÍOS S.A.U</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>CONCURSO DE PRECIOS</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>322/2026</t>
-        </is>
-      </c>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr"/>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>REPARACION DE MOTOR COMPLETO SEGUN DETALLES</t>
+          <t>Contratación de Servicio de Viandas para el Hospital de la Baxada</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>16/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026 08:15</t>
+          <t>Hospital de la Baxada, calle Gral. Al varado Nº 2.250 Paraná, Entre Ríos, el día 19/10/2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -1670,7 +1662,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K16" s="4" t="inlineStr"/>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
       <c r="L16" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1683,19 +1679,19 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>id-823d486904965498</t>
+          <t>id-d35d5e849089d7ac</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1703,14 +1699,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>SALUD ENTRE RÍOS S.A.U</t>
+          <t>VILLAGUAY — MUNICIPALIDAD DE VILLAGUAY</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1721,17 +1717,17 @@
       <c r="F17" s="4" t="inlineStr"/>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Contratación de Servicio de Viandas para el Hospital de la Baxada</t>
+          <t>Provisión de una (1) camioneta usada destinada al Parque Automotor Municipal</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>Hospital de la Baxada, calle Gral. Al varado Nº 2.250 Paraná, Entre Ríos, el día 19/10/2026 a las 10:00 hs</t>
+          <t>21 de octubre del año 2026 a las 10:00 Horas, la que se realizara en la Oficina de suministros de la Municipalidad de Vi</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1741,7 +1737,7 @@
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>$10.000,00</t>
         </is>
       </c>
       <c r="L17" s="6" t="inlineStr">
@@ -1761,14 +1757,14 @@
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>id-d35d5e849089d7ac</t>
+          <t>id-2d3dded56e6c6f6a</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1776,14 +1772,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>VILLAGUAY — MUNICIPALIDAD DE VILLAGUAY</t>
+          <t>PARANA — SALUD ENTRE RÍOS S.A.U</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1794,7 +1790,7 @@
       <c r="F18" s="4" t="inlineStr"/>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Provisión de una (1) camioneta usada destinada al Parque Automotor Municipal</t>
+          <t>Servicio de Recolección, Lavado, Desinfección, Secado, Planchado y Transporte de Ropa Hospitalaria</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
@@ -1804,7 +1800,7 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>21 de octubre del año 2026 a las 10:00 Horas, la que se realizara en la Oficina de suministros de la Municipalidad de Vi</t>
+          <t>Hospital de la Baxada, calle Gral. Alvarado Nº 2.250 Paraná, Entre Ríos, el día 21/10/2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1814,7 +1810,7 @@
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>$10.000,00</t>
+          <t>Ninguno</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr">
@@ -1834,7 +1830,7 @@
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>id-2d3dded56e6c6f6a</t>
+          <t>id-6b955df9d3f6241a</t>
         </is>
       </c>
     </row>
@@ -1849,14 +1845,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>PARANA — SALUD ENTRE RÍOS S.A.U</t>
+          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1864,20 +1860,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr"/>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>11/26</t>
+        </is>
+      </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Servicio de Recolección, Lavado, Desinfección, Secado, Planchado y Transporte de Ropa Hospitalaria</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “TERMINACION ESCUELA Nº 40 “JOSÉ ENRIQUE RODÓ”-SEPTIMO DISTRITO-DEPARTAMENTO GUALEGUAY.”</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>21/10/2026</t>
+          <t>23/10/2026</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>Hospital de la Baxada, calle Gral. Alvarado Nº 2.250 Paraná, Entre Ríos, el día 21/10/2026 a las 10:00 hs</t>
+          <t>DE LAS OFERTAS: el día 23 de Octubre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1887,7 +1887,7 @@
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>$ 100 (Cien)</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr">
@@ -1907,14 +1907,14 @@
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>id-6b955df9d3f6241a</t>
+          <t>id-86cc9c230734c462</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -1929,7 +1929,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1939,12 +1939,12 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>11/26</t>
+          <t>11/2026</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “TERMINACION ESCUELA Nº 40 “JOSÉ ENRIQUE RODÓ”-SEPTIMO DISTRITO-DEPARTAMENTO GUALEGUAY.”</t>
+          <t>Terminación Escuela N° 40 "José Enrique Rodó", Séptimo Distrito</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 23 de Octubre de 2026 a las 10:00 hs</t>
+          <t>viernes, 23 de octubre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1962,11 +1962,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K20" s="4" t="inlineStr">
-        <is>
-          <t>$ 100 (Cien)</t>
-        </is>
-      </c>
+      <c r="K20" s="4" t="inlineStr"/>
       <c r="L20" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1979,12 +1975,12 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>id-86cc9c230734c462</t>
+          <t>id-322a40f5e43af35d</t>
         </is>
       </c>
     </row>
@@ -1999,14 +1995,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>COMUNA DE EL PALENQUE</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2016,22 +2012,22 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>11/2026</t>
+          <t>06/26</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Terminación Escuela N° 40 "José Enrique Rodó", Séptimo Distrito</t>
+          <t>Adquisición de UNA (1) PALA CARGADORA 0 KM destinada a trabajos en la Comuna</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>23/10/2026</t>
+          <t>26/10/2026</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>viernes, 23 de octubre de 2026 - 10:00hs</t>
+          <t>26/10/2026, 12:30 horas, Lugar: Sede Administrativa de la Comuna de El Palenque, sito en calle San Martín sin número, El</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -2039,7 +2035,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K21" s="4" t="inlineStr"/>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>pesos cero ($0,00)</t>
+        </is>
+      </c>
       <c r="L21" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2052,19 +2052,19 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-322a40f5e43af35d</t>
+          <t>id-4b7dfe1bdd0c2ac6</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -2089,22 +2089,22 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>06/26</t>
+          <t>07/26</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de UNA (1) PALA CARGADORA 0 KM destinada a trabajos en la Comuna</t>
+          <t>Adquisición de UN (1) TRACTOR AGRÍCOLA 0 KM DE HASTA 90 HP, CABINADO 4 x4, CON PALA FRONTAL destinado a trabajos en la Comuna</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>26/10/2026</t>
+          <t>28/10/2026</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>26/10/2026, 12:30 horas, Lugar: Sede Administrativa de la Comuna de El Palenque, sito en calle San Martín sin número, El</t>
+          <t>28/10/2026, 12:40 horas, Lugar: Sede Administrativa de la Comuna de El Palenque, sito en calle San Martín sin número, El</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
-          <t>pesos cero ($0,00)</t>
+          <t>pesos cero ($ 0,00)</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr">
@@ -2134,14 +2134,14 @@
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-4b7dfe1bdd0c2ac6</t>
+          <t>id-54e2b94544e5c76f</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>12/10/2026</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -2156,7 +2156,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>COMUNA DE EL PALENQUE</t>
+          <t>VILLAGUAY — COMUNA DE MOJONES SUD YY PARAJE LOS ALGARROBOS</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2164,24 +2164,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>07/26</t>
-        </is>
-      </c>
+      <c r="F23" s="4" t="inlineStr"/>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de UN (1) TRACTOR AGRÍCOLA 0 KM DE HASTA 90 HP, CABINADO 4 x4, CON PALA FRONTAL destinado a trabajos en la Comuna</t>
+          <t>ADQUISICIÓN DE MOTONIVELADORA USADA</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>28/10/2026</t>
+          <t>29/10/2026</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>28/10/2026, 12:40 horas, Lugar: Sede Administrativa de la Comuna de El Palenque, sito en calle San Martín sin número, El</t>
+          <t>29/10/2026 a las 16:30 hs</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2191,7 +2187,7 @@
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t>pesos cero ($ 0,00)</t>
+          <t>$ 10.000 (PESOS DIEZ MIL)</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr">
@@ -2211,7 +2207,7 @@
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-54e2b94544e5c76f</t>
+          <t>id-2aa97e0762afa9ea</t>
         </is>
       </c>
     </row>
@@ -2221,9 +2217,9 @@
           <t>12/10/2026</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
@@ -2233,7 +2229,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>VILLAGUAY — COMUNA DE MOJONES SUD YY PARAJE LOS ALGARROBOS</t>
+          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2241,20 +2237,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr"/>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>002/26</t>
+        </is>
+      </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN DE MOTONIVELADORA USADA</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>29/10/2026</t>
-        </is>
-      </c>
+          <t>ADQUISICIÓN de UN (1) TRACTOR 4 x4 C/CABINA DE 90 A 100 HP - 0 Km. con destino a Secretaria de Obras y Servicios Publicos</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr"/>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>29/10/2026 a las 16:30 hs</t>
+          <t>DE LAS PROPUESTAS: 28 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -2262,11 +2258,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K24" s="4" t="inlineStr">
-        <is>
-          <t>$ 10.000 (PESOS DIEZ MIL)</t>
-        </is>
-      </c>
+      <c r="K24" s="4" t="inlineStr"/>
       <c r="L24" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2284,14 +2276,14 @@
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-2aa97e0762afa9ea</t>
+          <t>id-da43a5f725393cbf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2299,14 +2291,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
+          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2316,18 +2308,18 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>002/26</t>
+          <t>07/2026</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN de UN (1) TRACTOR 4 x4 C/CABINA DE 90 A 100 HP - 0 Km. con destino a Secretaria de Obras y Servicios Publicos</t>
+          <t>Transporte de mil doscientos cincuenta metros cúbicos (1.250 m³) de broza grillada desde Cantera “Tayreta” (Ruta Nacional N° 14 km 135) hasta jurisdicción de la comuna, de acuerdo a los Pliegos de Bases, Condiciones Part iculares y demás documentación</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr"/>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>DE LAS PROPUESTAS: 28 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
+          <t>Viernes 09 de octubre del corriente año a las 10:00 hs en la Oficina de la Sede de la Comuna</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2353,14 +2345,14 @@
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-da43a5f725393cbf</t>
+          <t>id-24e9015ecceeff7f</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2368,14 +2360,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C26" s="10" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
+          <t>DIAMANTE — MUNICIPALIDAD DE DIAMANTE -- ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2383,20 +2375,16 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>07/2026</t>
-        </is>
-      </c>
+      <c r="F26" s="4" t="inlineStr"/>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Transporte de mil doscientos cincuenta metros cúbicos (1.250 m³) de broza grillada desde Cantera “Tayreta” (Ruta Nacional N° 14 km 135) hasta jurisdicción de la comuna, de acuerdo a los Pliegos de Bases, Condiciones Part iculares y demás documentación</t>
+          <t>Solicitar Contratación de una empresa para la Obra de “22 (veintidós) cuadras de pavimento urbano” – Grupo 1- según Expte. Letra “D” Nº 2196</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>Viernes 09 de octubre del corriente año a las 10:00 hs en la Oficina de la Sede de la Comuna</t>
+          <t>viernes 23 de octubre de 2.026, a la hora diez (10.00)</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2422,14 +2410,14 @@
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-24e9015ecceeff7f</t>
+          <t>id-4f207bef5c709ad6</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2444,24 +2432,24 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>DIAMANTE — MUNICIPALIDAD DE DIAMANTE -- ENTRE RÍOS</t>
+          <t>CONCORDIA — APEX S.A.S</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr"/>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>Solicitar Contratación de una empresa para la Obra de “22 (veintidós) cuadras de pavimento urbano” – Grupo 1- según Expte. Letra “D” Nº 2196</t>
+          <t>instalaciones eléctricas, sanitarias, hidráulicas, mecánicas o de cualquier otra naturaleza relacionada con el sector</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>viernes 23 de octubre de 2.026, a la hora diez (10.00)</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -2487,7 +2475,7 @@
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-4f207bef5c709ad6</t>
+          <t>id-a20c6b2b6fcf36a2</t>
         </is>
       </c>
     </row>
@@ -2502,25 +2490,25 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>CONCORDIA — APEX S.A.S</t>
+          <t>Boletín Oficial</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Licitación</t>
+          <t>Remate</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr"/>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>instalaciones eléctricas, sanitarias, hidráulicas, mecánicas o de cualquier otra naturaleza relacionada con el sector</t>
+          <t>los vehículos se encuentran en exhibición por lo cuál la información registral, de rentas y de infracciones puede ser</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
@@ -2552,14 +2540,14 @@
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-a20c6b2b6fcf36a2</t>
+          <t>id-fb8d7dc09e202fea</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2574,24 +2562,28 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Boletín Oficial</t>
+          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Remate</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>001/26</t>
+        </is>
+      </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>los vehículos se encuentran en exhibición por lo cuál la información registral, de rentas y de infracciones puede ser</t>
+          <t>ADQUISICIÓN de UN (1) FURGON UTILITARIO CHICO con 5 asientos 0 KM. con destino a Subsecretaria de Asistencia Directa y Emergencia</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>DE LAS PROPUESTAS: 20 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2617,7 +2609,7 @@
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-fb8d7dc09e202fea</t>
+          <t>id-ca205f0874380f69</t>
         </is>
       </c>
     </row>
@@ -2632,35 +2624,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C30" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
+          <t>INSTITUTO CARBÓ S.R.L</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>001/26</t>
-        </is>
-      </c>
+          <t>Licitación</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr"/>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN de UN (1) FURGON UTILITARIO CHICO con 5 asientos 0 KM. con destino a Subsecretaria de Asistencia Directa y Emergencia</t>
+          <t>sin internación en materia de salud, pre- hospitalarias, atención médica, domiciliaria y traslados sanitarios de alta</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>DE LAS PROPUESTAS: 20 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2686,7 +2674,7 @@
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-ca205f0874380f69</t>
+          <t>id-6aa57c7437a30ca3</t>
         </is>
       </c>
     </row>
@@ -2708,18 +2696,22 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>INSTITUTO CARBÓ S.R.L</t>
+          <t>MUNICIPALIDAD DE VIALE</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Licitación</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>08/26</t>
+        </is>
+      </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>sin internación en materia de salud, pre- hospitalarias, atención médica, domiciliaria y traslados sanitarios de alta</t>
+          <t>de asf alto 70-16 destinado a la producción de pavimento de la Planta Asfáltica, y que a continuación se detalla y</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
@@ -2751,14 +2743,14 @@
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-6aa57c7437a30ca3</t>
+          <t>id-ef1ddb923c7e7fdb</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2773,7 +2765,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE VIALE</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -2783,18 +2775,18 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>08/26</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>de asf alto 70-16 destinado a la producción de pavimento de la Planta Asfáltica, y que a continuación se detalla y</t>
+          <t>TERMINACIÓN CONCEPCIÓN DEL URUGUAY 63 VIV</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Publicada 06/10/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2815,12 +2807,12 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-ef1ddb923c7e7fdb</t>
+          <t>id-1a3c1f8e036ac91e</t>
         </is>
       </c>
     </row>
@@ -2852,18 +2844,18 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>05/2026</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN CONCEPCIÓN DEL URUGUAY 63 VIV</t>
+          <t>COMPLEJO HABITACIONAL SAN AGUSTÍN (P</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2026 — ver pliego</t>
+          <t>Publicada 05/10/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2889,14 +2881,14 @@
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-1a3c1f8e036ac91e</t>
+          <t>id-ccb22bcad9356438</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2921,18 +2913,18 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>05/2026</t>
+          <t>03/26</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>COMPLEJO HABITACIONAL SAN AGUSTÍN (P</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/10/2026 — ver pliego</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -2958,7 +2950,7 @@
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-ccb22bcad9356438</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
@@ -2990,18 +2982,18 @@
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>03/26</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3027,7 +3019,7 @@
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
@@ -3059,18 +3051,18 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>02/2026</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3096,7 +3088,7 @@
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
@@ -3128,18 +3120,18 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>05/2025</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3165,7 +3157,7 @@
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
@@ -3197,18 +3189,18 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>05/2025</t>
+          <t>06/2025</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -3234,7 +3226,7 @@
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
@@ -3264,20 +3256,16 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F39" s="4" t="inlineStr">
-        <is>
-          <t>06/2025</t>
-        </is>
-      </c>
+      <c r="F39" s="4" t="inlineStr"/>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -3303,7 +3291,7 @@
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
@@ -3333,16 +3321,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F40" s="4" t="inlineStr"/>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>04/2025</t>
+        </is>
+      </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr"/>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
@@ -3368,7 +3360,7 @@
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
-          <t>id-ebeeb6a87e688d85</t>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
@@ -3400,18 +3392,18 @@
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>04/2025</t>
+          <t>03/2025</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
@@ -3437,7 +3429,7 @@
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
-          <t>id-34c85bcdb9b1123f</t>
+          <t>id-75bfffae63b7eedc</t>
         </is>
       </c>
     </row>
@@ -3459,28 +3451,24 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="inlineStr">
-        <is>
-          <t>03/2025</t>
-        </is>
-      </c>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr"/>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+          <t>CONSTRUCCIÓN DE OBRAS DE ARTE EN EL DEPARTAMENTO LA PAZ. 1) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE EN R.P. S/Nº SOBRE Aº ESTACAS – “CAMINO SAUCECITO” – TRAMO: R.P.Nº 1 – ESCUELA Nº 62 – DISTRITO ESTACAS – DEPARTAMENTO LA PAZ – 2) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE SOBRE Aº ESTACAS SAN GUSTAVO – TRAMO: […]</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr"/>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr">
@@ -3501,19 +3489,19 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O42" s="4" t="inlineStr">
         <is>
-          <t>id-75bfffae63b7eedc</t>
+          <t>id-3d7728874996f284</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -3521,9 +3509,9 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C43" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -3539,7 +3527,7 @@
       <c r="F43" s="4" t="inlineStr"/>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>CONSTRUCCIÓN DE OBRAS DE ARTE EN EL DEPARTAMENTO LA PAZ. 1) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE EN R.P. S/Nº SOBRE Aº ESTACAS – “CAMINO SAUCECITO” – TRAMO: R.P.Nº 1 – ESCUELA Nº 62 – DISTRITO ESTACAS – DEPARTAMENTO LA PAZ – 2) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE SOBRE Aº ESTACAS SAN GUSTAVO – TRAMO: […]</t>
+          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
         </is>
       </c>
       <c r="H43" s="4" t="inlineStr"/>
@@ -3571,7 +3559,7 @@
       </c>
       <c r="O43" s="4" t="inlineStr">
         <is>
-          <t>id-3d7728874996f284</t>
+          <t>id-654eebef400f89cd</t>
         </is>
       </c>
     </row>
@@ -3586,9 +3574,9 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C44" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -3598,13 +3586,17 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F44" s="4" t="inlineStr"/>
+          <t>Concurso</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>01/26</t>
+        </is>
+      </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr"/>
@@ -3636,7 +3628,7 @@
       </c>
       <c r="O44" s="4" t="inlineStr">
         <is>
-          <t>id-654eebef400f89cd</t>
+          <t>id-9a16884dd5a64a49</t>
         </is>
       </c>
     </row>
@@ -3651,29 +3643,29 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Concurso</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>01/26</t>
+          <t>2026-1227</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr"/>
@@ -3700,86 +3692,17 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="O45" s="4" t="inlineStr">
         <is>
-          <t>id-9a16884dd5a64a49</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>ENERSA</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Licitación</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="inlineStr">
-        <is>
-          <t>2026-1227</t>
-        </is>
-      </c>
-      <c r="G46" s="5" t="inlineStr">
-        <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
-        </is>
-      </c>
-      <c r="H46" s="4" t="inlineStr"/>
-      <c r="I46" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J46" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K46" s="4" t="inlineStr"/>
-      <c r="L46" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M46" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>ENERSA</t>
-        </is>
-      </c>
-      <c r="O46" s="4" t="inlineStr">
-        <is>
           <t>id-0691eb485d7548eb</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O46"/>
+  <autoFilter ref="A1:O45"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -3869,8 +3792,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId86"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId87"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId90"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Licitaciones desde la Mac (incluye Paraná) - 15/10/2026 08:05
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O45"/>
+  <dimension ref="A1:O41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -803,7 +803,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -811,25 +811,29 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>COLON — MUNICIPALIDAD DE COLON</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr"/>
+          <t>LICITACIÓN PÚBLICA</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>89/2026</t>
+        </is>
+      </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>“ADQUISICIÓN DE MATERIALES ELÉCTRICOS PARA EJECUCIÓN DEL PROYECTO DE RECONVERSIÓN Y OPTIMIZACIÓN DEL ALUMBRADO PÚBLICO DE LA CIUDAD DE COLÓN”</t>
+          <t>ADQUISICION DE BALANZA BASCULA PARA PESAJE DE EJESDE CAMIONES</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -839,7 +843,7 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>14 de OCTUBRE de 2026</t>
+          <t>14-10-2026 08:00</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -847,11 +851,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t>Sin Cargo</t>
-        </is>
-      </c>
+      <c r="K5" s="4" t="inlineStr"/>
       <c r="L5" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -864,19 +864,19 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>id-9e122d52de12ffef</t>
+          <t>id-4ee814ba6420f0cc</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>12/10/2026</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -884,29 +884,29 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>DIAMANTE — COMUNA ALDEA PROTESTANTE -- DIAMANTE -- ENTRE RÍOS</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>LICITACION PRIVADA</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>03/2026</t>
+          <t>77/2026</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Conforme a lo autorizado por decreto Nº 290/26 llámese a licitación pública Nº 03/26 con el objeto de comprar 10 toneladas de emulsión catiónica súper estable (asfalto de imprimación), puesto en Aldea Protestante</t>
+          <t>SERVICIO DE ALQUILER DE RETROEXCAVADORA, MINICARGADORA, CAMION VOLCADOR Y PISON VIBRATORIO</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>miércoles 14 de octubre de 2026 – Hora nueve (09:00) Lugar de presentación de la oferta: Sede Comuna Aldea Protestan</t>
+          <t>14-10-2026 09:00</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -937,19 +937,19 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>id-c2f3a25cfb37fd38</t>
+          <t>id-12335630ae6fd191</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -964,7 +964,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>FEDERACION — MUNICIPALIDAD DE CHAJARI</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -974,12 +974,12 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>017/2026</t>
+          <t>89/2026</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Llamar a LICITACION PUBLICA tendiente a la provisión de UNA (1) MOTONIVELADORA, nueva, sin uso, cero km, con una potencia entre 220/240 HP, con opción a implementos, que será utilizada para el área del corralón municipal</t>
+          <t>Adquisición de balanzas básculas para pesaje de ejes de camiones</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -989,7 +989,7 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>14 DE OCTUBRE DE 2026 - HORA: 10:00. (DIEZ)</t>
+          <t>miércoles, 14 de octubre de 2026 a las 08:00</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -997,11 +997,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr">
-        <is>
-          <t>$100.000,00. - (PESOS CIEN MIL CON 00/100) PRESUPUESTO OFICIAL ESTIMAD</t>
-        </is>
-      </c>
+      <c r="K7" s="4" t="inlineStr"/>
       <c r="L7" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1014,19 +1010,19 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Boletín Oficial Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>id-4c3b33859e596759</t>
+          <t>id-d963348e34fcb0d3</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1041,7 +1037,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>VICTORIA — MUNICIPALIDAD DE VICTORIA</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE ALDEA SAN ANTONIO</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1051,22 +1047,22 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>008/2026</t>
+          <t>002/2026</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Proveer a la Municipalidad de Victoria, Entre Ríos, de Veinticinco Mil (25.000) litros de Diésel 500, para movilidad de vehículos y maquinarias viales , Ocho Mil (8.000) litros de Gasoil Tipo euro o similar y Ocho (8.000) litros de nafta súper para vehículos y áreas afectadas a la Secretaria de Planeamiento y Dirección de Ambiente y Desarrollo sostenible;</t>
+          <t>ADQUISICIÓN DE UNA MÁQUINA MOTONIVELADORA PARA INCORPORAR AL PARQUE AUTOMOTOR DE LA MUNICIPALIDAD DE ALDEA SAN ANTONIO</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>14/10/2026</t>
+          <t>15/10/2026</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>14 de octubre de 2026 a las 09:00 hs., en la Oficina de Compras de la Municipalidad de Victoria, Entr</t>
+          <t>15 de octubre de 2026, a las 08:00 horas, en el Edificio Municipal</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -1074,7 +1070,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr"/>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>PESOS CIEN MIL con 00/100 ($ 100.000,00. -)</t>
+        </is>
+      </c>
       <c r="L8" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1092,14 +1092,14 @@
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>id-a9af9f59c8c487c8</t>
+          <t>id-95a507b67b7b1450</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1107,39 +1107,39 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>MINISTERIO DE SALUD — GOBIERNO DE ENTRE RIOS</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>89/2026</t>
+          <t>18/26</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICION DE BALANZA BASCULA PARA PESAJE DE EJESDE CAMIONES</t>
+          <t>Adquirir Sesenta Mil (60.000) Kilogramos de Leche Entera en Polvo Instantánea, Fortificada con Hierro, Zinc y Ácido Ascórbico</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>14/10/2026</t>
+          <t>16/10/2026</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>14-10-2026 08:00</t>
+          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1147,7 +1147,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr"/>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>PESOS TRES MIL QUINIENTOS ($ 3.500,00)</t>
+        </is>
+      </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1160,19 +1164,19 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>id-4ee814ba6420f0cc</t>
+          <t>id-04a917d50ccab2e3</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>12/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1180,39 +1184,35 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>VILLAGUAY — MUNICIPALIDAD DE VILLAGUAY</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>LICITACION PRIVADA</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>77/2026</t>
-        </is>
-      </c>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr"/>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE ALQUILER DE RETROEXCAVADORA, MINICARGADORA, CAMION VOLCADOR Y PISON VIBRATORIO</t>
+          <t>Contratación, ejecución, liquidación, pago y recepción de la obra destinada a la elaboración del Proyecto Ejecutivo, provisión de materiales, mano de obra, equipos, ejecución, ensayos, habilitación y puesta en servicio de la instalación de gas natural para la Planta Municipal de Elaboración de Mezcla Asfáltica en Caliente, ubicada en el Lote N.º 4 de la Chacra N.º 263 del Parque Industrial de Villaguay, Provincia de Entre Ríos. La contratación comprender á una solución integral bajo modalidad “llave en mano”, incluyendo todos los trabajos, provisiones, trámites, representaciones técnicas, insp</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>14/10/2026</t>
+          <t>16/10/2026</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>14-10-2026 09:00</t>
+          <t>16 de octubre del año 2026 a las 10:00 Horas, la que se reali zara en la Oficina de suministros de la Municipalidad de V</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1220,7 +1220,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr"/>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>$ 50.000,00</t>
+        </is>
+      </c>
       <c r="L10" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1233,19 +1237,19 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O10" s="4" t="inlineStr">
         <is>
-          <t>id-12335630ae6fd191</t>
+          <t>id-55f1e5ca423a9262</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>12/10/2026</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1253,9 +1257,9 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1265,27 +1269,27 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>CONCURSO DE PRECIOS</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>89/2026</t>
+          <t>322/2026</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de balanzas básculas para pesaje de ejes de camiones</t>
+          <t>REPARACION DE MOTOR COMPLETO SEGUN DETALLES</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>14/10/2026</t>
+          <t>16/10/2026</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 14 de octubre de 2026 a las 08:00</t>
+          <t>16-10-2026 08:15</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
@@ -1306,19 +1310,19 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Boletín Oficial Municipalidad de Paraná</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
-          <t>id-d963348e34fcb0d3</t>
+          <t>id-823d486904965498</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1326,14 +1330,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE ALDEA SAN ANTONIO</t>
+          <t>SALUD ENTRE RÍOS S.A.U</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1341,24 +1345,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>002/2026</t>
-        </is>
-      </c>
+      <c r="F12" s="4" t="inlineStr"/>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN DE UNA MÁQUINA MOTONIVELADORA PARA INCORPORAR AL PARQUE AUTOMOTOR DE LA MUNICIPALIDAD DE ALDEA SAN ANTONIO</t>
+          <t>Contratación de Servicio de Viandas para el Hospital de la Baxada</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>15/10/2026</t>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>15 de octubre de 2026, a las 08:00 horas, en el Edificio Municipal</t>
+          <t>Hospital de la Baxada, calle Gral. Al varado Nº 2.250 Paraná, Entre Ríos, el día 19/10/2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>PESOS CIEN MIL con 00/100 ($ 100.000,00. -)</t>
+          <t>Ninguno</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
@@ -1388,14 +1388,14 @@
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>id-95a507b67b7b1450</t>
+          <t>id-d35d5e849089d7ac</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1403,14 +1403,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>MINISTERIO DE SALUD — GOBIERNO DE ENTRE RIOS</t>
+          <t>VILLAGUAY — MUNICIPALIDAD DE VILLAGUAY</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1418,24 +1418,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>18/26</t>
-        </is>
-      </c>
+      <c r="F13" s="4" t="inlineStr"/>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Adquirir Sesenta Mil (60.000) Kilogramos de Leche Entera en Polvo Instantánea, Fortificada con Hierro, Zinc y Ácido Ascórbico</t>
+          <t>Provisión de una (1) camioneta usada destinada al Parque Automotor Municipal</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>16/10/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
+          <t>21 de octubre del año 2026 a las 10:00 Horas, la que se realizara en la Oficina de suministros de la Municipalidad de Vi</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
@@ -1445,7 +1441,7 @@
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>PESOS TRES MIL QUINIENTOS ($ 3.500,00)</t>
+          <t>$10.000,00</t>
         </is>
       </c>
       <c r="L13" s="6" t="inlineStr">
@@ -1465,7 +1461,7 @@
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
-          <t>id-04a917d50ccab2e3</t>
+          <t>id-2d3dded56e6c6f6a</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1483,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>VILLAGUAY — MUNICIPALIDAD DE VILLAGUAY</t>
+          <t>PARANA — SALUD ENTRE RÍOS S.A.U</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1498,17 +1494,17 @@
       <c r="F14" s="4" t="inlineStr"/>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Contratación, ejecución, liquidación, pago y recepción de la obra destinada a la elaboración del Proyecto Ejecutivo, provisión de materiales, mano de obra, equipos, ejecución, ensayos, habilitación y puesta en servicio de la instalación de gas natural para la Planta Municipal de Elaboración de Mezcla Asfáltica en Caliente, ubicada en el Lote N.º 4 de la Chacra N.º 263 del Parque Industrial de Villaguay, Provincia de Entre Ríos. La contratación comprender á una solución integral bajo modalidad “llave en mano”, incluyendo todos los trabajos, provisiones, trámites, representaciones técnicas, insp</t>
+          <t>Servicio de Recolección, Lavado, Desinfección, Secado, Planchado y Transporte de Ropa Hospitalaria</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>16/10/2026</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>16 de octubre del año 2026 a las 10:00 Horas, la que se reali zara en la Oficina de suministros de la Municipalidad de V</t>
+          <t>Hospital de la Baxada, calle Gral. Alvarado Nº 2.250 Paraná, Entre Ríos, el día 21/10/2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -1518,7 +1514,7 @@
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
-          <t>$ 50.000,00</t>
+          <t>Ninguno</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr">
@@ -1538,14 +1534,14 @@
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>id-55f1e5ca423a9262</t>
+          <t>id-6b955df9d3f6241a</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>12/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1560,32 +1556,32 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>CONCURSO DE PRECIOS</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>322/2026</t>
+          <t>11/26</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>REPARACION DE MOTOR COMPLETO SEGUN DETALLES</t>
+          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “TERMINACION ESCUELA Nº 40 “JOSÉ ENRIQUE RODÓ”-SEPTIMO DISTRITO-DEPARTAMENTO GUALEGUAY.”</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>16/10/2026</t>
+          <t>23/10/2026</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>16-10-2026 08:15</t>
+          <t>DE LAS OFERTAS: el día 23 de Octubre de 2026 a las 10:00 hs</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1593,7 +1589,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K15" s="4" t="inlineStr"/>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>$ 100 (Cien)</t>
+        </is>
+      </c>
       <c r="L15" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1606,19 +1606,19 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O15" s="4" t="inlineStr">
         <is>
-          <t>id-823d486904965498</t>
+          <t>id-86cc9c230734c462</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1626,14 +1626,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>SALUD ENTRE RÍOS S.A.U</t>
+          <t>Arquitectura y Construcciones (DGAyC)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1641,20 +1641,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr"/>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>11/2026</t>
+        </is>
+      </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Contratación de Servicio de Viandas para el Hospital de la Baxada</t>
+          <t>Terminación Escuela N° 40 "José Enrique Rodó", Séptimo Distrito</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>19/10/2026</t>
+          <t>23/10/2026</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Hospital de la Baxada, calle Gral. Al varado Nº 2.250 Paraná, Entre Ríos, el día 19/10/2026 a las 10:00 hs</t>
+          <t>viernes, 23 de octubre de 2026 - 10:00hs</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -1662,11 +1666,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K16" s="4" t="inlineStr">
-        <is>
-          <t>Ninguno</t>
-        </is>
-      </c>
+      <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1679,19 +1679,19 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Min. Planeamiento (provincia)</t>
         </is>
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>id-d35d5e849089d7ac</t>
+          <t>id-322a40f5e43af35d</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1706,7 +1706,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>VILLAGUAY — MUNICIPALIDAD DE VILLAGUAY</t>
+          <t>COMUNA DE EL PALENQUE</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1714,20 +1714,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr"/>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>06/26</t>
+        </is>
+      </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Provisión de una (1) camioneta usada destinada al Parque Automotor Municipal</t>
+          <t>Adquisición de UNA (1) PALA CARGADORA 0 KM destinada a trabajos en la Comuna</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>21/10/2026</t>
+          <t>26/10/2026</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>21 de octubre del año 2026 a las 10:00 Horas, la que se realizara en la Oficina de suministros de la Municipalidad de Vi</t>
+          <t>26/10/2026, 12:30 horas, Lugar: Sede Administrativa de la Comuna de El Palenque, sito en calle San Martín sin número, El</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
@@ -1737,7 +1741,7 @@
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t>$10.000,00</t>
+          <t>pesos cero ($0,00)</t>
         </is>
       </c>
       <c r="L17" s="6" t="inlineStr">
@@ -1757,14 +1761,14 @@
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
-          <t>id-2d3dded56e6c6f6a</t>
+          <t>id-4b7dfe1bdd0c2ac6</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>08/10/2026</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1772,14 +1776,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>PARANA — SALUD ENTRE RÍOS S.A.U</t>
+          <t>COMUNA DE EL PALENQUE</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1787,20 +1791,24 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr"/>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>07/26</t>
+        </is>
+      </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Servicio de Recolección, Lavado, Desinfección, Secado, Planchado y Transporte de Ropa Hospitalaria</t>
+          <t>Adquisición de UN (1) TRACTOR AGRÍCOLA 0 KM DE HASTA 90 HP, CABINADO 4 x4, CON PALA FRONTAL destinado a trabajos en la Comuna</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>21/10/2026</t>
+          <t>28/10/2026</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>Hospital de la Baxada, calle Gral. Alvarado Nº 2.250 Paraná, Entre Ríos, el día 21/10/2026 a las 10:00 hs</t>
+          <t>28/10/2026, 12:40 horas, Lugar: Sede Administrativa de la Comuna de El Palenque, sito en calle San Martín sin número, El</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -1810,7 +1818,7 @@
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>Ninguno</t>
+          <t>pesos cero ($ 0,00)</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr">
@@ -1830,14 +1838,14 @@
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>id-6b955df9d3f6241a</t>
+          <t>id-54e2b94544e5c76f</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>12/10/2026</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1845,14 +1853,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>PARANA — MINISTERIO DE PLANEAMIENTO EE INFRAESTRUCTURA</t>
+          <t>VILLAGUAY — COMUNA DE MOJONES SUD YY PARAJE LOS ALGARROBOS</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1860,24 +1868,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>11/26</t>
-        </is>
-      </c>
+      <c r="F19" s="4" t="inlineStr"/>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Provisión de Materiales y Mano de Obra según Pliego para la Obra: “TERMINACION ESCUELA Nº 40 “JOSÉ ENRIQUE RODÓ”-SEPTIMO DISTRITO-DEPARTAMENTO GUALEGUAY.”</t>
+          <t>ADQUISICIÓN DE MOTONIVELADORA USADA</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>23/10/2026</t>
+          <t>29/10/2026</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>DE LAS OFERTAS: el día 23 de Octubre de 2026 a las 10:00 hs</t>
+          <t>29/10/2026 a las 16:30 hs</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1887,7 +1891,7 @@
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>$ 100 (Cien)</t>
+          <t>$ 10.000 (PESOS DIEZ MIL)</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr">
@@ -1907,29 +1911,29 @@
       </c>
       <c r="O19" s="4" t="inlineStr">
         <is>
-          <t>id-86cc9c230734c462</t>
+          <t>id-2aa97e0762afa9ea</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C20" s="9" t="inlineStr">
-        <is>
-          <t>Arquitectura</t>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Arquitectura y Construcciones (DGAyC)</t>
+          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1939,22 +1943,18 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>11/2026</t>
+          <t>002/26</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Terminación Escuela N° 40 "José Enrique Rodó", Séptimo Distrito</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>23/10/2026</t>
-        </is>
-      </c>
+          <t>ADQUISICIÓN de UN (1) TRACTOR 4 x4 C/CABINA DE 90 A 100 HP - 0 Km. con destino a Secretaria de Obras y Servicios Publicos</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr"/>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>viernes, 23 de octubre de 2026 - 10:00hs</t>
+          <t>DE LAS PROPUESTAS: 28 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -1975,34 +1975,34 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Min. Planeamiento (provincia)</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>id-322a40f5e43af35d</t>
+          <t>id-da43a5f725393cbf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>Áridos</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>COMUNA DE EL PALENQUE</t>
+          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2012,22 +2012,18 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>06/26</t>
+          <t>07/2026</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de UNA (1) PALA CARGADORA 0 KM destinada a trabajos en la Comuna</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>26/10/2026</t>
-        </is>
-      </c>
+          <t>Transporte de mil doscientos cincuenta metros cúbicos (1.250 m³) de broza grillada desde Cantera “Tayreta” (Ruta Nacional N° 14 km 135) hasta jurisdicción de la comuna, de acuerdo a los Pliegos de Bases, Condiciones Part iculares y demás documentación</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr"/>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>26/10/2026, 12:30 horas, Lugar: Sede Administrativa de la Comuna de El Palenque, sito en calle San Martín sin número, El</t>
+          <t>Viernes 09 de octubre del corriente año a las 10:00 hs en la Oficina de la Sede de la Comuna</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
@@ -2035,11 +2031,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K21" s="4" t="inlineStr">
-        <is>
-          <t>pesos cero ($0,00)</t>
-        </is>
-      </c>
+      <c r="K21" s="4" t="inlineStr"/>
       <c r="L21" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2057,29 +2049,29 @@
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
-          <t>id-4b7dfe1bdd0c2ac6</t>
+          <t>id-24e9015ecceeff7f</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>COMUNA DE EL PALENQUE</t>
+          <t>DIAMANTE — MUNICIPALIDAD DE DIAMANTE -- ENTRE RÍOS</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2087,24 +2079,16 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>07/26</t>
-        </is>
-      </c>
+      <c r="F22" s="4" t="inlineStr"/>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de UN (1) TRACTOR AGRÍCOLA 0 KM DE HASTA 90 HP, CABINADO 4 x4, CON PALA FRONTAL destinado a trabajos en la Comuna</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr">
-        <is>
-          <t>28/10/2026</t>
-        </is>
-      </c>
+          <t>Solicitar Contratación de una empresa para la Obra de “22 (veintidós) cuadras de pavimento urbano” – Grupo 1- según Expte. Letra “D” Nº 2196</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr"/>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>28/10/2026, 12:40 horas, Lugar: Sede Administrativa de la Comuna de El Palenque, sito en calle San Martín sin número, El</t>
+          <t>viernes 23 de octubre de 2.026, a la hora diez (10.00)</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
@@ -2112,11 +2096,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K22" s="4" t="inlineStr">
-        <is>
-          <t>pesos cero ($ 0,00)</t>
-        </is>
-      </c>
+      <c r="K22" s="4" t="inlineStr"/>
       <c r="L22" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2134,50 +2114,46 @@
       </c>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>id-54e2b94544e5c76f</t>
+          <t>id-4f207bef5c709ad6</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>12/10/2026</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Vigente</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+          <t>07/10/2026</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Revisar fecha</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>VILLAGUAY — COMUNA DE MOJONES SUD YY PARAJE LOS ALGARROBOS</t>
+          <t>CONCORDIA — APEX S.A.S</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr"/>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN DE MOTONIVELADORA USADA</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t>29/10/2026</t>
-        </is>
-      </c>
+          <t>instalaciones eléctricas, sanitarias, hidráulicas, mecánicas o de cualquier otra naturaleza relacionada con el sector</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr"/>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>29/10/2026 a las 16:30 hs</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2185,11 +2161,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K23" s="4" t="inlineStr">
-        <is>
-          <t>$ 10.000 (PESOS DIEZ MIL)</t>
-        </is>
-      </c>
+      <c r="K23" s="4" t="inlineStr"/>
       <c r="L23" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -2207,14 +2179,14 @@
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>id-2aa97e0762afa9ea</t>
+          <t>id-a20c6b2b6fcf36a2</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2229,28 +2201,24 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
+          <t>Boletín Oficial</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>002/26</t>
-        </is>
-      </c>
+          <t>Remate</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr"/>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN de UN (1) TRACTOR 4 x4 C/CABINA DE 90 A 100 HP - 0 Km. con destino a Secretaria de Obras y Servicios Publicos</t>
+          <t>los vehículos se encuentran en exhibición por lo cuál la información registral, de rentas y de infracciones puede ser</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr"/>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>DE LAS PROPUESTAS: 28 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -2276,7 +2244,7 @@
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>id-da43a5f725393cbf</t>
+          <t>id-fb8d7dc09e202fea</t>
         </is>
       </c>
     </row>
@@ -2291,14 +2259,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C25" s="10" t="inlineStr">
-        <is>
-          <t>Áridos</t>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Vehículos</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>SAN SALVADOR — COMUNA COLONIA BAYLINA</t>
+          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2308,18 +2276,18 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>07/2026</t>
+          <t>001/26</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>Transporte de mil doscientos cincuenta metros cúbicos (1.250 m³) de broza grillada desde Cantera “Tayreta” (Ruta Nacional N° 14 km 135) hasta jurisdicción de la comuna, de acuerdo a los Pliegos de Bases, Condiciones Part iculares y demás documentación</t>
+          <t>ADQUISICIÓN de UN (1) FURGON UTILITARIO CHICO con 5 asientos 0 KM. con destino a Subsecretaria de Asistencia Directa y Emergencia</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr"/>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>Viernes 09 de octubre del corriente año a las 10:00 hs en la Oficina de la Sede de la Comuna</t>
+          <t>DE LAS PROPUESTAS: 20 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -2345,14 +2313,14 @@
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>id-24e9015ecceeff7f</t>
+          <t>id-ca205f0874380f69</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2367,24 +2335,24 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>DIAMANTE — MUNICIPALIDAD DE DIAMANTE -- ENTRE RÍOS</t>
+          <t>INSTITUTO CARBÓ S.R.L</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr"/>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Solicitar Contratación de una empresa para la Obra de “22 (veintidós) cuadras de pavimento urbano” – Grupo 1- según Expte. Letra “D” Nº 2196</t>
+          <t>sin internación en materia de salud, pre- hospitalarias, atención médica, domiciliaria y traslados sanitarios de alta</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>viernes 23 de octubre de 2.026, a la hora diez (10.00)</t>
+          <t>Ver boletín</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2410,14 +2378,14 @@
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>id-4f207bef5c709ad6</t>
+          <t>id-6aa57c7437a30ca3</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2432,18 +2400,22 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>CONCORDIA — APEX S.A.S</t>
+          <t>MUNICIPALIDAD DE VIALE</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Licitación</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>08/26</t>
+        </is>
+      </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>instalaciones eléctricas, sanitarias, hidráulicas, mecánicas o de cualquier otra naturaleza relacionada con el sector</t>
+          <t>de asf alto 70-16 destinado a la producción de pavimento de la Planta Asfáltica, y que a continuación se detalla y</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
@@ -2475,7 +2447,7 @@
       </c>
       <c r="O27" s="4" t="inlineStr">
         <is>
-          <t>id-a20c6b2b6fcf36a2</t>
+          <t>id-ef1ddb923c7e7fdb</t>
         </is>
       </c>
     </row>
@@ -2490,31 +2462,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Boletín Oficial</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Remate</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>04/2026</t>
+        </is>
+      </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>los vehículos se encuentran en exhibición por lo cuál la información registral, de rentas y de infracciones puede ser</t>
+          <t>TERMINACIÓN CONCEPCIÓN DEL URUGUAY 63 VIV</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Publicada 06/10/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2535,19 +2511,19 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>id-fb8d7dc09e202fea</t>
+          <t>id-1a3c1f8e036ac91e</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>07/10/2026</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2555,14 +2531,14 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>ISLAS DEL IBICUY — MUNICIPALIDAD DE VILLA PARANACITO</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2572,18 +2548,18 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>001/26</t>
+          <t>05/2026</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN de UN (1) FURGON UTILITARIO CHICO con 5 asientos 0 KM. con destino a Subsecretaria de Asistencia Directa y Emergencia</t>
+          <t>COMPLEJO HABITACIONAL SAN AGUSTÍN (P</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>DE LAS PROPUESTAS: 20 de Octubre de 2.026, a las 11:00 Hs. en el salón de reuniones sito en Av. Entre Rios 941 de la loc</t>
+          <t>Publicada 05/10/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2604,19 +2580,19 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O29" s="4" t="inlineStr">
         <is>
-          <t>id-ca205f0874380f69</t>
+          <t>id-ccb22bcad9356438</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2631,24 +2607,28 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>INSTITUTO CARBÓ S.R.L</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Licitación</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr"/>
+          <t>Licitación Pública</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>03/26</t>
+        </is>
+      </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>sin internación en materia de salud, pre- hospitalarias, atención médica, domiciliaria y traslados sanitarios de alta</t>
+          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Publicada 21/08/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
@@ -2669,19 +2649,19 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O30" s="4" t="inlineStr">
         <is>
-          <t>id-6aa57c7437a30ca3</t>
+          <t>id-2b877612500f72b1</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2696,7 +2676,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>MUNICIPALIDAD DE VIALE</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2706,18 +2686,18 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>08/26</t>
+          <t>02/2026</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>de asf alto 70-16 destinado a la producción de pavimento de la Planta Asfáltica, y que a continuación se detalla y</t>
+          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>Ver boletín</t>
+          <t>Publicada 09/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
@@ -2738,19 +2718,19 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O31" s="4" t="inlineStr">
         <is>
-          <t>id-ef1ddb923c7e7fdb</t>
+          <t>id-b8ac4ddaa39b00be</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2775,18 +2755,18 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>01/2026</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN CONCEPCIÓN DEL URUGUAY 63 VIV</t>
+          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Publicada 06/10/2026 — ver pliego</t>
+          <t>Publicada 05/06/2026 — ver pliego</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr">
@@ -2812,14 +2792,14 @@
       </c>
       <c r="O32" s="4" t="inlineStr">
         <is>
-          <t>id-1a3c1f8e036ac91e</t>
+          <t>id-d0b9714db86e5226</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>03/10/2026</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2844,18 +2824,18 @@
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>05/2026</t>
+          <t>05/2025</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>COMPLEJO HABITACIONAL SAN AGUSTÍN (P</t>
+          <t>NOGOYA 19 VIVIENDAS</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/10/2026 — ver pliego</t>
+          <t>Publicada 11/12/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2881,7 +2861,7 @@
       </c>
       <c r="O33" s="4" t="inlineStr">
         <is>
-          <t>id-ccb22bcad9356438</t>
+          <t>id-22811eab8859abaf</t>
         </is>
       </c>
     </row>
@@ -2913,18 +2893,18 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>03/26</t>
+          <t>06/2025</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN VILLA PARANECITO 50 VIVIENDAS - DEPARTAMENTO ISLAS DEL IBICUY</t>
+          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Publicada 21/08/2026 — ver pliego</t>
+          <t>Publicada 18/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr">
@@ -2950,7 +2930,7 @@
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>id-2b877612500f72b1</t>
+          <t>id-c019bf4a08989c09</t>
         </is>
       </c>
     </row>
@@ -2980,20 +2960,16 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F35" s="4" t="inlineStr">
-        <is>
-          <t>02/2026</t>
-        </is>
-      </c>
+      <c r="F35" s="4" t="inlineStr"/>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>HERRERA 18 VIVIENDAS - DEPARTAMENTO URUGUAY</t>
+          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>Publicada 09/06/2026 — ver pliego</t>
+          <t>Publicada 11/11/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -3019,7 +2995,7 @@
       </c>
       <c r="O35" s="4" t="inlineStr">
         <is>
-          <t>id-b8ac4ddaa39b00be</t>
+          <t>id-ebeeb6a87e688d85</t>
         </is>
       </c>
     </row>
@@ -3051,18 +3027,18 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>01/2026</t>
+          <t>04/2025</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>LARROQUE 18 VIVIENDAS - DEPARTAMENTO GUALEGUAYCHU</t>
+          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Publicada 05/06/2026 — ver pliego</t>
+          <t>Publicada 23/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr">
@@ -3088,7 +3064,7 @@
       </c>
       <c r="O36" s="4" t="inlineStr">
         <is>
-          <t>id-d0b9714db86e5226</t>
+          <t>id-34c85bcdb9b1123f</t>
         </is>
       </c>
     </row>
@@ -3120,18 +3096,18 @@
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>05/2025</t>
+          <t>03/2025</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>NOGOYA 19 VIVIENDAS</t>
+          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
         </is>
       </c>
       <c r="H37" s="4" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/12/2025 — ver pliego</t>
+          <t>Publicada 08/10/2025 — ver pliego</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -3157,7 +3133,7 @@
       </c>
       <c r="O37" s="4" t="inlineStr">
         <is>
-          <t>id-22811eab8859abaf</t>
+          <t>id-75bfffae63b7eedc</t>
         </is>
       </c>
     </row>
@@ -3179,28 +3155,24 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F38" s="4" t="inlineStr">
-        <is>
-          <t>06/2025</t>
-        </is>
-      </c>
+          <t>Contratación Directa</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr"/>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>SAN JAIME DE LA FRONTERA 15 VIVIENDAS</t>
+          <t>CONSTRUCCIÓN DE OBRAS DE ARTE EN EL DEPARTAMENTO LA PAZ. 1) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE EN R.P. S/Nº SOBRE Aº ESTACAS – “CAMINO SAUCECITO” – TRAMO: R.P.Nº 1 – ESCUELA Nº 62 – DISTRITO ESTACAS – DEPARTAMENTO LA PAZ – 2) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE SOBRE Aº ESTACAS SAN GUSTAVO – TRAMO: […]</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Publicada 18/11/2025 — ver pliego</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr">
@@ -3221,19 +3193,19 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>id-c019bf4a08989c09</t>
+          <t>id-3d7728874996f284</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3241,31 +3213,31 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Contratación Directa</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr"/>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>PARANÁ 2 VIVIENDAS - PROTOTIPO DUPLEX 2 DORMITORIOS</t>
+          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
         </is>
       </c>
       <c r="H39" s="4" t="inlineStr"/>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>Publicada 11/11/2025 — ver pliego</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -3286,19 +3258,19 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O39" s="4" t="inlineStr">
         <is>
-          <t>id-ebeeb6a87e688d85</t>
+          <t>id-654eebef400f89cd</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3313,28 +3285,28 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Concurso</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>04/2025</t>
+          <t>01/26</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>CHAJARI 10 VIVIENDAS - MAIPER (P</t>
+          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr"/>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>Publicada 23/10/2025 — ver pliego</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr">
@@ -3355,19 +3327,19 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>Vialidad Entre Ríos (DPV)</t>
         </is>
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
-          <t>id-34c85bcdb9b1123f</t>
+          <t>id-9a16884dd5a64a49</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>01/10/2026</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3375,35 +3347,35 @@
           <t>Revisar fecha</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>IAPV (Vivienda)</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>03/2025</t>
+          <t>2026-1227</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>TERMINACIÓN PARANÁ 30 VIVIENDAS - VICOER</t>
+          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
         </is>
       </c>
       <c r="H41" s="4" t="inlineStr"/>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Publicada 08/10/2025 — ver pliego</t>
+          <t>Ver pliego</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
@@ -3424,285 +3396,17 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>IAPV — Viviendas</t>
+          <t>ENERSA</t>
         </is>
       </c>
       <c r="O41" s="4" t="inlineStr">
         <is>
-          <t>id-75bfffae63b7eedc</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>03/10/2026</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="inlineStr"/>
-      <c r="G42" s="5" t="inlineStr">
-        <is>
-          <t>CONSTRUCCIÓN DE OBRAS DE ARTE EN EL DEPARTAMENTO LA PAZ. 1) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE EN R.P. S/Nº SOBRE Aº ESTACAS – “CAMINO SAUCECITO” – TRAMO: R.P.Nº 1 – ESCUELA Nº 62 – DISTRITO ESTACAS – DEPARTAMENTO LA PAZ – 2) OBRA: CONSTRUCCIÓN DE CALZADA SUMERGIBLE SOBRE Aº ESTACAS SAN GUSTAVO – TRAMO: […]</t>
-        </is>
-      </c>
-      <c r="H42" s="4" t="inlineStr"/>
-      <c r="I42" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J42" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K42" s="4" t="inlineStr"/>
-      <c r="L42" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M42" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
-        </is>
-      </c>
-      <c r="O42" s="4" t="inlineStr">
-        <is>
-          <t>id-3d7728874996f284</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C43" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Contratación Directa</t>
-        </is>
-      </c>
-      <c r="F43" s="4" t="inlineStr"/>
-      <c r="G43" s="5" t="inlineStr">
-        <is>
-          <t>REFUERZO DE SEÑALIZACIÓN VERTICAL EN ZONA TÚNEL SUBFLUVIAL – TRAMO: ACC. TÚNEL SUBFLUVIAL “RAÚL URANGA – CARLOS SILVESTRE BEGNIS” – AV. CIRCUNVALACIÓN JOSÉ HERNÁNDEZ – DISTRITO SAUCE – DEPARTAMENTO PARANÁ – ZONAL XIX PARANÁ. – CONSULTA DE PLIEGOS: www.dpver.gov.ar – despacho.licitaciones@vialidadentrerios.gob.ar APERTURA DE LAS OFERTAS: El Acto de Apertura de las propuestas se llevará […]</t>
-        </is>
-      </c>
-      <c r="H43" s="4" t="inlineStr"/>
-      <c r="I43" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J43" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K43" s="4" t="inlineStr"/>
-      <c r="L43" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M43" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N43" t="inlineStr">
-        <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
-        </is>
-      </c>
-      <c r="O43" s="4" t="inlineStr">
-        <is>
-          <t>id-654eebef400f89cd</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>Concurso</t>
-        </is>
-      </c>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t>01/26</t>
-        </is>
-      </c>
-      <c r="G44" s="5" t="inlineStr">
-        <is>
-          <t>PROYECTO EJECUTIVO DE LA OBRA: RUTA PROVINCIAL A08 – TRAMO: R.N. Nº12 – VILLA PARANACITO – CONSTRUCCIÓN DE CALZADA, RECONSTRUCCIÓN DE LA CALZADA EXISTENTE, VERIFICACIÓN, REPARACIÓN Y DISEÑO DE OBRAS DE ARTE -DEPARTAMENTO: ISLAS DEL IBICUY – PROVINCIA: ENTRE RÍOS – LONGITUD APROXIMADA DEL TRAMO: 20,685 km.- CONSULTA DE PLIEGOS: www.dpver.gov.ar – […]</t>
-        </is>
-      </c>
-      <c r="H44" s="4" t="inlineStr"/>
-      <c r="I44" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J44" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K44" s="4" t="inlineStr"/>
-      <c r="L44" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M44" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N44" t="inlineStr">
-        <is>
-          <t>Vialidad Entre Ríos (DPV)</t>
-        </is>
-      </c>
-      <c r="O44" s="4" t="inlineStr">
-        <is>
-          <t>id-9a16884dd5a64a49</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>01/10/2026</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Revisar fecha</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>ENERSA</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Licitación</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="inlineStr">
-        <is>
-          <t>2026-1227</t>
-        </is>
-      </c>
-      <c r="G45" s="5" t="inlineStr">
-        <is>
-          <t>Adquisición Postes de hormigón para líneas aéreas de energía eléctrica</t>
-        </is>
-      </c>
-      <c r="H45" s="4" t="inlineStr"/>
-      <c r="I45" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="J45" s="4" t="inlineStr">
-        <is>
-          <t>Ver pliego</t>
-        </is>
-      </c>
-      <c r="K45" s="4" t="inlineStr"/>
-      <c r="L45" s="6" t="inlineStr">
-        <is>
-          <t>ver licitación</t>
-        </is>
-      </c>
-      <c r="M45" s="6" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>ENERSA</t>
-        </is>
-      </c>
-      <c r="O45" s="4" t="inlineStr">
-        <is>
           <t>id-0691eb485d7548eb</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O45"/>
+  <autoFilter ref="A1:O41"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
@@ -3784,14 +3488,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M40" r:id="rId78"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId79"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M41" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M42" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L43" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M43" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId88"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Publicar el diagnóstico de fuentes (estaba congelado hace dos semanas)
El scraper genera diagnostico.csv en cada corrida, pero ni el workflow ni
correr.sh lo incluían en el commit: la hoja Fuentes mostraba el estado del
01/10/2026 aunque el sistema corriera todos los días. Por eso Min. Planeamiento
figuraba en ERROR con un timeout de ese día, cuando hace rato responde normal
(0,4s).

Incluye además el arreglo pendiente del Resumen:
- Los contadores salían como porcentaje ('3000%' por 30 descartadas): clear()
  no borra el formato de número.
- 'VIGENTES' mostraba sólo las no descartadas (4 de 24). Ahora se ven las dos
  cifras: el total vigente y las que siguen en carrera.
- La ventana de próximas aperturas pasa de 15 a 30 días.
</commit_message>
<xml_diff>
--- a/Licitaciones-Entre-Rios.xlsx
+++ b/Licitaciones-Entre-Rios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licitaciones" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Licitaciones'!$A$1:$O$32</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O41"/>
+  <dimension ref="A1:O32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -572,7 +572,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>15/10/2026</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -649,7 +649,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>08/10/2026</t>
+          <t>15/10/2026</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -657,14 +657,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>COLON — MUNICIPALIDAD DE VILLA ELISA (E.R.)</t>
+          <t>IAPV (Vivienda)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -674,22 +674,22 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>004/26</t>
+          <t>05/2026</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN DE UN (1) VEHÍCULO PARA TRANSPORTE DE PASAJEROS DE (5) CINCO PLAZAS 0 KM - MODELO/AÑO 2026, PARA LA MUNICIPALIDAD DE LA CIUDAD DE VILLA ELISA, ENTRE RÍOS</t>
+          <t>COMPLEJO HABITACIONAL SAN AGUSTÍN (P</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>12/11/2026</t>
+          <t>01/12/2026</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>12 de NOVIEMBRE de 2026 a la hora 10:00 en la Oficina de Compras de la Municipalidad de Villa Elisa, Entre Ríos</t>
+          <t>01/12/2026 (leído del aviso)</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -699,7 +699,7 @@
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">$ 20.000,00 (Pesos Veinte mil con 00/100) el que se puede adquirir en </t>
+          <t>$ 299.794,33</t>
         </is>
       </c>
       <c r="L3" s="6" t="inlineStr">
@@ -714,19 +714,19 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>IAPV — Viviendas</t>
         </is>
       </c>
       <c r="O3" s="4" t="inlineStr">
         <is>
-          <t>id-bb3703ff360c8c43</t>
+          <t>id-ccb22bcad9356438</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>15/10/2026</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -741,32 +741,32 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>MUNICIPALIDAD DE SANTA ANA</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>Licitación Publica</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>87/2026</t>
+          <t>06/2026</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Contratar la ejecución de la obra denominada “Construcción de Red Cloacal Subsidiaria del Colector Noroeste Barrio Ciudad Paisaje”</t>
+          <t>Provisión de mano de obra, materiales, maquinarias y herramientas para pavimento asfáltico en Santa Ana</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>13/10/2026</t>
+          <t>06/11/2026</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>martes, 13 de octubre de 2026 a las 10:00</t>
+          <t>Viernes 06 de Noviembre de 2026, 10 hs</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>$ 10.000 (pesos diez mil)</t>
+          <t>$ 150.000, 00.- (Pesos Ciento Cincuenta Mil)</t>
         </is>
       </c>
       <c r="L4" s="6" t="inlineStr">
@@ -791,19 +791,19 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Boletín Oficial Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
-          <t>id-ceeb594e8bcc4ff7</t>
+          <t>id-270211eda8d9288f</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>15/10/2026</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -818,32 +818,32 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>COLON — MUNICIPALIDAD DE VILLA ELISA (E.R.)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>LICITACIÓN PÚBLICA</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>89/2026</t>
+          <t>004/26</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICION DE BALANZA BASCULA PARA PESAJE DE EJESDE CAMIONES</t>
+          <t>ADQUISICIÓN DE UN (1) VEHÍCULO PARA TRANSPORTE DE PASAJEROS DE (5) CINCO PLAZAS 0 KM - MODELO/AÑO 2026, PARA LA MUNICIPALIDAD DE LA CIUDAD DE VILLA ELISA, ENTRE RÍOS</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>14/10/2026</t>
+          <t>12/11/2026</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>14-10-2026 08:00</t>
+          <t>12 de NOVIEMBRE de 2026 a la hora 10:00 en la Oficina de Compras de la Municipalidad de Villa Elisa, Entre Ríos</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
@@ -851,7 +851,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr"/>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">$ 20.000,00 (Pesos Veinte mil con 00/100) el que se puede adquirir en </t>
+        </is>
+      </c>
       <c r="L5" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -864,19 +868,19 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
-          <t>id-4ee814ba6420f0cc</t>
+          <t>id-bb3703ff360c8c43</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>12/10/2026</t>
+          <t>15/10/2026</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -891,32 +895,32 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>GUALEGUAYCHU — MUNICIPIO DE ALDEA SAN ANTONIO</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>LICITACION PRIVADA</t>
+          <t>Licitación Pública</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>77/2026</t>
+          <t>002/2026</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>SERVICIO DE ALQUILER DE RETROEXCAVADORA, MINICARGADORA, CAMION VOLCADOR Y PISON VIBRATORIO</t>
+          <t>ADQUISICIÓN DE UNA MÁQUINA MOTONIVELADORA PARA INCORPORAR AL PARQUE AUTOMOTOR DE LA MUNICIPALIDAD DE ALDEA SAN ANTONIO</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>14/10/2026</t>
+          <t>15/10/2026</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>14-10-2026 09:00</t>
+          <t>15 de octubre de 2026, a las 08:00 horas, en el Edificio Municipal</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -924,7 +928,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr"/>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>PESOS CIEN MIL con 00/100 ($ 100.000,00. -)</t>
+        </is>
+      </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -937,19 +945,19 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>id-12335630ae6fd191</t>
+          <t>id-95a507b67b7b1450</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>15/10/2026</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -957,14 +965,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Materiales</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Municipalidad de Paraná</t>
+          <t>MINISTERIO DE SALUD — GOBIERNO DE ENTRE RIOS</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -974,22 +982,22 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>89/2026</t>
+          <t>18/26</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Adquisición de balanzas básculas para pesaje de ejes de camiones</t>
+          <t>Adquirir Sesenta Mil (60.000) Kilogramos de Leche Entera en Polvo Instantánea, Fortificada con Hierro, Zinc y Ácido Ascórbico</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>14/10/2026</t>
+          <t>16/10/2026</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>miércoles, 14 de octubre de 2026 a las 08:00</t>
+          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -997,7 +1005,11 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr"/>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>PESOS TRES MIL QUINIENTOS ($ 3.500,00)</t>
+        </is>
+      </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1010,19 +1022,19 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Boletín Oficial Municipalidad de Paraná</t>
+          <t>Boletín Oficial de Entre Ríos</t>
         </is>
       </c>
       <c r="O7" s="4" t="inlineStr">
         <is>
-          <t>id-d963348e34fcb0d3</t>
+          <t>id-04a917d50ccab2e3</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>07/10/2026</t>
+          <t>15/10/2026</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -1030,14 +1042,14 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Vehículos</t>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Infraestructura</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>GUALEGUAYCHU — MUNICIPIO DE ALDEA SAN ANTONIO</t>
+          <t>VILLAGUAY — MUNICIPALIDAD DE VILLAGUAY</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1045,24 +1057,20 @@
           <t>Licitación Pública</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>002/2026</t>
-        </is>
-      </c>
+      <c r="F8" s="4" t="inlineStr"/>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>ADQUISICIÓN DE UNA MÁQUINA MOTONIVELADORA PARA INCORPORAR AL PARQUE AUTOMOTOR DE LA MUNICIPALIDAD DE ALDEA SAN ANTONIO</t>
+          <t>Contratación, ejecución, liquidación, pago y recepción de la obra destinada a la elaboración del Proyecto Ejecutivo, provisión de materiales, mano de obra, equipos, ejecución, ensayos, habilitación y puesta en servicio de la instalación de gas natural para la Planta Municipal de Elaboración de Mezcla Asfáltica en Caliente, ubicada en el Lote N.º 4 de la Chacra N.º 263 del Parque Industrial de Villaguay, Provincia de Entre Ríos. La contratación comprender á una solución integral bajo modalidad “llave en mano”, incluyendo todos los trabajos, provisiones, trámites, representaciones técnicas, insp</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>15/10/2026</t>
+          <t>16/10/2026</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>15 de octubre de 2026, a las 08:00 horas, en el Edificio Municipal</t>
+          <t>16 de octubre del año 2026 a las 10:00 Horas, la que se reali zara en la Oficina de suministros de la Municipalidad de V</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -1072,7 +1080,7 @@
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>PESOS CIEN MIL con 00/100 ($ 100.000,00. -)</t>
+          <t>$ 50.000,00</t>
         </is>
       </c>
       <c r="L8" s="6" t="inlineStr">
@@ -1092,14 +1100,14 @@
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
-          <t>id-95a507b67b7b1450</t>
+          <t>id-55f1e5ca423a9262</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>15/10/2026</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1107,29 +1115,29 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>Materiales</t>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>MINISTERIO DE SALUD — GOBIERNO DE ENTRE RIOS</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
+          <t>CONCURSO DE PRECIOS</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>18/26</t>
+          <t>322/2026</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Adquirir Sesenta Mil (60.000) Kilogramos de Leche Entera en Polvo Instantánea, Fortificada con Hierro, Zinc y Ácido Ascórbico</t>
+          <t>REPARACION DE MOTOR COMPLETO SEGUN DETALLES</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -1139,7 +1147,7 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>Sala de reuniones de la Dirección de Contrataciones del Ministerio de Salud, sito en calle 25 de Mayo N° 181, segundo pi</t>
+          <t>16-10-2026 08:15</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1147,11 +1155,7 @@
           <t>Ver pliego</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>PESOS TRES MIL QUINIENTOS ($ 3.500,00)</t>
-        </is>
-      </c>
+      <c r="K9" s="4" t="inlineStr"/>
       <c r="L9" s="6" t="inlineStr">
         <is>
           <t>ver licitación</t>
@@ -1164,19 +1168,19 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Boletín Oficial de Entre Ríos</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
-          <t>id-04a917d50ccab2e3</t>
+          <t>id-823d486904965498</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>01/10/2026</t>
+          <t>15/10/2026</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1184,25 +1188,29 @@
           <t>Vigente</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Infraestructura</t>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Arquitectura</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>VILLAGUAY — MUNICIPALIDAD DE VILLAGUAY</t>
+          <t>Municipalidad de Paraná</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Licitación Pública</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr"/>
+          <t>LICITACION PRIVADA</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>78/2026</t>
+        </is>
+      </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Contratación, ejecución, liquidación, pago y recepción de la obra destinada a la elaboración del Proyecto Ejecutivo, provisión de materi